<commit_message>
📊 Daily StockIQ Insights update (2026-01-12)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O81"/>
+  <dimension ref="A1:O101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5844,6 +5844,1266 @@
       <c r="O81" t="inlineStr">
         <is>
           <t>11 Jan 2026, 06:39:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>1475.3</v>
+      </c>
+      <c r="F82" t="n">
+        <v>1674.38</v>
+      </c>
+      <c r="G82" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="H82" t="n">
+        <v>1459.489990234375</v>
+      </c>
+      <c r="I82" t="n">
+        <v>-1.070000052452087</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K82" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N82" t="n">
+        <v>83.23999999999999</v>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>3207.8</v>
+      </c>
+      <c r="F83" t="n">
+        <v>3283.66</v>
+      </c>
+      <c r="G83" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="H83" t="n">
+        <v>3132.169921875</v>
+      </c>
+      <c r="I83" t="n">
+        <v>-2.359999895095825</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K83" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N83" t="n">
+        <v>62.35</v>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>1614.1</v>
+      </c>
+      <c r="F84" t="n">
+        <v>1648.35</v>
+      </c>
+      <c r="G84" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="H84" t="n">
+        <v>1647.010009765625</v>
+      </c>
+      <c r="I84" t="n">
+        <v>2.039999961853027</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K84" t="n">
+        <v>-0.273</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N84" t="n">
+        <v>47.72</v>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>939</v>
+      </c>
+      <c r="F85" t="n">
+        <v>921.97</v>
+      </c>
+      <c r="G85" t="n">
+        <v>-1.81</v>
+      </c>
+      <c r="H85" t="n">
+        <v>1113.430053710938</v>
+      </c>
+      <c r="I85" t="n">
+        <v>18.57999992370605</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K85" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N85" t="n">
+        <v>56.46</v>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>1404.3</v>
+      </c>
+      <c r="F86" t="n">
+        <v>1322.19</v>
+      </c>
+      <c r="G86" t="n">
+        <v>-5.85</v>
+      </c>
+      <c r="H86" t="n">
+        <v>1388.81005859375</v>
+      </c>
+      <c r="I86" t="n">
+        <v>-1.100000023841858</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K86" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N86" t="n">
+        <v>28.23</v>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>1000.5</v>
+      </c>
+      <c r="F87" t="n">
+        <v>977.95</v>
+      </c>
+      <c r="G87" t="n">
+        <v>-2.25</v>
+      </c>
+      <c r="H87" t="n">
+        <v>851.6900024414062</v>
+      </c>
+      <c r="I87" t="n">
+        <v>-14.86999988555908</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K87" t="n">
+        <v>-0.572</v>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N87" t="n">
+        <v>35.18</v>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>2372.6</v>
+      </c>
+      <c r="F88" t="n">
+        <v>2321.5</v>
+      </c>
+      <c r="G88" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="H88" t="n">
+        <v>2461.5400390625</v>
+      </c>
+      <c r="I88" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K88" t="n">
+        <v>0.681</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N88" t="n">
+        <v>60.39</v>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>337.15</v>
+      </c>
+      <c r="F89" t="n">
+        <v>376.52</v>
+      </c>
+      <c r="G89" t="n">
+        <v>11.68</v>
+      </c>
+      <c r="H89" t="n">
+        <v>379.1700134277344</v>
+      </c>
+      <c r="I89" t="n">
+        <v>12.46000003814697</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K89" t="n">
+        <v>0.751</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N89" t="n">
+        <v>82.54000000000001</v>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>4025.2</v>
+      </c>
+      <c r="F90" t="n">
+        <v>3956.72</v>
+      </c>
+      <c r="G90" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="H90" t="n">
+        <v>4316.5</v>
+      </c>
+      <c r="I90" t="n">
+        <v>7.239999771118164</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K90" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N90" t="n">
+        <v>54.25</v>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>959.6</v>
+      </c>
+      <c r="F91" t="n">
+        <v>1024.94</v>
+      </c>
+      <c r="G91" t="n">
+        <v>6.81</v>
+      </c>
+      <c r="H91" t="n">
+        <v>897.5499877929688</v>
+      </c>
+      <c r="I91" t="n">
+        <v>-6.46999979019165</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N91" t="n">
+        <v>60.21</v>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>2027.1</v>
+      </c>
+      <c r="F92" t="n">
+        <v>2217.28</v>
+      </c>
+      <c r="G92" t="n">
+        <v>9.380000000000001</v>
+      </c>
+      <c r="H92" t="n">
+        <v>2067.449951171875</v>
+      </c>
+      <c r="I92" t="n">
+        <v>1.990000009536743</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K92" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N92" t="n">
+        <v>76.56999999999999</v>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>2825.5</v>
+      </c>
+      <c r="F93" t="n">
+        <v>2758.41</v>
+      </c>
+      <c r="G93" t="n">
+        <v>-2.37</v>
+      </c>
+      <c r="H93" t="n">
+        <v>2792.489990234375</v>
+      </c>
+      <c r="I93" t="n">
+        <v>-1.169999957084656</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K93" t="n">
+        <v>0.8129999999999999</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N93" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>1272</v>
+      </c>
+      <c r="F94" t="n">
+        <v>1200.92</v>
+      </c>
+      <c r="G94" t="n">
+        <v>-5.59</v>
+      </c>
+      <c r="H94" t="n">
+        <v>1146.839965820312</v>
+      </c>
+      <c r="I94" t="n">
+        <v>-9.840000152587891</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K94" t="n">
+        <v>0.852</v>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N94" t="n">
+        <v>58.66</v>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>16501</v>
+      </c>
+      <c r="F95" t="n">
+        <v>18406.29</v>
+      </c>
+      <c r="G95" t="n">
+        <v>11.55</v>
+      </c>
+      <c r="H95" t="n">
+        <v>17159.16015625</v>
+      </c>
+      <c r="I95" t="n">
+        <v>3.990000009536743</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K95" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N95" t="n">
+        <v>80.31999999999999</v>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>1729.9</v>
+      </c>
+      <c r="F96" t="n">
+        <v>1821.69</v>
+      </c>
+      <c r="G96" t="n">
+        <v>5.31</v>
+      </c>
+      <c r="H96" t="n">
+        <v>1906.4599609375</v>
+      </c>
+      <c r="I96" t="n">
+        <v>10.21000003814697</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K96" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N96" t="n">
+        <v>70.95999999999999</v>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>261.95</v>
+      </c>
+      <c r="F97" t="n">
+        <v>280.01</v>
+      </c>
+      <c r="G97" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="H97" t="n">
+        <v>304.3999938964844</v>
+      </c>
+      <c r="I97" t="n">
+        <v>16.20000076293945</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K97" t="n">
+        <v>-0.361</v>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N97" t="n">
+        <v>53.12</v>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>11937</v>
+      </c>
+      <c r="F98" t="n">
+        <v>11560.26</v>
+      </c>
+      <c r="G98" t="n">
+        <v>-3.16</v>
+      </c>
+      <c r="H98" t="n">
+        <v>12397.1796875</v>
+      </c>
+      <c r="I98" t="n">
+        <v>3.859999895095825</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K98" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N98" t="n">
+        <v>58.27</v>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>336</v>
+      </c>
+      <c r="F99" t="n">
+        <v>327.14</v>
+      </c>
+      <c r="G99" t="n">
+        <v>-2.64</v>
+      </c>
+      <c r="H99" t="n">
+        <v>310.1900024414062</v>
+      </c>
+      <c r="I99" t="n">
+        <v>-7.679999828338623</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K99" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N99" t="n">
+        <v>59.05</v>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>258</v>
+      </c>
+      <c r="F100" t="n">
+        <v>256.24</v>
+      </c>
+      <c r="G100" t="n">
+        <v>-0.68</v>
+      </c>
+      <c r="H100" t="n">
+        <v>267.9400024414062</v>
+      </c>
+      <c r="I100" t="n">
+        <v>3.849999904632568</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K100" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N100" t="n">
+        <v>61.98</v>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>4201.8</v>
+      </c>
+      <c r="F101" t="n">
+        <v>4110.33</v>
+      </c>
+      <c r="G101" t="n">
+        <v>-2.18</v>
+      </c>
+      <c r="H101" t="n">
+        <v>4174.60986328125</v>
+      </c>
+      <c r="I101" t="n">
+        <v>-0.6499999761581421</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K101" t="n">
+        <v>0.765</v>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N101" t="n">
+        <v>62.03</v>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
         </is>
       </c>
     </row>
@@ -5858,7 +7118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8595,6 +9855,636 @@
       <c r="O41" t="inlineStr">
         <is>
           <t>11 Jan 2026, 06:39:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1475.3</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1683.66</v>
+      </c>
+      <c r="G42" t="n">
+        <v>14.12</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1289.329956054688</v>
+      </c>
+      <c r="I42" t="n">
+        <v>-12.60999965667725</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K42" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N42" t="n">
+        <v>84.18000000000001</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>3208</v>
+      </c>
+      <c r="F43" t="n">
+        <v>3262.9</v>
+      </c>
+      <c r="G43" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="H43" t="n">
+        <v>3156.110107421875</v>
+      </c>
+      <c r="I43" t="n">
+        <v>-1.620000004768372</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K43" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N43" t="n">
+        <v>61.37</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1614.75</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1667.62</v>
+      </c>
+      <c r="G44" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="H44" t="n">
+        <v>1669.219970703125</v>
+      </c>
+      <c r="I44" t="n">
+        <v>3.369999885559082</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
+        <v>-0.273</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N44" t="n">
+        <v>49.45</v>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>938.7</v>
+      </c>
+      <c r="F45" t="n">
+        <v>925.67</v>
+      </c>
+      <c r="G45" t="n">
+        <v>-1.39</v>
+      </c>
+      <c r="H45" t="n">
+        <v>937.6300048828125</v>
+      </c>
+      <c r="I45" t="n">
+        <v>-0.1099999994039536</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K45" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1403.55</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1328.8</v>
+      </c>
+      <c r="G46" t="n">
+        <v>-5.33</v>
+      </c>
+      <c r="H46" t="n">
+        <v>1419.160034179688</v>
+      </c>
+      <c r="I46" t="n">
+        <v>1.110000014305115</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K46" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F47" t="n">
+        <v>982.72</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-1.73</v>
+      </c>
+      <c r="H47" t="n">
+        <v>821.22998046875</v>
+      </c>
+      <c r="I47" t="n">
+        <v>-17.8799991607666</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K47" t="n">
+        <v>-0.572</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N47" t="n">
+        <v>35.97</v>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>337.1</v>
+      </c>
+      <c r="F48" t="n">
+        <v>370.84</v>
+      </c>
+      <c r="G48" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="H48" t="n">
+        <v>379.3699951171875</v>
+      </c>
+      <c r="I48" t="n">
+        <v>12.53999996185303</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K48" t="n">
+        <v>0.751</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N48" t="n">
+        <v>80.03</v>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>4026.75</v>
+      </c>
+      <c r="F49" t="n">
+        <v>3963.48</v>
+      </c>
+      <c r="G49" t="n">
+        <v>-1.57</v>
+      </c>
+      <c r="H49" t="n">
+        <v>3734.35009765625</v>
+      </c>
+      <c r="I49" t="n">
+        <v>-7.260000228881836</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N49" t="n">
+        <v>54.44</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>1271.95</v>
+      </c>
+      <c r="F50" t="n">
+        <v>1212.34</v>
+      </c>
+      <c r="G50" t="n">
+        <v>-4.69</v>
+      </c>
+      <c r="H50" t="n">
+        <v>1067.52001953125</v>
+      </c>
+      <c r="I50" t="n">
+        <v>-16.06999969482422</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K50" t="n">
+        <v>0.852</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N50" t="n">
+        <v>60.01</v>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>16501</v>
+      </c>
+      <c r="F51" t="n">
+        <v>18546.53</v>
+      </c>
+      <c r="G51" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="H51" t="n">
+        <v>16628.349609375</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0.7699999809265137</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K51" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N51" t="n">
+        <v>81.59</v>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
         </is>
       </c>
     </row>
@@ -8609,7 +10499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O81"/>
+  <dimension ref="A1:O101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14009,6 +15899,1266 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>259.37</v>
+      </c>
+      <c r="F82" t="n">
+        <v>286.91</v>
+      </c>
+      <c r="G82" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="H82" t="n">
+        <v>243.1199951171875</v>
+      </c>
+      <c r="I82" t="n">
+        <v>-6.260000228881836</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K82" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N82" t="n">
+        <v>77.64</v>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>479.28</v>
+      </c>
+      <c r="F83" t="n">
+        <v>478.9</v>
+      </c>
+      <c r="G83" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="H83" t="n">
+        <v>439.4100036621094</v>
+      </c>
+      <c r="I83" t="n">
+        <v>-8.319999694824219</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K83" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N83" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>328.57</v>
+      </c>
+      <c r="F84" t="n">
+        <v>358.55</v>
+      </c>
+      <c r="G84" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="H84" t="n">
+        <v>317.1499938964844</v>
+      </c>
+      <c r="I84" t="n">
+        <v>-3.480000019073486</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K84" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N84" t="n">
+        <v>77.51000000000001</v>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>247.38</v>
+      </c>
+      <c r="F85" t="n">
+        <v>251.23</v>
+      </c>
+      <c r="G85" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="H85" t="n">
+        <v>239.7700042724609</v>
+      </c>
+      <c r="I85" t="n">
+        <v>-3.079999923706055</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K85" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N85" t="n">
+        <v>62.55</v>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>653.0599999999999</v>
+      </c>
+      <c r="F86" t="n">
+        <v>719.26</v>
+      </c>
+      <c r="G86" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="H86" t="n">
+        <v>802.4600219726562</v>
+      </c>
+      <c r="I86" t="n">
+        <v>22.8799991607666</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K86" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N86" t="n">
+        <v>78.61</v>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>445.01</v>
+      </c>
+      <c r="F87" t="n">
+        <v>452.26</v>
+      </c>
+      <c r="G87" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="H87" t="n">
+        <v>506.4700012207031</v>
+      </c>
+      <c r="I87" t="n">
+        <v>13.8100004196167</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K87" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N87" t="n">
+        <v>59.24</v>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>184.86</v>
+      </c>
+      <c r="F88" t="n">
+        <v>200.37</v>
+      </c>
+      <c r="G88" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="H88" t="n">
+        <v>164.7899932861328</v>
+      </c>
+      <c r="I88" t="n">
+        <v>-10.85999965667725</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K88" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N88" t="n">
+        <v>75.78</v>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>329.19</v>
+      </c>
+      <c r="F89" t="n">
+        <v>343.86</v>
+      </c>
+      <c r="G89" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="H89" t="n">
+        <v>340.7799987792969</v>
+      </c>
+      <c r="I89" t="n">
+        <v>3.519999980926514</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K89" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N89" t="n">
+        <v>66.91</v>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>349.77</v>
+      </c>
+      <c r="F90" t="n">
+        <v>358.48</v>
+      </c>
+      <c r="G90" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="H90" t="n">
+        <v>364.4299926757812</v>
+      </c>
+      <c r="I90" t="n">
+        <v>4.190000057220459</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K90" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N90" t="n">
+        <v>63.61</v>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>204.39</v>
+      </c>
+      <c r="F91" t="n">
+        <v>219.29</v>
+      </c>
+      <c r="G91" t="n">
+        <v>7.29</v>
+      </c>
+      <c r="H91" t="n">
+        <v>227.0800018310547</v>
+      </c>
+      <c r="I91" t="n">
+        <v>11.10000038146973</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K91" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N91" t="n">
+        <v>68.56999999999999</v>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>114.53</v>
+      </c>
+      <c r="F92" t="n">
+        <v>117.82</v>
+      </c>
+      <c r="G92" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="H92" t="n">
+        <v>111.3300018310547</v>
+      </c>
+      <c r="I92" t="n">
+        <v>-2.799999952316284</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K92" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N92" t="n">
+        <v>54.31</v>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>141.87</v>
+      </c>
+      <c r="F93" t="n">
+        <v>143.78</v>
+      </c>
+      <c r="G93" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="H93" t="n">
+        <v>145.1699981689453</v>
+      </c>
+      <c r="I93" t="n">
+        <v>2.329999923706055</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K93" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N93" t="n">
+        <v>65.42</v>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>575.54</v>
+      </c>
+      <c r="F94" t="n">
+        <v>583.6</v>
+      </c>
+      <c r="G94" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H94" t="n">
+        <v>546.989990234375</v>
+      </c>
+      <c r="I94" t="n">
+        <v>-4.960000038146973</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K94" t="n">
+        <v>0.637</v>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N94" t="n">
+        <v>64.84</v>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>343.98</v>
+      </c>
+      <c r="F95" t="n">
+        <v>316.28</v>
+      </c>
+      <c r="G95" t="n">
+        <v>-8.050000000000001</v>
+      </c>
+      <c r="H95" t="n">
+        <v>333.7000122070312</v>
+      </c>
+      <c r="I95" t="n">
+        <v>-2.990000009536743</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K95" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N95" t="n">
+        <v>53.48</v>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>374.64</v>
+      </c>
+      <c r="F96" t="n">
+        <v>344.48</v>
+      </c>
+      <c r="G96" t="n">
+        <v>-8.050000000000001</v>
+      </c>
+      <c r="H96" t="n">
+        <v>349.7200012207031</v>
+      </c>
+      <c r="I96" t="n">
+        <v>-6.650000095367432</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K96" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N96" t="n">
+        <v>50.92</v>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>55.85</v>
+      </c>
+      <c r="F97" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="G97" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="H97" t="n">
+        <v>46.61999893188477</v>
+      </c>
+      <c r="I97" t="n">
+        <v>-16.52000045776367</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K97" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N97" t="n">
+        <v>67.31999999999999</v>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>124.61</v>
+      </c>
+      <c r="F98" t="n">
+        <v>120.53</v>
+      </c>
+      <c r="G98" t="n">
+        <v>-3.27</v>
+      </c>
+      <c r="H98" t="n">
+        <v>117.2900009155273</v>
+      </c>
+      <c r="I98" t="n">
+        <v>-5.880000114440918</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K98" t="n">
+        <v>-0.703</v>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N98" t="n">
+        <v>31.03</v>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>344.97</v>
+      </c>
+      <c r="F99" t="n">
+        <v>415.28</v>
+      </c>
+      <c r="G99" t="n">
+        <v>20.38</v>
+      </c>
+      <c r="H99" t="n">
+        <v>345.6000061035156</v>
+      </c>
+      <c r="I99" t="n">
+        <v>0.1800000071525574</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K99" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N99" t="n">
+        <v>87.64</v>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>924.88</v>
+      </c>
+      <c r="F100" t="n">
+        <v>912.54</v>
+      </c>
+      <c r="G100" t="n">
+        <v>-1.33</v>
+      </c>
+      <c r="H100" t="n">
+        <v>1065.699951171875</v>
+      </c>
+      <c r="I100" t="n">
+        <v>15.22999954223633</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K100" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N100" t="n">
+        <v>61.4</v>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>139.91</v>
+      </c>
+      <c r="F101" t="n">
+        <v>150.44</v>
+      </c>
+      <c r="G101" t="n">
+        <v>7.53</v>
+      </c>
+      <c r="H101" t="n">
+        <v>140.9799957275391</v>
+      </c>
+      <c r="I101" t="n">
+        <v>0.7599999904632568</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K101" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N101" t="n">
+        <v>74.48999999999999</v>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-13)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O101"/>
+  <dimension ref="A1:O121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7104,6 +7104,1266 @@
       <c r="O101" t="inlineStr">
         <is>
           <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>1483.2</v>
+      </c>
+      <c r="F102" t="n">
+        <v>1662.04</v>
+      </c>
+      <c r="G102" t="n">
+        <v>12.06</v>
+      </c>
+      <c r="H102" t="n">
+        <v>1775.530029296875</v>
+      </c>
+      <c r="I102" t="n">
+        <v>19.70999908447266</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K102" t="n">
+        <v>-0.796</v>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N102" t="n">
+        <v>52.17</v>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>3239.6</v>
+      </c>
+      <c r="F103" t="n">
+        <v>3255.03</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="H103" t="n">
+        <v>3426.14990234375</v>
+      </c>
+      <c r="I103" t="n">
+        <v>5.760000228881836</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K103" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N103" t="n">
+        <v>58.35</v>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>1595.9</v>
+      </c>
+      <c r="F104" t="n">
+        <v>1645.85</v>
+      </c>
+      <c r="G104" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="H104" t="n">
+        <v>1616.640014648438</v>
+      </c>
+      <c r="I104" t="n">
+        <v>1.299999952316284</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K104" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N104" t="n">
+        <v>67.69</v>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>936.95</v>
+      </c>
+      <c r="F105" t="n">
+        <v>925.05</v>
+      </c>
+      <c r="G105" t="n">
+        <v>-1.27</v>
+      </c>
+      <c r="H105" t="n">
+        <v>899.6400146484375</v>
+      </c>
+      <c r="I105" t="n">
+        <v>-3.980000019073486</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K105" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N105" t="n">
+        <v>56.13</v>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>1413.1</v>
+      </c>
+      <c r="F106" t="n">
+        <v>1330.46</v>
+      </c>
+      <c r="G106" t="n">
+        <v>-5.85</v>
+      </c>
+      <c r="H106" t="n">
+        <v>1419.5400390625</v>
+      </c>
+      <c r="I106" t="n">
+        <v>0.4600000083446503</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K106" t="n">
+        <v>-0.459</v>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N106" t="n">
+        <v>32.05</v>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>1015.15</v>
+      </c>
+      <c r="F107" t="n">
+        <v>980.13</v>
+      </c>
+      <c r="G107" t="n">
+        <v>-3.45</v>
+      </c>
+      <c r="H107" t="n">
+        <v>1025.390014648438</v>
+      </c>
+      <c r="I107" t="n">
+        <v>1.009999990463257</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K107" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N107" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>2406.2</v>
+      </c>
+      <c r="F108" t="n">
+        <v>2312.55</v>
+      </c>
+      <c r="G108" t="n">
+        <v>-3.89</v>
+      </c>
+      <c r="H108" t="n">
+        <v>2694.159912109375</v>
+      </c>
+      <c r="I108" t="n">
+        <v>11.97000026702881</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K108" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N108" t="n">
+        <v>57.36</v>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>338.4</v>
+      </c>
+      <c r="F109" t="n">
+        <v>358.62</v>
+      </c>
+      <c r="G109" t="n">
+        <v>5.97</v>
+      </c>
+      <c r="H109" t="n">
+        <v>392.9599914550781</v>
+      </c>
+      <c r="I109" t="n">
+        <v>16.1200008392334</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K109" t="n">
+        <v>0.329</v>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N109" t="n">
+        <v>65.54000000000001</v>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>4019</v>
+      </c>
+      <c r="F110" t="n">
+        <v>3925.74</v>
+      </c>
+      <c r="G110" t="n">
+        <v>-2.32</v>
+      </c>
+      <c r="H110" t="n">
+        <v>4404.41015625</v>
+      </c>
+      <c r="I110" t="n">
+        <v>9.590000152587891</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K110" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N110" t="n">
+        <v>50.08</v>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>951.9</v>
+      </c>
+      <c r="F111" t="n">
+        <v>1018.97</v>
+      </c>
+      <c r="G111" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="H111" t="n">
+        <v>967.3400268554688</v>
+      </c>
+      <c r="I111" t="n">
+        <v>1.620000004768372</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K111" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N111" t="n">
+        <v>74.56999999999999</v>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>2044</v>
+      </c>
+      <c r="F112" t="n">
+        <v>2219.42</v>
+      </c>
+      <c r="G112" t="n">
+        <v>8.58</v>
+      </c>
+      <c r="H112" t="n">
+        <v>1991.349975585938</v>
+      </c>
+      <c r="I112" t="n">
+        <v>-2.579999923706055</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K112" t="n">
+        <v>-0.735</v>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N112" t="n">
+        <v>48.17</v>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>2896.4</v>
+      </c>
+      <c r="F113" t="n">
+        <v>2720.45</v>
+      </c>
+      <c r="G113" t="n">
+        <v>-6.07</v>
+      </c>
+      <c r="H113" t="n">
+        <v>3202.8798828125</v>
+      </c>
+      <c r="I113" t="n">
+        <v>10.57999992370605</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K113" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N113" t="n">
+        <v>54.09</v>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>1274.2</v>
+      </c>
+      <c r="F114" t="n">
+        <v>1191.91</v>
+      </c>
+      <c r="G114" t="n">
+        <v>-6.46</v>
+      </c>
+      <c r="H114" t="n">
+        <v>1335.650024414062</v>
+      </c>
+      <c r="I114" t="n">
+        <v>4.820000171661377</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K114" t="n">
+        <v>0.718</v>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N114" t="n">
+        <v>54.67</v>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>16582</v>
+      </c>
+      <c r="F115" t="n">
+        <v>18424.06</v>
+      </c>
+      <c r="G115" t="n">
+        <v>11.11</v>
+      </c>
+      <c r="H115" t="n">
+        <v>16554.580078125</v>
+      </c>
+      <c r="I115" t="n">
+        <v>-0.1700000017881393</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K115" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N115" t="n">
+        <v>79.66</v>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>1736</v>
+      </c>
+      <c r="F116" t="n">
+        <v>1819.99</v>
+      </c>
+      <c r="G116" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="H116" t="n">
+        <v>1692.599975585938</v>
+      </c>
+      <c r="I116" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K116" t="n">
+        <v>0.8129999999999999</v>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N116" t="n">
+        <v>73.52</v>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>263.1</v>
+      </c>
+      <c r="F117" t="n">
+        <v>276.96</v>
+      </c>
+      <c r="G117" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="H117" t="n">
+        <v>240.9799957275391</v>
+      </c>
+      <c r="I117" t="n">
+        <v>-8.409999847412109</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K117" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N117" t="n">
+        <v>70.90000000000001</v>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>12098</v>
+      </c>
+      <c r="F118" t="n">
+        <v>11651.22</v>
+      </c>
+      <c r="G118" t="n">
+        <v>-3.69</v>
+      </c>
+      <c r="H118" t="n">
+        <v>9949.4296875</v>
+      </c>
+      <c r="I118" t="n">
+        <v>-17.76000022888184</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K118" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N118" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>337.45</v>
+      </c>
+      <c r="F119" t="n">
+        <v>327.98</v>
+      </c>
+      <c r="G119" t="n">
+        <v>-2.81</v>
+      </c>
+      <c r="H119" t="n">
+        <v>379.5</v>
+      </c>
+      <c r="I119" t="n">
+        <v>12.46000003814697</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K119" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N119" t="n">
+        <v>58.79</v>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>258.55</v>
+      </c>
+      <c r="F120" t="n">
+        <v>256.7</v>
+      </c>
+      <c r="G120" t="n">
+        <v>-0.72</v>
+      </c>
+      <c r="H120" t="n">
+        <v>289.2699890136719</v>
+      </c>
+      <c r="I120" t="n">
+        <v>11.88000011444092</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K120" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N120" t="n">
+        <v>61.93</v>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>4231.6</v>
+      </c>
+      <c r="F121" t="n">
+        <v>4045.92</v>
+      </c>
+      <c r="G121" t="n">
+        <v>-4.39</v>
+      </c>
+      <c r="H121" t="n">
+        <v>3808.429931640625</v>
+      </c>
+      <c r="I121" t="n">
+        <v>-10</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K121" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N121" t="n">
+        <v>59.34</v>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
         </is>
       </c>
     </row>
@@ -7118,7 +8378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10485,6 +11745,636 @@
       <c r="O51" t="inlineStr">
         <is>
           <t>12 Jan 2026, 06:55:07 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1483.3</v>
+      </c>
+      <c r="F52" t="n">
+        <v>1667.85</v>
+      </c>
+      <c r="G52" t="n">
+        <v>12.44</v>
+      </c>
+      <c r="H52" t="n">
+        <v>1541.77001953125</v>
+      </c>
+      <c r="I52" t="n">
+        <v>3.940000057220459</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K52" t="n">
+        <v>-0.796</v>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N52" t="n">
+        <v>52.74</v>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>3235.7</v>
+      </c>
+      <c r="F53" t="n">
+        <v>3243</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="H53" t="n">
+        <v>3342.080078125</v>
+      </c>
+      <c r="I53" t="n">
+        <v>3.289999961853027</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K53" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N53" t="n">
+        <v>57.98</v>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1595.95</v>
+      </c>
+      <c r="F54" t="n">
+        <v>1651.31</v>
+      </c>
+      <c r="G54" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="H54" t="n">
+        <v>1621.530029296875</v>
+      </c>
+      <c r="I54" t="n">
+        <v>1.600000023841858</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K54" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N54" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>936.65</v>
+      </c>
+      <c r="F55" t="n">
+        <v>927.78</v>
+      </c>
+      <c r="G55" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="H55" t="n">
+        <v>1026.050048828125</v>
+      </c>
+      <c r="I55" t="n">
+        <v>9.550000190734863</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K55" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N55" t="n">
+        <v>56.62</v>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>1413.15</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1339.74</v>
+      </c>
+      <c r="G56" t="n">
+        <v>-5.19</v>
+      </c>
+      <c r="H56" t="n">
+        <v>1346.369995117188</v>
+      </c>
+      <c r="I56" t="n">
+        <v>-4.730000019073486</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K56" t="n">
+        <v>-0.459</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N56" t="n">
+        <v>33.03</v>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>1015.05</v>
+      </c>
+      <c r="F57" t="n">
+        <v>986.16</v>
+      </c>
+      <c r="G57" t="n">
+        <v>-2.85</v>
+      </c>
+      <c r="H57" t="n">
+        <v>847.7999877929688</v>
+      </c>
+      <c r="I57" t="n">
+        <v>-16.47999954223633</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K57" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N57" t="n">
+        <v>53.77</v>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>338.35</v>
+      </c>
+      <c r="F58" t="n">
+        <v>365.91</v>
+      </c>
+      <c r="G58" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="H58" t="n">
+        <v>374.8099975585938</v>
+      </c>
+      <c r="I58" t="n">
+        <v>10.77999973297119</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K58" t="n">
+        <v>0.329</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N58" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>4018.5</v>
+      </c>
+      <c r="F59" t="n">
+        <v>3936.56</v>
+      </c>
+      <c r="G59" t="n">
+        <v>-2.04</v>
+      </c>
+      <c r="H59" t="n">
+        <v>4084.909912109375</v>
+      </c>
+      <c r="I59" t="n">
+        <v>1.649999976158142</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K59" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N59" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>1274.25</v>
+      </c>
+      <c r="F60" t="n">
+        <v>1223.64</v>
+      </c>
+      <c r="G60" t="n">
+        <v>-3.97</v>
+      </c>
+      <c r="H60" t="n">
+        <v>1183.339965820312</v>
+      </c>
+      <c r="I60" t="n">
+        <v>-7.130000114440918</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K60" t="n">
+        <v>0.718</v>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N60" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>16588.85</v>
+      </c>
+      <c r="F61" t="n">
+        <v>18549.22</v>
+      </c>
+      <c r="G61" t="n">
+        <v>11.82</v>
+      </c>
+      <c r="H61" t="n">
+        <v>15497</v>
+      </c>
+      <c r="I61" t="n">
+        <v>-6.579999923706055</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K61" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N61" t="n">
+        <v>80.73</v>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
         </is>
       </c>
     </row>
@@ -10499,7 +12389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O101"/>
+  <dimension ref="A1:O121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17159,6 +19049,1266 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>260.25</v>
+      </c>
+      <c r="F102" t="n">
+        <v>286.16</v>
+      </c>
+      <c r="G102" t="n">
+        <v>9.960000000000001</v>
+      </c>
+      <c r="H102" t="n">
+        <v>271.239990234375</v>
+      </c>
+      <c r="I102" t="n">
+        <v>4.21999979019165</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K102" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N102" t="n">
+        <v>76.66</v>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>477.18</v>
+      </c>
+      <c r="F103" t="n">
+        <v>476.58</v>
+      </c>
+      <c r="G103" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="H103" t="n">
+        <v>441.8399963378906</v>
+      </c>
+      <c r="I103" t="n">
+        <v>-7.409999847412109</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K103" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N103" t="n">
+        <v>60.95</v>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>331.86</v>
+      </c>
+      <c r="F104" t="n">
+        <v>357.54</v>
+      </c>
+      <c r="G104" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="H104" t="n">
+        <v>379.239990234375</v>
+      </c>
+      <c r="I104" t="n">
+        <v>14.27999973297119</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K104" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N104" t="n">
+        <v>74.81</v>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>246.47</v>
+      </c>
+      <c r="F105" t="n">
+        <v>253.56</v>
+      </c>
+      <c r="G105" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="H105" t="n">
+        <v>229.3600006103516</v>
+      </c>
+      <c r="I105" t="n">
+        <v>-6.940000057220459</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K105" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N105" t="n">
+        <v>57.88</v>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>641.97</v>
+      </c>
+      <c r="F106" t="n">
+        <v>733.35</v>
+      </c>
+      <c r="G106" t="n">
+        <v>14.23</v>
+      </c>
+      <c r="H106" t="n">
+        <v>807.6900024414062</v>
+      </c>
+      <c r="I106" t="n">
+        <v>25.80999946594238</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K106" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N106" t="n">
+        <v>58.35</v>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>448.96</v>
+      </c>
+      <c r="F107" t="n">
+        <v>450.53</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="H107" t="n">
+        <v>572.1500244140625</v>
+      </c>
+      <c r="I107" t="n">
+        <v>27.44000053405762</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K107" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N107" t="n">
+        <v>64.52</v>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>184.94</v>
+      </c>
+      <c r="F108" t="n">
+        <v>202.68</v>
+      </c>
+      <c r="G108" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="H108" t="n">
+        <v>163.1100006103516</v>
+      </c>
+      <c r="I108" t="n">
+        <v>-11.80000019073486</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K108" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N108" t="n">
+        <v>79.95</v>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>324.49</v>
+      </c>
+      <c r="F109" t="n">
+        <v>345.57</v>
+      </c>
+      <c r="G109" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H109" t="n">
+        <v>333.8399963378906</v>
+      </c>
+      <c r="I109" t="n">
+        <v>2.880000114440918</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K109" t="n">
+        <v>0.485</v>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N109" t="n">
+        <v>69.44</v>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>343.2</v>
+      </c>
+      <c r="F110" t="n">
+        <v>359.53</v>
+      </c>
+      <c r="G110" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="H110" t="n">
+        <v>334.7200012207031</v>
+      </c>
+      <c r="I110" t="n">
+        <v>-2.470000028610229</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K110" t="n">
+        <v>-0.296</v>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N110" t="n">
+        <v>51.22</v>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>209.72</v>
+      </c>
+      <c r="F111" t="n">
+        <v>218.8</v>
+      </c>
+      <c r="G111" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="H111" t="n">
+        <v>190.6300048828125</v>
+      </c>
+      <c r="I111" t="n">
+        <v>-9.100000381469727</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K111" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N111" t="n">
+        <v>64.13</v>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>117.97</v>
+      </c>
+      <c r="F112" t="n">
+        <v>117.95</v>
+      </c>
+      <c r="G112" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="H112" t="n">
+        <v>107.8600006103516</v>
+      </c>
+      <c r="I112" t="n">
+        <v>-8.569999694824219</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K112" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N112" t="n">
+        <v>56.33</v>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>143.46</v>
+      </c>
+      <c r="F113" t="n">
+        <v>143.53</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H113" t="n">
+        <v>145.7899932861328</v>
+      </c>
+      <c r="I113" t="n">
+        <v>1.620000004768372</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K113" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N113" t="n">
+        <v>63.27</v>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>566.28</v>
+      </c>
+      <c r="F114" t="n">
+        <v>588.36</v>
+      </c>
+      <c r="G114" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="H114" t="n">
+        <v>586.9600219726562</v>
+      </c>
+      <c r="I114" t="n">
+        <v>3.650000095367432</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K114" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N114" t="n">
+        <v>66.06999999999999</v>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>340.51</v>
+      </c>
+      <c r="F115" t="n">
+        <v>311.17</v>
+      </c>
+      <c r="G115" t="n">
+        <v>-8.619999999999999</v>
+      </c>
+      <c r="H115" t="n">
+        <v>460.8500061035156</v>
+      </c>
+      <c r="I115" t="n">
+        <v>35.34000015258789</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K115" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N115" t="n">
+        <v>24.07</v>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>374.94</v>
+      </c>
+      <c r="F116" t="n">
+        <v>346.21</v>
+      </c>
+      <c r="G116" t="n">
+        <v>-7.66</v>
+      </c>
+      <c r="H116" t="n">
+        <v>389.9700012207031</v>
+      </c>
+      <c r="I116" t="n">
+        <v>4.010000228881836</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K116" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N116" t="n">
+        <v>51.51</v>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>55.19</v>
+      </c>
+      <c r="F117" t="n">
+        <v>57.52</v>
+      </c>
+      <c r="G117" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="H117" t="n">
+        <v>65.73999786376953</v>
+      </c>
+      <c r="I117" t="n">
+        <v>19.11000061035156</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K117" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N117" t="n">
+        <v>69.52</v>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>124.03</v>
+      </c>
+      <c r="F118" t="n">
+        <v>122.24</v>
+      </c>
+      <c r="G118" t="n">
+        <v>-1.44</v>
+      </c>
+      <c r="H118" t="n">
+        <v>143.1600036621094</v>
+      </c>
+      <c r="I118" t="n">
+        <v>15.43000030517578</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K118" t="n">
+        <v>-0.703</v>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N118" t="n">
+        <v>33.78</v>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>352.21</v>
+      </c>
+      <c r="F119" t="n">
+        <v>412.16</v>
+      </c>
+      <c r="G119" t="n">
+        <v>17.02</v>
+      </c>
+      <c r="H119" t="n">
+        <v>364.8699951171875</v>
+      </c>
+      <c r="I119" t="n">
+        <v>3.589999914169312</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K119" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N119" t="n">
+        <v>90.69</v>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>943.08</v>
+      </c>
+      <c r="F120" t="n">
+        <v>921.72</v>
+      </c>
+      <c r="G120" t="n">
+        <v>-2.26</v>
+      </c>
+      <c r="H120" t="n">
+        <v>951.4199829101562</v>
+      </c>
+      <c r="I120" t="n">
+        <v>0.8799999952316284</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K120" t="n">
+        <v>0.681</v>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N120" t="n">
+        <v>60.22</v>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>141.36</v>
+      </c>
+      <c r="F121" t="n">
+        <v>146.31</v>
+      </c>
+      <c r="G121" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H121" t="n">
+        <v>147.6300048828125</v>
+      </c>
+      <c r="I121" t="n">
+        <v>4.429999828338623</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K121" t="n">
+        <v>0.681</v>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N121" t="n">
+        <v>68.87</v>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-14)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O121"/>
+  <dimension ref="A1:O141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8364,6 +8364,1266 @@
       <c r="O121" t="inlineStr">
         <is>
           <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>1452.8</v>
+      </c>
+      <c r="F122" t="n">
+        <v>1651.26</v>
+      </c>
+      <c r="G122" t="n">
+        <v>13.66</v>
+      </c>
+      <c r="H122" t="n">
+        <v>1217.099975585938</v>
+      </c>
+      <c r="I122" t="n">
+        <v>-16.21999931335449</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K122" t="n">
+        <v>0.359</v>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N122" t="n">
+        <v>77.67</v>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>3268</v>
+      </c>
+      <c r="F123" t="n">
+        <v>3236.46</v>
+      </c>
+      <c r="G123" t="n">
+        <v>-0.96</v>
+      </c>
+      <c r="H123" t="n">
+        <v>3180.3798828125</v>
+      </c>
+      <c r="I123" t="n">
+        <v>-2.680000066757202</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K123" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N123" t="n">
+        <v>61.55</v>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>1599</v>
+      </c>
+      <c r="F124" t="n">
+        <v>1633.43</v>
+      </c>
+      <c r="G124" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="H124" t="n">
+        <v>1574.469970703125</v>
+      </c>
+      <c r="I124" t="n">
+        <v>-1.529999971389771</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K124" t="n">
+        <v>0.863</v>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N124" t="n">
+        <v>70.48999999999999</v>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>937.35</v>
+      </c>
+      <c r="F125" t="n">
+        <v>925.04</v>
+      </c>
+      <c r="G125" t="n">
+        <v>-1.31</v>
+      </c>
+      <c r="H125" t="n">
+        <v>992.6799926757812</v>
+      </c>
+      <c r="I125" t="n">
+        <v>5.900000095367432</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K125" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N125" t="n">
+        <v>59.17</v>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>1437</v>
+      </c>
+      <c r="F126" t="n">
+        <v>1337.85</v>
+      </c>
+      <c r="G126" t="n">
+        <v>-6.9</v>
+      </c>
+      <c r="H126" t="n">
+        <v>1396.150024414062</v>
+      </c>
+      <c r="I126" t="n">
+        <v>-2.839999914169312</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K126" t="n">
+        <v>0.827</v>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N126" t="n">
+        <v>56.19</v>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>1028.45</v>
+      </c>
+      <c r="F127" t="n">
+        <v>987</v>
+      </c>
+      <c r="G127" t="n">
+        <v>-4.03</v>
+      </c>
+      <c r="H127" t="n">
+        <v>1349.77001953125</v>
+      </c>
+      <c r="I127" t="n">
+        <v>31.23999977111816</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K127" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N127" t="n">
+        <v>49.87</v>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>2389.5</v>
+      </c>
+      <c r="F128" t="n">
+        <v>2302.58</v>
+      </c>
+      <c r="G128" t="n">
+        <v>-3.64</v>
+      </c>
+      <c r="H128" t="n">
+        <v>2319.330078125</v>
+      </c>
+      <c r="I128" t="n">
+        <v>-2.940000057220459</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K128" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N128" t="n">
+        <v>57.04</v>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>334.7</v>
+      </c>
+      <c r="F129" t="n">
+        <v>358.65</v>
+      </c>
+      <c r="G129" t="n">
+        <v>7.16</v>
+      </c>
+      <c r="H129" t="n">
+        <v>375.7000122070312</v>
+      </c>
+      <c r="I129" t="n">
+        <v>12.25</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K129" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N129" t="n">
+        <v>68.37</v>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>3887.4</v>
+      </c>
+      <c r="F130" t="n">
+        <v>3921.05</v>
+      </c>
+      <c r="G130" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="H130" t="n">
+        <v>3621.090087890625</v>
+      </c>
+      <c r="I130" t="n">
+        <v>-6.849999904632568</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K130" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N130" t="n">
+        <v>57.66</v>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>949</v>
+      </c>
+      <c r="F131" t="n">
+        <v>1018.17</v>
+      </c>
+      <c r="G131" t="n">
+        <v>7.29</v>
+      </c>
+      <c r="H131" t="n">
+        <v>1023.900024414062</v>
+      </c>
+      <c r="I131" t="n">
+        <v>7.889999866485596</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K131" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N131" t="n">
+        <v>78.48999999999999</v>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>2026.9</v>
+      </c>
+      <c r="F132" t="n">
+        <v>2205.81</v>
+      </c>
+      <c r="G132" t="n">
+        <v>8.83</v>
+      </c>
+      <c r="H132" t="n">
+        <v>2074.0400390625</v>
+      </c>
+      <c r="I132" t="n">
+        <v>2.329999923706055</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K132" t="n">
+        <v>-0.735</v>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N132" t="n">
+        <v>48.54</v>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>2886.3</v>
+      </c>
+      <c r="F133" t="n">
+        <v>2734.12</v>
+      </c>
+      <c r="G133" t="n">
+        <v>-5.27</v>
+      </c>
+      <c r="H133" t="n">
+        <v>2768.449951171875</v>
+      </c>
+      <c r="I133" t="n">
+        <v>-4.079999923706055</v>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K133" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N133" t="n">
+        <v>48.45</v>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>1262</v>
+      </c>
+      <c r="F134" t="n">
+        <v>1183.72</v>
+      </c>
+      <c r="G134" t="n">
+        <v>-6.2</v>
+      </c>
+      <c r="H134" t="n">
+        <v>1221.030029296875</v>
+      </c>
+      <c r="I134" t="n">
+        <v>-3.25</v>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K134" t="n">
+        <v>0</v>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N134" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>16426</v>
+      </c>
+      <c r="F135" t="n">
+        <v>18408.18</v>
+      </c>
+      <c r="G135" t="n">
+        <v>12.07</v>
+      </c>
+      <c r="H135" t="n">
+        <v>15818.2802734375</v>
+      </c>
+      <c r="I135" t="n">
+        <v>-3.700000047683716</v>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K135" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N135" t="n">
+        <v>81.09999999999999</v>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>1728.7</v>
+      </c>
+      <c r="F136" t="n">
+        <v>1812.86</v>
+      </c>
+      <c r="G136" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="H136" t="n">
+        <v>1837.119995117188</v>
+      </c>
+      <c r="I136" t="n">
+        <v>6.269999980926514</v>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K136" t="n">
+        <v>0.8129999999999999</v>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N136" t="n">
+        <v>73.56</v>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>264.2</v>
+      </c>
+      <c r="F137" t="n">
+        <v>275.9</v>
+      </c>
+      <c r="G137" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="H137" t="n">
+        <v>268.3599853515625</v>
+      </c>
+      <c r="I137" t="n">
+        <v>1.580000042915344</v>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K137" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N137" t="n">
+        <v>70.64</v>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>12044</v>
+      </c>
+      <c r="F138" t="n">
+        <v>11662.98</v>
+      </c>
+      <c r="G138" t="n">
+        <v>-3.16</v>
+      </c>
+      <c r="H138" t="n">
+        <v>12304.9697265625</v>
+      </c>
+      <c r="I138" t="n">
+        <v>2.170000076293945</v>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K138" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N138" t="n">
+        <v>50.71</v>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>337.9</v>
+      </c>
+      <c r="F139" t="n">
+        <v>328.34</v>
+      </c>
+      <c r="G139" t="n">
+        <v>-2.83</v>
+      </c>
+      <c r="H139" t="n">
+        <v>330.3500061035156</v>
+      </c>
+      <c r="I139" t="n">
+        <v>-2.230000019073486</v>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K139" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N139" t="n">
+        <v>58.76</v>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>258.8</v>
+      </c>
+      <c r="F140" t="n">
+        <v>256.88</v>
+      </c>
+      <c r="G140" t="n">
+        <v>-0.74</v>
+      </c>
+      <c r="H140" t="n">
+        <v>294.9200134277344</v>
+      </c>
+      <c r="I140" t="n">
+        <v>13.96000003814697</v>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K140" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N140" t="n">
+        <v>61.89</v>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>4239.2</v>
+      </c>
+      <c r="F141" t="n">
+        <v>4051.3</v>
+      </c>
+      <c r="G141" t="n">
+        <v>-4.43</v>
+      </c>
+      <c r="H141" t="n">
+        <v>3241.75</v>
+      </c>
+      <c r="I141" t="n">
+        <v>-23.53000068664551</v>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K141" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N141" t="n">
+        <v>59.27</v>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
         </is>
       </c>
     </row>
@@ -8378,7 +9638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O61"/>
+  <dimension ref="A1:O71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12375,6 +13635,636 @@
       <c r="O61" t="inlineStr">
         <is>
           <t>13 Jan 2026, 06:54:51 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>1451.5</v>
+      </c>
+      <c r="F62" t="n">
+        <v>1664.08</v>
+      </c>
+      <c r="G62" t="n">
+        <v>14.65</v>
+      </c>
+      <c r="H62" t="n">
+        <v>1567.579956054688</v>
+      </c>
+      <c r="I62" t="n">
+        <v>8</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K62" t="n">
+        <v>0.359</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N62" t="n">
+        <v>79.15000000000001</v>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>3267.6</v>
+      </c>
+      <c r="F63" t="n">
+        <v>3247.41</v>
+      </c>
+      <c r="G63" t="n">
+        <v>-0.62</v>
+      </c>
+      <c r="H63" t="n">
+        <v>3385.68994140625</v>
+      </c>
+      <c r="I63" t="n">
+        <v>3.609999895095825</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K63" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N63" t="n">
+        <v>62.07</v>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>1597.95</v>
+      </c>
+      <c r="F64" t="n">
+        <v>1647.71</v>
+      </c>
+      <c r="G64" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="H64" t="n">
+        <v>1439.819946289062</v>
+      </c>
+      <c r="I64" t="n">
+        <v>-9.899999618530273</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K64" t="n">
+        <v>0.863</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N64" t="n">
+        <v>71.93000000000001</v>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>937.25</v>
+      </c>
+      <c r="F65" t="n">
+        <v>928.03</v>
+      </c>
+      <c r="G65" t="n">
+        <v>-0.98</v>
+      </c>
+      <c r="H65" t="n">
+        <v>1013.390014648438</v>
+      </c>
+      <c r="I65" t="n">
+        <v>8.119999885559082</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K65" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N65" t="n">
+        <v>59.66</v>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>1436.55</v>
+      </c>
+      <c r="F66" t="n">
+        <v>1342.45</v>
+      </c>
+      <c r="G66" t="n">
+        <v>-6.55</v>
+      </c>
+      <c r="H66" t="n">
+        <v>1417.170043945312</v>
+      </c>
+      <c r="I66" t="n">
+        <v>-1.350000023841858</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K66" t="n">
+        <v>0.827</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N66" t="n">
+        <v>56.71</v>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>1028.45</v>
+      </c>
+      <c r="F67" t="n">
+        <v>993.3</v>
+      </c>
+      <c r="G67" t="n">
+        <v>-3.42</v>
+      </c>
+      <c r="H67" t="n">
+        <v>1047.0400390625</v>
+      </c>
+      <c r="I67" t="n">
+        <v>1.809999942779541</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K67" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N67" t="n">
+        <v>50.79</v>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>334.65</v>
+      </c>
+      <c r="F68" t="n">
+        <v>362.55</v>
+      </c>
+      <c r="G68" t="n">
+        <v>8.34</v>
+      </c>
+      <c r="H68" t="n">
+        <v>386.7799987792969</v>
+      </c>
+      <c r="I68" t="n">
+        <v>15.57999992370605</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K68" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N68" t="n">
+        <v>70.55</v>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>3888.05</v>
+      </c>
+      <c r="F69" t="n">
+        <v>3932.11</v>
+      </c>
+      <c r="G69" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="H69" t="n">
+        <v>4253.0400390625</v>
+      </c>
+      <c r="I69" t="n">
+        <v>9.390000343322754</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K69" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N69" t="n">
+        <v>58.06</v>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>1261.9</v>
+      </c>
+      <c r="F70" t="n">
+        <v>1230.27</v>
+      </c>
+      <c r="G70" t="n">
+        <v>-2.51</v>
+      </c>
+      <c r="H70" t="n">
+        <v>1241.949951171875</v>
+      </c>
+      <c r="I70" t="n">
+        <v>-1.580000042915344</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K70" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N70" t="n">
+        <v>58.48</v>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>16425.8</v>
+      </c>
+      <c r="F71" t="n">
+        <v>18487.29</v>
+      </c>
+      <c r="G71" t="n">
+        <v>12.55</v>
+      </c>
+      <c r="H71" t="n">
+        <v>22186.390625</v>
+      </c>
+      <c r="I71" t="n">
+        <v>35.06999969482422</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K71" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N71" t="n">
+        <v>81.83</v>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
         </is>
       </c>
     </row>
@@ -12389,7 +14279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O121"/>
+  <dimension ref="A1:O141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20309,6 +22199,1266 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>261.05</v>
+      </c>
+      <c r="F122" t="n">
+        <v>286.88</v>
+      </c>
+      <c r="G122" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="H122" t="n">
+        <v>289.9599914550781</v>
+      </c>
+      <c r="I122" t="n">
+        <v>11.06999969482422</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K122" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N122" t="n">
+        <v>78.04000000000001</v>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>470.67</v>
+      </c>
+      <c r="F123" t="n">
+        <v>476.14</v>
+      </c>
+      <c r="G123" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="H123" t="n">
+        <v>451.7200012207031</v>
+      </c>
+      <c r="I123" t="n">
+        <v>-4.03000020980835</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K123" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N123" t="n">
+        <v>60.54</v>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>335.97</v>
+      </c>
+      <c r="F124" t="n">
+        <v>357.01</v>
+      </c>
+      <c r="G124" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="H124" t="n">
+        <v>318.3800048828125</v>
+      </c>
+      <c r="I124" t="n">
+        <v>-5.230000019073486</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K124" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N124" t="n">
+        <v>68.58</v>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>242.6</v>
+      </c>
+      <c r="F125" t="n">
+        <v>255.03</v>
+      </c>
+      <c r="G125" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="H125" t="n">
+        <v>264.739990234375</v>
+      </c>
+      <c r="I125" t="n">
+        <v>9.130000114440918</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K125" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N125" t="n">
+        <v>68.81999999999999</v>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>631.09</v>
+      </c>
+      <c r="F126" t="n">
+        <v>729.49</v>
+      </c>
+      <c r="G126" t="n">
+        <v>15.59</v>
+      </c>
+      <c r="H126" t="n">
+        <v>768.219970703125</v>
+      </c>
+      <c r="I126" t="n">
+        <v>21.72999954223633</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K126" t="n">
+        <v>0.791</v>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N126" t="n">
+        <v>89.20999999999999</v>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>447.2</v>
+      </c>
+      <c r="F127" t="n">
+        <v>450.06</v>
+      </c>
+      <c r="G127" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="H127" t="n">
+        <v>339.0499877929688</v>
+      </c>
+      <c r="I127" t="n">
+        <v>-24.18000030517578</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K127" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N127" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>185.81</v>
+      </c>
+      <c r="F128" t="n">
+        <v>203.1</v>
+      </c>
+      <c r="G128" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="H128" t="n">
+        <v>156.1699981689453</v>
+      </c>
+      <c r="I128" t="n">
+        <v>-15.94999980926514</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K128" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N128" t="n">
+        <v>75.68000000000001</v>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>310.9</v>
+      </c>
+      <c r="F129" t="n">
+        <v>344.64</v>
+      </c>
+      <c r="G129" t="n">
+        <v>10.85</v>
+      </c>
+      <c r="H129" t="n">
+        <v>347.1300048828125</v>
+      </c>
+      <c r="I129" t="n">
+        <v>11.64999961853027</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K129" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N129" t="n">
+        <v>73.92</v>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>327.88</v>
+      </c>
+      <c r="F130" t="n">
+        <v>358.17</v>
+      </c>
+      <c r="G130" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="H130" t="n">
+        <v>353.2300109863281</v>
+      </c>
+      <c r="I130" t="n">
+        <v>7.730000019073486</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K130" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N130" t="n">
+        <v>77.26000000000001</v>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>213.65</v>
+      </c>
+      <c r="F131" t="n">
+        <v>219.43</v>
+      </c>
+      <c r="G131" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H131" t="n">
+        <v>229.4499969482422</v>
+      </c>
+      <c r="I131" t="n">
+        <v>7.389999866485596</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K131" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N131" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>120.36</v>
+      </c>
+      <c r="F132" t="n">
+        <v>118.59</v>
+      </c>
+      <c r="G132" t="n">
+        <v>-1.47</v>
+      </c>
+      <c r="H132" t="n">
+        <v>116.370002746582</v>
+      </c>
+      <c r="I132" t="n">
+        <v>-3.309999942779541</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K132" t="n">
+        <v>0</v>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N132" t="n">
+        <v>47.79</v>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>144.24</v>
+      </c>
+      <c r="F133" t="n">
+        <v>143.58</v>
+      </c>
+      <c r="G133" t="n">
+        <v>-0.46</v>
+      </c>
+      <c r="H133" t="n">
+        <v>144.3999938964844</v>
+      </c>
+      <c r="I133" t="n">
+        <v>0.1099999994039536</v>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K133" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N133" t="n">
+        <v>59.19</v>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>544.99</v>
+      </c>
+      <c r="F134" t="n">
+        <v>587.52</v>
+      </c>
+      <c r="G134" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="H134" t="n">
+        <v>601.5700073242188</v>
+      </c>
+      <c r="I134" t="n">
+        <v>10.38000011444092</v>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K134" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N134" t="n">
+        <v>67.63</v>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>333.93</v>
+      </c>
+      <c r="F135" t="n">
+        <v>309.4</v>
+      </c>
+      <c r="G135" t="n">
+        <v>-7.35</v>
+      </c>
+      <c r="H135" t="n">
+        <v>327.8599853515625</v>
+      </c>
+      <c r="I135" t="n">
+        <v>-1.820000052452087</v>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K135" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N135" t="n">
+        <v>25.98</v>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>379.74</v>
+      </c>
+      <c r="F136" t="n">
+        <v>346.91</v>
+      </c>
+      <c r="G136" t="n">
+        <v>-8.65</v>
+      </c>
+      <c r="H136" t="n">
+        <v>338.510009765625</v>
+      </c>
+      <c r="I136" t="n">
+        <v>-10.85999965667725</v>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K136" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N136" t="n">
+        <v>50.03</v>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>54.54</v>
+      </c>
+      <c r="F137" t="n">
+        <v>57.15</v>
+      </c>
+      <c r="G137" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="H137" t="n">
+        <v>60.36999893188477</v>
+      </c>
+      <c r="I137" t="n">
+        <v>10.6899995803833</v>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K137" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N137" t="n">
+        <v>70.59</v>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>126.54</v>
+      </c>
+      <c r="F138" t="n">
+        <v>123.33</v>
+      </c>
+      <c r="G138" t="n">
+        <v>-2.54</v>
+      </c>
+      <c r="H138" t="n">
+        <v>122.7300033569336</v>
+      </c>
+      <c r="I138" t="n">
+        <v>-3.009999990463257</v>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K138" t="n">
+        <v>0.735</v>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N138" t="n">
+        <v>60.89</v>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>354.61</v>
+      </c>
+      <c r="F139" t="n">
+        <v>407.46</v>
+      </c>
+      <c r="G139" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="H139" t="n">
+        <v>351.4800109863281</v>
+      </c>
+      <c r="I139" t="n">
+        <v>-0.8799999952316284</v>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K139" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N139" t="n">
+        <v>86.55</v>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>941.9299999999999</v>
+      </c>
+      <c r="F140" t="n">
+        <v>925.86</v>
+      </c>
+      <c r="G140" t="n">
+        <v>-1.71</v>
+      </c>
+      <c r="H140" t="n">
+        <v>954.1500244140625</v>
+      </c>
+      <c r="I140" t="n">
+        <v>1.299999952316284</v>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K140" t="n">
+        <v>0.681</v>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N140" t="n">
+        <v>61.06</v>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>143.48</v>
+      </c>
+      <c r="F141" t="n">
+        <v>147.87</v>
+      </c>
+      <c r="G141" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="H141" t="n">
+        <v>141.3699951171875</v>
+      </c>
+      <c r="I141" t="n">
+        <v>-1.470000028610229</v>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K141" t="n">
+        <v>-0.612</v>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N141" t="n">
+        <v>42.35</v>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-15)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O141"/>
+  <dimension ref="A1:O161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9624,6 +9624,1266 @@
       <c r="O141" t="inlineStr">
         <is>
           <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>1458.8</v>
+      </c>
+      <c r="F142" t="n">
+        <v>1648.88</v>
+      </c>
+      <c r="G142" t="n">
+        <v>13.03</v>
+      </c>
+      <c r="H142" t="n">
+        <v>1395.880004882812</v>
+      </c>
+      <c r="I142" t="n">
+        <v>-4.309999942779541</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K142" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N142" t="n">
+        <v>82.54000000000001</v>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>3192.5</v>
+      </c>
+      <c r="F143" t="n">
+        <v>3232.1</v>
+      </c>
+      <c r="G143" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="H143" t="n">
+        <v>3785.639892578125</v>
+      </c>
+      <c r="I143" t="n">
+        <v>18.57999992370605</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K143" t="n">
+        <v>0.888</v>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N143" t="n">
+        <v>69.62</v>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>1599.8</v>
+      </c>
+      <c r="F144" t="n">
+        <v>1625.98</v>
+      </c>
+      <c r="G144" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="H144" t="n">
+        <v>1534.550048828125</v>
+      </c>
+      <c r="I144" t="n">
+        <v>-4.079999923706055</v>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K144" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N144" t="n">
+        <v>62.68</v>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>925.45</v>
+      </c>
+      <c r="F145" t="n">
+        <v>923.16</v>
+      </c>
+      <c r="G145" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="H145" t="n">
+        <v>1035.589965820312</v>
+      </c>
+      <c r="I145" t="n">
+        <v>11.89999961853027</v>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K145" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N145" t="n">
+        <v>59.17</v>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>1418.4</v>
+      </c>
+      <c r="F146" t="n">
+        <v>1343.25</v>
+      </c>
+      <c r="G146" t="n">
+        <v>-5.3</v>
+      </c>
+      <c r="H146" t="n">
+        <v>1404.75</v>
+      </c>
+      <c r="I146" t="n">
+        <v>-0.9599999785423279</v>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K146" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N146" t="n">
+        <v>54.29</v>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>1028.35</v>
+      </c>
+      <c r="F147" t="n">
+        <v>992.53</v>
+      </c>
+      <c r="G147" t="n">
+        <v>-3.48</v>
+      </c>
+      <c r="H147" t="n">
+        <v>1101.9599609375</v>
+      </c>
+      <c r="I147" t="n">
+        <v>7.159999847412109</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K147" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N147" t="n">
+        <v>57.78</v>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>2353.5</v>
+      </c>
+      <c r="F148" t="n">
+        <v>2301.76</v>
+      </c>
+      <c r="G148" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="H148" t="n">
+        <v>2271.64990234375</v>
+      </c>
+      <c r="I148" t="n">
+        <v>-3.480000019073486</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K148" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N148" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>334.75</v>
+      </c>
+      <c r="F149" t="n">
+        <v>356.4</v>
+      </c>
+      <c r="G149" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="H149" t="n">
+        <v>373.1199951171875</v>
+      </c>
+      <c r="I149" t="n">
+        <v>11.46000003814697</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K149" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N149" t="n">
+        <v>55.18</v>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>3865.8</v>
+      </c>
+      <c r="F150" t="n">
+        <v>3906.65</v>
+      </c>
+      <c r="G150" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="H150" t="n">
+        <v>3903.47998046875</v>
+      </c>
+      <c r="I150" t="n">
+        <v>0.9700000286102295</v>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K150" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N150" t="n">
+        <v>57.95</v>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>945.95</v>
+      </c>
+      <c r="F151" t="n">
+        <v>1017.86</v>
+      </c>
+      <c r="G151" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="H151" t="n">
+        <v>1049.77001953125</v>
+      </c>
+      <c r="I151" t="n">
+        <v>10.97999954223633</v>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K151" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N151" t="n">
+        <v>73.64</v>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>2022.5</v>
+      </c>
+      <c r="F152" t="n">
+        <v>2192.69</v>
+      </c>
+      <c r="G152" t="n">
+        <v>8.41</v>
+      </c>
+      <c r="H152" t="n">
+        <v>1939.5</v>
+      </c>
+      <c r="I152" t="n">
+        <v>-4.099999904632568</v>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K152" t="n">
+        <v>-0.735</v>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N152" t="n">
+        <v>47.92</v>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>2813.9</v>
+      </c>
+      <c r="F153" t="n">
+        <v>2698.86</v>
+      </c>
+      <c r="G153" t="n">
+        <v>-4.09</v>
+      </c>
+      <c r="H153" t="n">
+        <v>2784.669921875</v>
+      </c>
+      <c r="I153" t="n">
+        <v>-1.039999961853027</v>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K153" t="n">
+        <v>-0.459</v>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N153" t="n">
+        <v>34.69</v>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>1298.8</v>
+      </c>
+      <c r="F154" t="n">
+        <v>1215.26</v>
+      </c>
+      <c r="G154" t="n">
+        <v>-6.43</v>
+      </c>
+      <c r="H154" t="n">
+        <v>1417</v>
+      </c>
+      <c r="I154" t="n">
+        <v>9.100000381469727</v>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K154" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N154" t="n">
+        <v>55.91</v>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>16152</v>
+      </c>
+      <c r="F155" t="n">
+        <v>18420.98</v>
+      </c>
+      <c r="G155" t="n">
+        <v>14.05</v>
+      </c>
+      <c r="H155" t="n">
+        <v>19509.30078125</v>
+      </c>
+      <c r="I155" t="n">
+        <v>20.79000091552734</v>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K155" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N155" t="n">
+        <v>84.06999999999999</v>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>1700.7</v>
+      </c>
+      <c r="F156" t="n">
+        <v>1801.71</v>
+      </c>
+      <c r="G156" t="n">
+        <v>5.94</v>
+      </c>
+      <c r="H156" t="n">
+        <v>1726.900024414062</v>
+      </c>
+      <c r="I156" t="n">
+        <v>1.539999961853027</v>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K156" t="n">
+        <v>0.8129999999999999</v>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N156" t="n">
+        <v>75.17</v>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>260.2</v>
+      </c>
+      <c r="F157" t="n">
+        <v>276.17</v>
+      </c>
+      <c r="G157" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="H157" t="n">
+        <v>247.5099945068359</v>
+      </c>
+      <c r="I157" t="n">
+        <v>-4.880000114440918</v>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K157" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N157" t="n">
+        <v>71.70999999999999</v>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>12255</v>
+      </c>
+      <c r="F158" t="n">
+        <v>11660.63</v>
+      </c>
+      <c r="G158" t="n">
+        <v>-4.85</v>
+      </c>
+      <c r="H158" t="n">
+        <v>11343.1201171875</v>
+      </c>
+      <c r="I158" t="n">
+        <v>-7.440000057220459</v>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K158" t="n">
+        <v>-0.625</v>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N158" t="n">
+        <v>30.23</v>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>349.1</v>
+      </c>
+      <c r="F159" t="n">
+        <v>332.16</v>
+      </c>
+      <c r="G159" t="n">
+        <v>-4.85</v>
+      </c>
+      <c r="H159" t="n">
+        <v>355.1400146484375</v>
+      </c>
+      <c r="I159" t="n">
+        <v>1.730000019073486</v>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K159" t="n">
+        <v>0.718</v>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N159" t="n">
+        <v>57.08</v>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>258.35</v>
+      </c>
+      <c r="F160" t="n">
+        <v>255.74</v>
+      </c>
+      <c r="G160" t="n">
+        <v>-1.01</v>
+      </c>
+      <c r="H160" t="n">
+        <v>253.3600006103516</v>
+      </c>
+      <c r="I160" t="n">
+        <v>-1.929999947547913</v>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K160" t="n">
+        <v>-0.625</v>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N160" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>4221.5</v>
+      </c>
+      <c r="F161" t="n">
+        <v>4062.59</v>
+      </c>
+      <c r="G161" t="n">
+        <v>-3.76</v>
+      </c>
+      <c r="H161" t="n">
+        <v>4095.39990234375</v>
+      </c>
+      <c r="I161" t="n">
+        <v>-2.990000009536743</v>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K161" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N161" t="n">
+        <v>60.27</v>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
         </is>
       </c>
     </row>
@@ -9638,7 +10898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O71"/>
+  <dimension ref="A1:O81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14265,6 +15525,636 @@
       <c r="O71" t="inlineStr">
         <is>
           <t>14 Jan 2026, 06:54:40 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1458.45</v>
+      </c>
+      <c r="F72" t="n">
+        <v>1652.83</v>
+      </c>
+      <c r="G72" t="n">
+        <v>13.33</v>
+      </c>
+      <c r="H72" t="n">
+        <v>1439.119995117188</v>
+      </c>
+      <c r="I72" t="n">
+        <v>-1.330000042915344</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K72" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N72" t="n">
+        <v>82.98999999999999</v>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>3192.3</v>
+      </c>
+      <c r="F73" t="n">
+        <v>3245.7</v>
+      </c>
+      <c r="G73" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="H73" t="n">
+        <v>3481.919921875</v>
+      </c>
+      <c r="I73" t="n">
+        <v>9.069999694824219</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K73" t="n">
+        <v>0.888</v>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N73" t="n">
+        <v>70.27</v>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>1599.05</v>
+      </c>
+      <c r="F74" t="n">
+        <v>1633.24</v>
+      </c>
+      <c r="G74" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="H74" t="n">
+        <v>1824.650024414062</v>
+      </c>
+      <c r="I74" t="n">
+        <v>14.10999965667725</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K74" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N74" t="n">
+        <v>63.43</v>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>926</v>
+      </c>
+      <c r="F75" t="n">
+        <v>925.74</v>
+      </c>
+      <c r="G75" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="H75" t="n">
+        <v>948.4000244140625</v>
+      </c>
+      <c r="I75" t="n">
+        <v>2.420000076293945</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K75" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N75" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>1418.15</v>
+      </c>
+      <c r="F76" t="n">
+        <v>1356.06</v>
+      </c>
+      <c r="G76" t="n">
+        <v>-4.38</v>
+      </c>
+      <c r="H76" t="n">
+        <v>1471.430053710938</v>
+      </c>
+      <c r="I76" t="n">
+        <v>3.759999990463257</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K76" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N76" t="n">
+        <v>55.67</v>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>1028.3</v>
+      </c>
+      <c r="F77" t="n">
+        <v>1002.73</v>
+      </c>
+      <c r="G77" t="n">
+        <v>-2.49</v>
+      </c>
+      <c r="H77" t="n">
+        <v>1083.75</v>
+      </c>
+      <c r="I77" t="n">
+        <v>5.389999866485596</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K77" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N77" t="n">
+        <v>59.27</v>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>334.75</v>
+      </c>
+      <c r="F78" t="n">
+        <v>360.23</v>
+      </c>
+      <c r="G78" t="n">
+        <v>7.61</v>
+      </c>
+      <c r="H78" t="n">
+        <v>376.6099853515625</v>
+      </c>
+      <c r="I78" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K78" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N78" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>3865.5</v>
+      </c>
+      <c r="F79" t="n">
+        <v>3917.75</v>
+      </c>
+      <c r="G79" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="H79" t="n">
+        <v>3785.199951171875</v>
+      </c>
+      <c r="I79" t="n">
+        <v>-2.079999923706055</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K79" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N79" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>1298.5</v>
+      </c>
+      <c r="F80" t="n">
+        <v>1225.95</v>
+      </c>
+      <c r="G80" t="n">
+        <v>-5.59</v>
+      </c>
+      <c r="H80" t="n">
+        <v>1043.390014648438</v>
+      </c>
+      <c r="I80" t="n">
+        <v>-19.64999961853027</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K80" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N80" t="n">
+        <v>57.18</v>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>16144.05</v>
+      </c>
+      <c r="F81" t="n">
+        <v>18501.09</v>
+      </c>
+      <c r="G81" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="H81" t="n">
+        <v>16896.76953125</v>
+      </c>
+      <c r="I81" t="n">
+        <v>4.659999847412109</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K81" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N81" t="n">
+        <v>84.90000000000001</v>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
         </is>
       </c>
     </row>
@@ -14279,7 +16169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O141"/>
+  <dimension ref="A1:O161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23459,6 +25349,1266 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>259.96</v>
+      </c>
+      <c r="F142" t="n">
+        <v>285.03</v>
+      </c>
+      <c r="G142" t="n">
+        <v>9.65</v>
+      </c>
+      <c r="H142" t="n">
+        <v>335.2699890136719</v>
+      </c>
+      <c r="I142" t="n">
+        <v>28.96999931335449</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K142" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N142" t="n">
+        <v>77.67</v>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>459.38</v>
+      </c>
+      <c r="F143" t="n">
+        <v>475.12</v>
+      </c>
+      <c r="G143" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="H143" t="n">
+        <v>480.5400085449219</v>
+      </c>
+      <c r="I143" t="n">
+        <v>4.610000133514404</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K143" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N143" t="n">
+        <v>61.06</v>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>335.84</v>
+      </c>
+      <c r="F144" t="n">
+        <v>356.67</v>
+      </c>
+      <c r="G144" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="H144" t="n">
+        <v>343.9299926757812</v>
+      </c>
+      <c r="I144" t="n">
+        <v>2.410000085830688</v>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K144" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N144" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>236.65</v>
+      </c>
+      <c r="F145" t="n">
+        <v>254.01</v>
+      </c>
+      <c r="G145" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="H145" t="n">
+        <v>229.6399993896484</v>
+      </c>
+      <c r="I145" t="n">
+        <v>-2.960000038146973</v>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K145" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N145" t="n">
+        <v>72.14</v>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>615.52</v>
+      </c>
+      <c r="F146" t="n">
+        <v>723.89</v>
+      </c>
+      <c r="G146" t="n">
+        <v>17.61</v>
+      </c>
+      <c r="H146" t="n">
+        <v>692.6900024414062</v>
+      </c>
+      <c r="I146" t="n">
+        <v>12.53999996185303</v>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K146" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N146" t="n">
+        <v>63.41</v>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>439.2</v>
+      </c>
+      <c r="F147" t="n">
+        <v>448.91</v>
+      </c>
+      <c r="G147" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="H147" t="n">
+        <v>300.239990234375</v>
+      </c>
+      <c r="I147" t="n">
+        <v>-31.63999938964844</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K147" t="n">
+        <v>-0.637</v>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N147" t="n">
+        <v>40.58</v>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>183.14</v>
+      </c>
+      <c r="F148" t="n">
+        <v>202.11</v>
+      </c>
+      <c r="G148" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="H148" t="n">
+        <v>204.1799926757812</v>
+      </c>
+      <c r="I148" t="n">
+        <v>11.48999977111816</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K148" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N148" t="n">
+        <v>78.73999999999999</v>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>307.87</v>
+      </c>
+      <c r="F149" t="n">
+        <v>343.59</v>
+      </c>
+      <c r="G149" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H149" t="n">
+        <v>335.0400085449219</v>
+      </c>
+      <c r="I149" t="n">
+        <v>8.819999694824219</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K149" t="n">
+        <v>0</v>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N149" t="n">
+        <v>67.41</v>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>329.17</v>
+      </c>
+      <c r="F150" t="n">
+        <v>357.67</v>
+      </c>
+      <c r="G150" t="n">
+        <v>8.66</v>
+      </c>
+      <c r="H150" t="n">
+        <v>331.4100036621094</v>
+      </c>
+      <c r="I150" t="n">
+        <v>0.6800000071525574</v>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K150" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N150" t="n">
+        <v>76.19</v>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>218.55</v>
+      </c>
+      <c r="F151" t="n">
+        <v>220.2</v>
+      </c>
+      <c r="G151" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="H151" t="n">
+        <v>240.7899932861328</v>
+      </c>
+      <c r="I151" t="n">
+        <v>10.18000030517578</v>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K151" t="n">
+        <v>0</v>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N151" t="n">
+        <v>51.14</v>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>120.04</v>
+      </c>
+      <c r="F152" t="n">
+        <v>118.79</v>
+      </c>
+      <c r="G152" t="n">
+        <v>-1.04</v>
+      </c>
+      <c r="H152" t="n">
+        <v>109.9300003051758</v>
+      </c>
+      <c r="I152" t="n">
+        <v>-8.420000076293945</v>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K152" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N152" t="n">
+        <v>61.43</v>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>146.35</v>
+      </c>
+      <c r="F153" t="n">
+        <v>143.86</v>
+      </c>
+      <c r="G153" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="H153" t="n">
+        <v>148.3699951171875</v>
+      </c>
+      <c r="I153" t="n">
+        <v>1.379999995231628</v>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K153" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N153" t="n">
+        <v>53.36</v>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>546.8200000000001</v>
+      </c>
+      <c r="F154" t="n">
+        <v>585.6799999999999</v>
+      </c>
+      <c r="G154" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="H154" t="n">
+        <v>600.0800170898438</v>
+      </c>
+      <c r="I154" t="n">
+        <v>9.739999771118164</v>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K154" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N154" t="n">
+        <v>66.58</v>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>334.96</v>
+      </c>
+      <c r="F155" t="n">
+        <v>311.31</v>
+      </c>
+      <c r="G155" t="n">
+        <v>-7.06</v>
+      </c>
+      <c r="H155" t="n">
+        <v>378.8200073242188</v>
+      </c>
+      <c r="I155" t="n">
+        <v>13.09000015258789</v>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K155" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N155" t="n">
+        <v>50.85</v>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>375.95</v>
+      </c>
+      <c r="F156" t="n">
+        <v>348.4</v>
+      </c>
+      <c r="G156" t="n">
+        <v>-7.33</v>
+      </c>
+      <c r="H156" t="n">
+        <v>452.239990234375</v>
+      </c>
+      <c r="I156" t="n">
+        <v>20.29000091552734</v>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K156" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N156" t="n">
+        <v>47.05</v>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>52.48</v>
+      </c>
+      <c r="F157" t="n">
+        <v>57.18</v>
+      </c>
+      <c r="G157" t="n">
+        <v>8.949999999999999</v>
+      </c>
+      <c r="H157" t="n">
+        <v>52.40000152587891</v>
+      </c>
+      <c r="I157" t="n">
+        <v>-0.1599999964237213</v>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K157" t="n">
+        <v>0</v>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N157" t="n">
+        <v>63.42</v>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>130.2</v>
+      </c>
+      <c r="F158" t="n">
+        <v>123.88</v>
+      </c>
+      <c r="G158" t="n">
+        <v>-4.85</v>
+      </c>
+      <c r="H158" t="n">
+        <v>134.7700042724609</v>
+      </c>
+      <c r="I158" t="n">
+        <v>3.509999990463257</v>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K158" t="n">
+        <v>0.735</v>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N158" t="n">
+        <v>57.42</v>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>339.89</v>
+      </c>
+      <c r="F159" t="n">
+        <v>403.9</v>
+      </c>
+      <c r="G159" t="n">
+        <v>18.83</v>
+      </c>
+      <c r="H159" t="n">
+        <v>423.7300109863281</v>
+      </c>
+      <c r="I159" t="n">
+        <v>24.67000007629395</v>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K159" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N159" t="n">
+        <v>92.45</v>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>950.98</v>
+      </c>
+      <c r="F160" t="n">
+        <v>931.52</v>
+      </c>
+      <c r="G160" t="n">
+        <v>-2.05</v>
+      </c>
+      <c r="H160" t="n">
+        <v>830.2899780273438</v>
+      </c>
+      <c r="I160" t="n">
+        <v>-12.6899995803833</v>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K160" t="n">
+        <v>0.751</v>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N160" t="n">
+        <v>61.95</v>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>145.92</v>
+      </c>
+      <c r="F161" t="n">
+        <v>147.62</v>
+      </c>
+      <c r="G161" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="H161" t="n">
+        <v>142.3800048828125</v>
+      </c>
+      <c r="I161" t="n">
+        <v>-2.430000066757202</v>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K161" t="n">
+        <v>-0.612</v>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N161" t="n">
+        <v>39.51</v>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-16)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O161"/>
+  <dimension ref="A1:O181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10884,6 +10884,1266 @@
       <c r="O161" t="inlineStr">
         <is>
           <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>1458.8</v>
+      </c>
+      <c r="F162" t="n">
+        <v>1647.99</v>
+      </c>
+      <c r="G162" t="n">
+        <v>12.97</v>
+      </c>
+      <c r="H162" t="n">
+        <v>1331.430053710938</v>
+      </c>
+      <c r="I162" t="n">
+        <v>-8.729999542236328</v>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K162" t="n">
+        <v>0.526</v>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N162" t="n">
+        <v>79.97</v>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>3192.5</v>
+      </c>
+      <c r="F163" t="n">
+        <v>3238.01</v>
+      </c>
+      <c r="G163" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="H163" t="n">
+        <v>3353.949951171875</v>
+      </c>
+      <c r="I163" t="n">
+        <v>5.059999942779541</v>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K163" t="n">
+        <v>0.888</v>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N163" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>1599.8</v>
+      </c>
+      <c r="F164" t="n">
+        <v>1617.33</v>
+      </c>
+      <c r="G164" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H164" t="n">
+        <v>1381.869995117188</v>
+      </c>
+      <c r="I164" t="n">
+        <v>-13.61999988555908</v>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K164" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N164" t="n">
+        <v>64.84</v>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>925.45</v>
+      </c>
+      <c r="F165" t="n">
+        <v>923.4299999999999</v>
+      </c>
+      <c r="G165" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="H165" t="n">
+        <v>928.5999755859375</v>
+      </c>
+      <c r="I165" t="n">
+        <v>0.3400000035762787</v>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K165" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N165" t="n">
+        <v>65.34999999999999</v>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>1418.4</v>
+      </c>
+      <c r="F166" t="n">
+        <v>1345.57</v>
+      </c>
+      <c r="G166" t="n">
+        <v>-5.13</v>
+      </c>
+      <c r="H166" t="n">
+        <v>1359.619995117188</v>
+      </c>
+      <c r="I166" t="n">
+        <v>-4.139999866485596</v>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K166" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N166" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>1028.35</v>
+      </c>
+      <c r="F167" t="n">
+        <v>995.0700000000001</v>
+      </c>
+      <c r="G167" t="n">
+        <v>-3.24</v>
+      </c>
+      <c r="H167" t="n">
+        <v>1182.31005859375</v>
+      </c>
+      <c r="I167" t="n">
+        <v>14.97000026702881</v>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K167" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N167" t="n">
+        <v>54.68</v>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>2353.5</v>
+      </c>
+      <c r="F168" t="n">
+        <v>2299.71</v>
+      </c>
+      <c r="G168" t="n">
+        <v>-2.29</v>
+      </c>
+      <c r="H168" t="n">
+        <v>2503.320068359375</v>
+      </c>
+      <c r="I168" t="n">
+        <v>6.369999885559082</v>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K168" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N168" t="n">
+        <v>59.07</v>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>334.75</v>
+      </c>
+      <c r="F169" t="n">
+        <v>356.46</v>
+      </c>
+      <c r="G169" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="H169" t="n">
+        <v>375.25</v>
+      </c>
+      <c r="I169" t="n">
+        <v>12.10000038146973</v>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K169" t="n">
+        <v>-0.547</v>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N169" t="n">
+        <v>48.79</v>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>3865.8</v>
+      </c>
+      <c r="F170" t="n">
+        <v>3904.76</v>
+      </c>
+      <c r="G170" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="H170" t="n">
+        <v>3949.699951171875</v>
+      </c>
+      <c r="I170" t="n">
+        <v>2.170000076293945</v>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K170" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N170" t="n">
+        <v>64.70999999999999</v>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>945.95</v>
+      </c>
+      <c r="F171" t="n">
+        <v>1017.68</v>
+      </c>
+      <c r="G171" t="n">
+        <v>7.58</v>
+      </c>
+      <c r="H171" t="n">
+        <v>870.2999877929688</v>
+      </c>
+      <c r="I171" t="n">
+        <v>-8</v>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K171" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N171" t="n">
+        <v>74.37</v>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>2022.5</v>
+      </c>
+      <c r="F172" t="n">
+        <v>2195.32</v>
+      </c>
+      <c r="G172" t="n">
+        <v>8.550000000000001</v>
+      </c>
+      <c r="H172" t="n">
+        <v>2027.780029296875</v>
+      </c>
+      <c r="I172" t="n">
+        <v>0.2599999904632568</v>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K172" t="n">
+        <v>-0.318</v>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N172" t="n">
+        <v>56.46</v>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>2813.9</v>
+      </c>
+      <c r="F173" t="n">
+        <v>2729.67</v>
+      </c>
+      <c r="G173" t="n">
+        <v>-2.99</v>
+      </c>
+      <c r="H173" t="n">
+        <v>2751.989990234375</v>
+      </c>
+      <c r="I173" t="n">
+        <v>-2.200000047683716</v>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K173" t="n">
+        <v>0.727</v>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N173" t="n">
+        <v>60.05</v>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>1298.8</v>
+      </c>
+      <c r="F174" t="n">
+        <v>1215.26</v>
+      </c>
+      <c r="G174" t="n">
+        <v>-6.43</v>
+      </c>
+      <c r="H174" t="n">
+        <v>1485.319946289062</v>
+      </c>
+      <c r="I174" t="n">
+        <v>14.35999965667725</v>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K174" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N174" t="n">
+        <v>55.91</v>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>16152</v>
+      </c>
+      <c r="F175" t="n">
+        <v>18421.6</v>
+      </c>
+      <c r="G175" t="n">
+        <v>14.05</v>
+      </c>
+      <c r="H175" t="n">
+        <v>17008.169921875</v>
+      </c>
+      <c r="I175" t="n">
+        <v>5.300000190734863</v>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K175" t="n">
+        <v>0</v>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N175" t="n">
+        <v>71.08</v>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>1700.7</v>
+      </c>
+      <c r="F176" t="n">
+        <v>1810.8</v>
+      </c>
+      <c r="G176" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="H176" t="n">
+        <v>1938.010009765625</v>
+      </c>
+      <c r="I176" t="n">
+        <v>13.94999980926514</v>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K176" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N176" t="n">
+        <v>64.70999999999999</v>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>260.2</v>
+      </c>
+      <c r="F177" t="n">
+        <v>276.17</v>
+      </c>
+      <c r="G177" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="H177" t="n">
+        <v>241.4400024414062</v>
+      </c>
+      <c r="I177" t="n">
+        <v>-7.210000038146973</v>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K177" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N177" t="n">
+        <v>72.20999999999999</v>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>12255</v>
+      </c>
+      <c r="F178" t="n">
+        <v>11629.01</v>
+      </c>
+      <c r="G178" t="n">
+        <v>-5.11</v>
+      </c>
+      <c r="H178" t="n">
+        <v>11322.849609375</v>
+      </c>
+      <c r="I178" t="n">
+        <v>-7.610000133514404</v>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K178" t="n">
+        <v>-0.625</v>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N178" t="n">
+        <v>29.84</v>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E179" t="n">
+        <v>349.1</v>
+      </c>
+      <c r="F179" t="n">
+        <v>330.94</v>
+      </c>
+      <c r="G179" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="H179" t="n">
+        <v>385.3299865722656</v>
+      </c>
+      <c r="I179" t="n">
+        <v>10.38000011444092</v>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K179" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N179" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
+        <v>258.35</v>
+      </c>
+      <c r="F180" t="n">
+        <v>255.86</v>
+      </c>
+      <c r="G180" t="n">
+        <v>-0.96</v>
+      </c>
+      <c r="H180" t="n">
+        <v>257.7799987792969</v>
+      </c>
+      <c r="I180" t="n">
+        <v>-0.2199999988079071</v>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K180" t="n">
+        <v>0.727</v>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N180" t="n">
+        <v>63.09</v>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E181" t="n">
+        <v>4221.5</v>
+      </c>
+      <c r="F181" t="n">
+        <v>4049.06</v>
+      </c>
+      <c r="G181" t="n">
+        <v>-4.08</v>
+      </c>
+      <c r="H181" t="n">
+        <v>3987.580078125</v>
+      </c>
+      <c r="I181" t="n">
+        <v>-5.539999961853027</v>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K181" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N181" t="n">
+        <v>57.27</v>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
         </is>
       </c>
     </row>
@@ -10898,7 +12158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O81"/>
+  <dimension ref="A1:O91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16155,6 +17415,636 @@
       <c r="O81" t="inlineStr">
         <is>
           <t>15 Jan 2026, 06:53:24 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>1458.45</v>
+      </c>
+      <c r="F82" t="n">
+        <v>1652.8</v>
+      </c>
+      <c r="G82" t="n">
+        <v>13.33</v>
+      </c>
+      <c r="H82" t="n">
+        <v>1513.510009765625</v>
+      </c>
+      <c r="I82" t="n">
+        <v>3.769999980926514</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K82" t="n">
+        <v>0.526</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N82" t="n">
+        <v>80.51000000000001</v>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>3192.3</v>
+      </c>
+      <c r="F83" t="n">
+        <v>3235.05</v>
+      </c>
+      <c r="G83" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="H83" t="n">
+        <v>3444.75</v>
+      </c>
+      <c r="I83" t="n">
+        <v>7.909999847412109</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K83" t="n">
+        <v>0.888</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N83" t="n">
+        <v>69.77</v>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>1599.05</v>
+      </c>
+      <c r="F84" t="n">
+        <v>1636.1</v>
+      </c>
+      <c r="G84" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="H84" t="n">
+        <v>1595.160034179688</v>
+      </c>
+      <c r="I84" t="n">
+        <v>-0.239999994635582</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K84" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N84" t="n">
+        <v>66.68000000000001</v>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>926</v>
+      </c>
+      <c r="F85" t="n">
+        <v>927.71</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="H85" t="n">
+        <v>837.1699829101562</v>
+      </c>
+      <c r="I85" t="n">
+        <v>-9.590000152587891</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K85" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N85" t="n">
+        <v>65.95999999999999</v>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>1418.15</v>
+      </c>
+      <c r="F86" t="n">
+        <v>1359.7</v>
+      </c>
+      <c r="G86" t="n">
+        <v>-4.12</v>
+      </c>
+      <c r="H86" t="n">
+        <v>1424.069946289062</v>
+      </c>
+      <c r="I86" t="n">
+        <v>0.4199999868869781</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K86" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N86" t="n">
+        <v>57.22</v>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>1028.3</v>
+      </c>
+      <c r="F87" t="n">
+        <v>1000.12</v>
+      </c>
+      <c r="G87" t="n">
+        <v>-2.74</v>
+      </c>
+      <c r="H87" t="n">
+        <v>1191.170043945312</v>
+      </c>
+      <c r="I87" t="n">
+        <v>15.84000015258789</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K87" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N87" t="n">
+        <v>55.43</v>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>334.75</v>
+      </c>
+      <c r="F88" t="n">
+        <v>359.9</v>
+      </c>
+      <c r="G88" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="H88" t="n">
+        <v>370.4400024414062</v>
+      </c>
+      <c r="I88" t="n">
+        <v>10.65999984741211</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K88" t="n">
+        <v>-0.547</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N88" t="n">
+        <v>50.33</v>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>3865.5</v>
+      </c>
+      <c r="F89" t="n">
+        <v>3917.75</v>
+      </c>
+      <c r="G89" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="H89" t="n">
+        <v>4004.5</v>
+      </c>
+      <c r="I89" t="n">
+        <v>3.599999904632568</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K89" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N89" t="n">
+        <v>65.23</v>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>1298.5</v>
+      </c>
+      <c r="F90" t="n">
+        <v>1223.1</v>
+      </c>
+      <c r="G90" t="n">
+        <v>-5.81</v>
+      </c>
+      <c r="H90" t="n">
+        <v>1324.02001953125</v>
+      </c>
+      <c r="I90" t="n">
+        <v>1.970000028610229</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K90" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N90" t="n">
+        <v>56.85</v>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>16144.05</v>
+      </c>
+      <c r="F91" t="n">
+        <v>18501.09</v>
+      </c>
+      <c r="G91" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="H91" t="n">
+        <v>15929.3896484375</v>
+      </c>
+      <c r="I91" t="n">
+        <v>-1.330000042915344</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N91" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
         </is>
       </c>
     </row>
@@ -16169,7 +18059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O161"/>
+  <dimension ref="A1:O181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26609,6 +28499,1266 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>258.21</v>
+      </c>
+      <c r="F162" t="n">
+        <v>283.44</v>
+      </c>
+      <c r="G162" t="n">
+        <v>9.77</v>
+      </c>
+      <c r="H162" t="n">
+        <v>251.3899993896484</v>
+      </c>
+      <c r="I162" t="n">
+        <v>-2.640000104904175</v>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K162" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N162" t="n">
+        <v>76.37</v>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>456.66</v>
+      </c>
+      <c r="F163" t="n">
+        <v>469.76</v>
+      </c>
+      <c r="G163" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="H163" t="n">
+        <v>505.0799865722656</v>
+      </c>
+      <c r="I163" t="n">
+        <v>10.60000038146973</v>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K163" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N163" t="n">
+        <v>60.22</v>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>332.78</v>
+      </c>
+      <c r="F164" t="n">
+        <v>357.56</v>
+      </c>
+      <c r="G164" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="H164" t="n">
+        <v>356.2999877929688</v>
+      </c>
+      <c r="I164" t="n">
+        <v>7.070000171661377</v>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K164" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N164" t="n">
+        <v>48.17</v>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>238.18</v>
+      </c>
+      <c r="F165" t="n">
+        <v>252.34</v>
+      </c>
+      <c r="G165" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="H165" t="n">
+        <v>217.0899963378906</v>
+      </c>
+      <c r="I165" t="n">
+        <v>-8.850000381469727</v>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K165" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N165" t="n">
+        <v>70.36</v>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>620.8</v>
+      </c>
+      <c r="F166" t="n">
+        <v>715.64</v>
+      </c>
+      <c r="G166" t="n">
+        <v>15.28</v>
+      </c>
+      <c r="H166" t="n">
+        <v>565.8499755859375</v>
+      </c>
+      <c r="I166" t="n">
+        <v>-8.850000381469727</v>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K166" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N166" t="n">
+        <v>83.14</v>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>438.57</v>
+      </c>
+      <c r="F167" t="n">
+        <v>445.99</v>
+      </c>
+      <c r="G167" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="H167" t="n">
+        <v>447.1900024414062</v>
+      </c>
+      <c r="I167" t="n">
+        <v>1.970000028610229</v>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K167" t="n">
+        <v>-0.402</v>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N167" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>187.05</v>
+      </c>
+      <c r="F168" t="n">
+        <v>200.42</v>
+      </c>
+      <c r="G168" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="H168" t="n">
+        <v>164.8699951171875</v>
+      </c>
+      <c r="I168" t="n">
+        <v>-11.85999965667725</v>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K168" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N168" t="n">
+        <v>74.12</v>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>309.26</v>
+      </c>
+      <c r="F169" t="n">
+        <v>342.13</v>
+      </c>
+      <c r="G169" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="H169" t="n">
+        <v>331.1600036621094</v>
+      </c>
+      <c r="I169" t="n">
+        <v>7.079999923706055</v>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K169" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N169" t="n">
+        <v>77.38</v>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>327.75</v>
+      </c>
+      <c r="F170" t="n">
+        <v>355.28</v>
+      </c>
+      <c r="G170" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="H170" t="n">
+        <v>332.2699890136719</v>
+      </c>
+      <c r="I170" t="n">
+        <v>1.379999995231628</v>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K170" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N170" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>219.57</v>
+      </c>
+      <c r="F171" t="n">
+        <v>222.18</v>
+      </c>
+      <c r="G171" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="H171" t="n">
+        <v>263.2999877929688</v>
+      </c>
+      <c r="I171" t="n">
+        <v>19.92000007629395</v>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K171" t="n">
+        <v>0</v>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N171" t="n">
+        <v>51.78</v>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>119.2</v>
+      </c>
+      <c r="F172" t="n">
+        <v>119.99</v>
+      </c>
+      <c r="G172" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="H172" t="n">
+        <v>118.5999984741211</v>
+      </c>
+      <c r="I172" t="n">
+        <v>-0.5099999904632568</v>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K172" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N172" t="n">
+        <v>56.92</v>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>144.63</v>
+      </c>
+      <c r="F173" t="n">
+        <v>143.95</v>
+      </c>
+      <c r="G173" t="n">
+        <v>-0.47</v>
+      </c>
+      <c r="H173" t="n">
+        <v>148.6999969482422</v>
+      </c>
+      <c r="I173" t="n">
+        <v>2.819999933242798</v>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K173" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N173" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>542.65</v>
+      </c>
+      <c r="F174" t="n">
+        <v>579.73</v>
+      </c>
+      <c r="G174" t="n">
+        <v>6.83</v>
+      </c>
+      <c r="H174" t="n">
+        <v>568.3499755859375</v>
+      </c>
+      <c r="I174" t="n">
+        <v>4.739999771118164</v>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K174" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N174" t="n">
+        <v>66.17</v>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>338.96</v>
+      </c>
+      <c r="F175" t="n">
+        <v>319.13</v>
+      </c>
+      <c r="G175" t="n">
+        <v>-5.85</v>
+      </c>
+      <c r="H175" t="n">
+        <v>334.3699951171875</v>
+      </c>
+      <c r="I175" t="n">
+        <v>-1.350000023841858</v>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K175" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N175" t="n">
+        <v>54.62</v>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>379.16</v>
+      </c>
+      <c r="F176" t="n">
+        <v>347.86</v>
+      </c>
+      <c r="G176" t="n">
+        <v>-8.26</v>
+      </c>
+      <c r="H176" t="n">
+        <v>343.5299987792969</v>
+      </c>
+      <c r="I176" t="n">
+        <v>-9.399999618530273</v>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K176" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N176" t="n">
+        <v>50.82</v>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>52.59</v>
+      </c>
+      <c r="F177" t="n">
+        <v>56.96</v>
+      </c>
+      <c r="G177" t="n">
+        <v>8.31</v>
+      </c>
+      <c r="H177" t="n">
+        <v>61.54000091552734</v>
+      </c>
+      <c r="I177" t="n">
+        <v>17.01000022888184</v>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K177" t="n">
+        <v>0.649</v>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N177" t="n">
+        <v>75.44</v>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>129.13</v>
+      </c>
+      <c r="F178" t="n">
+        <v>125.61</v>
+      </c>
+      <c r="G178" t="n">
+        <v>-2.73</v>
+      </c>
+      <c r="H178" t="n">
+        <v>134.7599945068359</v>
+      </c>
+      <c r="I178" t="n">
+        <v>4.360000133514404</v>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K178" t="n">
+        <v>0.735</v>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N178" t="n">
+        <v>60.61</v>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E179" t="n">
+        <v>343.02</v>
+      </c>
+      <c r="F179" t="n">
+        <v>401.27</v>
+      </c>
+      <c r="G179" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="H179" t="n">
+        <v>311.1199951171875</v>
+      </c>
+      <c r="I179" t="n">
+        <v>-9.300000190734863</v>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K179" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N179" t="n">
+        <v>89.67</v>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
+        <v>956.75</v>
+      </c>
+      <c r="F180" t="n">
+        <v>934.54</v>
+      </c>
+      <c r="G180" t="n">
+        <v>-2.32</v>
+      </c>
+      <c r="H180" t="n">
+        <v>941.3400268554688</v>
+      </c>
+      <c r="I180" t="n">
+        <v>-1.610000014305115</v>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K180" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N180" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E181" t="n">
+        <v>146.57</v>
+      </c>
+      <c r="F181" t="n">
+        <v>148.17</v>
+      </c>
+      <c r="G181" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="H181" t="n">
+        <v>138.1799926757812</v>
+      </c>
+      <c r="I181" t="n">
+        <v>-5.71999979019165</v>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K181" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N181" t="n">
+        <v>63.36</v>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-17)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O181"/>
+  <dimension ref="A1:O201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12144,6 +12144,1266 @@
       <c r="O181" t="inlineStr">
         <is>
           <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>1457.9</v>
+      </c>
+      <c r="F182" t="n">
+        <v>1638.48</v>
+      </c>
+      <c r="G182" t="n">
+        <v>12.39</v>
+      </c>
+      <c r="H182" t="n">
+        <v>1404.280029296875</v>
+      </c>
+      <c r="I182" t="n">
+        <v>-3.680000066757202</v>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K182" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N182" t="n">
+        <v>77.38</v>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E183" t="n">
+        <v>3206.7</v>
+      </c>
+      <c r="F183" t="n">
+        <v>3178.85</v>
+      </c>
+      <c r="G183" t="n">
+        <v>-0.87</v>
+      </c>
+      <c r="H183" t="n">
+        <v>3203.969970703125</v>
+      </c>
+      <c r="I183" t="n">
+        <v>-0.09000000357627869</v>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K183" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N183" t="n">
+        <v>63.56</v>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E184" t="n">
+        <v>1689.8</v>
+      </c>
+      <c r="F184" t="n">
+        <v>1643.51</v>
+      </c>
+      <c r="G184" t="n">
+        <v>-2.74</v>
+      </c>
+      <c r="H184" t="n">
+        <v>1517.369995117188</v>
+      </c>
+      <c r="I184" t="n">
+        <v>-10.19999980926514</v>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K184" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N184" t="n">
+        <v>58.89</v>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E185" t="n">
+        <v>931.1</v>
+      </c>
+      <c r="F185" t="n">
+        <v>917.9</v>
+      </c>
+      <c r="G185" t="n">
+        <v>-1.42</v>
+      </c>
+      <c r="H185" t="n">
+        <v>1068.160034179688</v>
+      </c>
+      <c r="I185" t="n">
+        <v>14.72000026702881</v>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K185" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N185" t="n">
+        <v>61.87</v>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>1410.8</v>
+      </c>
+      <c r="F186" t="n">
+        <v>1367.06</v>
+      </c>
+      <c r="G186" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="H186" t="n">
+        <v>1469.199951171875</v>
+      </c>
+      <c r="I186" t="n">
+        <v>4.139999866485596</v>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K186" t="n">
+        <v>0.652</v>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N186" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E187" t="n">
+        <v>1042.3</v>
+      </c>
+      <c r="F187" t="n">
+        <v>1013.75</v>
+      </c>
+      <c r="G187" t="n">
+        <v>-2.74</v>
+      </c>
+      <c r="H187" t="n">
+        <v>1064.180053710938</v>
+      </c>
+      <c r="I187" t="n">
+        <v>2.099999904632568</v>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K187" t="n">
+        <v>-0.273</v>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N187" t="n">
+        <v>40.43</v>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E188" t="n">
+        <v>2360.4</v>
+      </c>
+      <c r="F188" t="n">
+        <v>2316.92</v>
+      </c>
+      <c r="G188" t="n">
+        <v>-1.84</v>
+      </c>
+      <c r="H188" t="n">
+        <v>2517.610107421875</v>
+      </c>
+      <c r="I188" t="n">
+        <v>6.659999847412109</v>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K188" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N188" t="n">
+        <v>57.78</v>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E189" t="n">
+        <v>329.2</v>
+      </c>
+      <c r="F189" t="n">
+        <v>352.32</v>
+      </c>
+      <c r="G189" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="H189" t="n">
+        <v>375.8599853515625</v>
+      </c>
+      <c r="I189" t="n">
+        <v>14.17000007629395</v>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K189" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N189" t="n">
+        <v>70.06999999999999</v>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E190" t="n">
+        <v>3856.4</v>
+      </c>
+      <c r="F190" t="n">
+        <v>3889.36</v>
+      </c>
+      <c r="G190" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H190" t="n">
+        <v>3835.949951171875</v>
+      </c>
+      <c r="I190" t="n">
+        <v>-0.5299999713897705</v>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K190" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N190" t="n">
+        <v>64.48</v>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E191" t="n">
+        <v>950.25</v>
+      </c>
+      <c r="F191" t="n">
+        <v>1020.28</v>
+      </c>
+      <c r="G191" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="H191" t="n">
+        <v>862.6799926757812</v>
+      </c>
+      <c r="I191" t="n">
+        <v>-9.220000267028809</v>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K191" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N191" t="n">
+        <v>70.93000000000001</v>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E192" t="n">
+        <v>2016.4</v>
+      </c>
+      <c r="F192" t="n">
+        <v>2177.21</v>
+      </c>
+      <c r="G192" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="H192" t="n">
+        <v>2073.169921875</v>
+      </c>
+      <c r="I192" t="n">
+        <v>2.819999933242798</v>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K192" t="n">
+        <v>-0.318</v>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N192" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E193" t="n">
+        <v>2756.9</v>
+      </c>
+      <c r="F193" t="n">
+        <v>2678.27</v>
+      </c>
+      <c r="G193" t="n">
+        <v>-2.85</v>
+      </c>
+      <c r="H193" t="n">
+        <v>2798.820068359375</v>
+      </c>
+      <c r="I193" t="n">
+        <v>1.519999980926514</v>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K193" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N193" t="n">
+        <v>58.72</v>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>1294.2</v>
+      </c>
+      <c r="F194" t="n">
+        <v>1231.81</v>
+      </c>
+      <c r="G194" t="n">
+        <v>-4.82</v>
+      </c>
+      <c r="H194" t="n">
+        <v>1281.52001953125</v>
+      </c>
+      <c r="I194" t="n">
+        <v>-0.9800000190734863</v>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K194" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N194" t="n">
+        <v>58.33</v>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E195" t="n">
+        <v>15859</v>
+      </c>
+      <c r="F195" t="n">
+        <v>18404.26</v>
+      </c>
+      <c r="G195" t="n">
+        <v>16.05</v>
+      </c>
+      <c r="H195" t="n">
+        <v>18219.26953125</v>
+      </c>
+      <c r="I195" t="n">
+        <v>14.88000011444092</v>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K195" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N195" t="n">
+        <v>81.70999999999999</v>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>1668.9</v>
+      </c>
+      <c r="F196" t="n">
+        <v>1794.92</v>
+      </c>
+      <c r="G196" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="H196" t="n">
+        <v>1498.050048828125</v>
+      </c>
+      <c r="I196" t="n">
+        <v>-10.23999977111816</v>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K196" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N196" t="n">
+        <v>66.33</v>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E197" t="n">
+        <v>267.45</v>
+      </c>
+      <c r="F197" t="n">
+        <v>278.82</v>
+      </c>
+      <c r="G197" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="H197" t="n">
+        <v>228.0899963378906</v>
+      </c>
+      <c r="I197" t="n">
+        <v>-14.72000026702881</v>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K197" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N197" t="n">
+        <v>43.38</v>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>12378</v>
+      </c>
+      <c r="F198" t="n">
+        <v>11685.05</v>
+      </c>
+      <c r="G198" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="H198" t="n">
+        <v>11988.6396484375</v>
+      </c>
+      <c r="I198" t="n">
+        <v>-3.150000095367432</v>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K198" t="n">
+        <v>-0.625</v>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N198" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E199" t="n">
+        <v>346.35</v>
+      </c>
+      <c r="F199" t="n">
+        <v>333.93</v>
+      </c>
+      <c r="G199" t="n">
+        <v>-3.59</v>
+      </c>
+      <c r="H199" t="n">
+        <v>374.4200134277344</v>
+      </c>
+      <c r="I199" t="n">
+        <v>8.100000381469727</v>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K199" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N199" t="n">
+        <v>56.86</v>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>257.3</v>
+      </c>
+      <c r="F200" t="n">
+        <v>254.15</v>
+      </c>
+      <c r="G200" t="n">
+        <v>-1.22</v>
+      </c>
+      <c r="H200" t="n">
+        <v>291.3800048828125</v>
+      </c>
+      <c r="I200" t="n">
+        <v>13.23999977111816</v>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K200" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N200" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E201" t="n">
+        <v>4196.9</v>
+      </c>
+      <c r="F201" t="n">
+        <v>4125.02</v>
+      </c>
+      <c r="G201" t="n">
+        <v>-1.71</v>
+      </c>
+      <c r="H201" t="n">
+        <v>3900.239990234375</v>
+      </c>
+      <c r="I201" t="n">
+        <v>-7.070000171661377</v>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K201" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N201" t="n">
+        <v>60.43</v>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
         </is>
       </c>
     </row>
@@ -12158,7 +13418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O91"/>
+  <dimension ref="A1:O101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18045,6 +19305,636 @@
       <c r="O91" t="inlineStr">
         <is>
           <t>16 Jan 2026, 06:44:03 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>1457.6</v>
+      </c>
+      <c r="F92" t="n">
+        <v>1648.18</v>
+      </c>
+      <c r="G92" t="n">
+        <v>13.07</v>
+      </c>
+      <c r="H92" t="n">
+        <v>1618.469970703125</v>
+      </c>
+      <c r="I92" t="n">
+        <v>11.03999996185303</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K92" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N92" t="n">
+        <v>78.41</v>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>3206.7</v>
+      </c>
+      <c r="F93" t="n">
+        <v>3237.55</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="H93" t="n">
+        <v>3528.56005859375</v>
+      </c>
+      <c r="I93" t="n">
+        <v>10.03999996185303</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K93" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N93" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>1689.4</v>
+      </c>
+      <c r="F94" t="n">
+        <v>1656.56</v>
+      </c>
+      <c r="G94" t="n">
+        <v>-1.94</v>
+      </c>
+      <c r="H94" t="n">
+        <v>1543.890014648438</v>
+      </c>
+      <c r="I94" t="n">
+        <v>-8.609999656677246</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K94" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N94" t="n">
+        <v>60.08</v>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>931.15</v>
+      </c>
+      <c r="F95" t="n">
+        <v>922.13</v>
+      </c>
+      <c r="G95" t="n">
+        <v>-0.97</v>
+      </c>
+      <c r="H95" t="n">
+        <v>886.989990234375</v>
+      </c>
+      <c r="I95" t="n">
+        <v>-4.739999771118164</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K95" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N95" t="n">
+        <v>62.55</v>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>1411.65</v>
+      </c>
+      <c r="F96" t="n">
+        <v>1364.89</v>
+      </c>
+      <c r="G96" t="n">
+        <v>-3.31</v>
+      </c>
+      <c r="H96" t="n">
+        <v>1285.150024414062</v>
+      </c>
+      <c r="I96" t="n">
+        <v>-8.960000038146973</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K96" t="n">
+        <v>0.652</v>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N96" t="n">
+        <v>58.07</v>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>1042.3</v>
+      </c>
+      <c r="F97" t="n">
+        <v>1018.62</v>
+      </c>
+      <c r="G97" t="n">
+        <v>-2.27</v>
+      </c>
+      <c r="H97" t="n">
+        <v>1020.619995117188</v>
+      </c>
+      <c r="I97" t="n">
+        <v>-2.079999923706055</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K97" t="n">
+        <v>-0.273</v>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N97" t="n">
+        <v>41.13</v>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>329.25</v>
+      </c>
+      <c r="F98" t="n">
+        <v>357.03</v>
+      </c>
+      <c r="G98" t="n">
+        <v>8.44</v>
+      </c>
+      <c r="H98" t="n">
+        <v>377.9100036621094</v>
+      </c>
+      <c r="I98" t="n">
+        <v>14.77999973297119</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K98" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N98" t="n">
+        <v>72.19</v>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>3855.9</v>
+      </c>
+      <c r="F99" t="n">
+        <v>3912.67</v>
+      </c>
+      <c r="G99" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="H99" t="n">
+        <v>3697.030029296875</v>
+      </c>
+      <c r="I99" t="n">
+        <v>-4.119999885559082</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K99" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N99" t="n">
+        <v>65.41</v>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>1294.55</v>
+      </c>
+      <c r="F100" t="n">
+        <v>1228.02</v>
+      </c>
+      <c r="G100" t="n">
+        <v>-5.14</v>
+      </c>
+      <c r="H100" t="n">
+        <v>1272</v>
+      </c>
+      <c r="I100" t="n">
+        <v>-1.740000009536743</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K100" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N100" t="n">
+        <v>57.85</v>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>15856.55</v>
+      </c>
+      <c r="F101" t="n">
+        <v>18489.42</v>
+      </c>
+      <c r="G101" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="H101" t="n">
+        <v>12949.7998046875</v>
+      </c>
+      <c r="I101" t="n">
+        <v>-18.32999992370605</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K101" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N101" t="n">
+        <v>82.55</v>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
         </is>
       </c>
     </row>
@@ -18059,7 +19949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O181"/>
+  <dimension ref="A1:O201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29759,6 +31649,1266 @@
         </is>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>255.53</v>
+      </c>
+      <c r="F182" t="n">
+        <v>279.62</v>
+      </c>
+      <c r="G182" t="n">
+        <v>9.43</v>
+      </c>
+      <c r="H182" t="n">
+        <v>268.2900085449219</v>
+      </c>
+      <c r="I182" t="n">
+        <v>5</v>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K182" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N182" t="n">
+        <v>77.34</v>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E183" t="n">
+        <v>459.86</v>
+      </c>
+      <c r="F183" t="n">
+        <v>467.27</v>
+      </c>
+      <c r="G183" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="H183" t="n">
+        <v>456.4200134277344</v>
+      </c>
+      <c r="I183" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K183" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N183" t="n">
+        <v>65.62</v>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E184" t="n">
+        <v>330</v>
+      </c>
+      <c r="F184" t="n">
+        <v>356.86</v>
+      </c>
+      <c r="G184" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="H184" t="n">
+        <v>341.5899963378906</v>
+      </c>
+      <c r="I184" t="n">
+        <v>3.509999990463257</v>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K184" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N184" t="n">
+        <v>77.06999999999999</v>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E185" t="n">
+        <v>239.12</v>
+      </c>
+      <c r="F185" t="n">
+        <v>251.08</v>
+      </c>
+      <c r="G185" t="n">
+        <v>5</v>
+      </c>
+      <c r="H185" t="n">
+        <v>214.1100006103516</v>
+      </c>
+      <c r="I185" t="n">
+        <v>-10.46000003814697</v>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K185" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N185" t="n">
+        <v>73.06</v>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>620.25</v>
+      </c>
+      <c r="F186" t="n">
+        <v>718.6900000000001</v>
+      </c>
+      <c r="G186" t="n">
+        <v>15.87</v>
+      </c>
+      <c r="H186" t="n">
+        <v>587.3400268554688</v>
+      </c>
+      <c r="I186" t="n">
+        <v>-5.309999942779541</v>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K186" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N186" t="n">
+        <v>85.79000000000001</v>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E187" t="n">
+        <v>437.5</v>
+      </c>
+      <c r="F187" t="n">
+        <v>445.22</v>
+      </c>
+      <c r="G187" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="H187" t="n">
+        <v>196.6600036621094</v>
+      </c>
+      <c r="I187" t="n">
+        <v>-55.04999923706055</v>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K187" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N187" t="n">
+        <v>62.53</v>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E188" t="n">
+        <v>186.23</v>
+      </c>
+      <c r="F188" t="n">
+        <v>199.23</v>
+      </c>
+      <c r="G188" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="H188" t="n">
+        <v>160.6799926757812</v>
+      </c>
+      <c r="I188" t="n">
+        <v>-13.72000026702881</v>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K188" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N188" t="n">
+        <v>73.67</v>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E189" t="n">
+        <v>312.47</v>
+      </c>
+      <c r="F189" t="n">
+        <v>340.98</v>
+      </c>
+      <c r="G189" t="n">
+        <v>9.119999999999999</v>
+      </c>
+      <c r="H189" t="n">
+        <v>299.5700073242188</v>
+      </c>
+      <c r="I189" t="n">
+        <v>-4.130000114440918</v>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K189" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N189" t="n">
+        <v>66.23999999999999</v>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E190" t="n">
+        <v>328.3</v>
+      </c>
+      <c r="F190" t="n">
+        <v>354.18</v>
+      </c>
+      <c r="G190" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="H190" t="n">
+        <v>320.2099914550781</v>
+      </c>
+      <c r="I190" t="n">
+        <v>-2.460000038146973</v>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K190" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N190" t="n">
+        <v>67.75</v>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E191" t="n">
+        <v>218.66</v>
+      </c>
+      <c r="F191" t="n">
+        <v>222.84</v>
+      </c>
+      <c r="G191" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="H191" t="n">
+        <v>222.5399932861328</v>
+      </c>
+      <c r="I191" t="n">
+        <v>1.769999980926514</v>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K191" t="n">
+        <v>0</v>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N191" t="n">
+        <v>52.86</v>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E192" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="F192" t="n">
+        <v>120.23</v>
+      </c>
+      <c r="G192" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="H192" t="n">
+        <v>134.3600006103516</v>
+      </c>
+      <c r="I192" t="n">
+        <v>12.23999977111816</v>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K192" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N192" t="n">
+        <v>56.58</v>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E193" t="n">
+        <v>144.53</v>
+      </c>
+      <c r="F193" t="n">
+        <v>144.45</v>
+      </c>
+      <c r="G193" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="H193" t="n">
+        <v>147.5200042724609</v>
+      </c>
+      <c r="I193" t="n">
+        <v>2.069999933242798</v>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K193" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N193" t="n">
+        <v>66.51000000000001</v>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>539.49</v>
+      </c>
+      <c r="F194" t="n">
+        <v>578.49</v>
+      </c>
+      <c r="G194" t="n">
+        <v>7.23</v>
+      </c>
+      <c r="H194" t="n">
+        <v>510.9599914550781</v>
+      </c>
+      <c r="I194" t="n">
+        <v>-5.289999961853027</v>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K194" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N194" t="n">
+        <v>66.76000000000001</v>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E195" t="n">
+        <v>331.02</v>
+      </c>
+      <c r="F195" t="n">
+        <v>320.75</v>
+      </c>
+      <c r="G195" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="H195" t="n">
+        <v>329.4800109863281</v>
+      </c>
+      <c r="I195" t="n">
+        <v>-0.4699999988079071</v>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K195" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N195" t="n">
+        <v>58.75</v>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>380.17</v>
+      </c>
+      <c r="F196" t="n">
+        <v>348.14</v>
+      </c>
+      <c r="G196" t="n">
+        <v>-8.43</v>
+      </c>
+      <c r="H196" t="n">
+        <v>349.7000122070312</v>
+      </c>
+      <c r="I196" t="n">
+        <v>-8.020000457763672</v>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K196" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N196" t="n">
+        <v>50.56</v>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E197" t="n">
+        <v>52.97</v>
+      </c>
+      <c r="F197" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="G197" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="H197" t="n">
+        <v>54.38000106811523</v>
+      </c>
+      <c r="I197" t="n">
+        <v>2.660000085830688</v>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K197" t="n">
+        <v>-0.604</v>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N197" t="n">
+        <v>48.19</v>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>129.89</v>
+      </c>
+      <c r="F198" t="n">
+        <v>125.12</v>
+      </c>
+      <c r="G198" t="n">
+        <v>-3.68</v>
+      </c>
+      <c r="H198" t="n">
+        <v>124.3600006103516</v>
+      </c>
+      <c r="I198" t="n">
+        <v>-4.260000228881836</v>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K198" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N198" t="n">
+        <v>50.41</v>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E199" t="n">
+        <v>351.71</v>
+      </c>
+      <c r="F199" t="n">
+        <v>401.41</v>
+      </c>
+      <c r="G199" t="n">
+        <v>14.13</v>
+      </c>
+      <c r="H199" t="n">
+        <v>369.1199951171875</v>
+      </c>
+      <c r="I199" t="n">
+        <v>4.949999809265137</v>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K199" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N199" t="n">
+        <v>82.34</v>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>963.61</v>
+      </c>
+      <c r="F200" t="n">
+        <v>939.1</v>
+      </c>
+      <c r="G200" t="n">
+        <v>-2.54</v>
+      </c>
+      <c r="H200" t="n">
+        <v>895.1900024414062</v>
+      </c>
+      <c r="I200" t="n">
+        <v>-7.099999904632568</v>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K200" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N200" t="n">
+        <v>56.41</v>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E201" t="n">
+        <v>146.32</v>
+      </c>
+      <c r="F201" t="n">
+        <v>148.49</v>
+      </c>
+      <c r="G201" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="H201" t="n">
+        <v>140.8899993896484</v>
+      </c>
+      <c r="I201" t="n">
+        <v>-3.710000038146973</v>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K201" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N201" t="n">
+        <v>65.43000000000001</v>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-18)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O201"/>
+  <dimension ref="A1:O221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13404,6 +13404,1266 @@
       <c r="O201" t="inlineStr">
         <is>
           <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E202" t="n">
+        <v>1457.9</v>
+      </c>
+      <c r="F202" t="n">
+        <v>1638.05</v>
+      </c>
+      <c r="G202" t="n">
+        <v>12.36</v>
+      </c>
+      <c r="H202" t="n">
+        <v>1494.22998046875</v>
+      </c>
+      <c r="I202" t="n">
+        <v>2.490000009536743</v>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K202" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N202" t="n">
+        <v>81.94</v>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E203" t="n">
+        <v>3206.7</v>
+      </c>
+      <c r="F203" t="n">
+        <v>3182.74</v>
+      </c>
+      <c r="G203" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="H203" t="n">
+        <v>3274.409912109375</v>
+      </c>
+      <c r="I203" t="n">
+        <v>2.109999895095825</v>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K203" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N203" t="n">
+        <v>57.68</v>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E204" t="n">
+        <v>1689.8</v>
+      </c>
+      <c r="F204" t="n">
+        <v>1641.63</v>
+      </c>
+      <c r="G204" t="n">
+        <v>-2.85</v>
+      </c>
+      <c r="H204" t="n">
+        <v>1576.359985351562</v>
+      </c>
+      <c r="I204" t="n">
+        <v>-6.710000038146973</v>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K204" t="n">
+        <v>-0.645</v>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N204" t="n">
+        <v>32.82</v>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E205" t="n">
+        <v>931.1</v>
+      </c>
+      <c r="F205" t="n">
+        <v>919.3099999999999</v>
+      </c>
+      <c r="G205" t="n">
+        <v>-1.27</v>
+      </c>
+      <c r="H205" t="n">
+        <v>963.0999755859375</v>
+      </c>
+      <c r="I205" t="n">
+        <v>3.440000057220459</v>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K205" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N205" t="n">
+        <v>62.1</v>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E206" t="n">
+        <v>1410.8</v>
+      </c>
+      <c r="F206" t="n">
+        <v>1365.09</v>
+      </c>
+      <c r="G206" t="n">
+        <v>-3.24</v>
+      </c>
+      <c r="H206" t="n">
+        <v>1556.280029296875</v>
+      </c>
+      <c r="I206" t="n">
+        <v>10.3100004196167</v>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K206" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N206" t="n">
+        <v>55.02</v>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E207" t="n">
+        <v>1042.3</v>
+      </c>
+      <c r="F207" t="n">
+        <v>1014.88</v>
+      </c>
+      <c r="G207" t="n">
+        <v>-2.63</v>
+      </c>
+      <c r="H207" t="n">
+        <v>1189.849975585938</v>
+      </c>
+      <c r="I207" t="n">
+        <v>14.15999984741211</v>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K207" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N207" t="n">
+        <v>55.93</v>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>2360.4</v>
+      </c>
+      <c r="F208" t="n">
+        <v>2317.61</v>
+      </c>
+      <c r="G208" t="n">
+        <v>-1.81</v>
+      </c>
+      <c r="H208" t="n">
+        <v>2230.68994140625</v>
+      </c>
+      <c r="I208" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K208" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N208" t="n">
+        <v>57.82</v>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E209" t="n">
+        <v>329.2</v>
+      </c>
+      <c r="F209" t="n">
+        <v>354.98</v>
+      </c>
+      <c r="G209" t="n">
+        <v>7.83</v>
+      </c>
+      <c r="H209" t="n">
+        <v>383.1499938964844</v>
+      </c>
+      <c r="I209" t="n">
+        <v>16.38999938964844</v>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K209" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N209" t="n">
+        <v>71.29000000000001</v>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>3856.4</v>
+      </c>
+      <c r="F210" t="n">
+        <v>3889.36</v>
+      </c>
+      <c r="G210" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H210" t="n">
+        <v>3642.199951171875</v>
+      </c>
+      <c r="I210" t="n">
+        <v>-5.550000190734863</v>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K210" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N210" t="n">
+        <v>57.64</v>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>950.25</v>
+      </c>
+      <c r="F211" t="n">
+        <v>1022.27</v>
+      </c>
+      <c r="G211" t="n">
+        <v>7.58</v>
+      </c>
+      <c r="H211" t="n">
+        <v>881.1300048828125</v>
+      </c>
+      <c r="I211" t="n">
+        <v>-7.269999980926514</v>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K211" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N211" t="n">
+        <v>71.25</v>
+      </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>2016.4</v>
+      </c>
+      <c r="F212" t="n">
+        <v>2177.21</v>
+      </c>
+      <c r="G212" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="H212" t="n">
+        <v>2096.570068359375</v>
+      </c>
+      <c r="I212" t="n">
+        <v>3.980000019073486</v>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K212" t="n">
+        <v>-0.318</v>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N212" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E213" t="n">
+        <v>2756.9</v>
+      </c>
+      <c r="F213" t="n">
+        <v>2756.49</v>
+      </c>
+      <c r="G213" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="H213" t="n">
+        <v>2860.219970703125</v>
+      </c>
+      <c r="I213" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K213" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N213" t="n">
+        <v>62.98</v>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>1294.2</v>
+      </c>
+      <c r="F214" t="n">
+        <v>1231.31</v>
+      </c>
+      <c r="G214" t="n">
+        <v>-4.86</v>
+      </c>
+      <c r="H214" t="n">
+        <v>1275.130004882812</v>
+      </c>
+      <c r="I214" t="n">
+        <v>-1.470000028610229</v>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K214" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N214" t="n">
+        <v>54.15</v>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E215" t="n">
+        <v>15859</v>
+      </c>
+      <c r="F215" t="n">
+        <v>18392.46</v>
+      </c>
+      <c r="G215" t="n">
+        <v>15.97</v>
+      </c>
+      <c r="H215" t="n">
+        <v>19957.05078125</v>
+      </c>
+      <c r="I215" t="n">
+        <v>25.84000015258789</v>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K215" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N215" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E216" t="n">
+        <v>1668.9</v>
+      </c>
+      <c r="F216" t="n">
+        <v>1795.06</v>
+      </c>
+      <c r="G216" t="n">
+        <v>7.56</v>
+      </c>
+      <c r="H216" t="n">
+        <v>1704.760009765625</v>
+      </c>
+      <c r="I216" t="n">
+        <v>2.150000095367432</v>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K216" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N216" t="n">
+        <v>66.34</v>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E217" t="n">
+        <v>267.45</v>
+      </c>
+      <c r="F217" t="n">
+        <v>278.92</v>
+      </c>
+      <c r="G217" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="H217" t="n">
+        <v>244.3999938964844</v>
+      </c>
+      <c r="I217" t="n">
+        <v>-8.619999885559082</v>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K217" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N217" t="n">
+        <v>69.43000000000001</v>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E218" t="n">
+        <v>12378</v>
+      </c>
+      <c r="F218" t="n">
+        <v>11713.83</v>
+      </c>
+      <c r="G218" t="n">
+        <v>-5.37</v>
+      </c>
+      <c r="H218" t="n">
+        <v>11667.6201171875</v>
+      </c>
+      <c r="I218" t="n">
+        <v>-5.739999771118164</v>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K218" t="n">
+        <v>-0.625</v>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N218" t="n">
+        <v>29.45</v>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E219" t="n">
+        <v>346.35</v>
+      </c>
+      <c r="F219" t="n">
+        <v>332.54</v>
+      </c>
+      <c r="G219" t="n">
+        <v>-3.99</v>
+      </c>
+      <c r="H219" t="n">
+        <v>350.7900085449219</v>
+      </c>
+      <c r="I219" t="n">
+        <v>1.279999971389771</v>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K219" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N219" t="n">
+        <v>57.22</v>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E220" t="n">
+        <v>257.3</v>
+      </c>
+      <c r="F220" t="n">
+        <v>254.53</v>
+      </c>
+      <c r="G220" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="H220" t="n">
+        <v>264.1400146484375</v>
+      </c>
+      <c r="I220" t="n">
+        <v>2.660000085830688</v>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K220" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N220" t="n">
+        <v>63.83</v>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E221" t="n">
+        <v>4196.9</v>
+      </c>
+      <c r="F221" t="n">
+        <v>4127.81</v>
+      </c>
+      <c r="G221" t="n">
+        <v>-1.65</v>
+      </c>
+      <c r="H221" t="n">
+        <v>3808.469970703125</v>
+      </c>
+      <c r="I221" t="n">
+        <v>-9.260000228881836</v>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K221" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N221" t="n">
+        <v>60.53</v>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
         </is>
       </c>
     </row>
@@ -13418,7 +14678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O101"/>
+  <dimension ref="A1:O111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19935,6 +21195,636 @@
       <c r="O101" t="inlineStr">
         <is>
           <t>17 Jan 2026, 06:37:44 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>1457.6</v>
+      </c>
+      <c r="F102" t="n">
+        <v>1646.13</v>
+      </c>
+      <c r="G102" t="n">
+        <v>12.93</v>
+      </c>
+      <c r="H102" t="n">
+        <v>1223.56005859375</v>
+      </c>
+      <c r="I102" t="n">
+        <v>-16.05999946594238</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K102" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N102" t="n">
+        <v>82.8</v>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>3206.7</v>
+      </c>
+      <c r="F103" t="n">
+        <v>3243.97</v>
+      </c>
+      <c r="G103" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="H103" t="n">
+        <v>3340.52001953125</v>
+      </c>
+      <c r="I103" t="n">
+        <v>4.170000076293945</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K103" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N103" t="n">
+        <v>60.54</v>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>1689.4</v>
+      </c>
+      <c r="F104" t="n">
+        <v>1656.94</v>
+      </c>
+      <c r="G104" t="n">
+        <v>-1.92</v>
+      </c>
+      <c r="H104" t="n">
+        <v>1812.089965820312</v>
+      </c>
+      <c r="I104" t="n">
+        <v>7.260000228881836</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K104" t="n">
+        <v>-0.645</v>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N104" t="n">
+        <v>34.22</v>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>931.15</v>
+      </c>
+      <c r="F105" t="n">
+        <v>920.36</v>
+      </c>
+      <c r="G105" t="n">
+        <v>-1.16</v>
+      </c>
+      <c r="H105" t="n">
+        <v>839</v>
+      </c>
+      <c r="I105" t="n">
+        <v>-9.899999618530273</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K105" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N105" t="n">
+        <v>62.26</v>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>1411.65</v>
+      </c>
+      <c r="F106" t="n">
+        <v>1364.89</v>
+      </c>
+      <c r="G106" t="n">
+        <v>-3.31</v>
+      </c>
+      <c r="H106" t="n">
+        <v>1394.800048828125</v>
+      </c>
+      <c r="I106" t="n">
+        <v>-1.190000057220459</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K106" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N106" t="n">
+        <v>54.91</v>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>1042.3</v>
+      </c>
+      <c r="F107" t="n">
+        <v>1020.64</v>
+      </c>
+      <c r="G107" t="n">
+        <v>-2.08</v>
+      </c>
+      <c r="H107" t="n">
+        <v>1115.589965820312</v>
+      </c>
+      <c r="I107" t="n">
+        <v>7.03000020980835</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K107" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N107" t="n">
+        <v>56.76</v>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>329.25</v>
+      </c>
+      <c r="F108" t="n">
+        <v>356.85</v>
+      </c>
+      <c r="G108" t="n">
+        <v>8.380000000000001</v>
+      </c>
+      <c r="H108" t="n">
+        <v>373.989990234375</v>
+      </c>
+      <c r="I108" t="n">
+        <v>13.59000015258789</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K108" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N108" t="n">
+        <v>72.11</v>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>3855.9</v>
+      </c>
+      <c r="F109" t="n">
+        <v>3910.24</v>
+      </c>
+      <c r="G109" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="H109" t="n">
+        <v>3774.31005859375</v>
+      </c>
+      <c r="I109" t="n">
+        <v>-2.119999885559082</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K109" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N109" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>1294.55</v>
+      </c>
+      <c r="F110" t="n">
+        <v>1236.54</v>
+      </c>
+      <c r="G110" t="n">
+        <v>-4.48</v>
+      </c>
+      <c r="H110" t="n">
+        <v>1306.609985351562</v>
+      </c>
+      <c r="I110" t="n">
+        <v>0.9300000071525574</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K110" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N110" t="n">
+        <v>54.72</v>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>15856.55</v>
+      </c>
+      <c r="F111" t="n">
+        <v>18530.09</v>
+      </c>
+      <c r="G111" t="n">
+        <v>16.86</v>
+      </c>
+      <c r="H111" t="n">
+        <v>15697.3896484375</v>
+      </c>
+      <c r="I111" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K111" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N111" t="n">
+        <v>82.93000000000001</v>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
         </is>
       </c>
     </row>
@@ -19949,7 +21839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O201"/>
+  <dimension ref="A1:O221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32909,6 +34799,1266 @@
         </is>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E202" t="n">
+        <v>255.53</v>
+      </c>
+      <c r="F202" t="n">
+        <v>282</v>
+      </c>
+      <c r="G202" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="H202" t="n">
+        <v>249.8300018310547</v>
+      </c>
+      <c r="I202" t="n">
+        <v>-2.230000019073486</v>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K202" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N202" t="n">
+        <v>78.73999999999999</v>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E203" t="n">
+        <v>459.86</v>
+      </c>
+      <c r="F203" t="n">
+        <v>467.88</v>
+      </c>
+      <c r="G203" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="H203" t="n">
+        <v>411.4800109863281</v>
+      </c>
+      <c r="I203" t="n">
+        <v>-10.52000045776367</v>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K203" t="n">
+        <v>0.635</v>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N203" t="n">
+        <v>65.31999999999999</v>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E204" t="n">
+        <v>330</v>
+      </c>
+      <c r="F204" t="n">
+        <v>356.88</v>
+      </c>
+      <c r="G204" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="H204" t="n">
+        <v>322.5599975585938</v>
+      </c>
+      <c r="I204" t="n">
+        <v>-2.259999990463257</v>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K204" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N204" t="n">
+        <v>75.22</v>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E205" t="n">
+        <v>239.12</v>
+      </c>
+      <c r="F205" t="n">
+        <v>251.08</v>
+      </c>
+      <c r="G205" t="n">
+        <v>5</v>
+      </c>
+      <c r="H205" t="n">
+        <v>210.5700073242188</v>
+      </c>
+      <c r="I205" t="n">
+        <v>-11.9399995803833</v>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K205" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N205" t="n">
+        <v>73.06</v>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E206" t="n">
+        <v>620.25</v>
+      </c>
+      <c r="F206" t="n">
+        <v>709.73</v>
+      </c>
+      <c r="G206" t="n">
+        <v>14.43</v>
+      </c>
+      <c r="H206" t="n">
+        <v>570.1500244140625</v>
+      </c>
+      <c r="I206" t="n">
+        <v>-8.079999923706055</v>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K206" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N206" t="n">
+        <v>84.64</v>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E207" t="n">
+        <v>437.5</v>
+      </c>
+      <c r="F207" t="n">
+        <v>445.22</v>
+      </c>
+      <c r="G207" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="H207" t="n">
+        <v>391.5400085449219</v>
+      </c>
+      <c r="I207" t="n">
+        <v>-10.51000022888184</v>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K207" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N207" t="n">
+        <v>63.79</v>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>186.23</v>
+      </c>
+      <c r="F208" t="n">
+        <v>200.31</v>
+      </c>
+      <c r="G208" t="n">
+        <v>7.56</v>
+      </c>
+      <c r="H208" t="n">
+        <v>167.9700012207031</v>
+      </c>
+      <c r="I208" t="n">
+        <v>-9.810000419616699</v>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K208" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N208" t="n">
+        <v>74.34</v>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E209" t="n">
+        <v>312.47</v>
+      </c>
+      <c r="F209" t="n">
+        <v>341.01</v>
+      </c>
+      <c r="G209" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="H209" t="n">
+        <v>308.6099853515625</v>
+      </c>
+      <c r="I209" t="n">
+        <v>-1.230000019073486</v>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K209" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N209" t="n">
+        <v>69.62</v>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>328.3</v>
+      </c>
+      <c r="F210" t="n">
+        <v>354.22</v>
+      </c>
+      <c r="G210" t="n">
+        <v>7.89</v>
+      </c>
+      <c r="H210" t="n">
+        <v>317.4700012207031</v>
+      </c>
+      <c r="I210" t="n">
+        <v>-3.299999952316284</v>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K210" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N210" t="n">
+        <v>71.72</v>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>218.66</v>
+      </c>
+      <c r="F211" t="n">
+        <v>222.75</v>
+      </c>
+      <c r="G211" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="H211" t="n">
+        <v>226.7799987792969</v>
+      </c>
+      <c r="I211" t="n">
+        <v>3.710000038146973</v>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K211" t="n">
+        <v>0</v>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N211" t="n">
+        <v>52.81</v>
+      </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="F212" t="n">
+        <v>120.28</v>
+      </c>
+      <c r="G212" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="H212" t="n">
+        <v>129.4400024414062</v>
+      </c>
+      <c r="I212" t="n">
+        <v>8.140000343322754</v>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K212" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N212" t="n">
+        <v>56.65</v>
+      </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E213" t="n">
+        <v>144.53</v>
+      </c>
+      <c r="F213" t="n">
+        <v>143.98</v>
+      </c>
+      <c r="G213" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="H213" t="n">
+        <v>150.5299987792969</v>
+      </c>
+      <c r="I213" t="n">
+        <v>4.150000095367432</v>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K213" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N213" t="n">
+        <v>66.03</v>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>539.49</v>
+      </c>
+      <c r="F214" t="n">
+        <v>579.3099999999999</v>
+      </c>
+      <c r="G214" t="n">
+        <v>7.38</v>
+      </c>
+      <c r="H214" t="n">
+        <v>555.75</v>
+      </c>
+      <c r="I214" t="n">
+        <v>3.009999990463257</v>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K214" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N214" t="n">
+        <v>66.98999999999999</v>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E215" t="n">
+        <v>331.02</v>
+      </c>
+      <c r="F215" t="n">
+        <v>317.72</v>
+      </c>
+      <c r="G215" t="n">
+        <v>-4.02</v>
+      </c>
+      <c r="H215" t="n">
+        <v>335.3299865722656</v>
+      </c>
+      <c r="I215" t="n">
+        <v>1.299999952316284</v>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K215" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N215" t="n">
+        <v>57.37</v>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E216" t="n">
+        <v>380.17</v>
+      </c>
+      <c r="F216" t="n">
+        <v>348.32</v>
+      </c>
+      <c r="G216" t="n">
+        <v>-8.380000000000001</v>
+      </c>
+      <c r="H216" t="n">
+        <v>428.25</v>
+      </c>
+      <c r="I216" t="n">
+        <v>12.64999961853027</v>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K216" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N216" t="n">
+        <v>50.63</v>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E217" t="n">
+        <v>52.97</v>
+      </c>
+      <c r="F217" t="n">
+        <v>56.69</v>
+      </c>
+      <c r="G217" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="H217" t="n">
+        <v>60.5099983215332</v>
+      </c>
+      <c r="I217" t="n">
+        <v>14.23999977111816</v>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K217" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N217" t="n">
+        <v>70.40000000000001</v>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E218" t="n">
+        <v>129.89</v>
+      </c>
+      <c r="F218" t="n">
+        <v>125.02</v>
+      </c>
+      <c r="G218" t="n">
+        <v>-3.75</v>
+      </c>
+      <c r="H218" t="n">
+        <v>125.2900009155273</v>
+      </c>
+      <c r="I218" t="n">
+        <v>-3.539999961853027</v>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K218" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N218" t="n">
+        <v>50.3</v>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E219" t="n">
+        <v>351.71</v>
+      </c>
+      <c r="F219" t="n">
+        <v>401.76</v>
+      </c>
+      <c r="G219" t="n">
+        <v>14.23</v>
+      </c>
+      <c r="H219" t="n">
+        <v>376.2099914550781</v>
+      </c>
+      <c r="I219" t="n">
+        <v>6.96999979019165</v>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K219" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N219" t="n">
+        <v>83.59</v>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E220" t="n">
+        <v>963.61</v>
+      </c>
+      <c r="F220" t="n">
+        <v>938.8200000000001</v>
+      </c>
+      <c r="G220" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="H220" t="n">
+        <v>965.239990234375</v>
+      </c>
+      <c r="I220" t="n">
+        <v>0.1700000017881393</v>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K220" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N220" t="n">
+        <v>58.38</v>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E221" t="n">
+        <v>146.32</v>
+      </c>
+      <c r="F221" t="n">
+        <v>148.66</v>
+      </c>
+      <c r="G221" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H221" t="n">
+        <v>146.4499969482422</v>
+      </c>
+      <c r="I221" t="n">
+        <v>0.09000000357627869</v>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K221" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N221" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-19)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O221"/>
+  <dimension ref="A1:O241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14664,6 +14664,1266 @@
       <c r="O221" t="inlineStr">
         <is>
           <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E222" t="n">
+        <v>1457.9</v>
+      </c>
+      <c r="F222" t="n">
+        <v>1638.05</v>
+      </c>
+      <c r="G222" t="n">
+        <v>12.36</v>
+      </c>
+      <c r="H222" t="n">
+        <v>1383.640014648438</v>
+      </c>
+      <c r="I222" t="n">
+        <v>-5.090000152587891</v>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K222" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N222" t="n">
+        <v>82.54000000000001</v>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E223" t="n">
+        <v>3206.7</v>
+      </c>
+      <c r="F223" t="n">
+        <v>3181.81</v>
+      </c>
+      <c r="G223" t="n">
+        <v>-0.78</v>
+      </c>
+      <c r="H223" t="n">
+        <v>3455.340087890625</v>
+      </c>
+      <c r="I223" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K223" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N223" t="n">
+        <v>57.64</v>
+      </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E224" t="n">
+        <v>1689.8</v>
+      </c>
+      <c r="F224" t="n">
+        <v>1646.37</v>
+      </c>
+      <c r="G224" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="H224" t="n">
+        <v>1455.530029296875</v>
+      </c>
+      <c r="I224" t="n">
+        <v>-13.85999965667725</v>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K224" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N224" t="n">
+        <v>59.14</v>
+      </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E225" t="n">
+        <v>931.1</v>
+      </c>
+      <c r="F225" t="n">
+        <v>919.0700000000001</v>
+      </c>
+      <c r="G225" t="n">
+        <v>-1.29</v>
+      </c>
+      <c r="H225" t="n">
+        <v>920.1699829101562</v>
+      </c>
+      <c r="I225" t="n">
+        <v>-1.169999957084656</v>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K225" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N225" t="n">
+        <v>53.98</v>
+      </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E226" t="n">
+        <v>1410.8</v>
+      </c>
+      <c r="F226" t="n">
+        <v>1365.08</v>
+      </c>
+      <c r="G226" t="n">
+        <v>-3.24</v>
+      </c>
+      <c r="H226" t="n">
+        <v>1481.7099609375</v>
+      </c>
+      <c r="I226" t="n">
+        <v>5.03000020980835</v>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K226" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N226" t="n">
+        <v>55.36</v>
+      </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E227" t="n">
+        <v>1042.3</v>
+      </c>
+      <c r="F227" t="n">
+        <v>1013.34</v>
+      </c>
+      <c r="G227" t="n">
+        <v>-2.78</v>
+      </c>
+      <c r="H227" t="n">
+        <v>1193.27001953125</v>
+      </c>
+      <c r="I227" t="n">
+        <v>14.47999954223633</v>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K227" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N227" t="n">
+        <v>53.47</v>
+      </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E228" t="n">
+        <v>2360.4</v>
+      </c>
+      <c r="F228" t="n">
+        <v>2314.3</v>
+      </c>
+      <c r="G228" t="n">
+        <v>-1.95</v>
+      </c>
+      <c r="H228" t="n">
+        <v>2415.35009765625</v>
+      </c>
+      <c r="I228" t="n">
+        <v>2.329999923706055</v>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K228" t="n">
+        <v>0.649</v>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N228" t="n">
+        <v>60.05</v>
+      </c>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E229" t="n">
+        <v>329.2</v>
+      </c>
+      <c r="F229" t="n">
+        <v>350.83</v>
+      </c>
+      <c r="G229" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="H229" t="n">
+        <v>383.6300048828125</v>
+      </c>
+      <c r="I229" t="n">
+        <v>16.53000068664551</v>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K229" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N229" t="n">
+        <v>73.05</v>
+      </c>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E230" t="n">
+        <v>3856.4</v>
+      </c>
+      <c r="F230" t="n">
+        <v>3891.8</v>
+      </c>
+      <c r="G230" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="H230" t="n">
+        <v>3349.89990234375</v>
+      </c>
+      <c r="I230" t="n">
+        <v>-13.13000011444092</v>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K230" t="n">
+        <v>0.542</v>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N230" t="n">
+        <v>62.22</v>
+      </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E231" t="n">
+        <v>950.25</v>
+      </c>
+      <c r="F231" t="n">
+        <v>1020.51</v>
+      </c>
+      <c r="G231" t="n">
+        <v>7.39</v>
+      </c>
+      <c r="H231" t="n">
+        <v>926.9199829101562</v>
+      </c>
+      <c r="I231" t="n">
+        <v>-2.450000047683716</v>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K231" t="n">
+        <v>0.493</v>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N231" t="n">
+        <v>70.95</v>
+      </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E232" t="n">
+        <v>2016.4</v>
+      </c>
+      <c r="F232" t="n">
+        <v>2173.03</v>
+      </c>
+      <c r="G232" t="n">
+        <v>7.77</v>
+      </c>
+      <c r="H232" t="n">
+        <v>2028.2900390625</v>
+      </c>
+      <c r="I232" t="n">
+        <v>0.5899999737739563</v>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K232" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N232" t="n">
+        <v>72.19</v>
+      </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E233" t="n">
+        <v>2756.9</v>
+      </c>
+      <c r="F233" t="n">
+        <v>2728.41</v>
+      </c>
+      <c r="G233" t="n">
+        <v>-1.03</v>
+      </c>
+      <c r="H233" t="n">
+        <v>2660.18994140625</v>
+      </c>
+      <c r="I233" t="n">
+        <v>-3.509999990463257</v>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K233" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N233" t="n">
+        <v>61.45</v>
+      </c>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E234" t="n">
+        <v>1294.2</v>
+      </c>
+      <c r="F234" t="n">
+        <v>1231.31</v>
+      </c>
+      <c r="G234" t="n">
+        <v>-4.86</v>
+      </c>
+      <c r="H234" t="n">
+        <v>1155.68994140625</v>
+      </c>
+      <c r="I234" t="n">
+        <v>-10.69999980926514</v>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K234" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N234" t="n">
+        <v>38.19</v>
+      </c>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E235" t="n">
+        <v>15859</v>
+      </c>
+      <c r="F235" t="n">
+        <v>18404.26</v>
+      </c>
+      <c r="G235" t="n">
+        <v>16.05</v>
+      </c>
+      <c r="H235" t="n">
+        <v>17913.8203125</v>
+      </c>
+      <c r="I235" t="n">
+        <v>12.96000003814697</v>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K235" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N235" t="n">
+        <v>87.06999999999999</v>
+      </c>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E236" t="n">
+        <v>1668.9</v>
+      </c>
+      <c r="F236" t="n">
+        <v>1796.02</v>
+      </c>
+      <c r="G236" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="H236" t="n">
+        <v>1715.2099609375</v>
+      </c>
+      <c r="I236" t="n">
+        <v>2.779999971389771</v>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K236" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N236" t="n">
+        <v>74.43000000000001</v>
+      </c>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E237" t="n">
+        <v>267.45</v>
+      </c>
+      <c r="F237" t="n">
+        <v>278.38</v>
+      </c>
+      <c r="G237" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="H237" t="n">
+        <v>271.8299865722656</v>
+      </c>
+      <c r="I237" t="n">
+        <v>1.639999985694885</v>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K237" t="n">
+        <v>0.727</v>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N237" t="n">
+        <v>70.67</v>
+      </c>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E238" t="n">
+        <v>12378</v>
+      </c>
+      <c r="F238" t="n">
+        <v>11674.44</v>
+      </c>
+      <c r="G238" t="n">
+        <v>-5.68</v>
+      </c>
+      <c r="H238" t="n">
+        <v>10655.58984375</v>
+      </c>
+      <c r="I238" t="n">
+        <v>-13.92000007629395</v>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K238" t="n">
+        <v>0.542</v>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N238" t="n">
+        <v>52.31</v>
+      </c>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E239" t="n">
+        <v>346.35</v>
+      </c>
+      <c r="F239" t="n">
+        <v>333.5</v>
+      </c>
+      <c r="G239" t="n">
+        <v>-3.71</v>
+      </c>
+      <c r="H239" t="n">
+        <v>366.8999938964844</v>
+      </c>
+      <c r="I239" t="n">
+        <v>5.929999828338623</v>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K239" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N239" t="n">
+        <v>55.87</v>
+      </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E240" t="n">
+        <v>257.3</v>
+      </c>
+      <c r="F240" t="n">
+        <v>254.83</v>
+      </c>
+      <c r="G240" t="n">
+        <v>-0.96</v>
+      </c>
+      <c r="H240" t="n">
+        <v>247.9299926757812</v>
+      </c>
+      <c r="I240" t="n">
+        <v>-3.640000104904175</v>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K240" t="n">
+        <v>0.791</v>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N240" t="n">
+        <v>64.38</v>
+      </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E241" t="n">
+        <v>4196.9</v>
+      </c>
+      <c r="F241" t="n">
+        <v>4128.98</v>
+      </c>
+      <c r="G241" t="n">
+        <v>-1.62</v>
+      </c>
+      <c r="H241" t="n">
+        <v>4105.85986328125</v>
+      </c>
+      <c r="I241" t="n">
+        <v>-2.170000076293945</v>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K241" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N241" t="n">
+        <v>60.57</v>
+      </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
         </is>
       </c>
     </row>
@@ -14678,7 +15938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O111"/>
+  <dimension ref="A1:O121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21825,6 +23085,636 @@
       <c r="O111" t="inlineStr">
         <is>
           <t>18 Jan 2026, 06:37:58 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>1457.6</v>
+      </c>
+      <c r="F112" t="n">
+        <v>1650.01</v>
+      </c>
+      <c r="G112" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="H112" t="n">
+        <v>1753.599975585938</v>
+      </c>
+      <c r="I112" t="n">
+        <v>20.30999946594238</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K112" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N112" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>3206.7</v>
+      </c>
+      <c r="F113" t="n">
+        <v>3241.23</v>
+      </c>
+      <c r="G113" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="H113" t="n">
+        <v>3386.570068359375</v>
+      </c>
+      <c r="I113" t="n">
+        <v>5.610000133514404</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K113" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N113" t="n">
+        <v>60.42</v>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>1689.4</v>
+      </c>
+      <c r="F114" t="n">
+        <v>1654.16</v>
+      </c>
+      <c r="G114" t="n">
+        <v>-2.09</v>
+      </c>
+      <c r="H114" t="n">
+        <v>1442.619995117188</v>
+      </c>
+      <c r="I114" t="n">
+        <v>-14.60999965667725</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K114" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N114" t="n">
+        <v>59.87</v>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>931.15</v>
+      </c>
+      <c r="F115" t="n">
+        <v>921.62</v>
+      </c>
+      <c r="G115" t="n">
+        <v>-1.02</v>
+      </c>
+      <c r="H115" t="n">
+        <v>894.4000244140625</v>
+      </c>
+      <c r="I115" t="n">
+        <v>-3.950000047683716</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K115" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N115" t="n">
+        <v>54.39</v>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>1411.65</v>
+      </c>
+      <c r="F116" t="n">
+        <v>1364.89</v>
+      </c>
+      <c r="G116" t="n">
+        <v>-3.31</v>
+      </c>
+      <c r="H116" t="n">
+        <v>1570.530029296875</v>
+      </c>
+      <c r="I116" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K116" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N116" t="n">
+        <v>55.25</v>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>1042.3</v>
+      </c>
+      <c r="F117" t="n">
+        <v>1020.64</v>
+      </c>
+      <c r="G117" t="n">
+        <v>-2.08</v>
+      </c>
+      <c r="H117" t="n">
+        <v>1125</v>
+      </c>
+      <c r="I117" t="n">
+        <v>7.929999828338623</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K117" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N117" t="n">
+        <v>54.52</v>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>329.25</v>
+      </c>
+      <c r="F118" t="n">
+        <v>357.25</v>
+      </c>
+      <c r="G118" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H118" t="n">
+        <v>384.0499877929688</v>
+      </c>
+      <c r="I118" t="n">
+        <v>16.63999938964844</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K118" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N118" t="n">
+        <v>75.95999999999999</v>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>3855.9</v>
+      </c>
+      <c r="F119" t="n">
+        <v>3910.24</v>
+      </c>
+      <c r="G119" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="H119" t="n">
+        <v>3985.72998046875</v>
+      </c>
+      <c r="I119" t="n">
+        <v>3.369999885559082</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K119" t="n">
+        <v>0.542</v>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N119" t="n">
+        <v>62.95</v>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>1294.55</v>
+      </c>
+      <c r="F120" t="n">
+        <v>1236.54</v>
+      </c>
+      <c r="G120" t="n">
+        <v>-4.48</v>
+      </c>
+      <c r="H120" t="n">
+        <v>1173.599975585938</v>
+      </c>
+      <c r="I120" t="n">
+        <v>-9.340000152587891</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K120" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N120" t="n">
+        <v>38.76</v>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>15856.55</v>
+      </c>
+      <c r="F121" t="n">
+        <v>18530.09</v>
+      </c>
+      <c r="G121" t="n">
+        <v>16.86</v>
+      </c>
+      <c r="H121" t="n">
+        <v>16301.26953125</v>
+      </c>
+      <c r="I121" t="n">
+        <v>2.799999952316284</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K121" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N121" t="n">
+        <v>88.29000000000001</v>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
         </is>
       </c>
     </row>
@@ -21839,7 +23729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O221"/>
+  <dimension ref="A1:O241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36059,6 +37949,1266 @@
         </is>
       </c>
     </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E222" t="n">
+        <v>255.53</v>
+      </c>
+      <c r="F222" t="n">
+        <v>280.23</v>
+      </c>
+      <c r="G222" t="n">
+        <v>9.66</v>
+      </c>
+      <c r="H222" t="n">
+        <v>252.9799957275391</v>
+      </c>
+      <c r="I222" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K222" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N222" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E223" t="n">
+        <v>459.86</v>
+      </c>
+      <c r="F223" t="n">
+        <v>466.91</v>
+      </c>
+      <c r="G223" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="H223" t="n">
+        <v>478.0199890136719</v>
+      </c>
+      <c r="I223" t="n">
+        <v>3.950000047683716</v>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K223" t="n">
+        <v>0.637</v>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N223" t="n">
+        <v>65.04000000000001</v>
+      </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E224" t="n">
+        <v>330</v>
+      </c>
+      <c r="F224" t="n">
+        <v>356.57</v>
+      </c>
+      <c r="G224" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="H224" t="n">
+        <v>357.75</v>
+      </c>
+      <c r="I224" t="n">
+        <v>8.409999847412109</v>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K224" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N224" t="n">
+        <v>75.08</v>
+      </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E225" t="n">
+        <v>239.12</v>
+      </c>
+      <c r="F225" t="n">
+        <v>251.08</v>
+      </c>
+      <c r="G225" t="n">
+        <v>5</v>
+      </c>
+      <c r="H225" t="n">
+        <v>214.6600036621094</v>
+      </c>
+      <c r="I225" t="n">
+        <v>-10.22999954223633</v>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K225" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N225" t="n">
+        <v>73.06</v>
+      </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E226" t="n">
+        <v>620.25</v>
+      </c>
+      <c r="F226" t="n">
+        <v>706.99</v>
+      </c>
+      <c r="G226" t="n">
+        <v>13.98</v>
+      </c>
+      <c r="H226" t="n">
+        <v>607.2899780273438</v>
+      </c>
+      <c r="I226" t="n">
+        <v>-2.089999914169312</v>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K226" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N226" t="n">
+        <v>83.98</v>
+      </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E227" t="n">
+        <v>437.5</v>
+      </c>
+      <c r="F227" t="n">
+        <v>445.22</v>
+      </c>
+      <c r="G227" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="H227" t="n">
+        <v>384.7900085449219</v>
+      </c>
+      <c r="I227" t="n">
+        <v>-12.05000019073486</v>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K227" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N227" t="n">
+        <v>65.84999999999999</v>
+      </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E228" t="n">
+        <v>186.23</v>
+      </c>
+      <c r="F228" t="n">
+        <v>200.02</v>
+      </c>
+      <c r="G228" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="H228" t="n">
+        <v>202.1600036621094</v>
+      </c>
+      <c r="I228" t="n">
+        <v>8.560000419616699</v>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K228" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N228" t="n">
+        <v>74.11</v>
+      </c>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E229" t="n">
+        <v>312.47</v>
+      </c>
+      <c r="F229" t="n">
+        <v>341.2</v>
+      </c>
+      <c r="G229" t="n">
+        <v>9.19</v>
+      </c>
+      <c r="H229" t="n">
+        <v>284.4100036621094</v>
+      </c>
+      <c r="I229" t="n">
+        <v>-8.979999542236328</v>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K229" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N229" t="n">
+        <v>66.34999999999999</v>
+      </c>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E230" t="n">
+        <v>328.3</v>
+      </c>
+      <c r="F230" t="n">
+        <v>354.48</v>
+      </c>
+      <c r="G230" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="H230" t="n">
+        <v>338.1799926757812</v>
+      </c>
+      <c r="I230" t="n">
+        <v>3.009999990463257</v>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K230" t="n">
+        <v>0.637</v>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N230" t="n">
+        <v>74.7</v>
+      </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E231" t="n">
+        <v>218.66</v>
+      </c>
+      <c r="F231" t="n">
+        <v>222.68</v>
+      </c>
+      <c r="G231" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="H231" t="n">
+        <v>223.0800018310547</v>
+      </c>
+      <c r="I231" t="n">
+        <v>2.019999980926514</v>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K231" t="n">
+        <v>0</v>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N231" t="n">
+        <v>52.76</v>
+      </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E232" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="F232" t="n">
+        <v>120.45</v>
+      </c>
+      <c r="G232" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="H232" t="n">
+        <v>114.9400024414062</v>
+      </c>
+      <c r="I232" t="n">
+        <v>-3.970000028610229</v>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K232" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N232" t="n">
+        <v>64.14</v>
+      </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E233" t="n">
+        <v>144.53</v>
+      </c>
+      <c r="F233" t="n">
+        <v>143.88</v>
+      </c>
+      <c r="G233" t="n">
+        <v>-0.45</v>
+      </c>
+      <c r="H233" t="n">
+        <v>151.1499938964844</v>
+      </c>
+      <c r="I233" t="n">
+        <v>4.579999923706055</v>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K233" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N233" t="n">
+        <v>65.93000000000001</v>
+      </c>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E234" t="n">
+        <v>539.49</v>
+      </c>
+      <c r="F234" t="n">
+        <v>578.9299999999999</v>
+      </c>
+      <c r="G234" t="n">
+        <v>7.31</v>
+      </c>
+      <c r="H234" t="n">
+        <v>610.02001953125</v>
+      </c>
+      <c r="I234" t="n">
+        <v>13.06999969482422</v>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K234" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N234" t="n">
+        <v>74.17</v>
+      </c>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E235" t="n">
+        <v>331.02</v>
+      </c>
+      <c r="F235" t="n">
+        <v>317.59</v>
+      </c>
+      <c r="G235" t="n">
+        <v>-4.06</v>
+      </c>
+      <c r="H235" t="n">
+        <v>410.0599975585938</v>
+      </c>
+      <c r="I235" t="n">
+        <v>23.8799991607666</v>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K235" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N235" t="n">
+        <v>57.73</v>
+      </c>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E236" t="n">
+        <v>380.17</v>
+      </c>
+      <c r="F236" t="n">
+        <v>348.59</v>
+      </c>
+      <c r="G236" t="n">
+        <v>-8.31</v>
+      </c>
+      <c r="H236" t="n">
+        <v>354.1199951171875</v>
+      </c>
+      <c r="I236" t="n">
+        <v>-6.849999904632568</v>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K236" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N236" t="n">
+        <v>50.74</v>
+      </c>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E237" t="n">
+        <v>52.97</v>
+      </c>
+      <c r="F237" t="n">
+        <v>56.72</v>
+      </c>
+      <c r="G237" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="H237" t="n">
+        <v>56.15999984741211</v>
+      </c>
+      <c r="I237" t="n">
+        <v>6.03000020980835</v>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K237" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N237" t="n">
+        <v>70.48999999999999</v>
+      </c>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E238" t="n">
+        <v>129.89</v>
+      </c>
+      <c r="F238" t="n">
+        <v>126.26</v>
+      </c>
+      <c r="G238" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="H238" t="n">
+        <v>121.4199981689453</v>
+      </c>
+      <c r="I238" t="n">
+        <v>-6.519999980926514</v>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K238" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N238" t="n">
+        <v>56.34</v>
+      </c>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E239" t="n">
+        <v>351.71</v>
+      </c>
+      <c r="F239" t="n">
+        <v>397.1</v>
+      </c>
+      <c r="G239" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="H239" t="n">
+        <v>305.5799865722656</v>
+      </c>
+      <c r="I239" t="n">
+        <v>-13.11999988555908</v>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K239" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N239" t="n">
+        <v>81.86</v>
+      </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E240" t="n">
+        <v>963.61</v>
+      </c>
+      <c r="F240" t="n">
+        <v>938.5700000000001</v>
+      </c>
+      <c r="G240" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="H240" t="n">
+        <v>838.0900268554688</v>
+      </c>
+      <c r="I240" t="n">
+        <v>-13.02999973297119</v>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K240" t="n">
+        <v>0.791</v>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N240" t="n">
+        <v>61.92</v>
+      </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E241" t="n">
+        <v>146.32</v>
+      </c>
+      <c r="F241" t="n">
+        <v>148.34</v>
+      </c>
+      <c r="G241" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="H241" t="n">
+        <v>146.0399932861328</v>
+      </c>
+      <c r="I241" t="n">
+        <v>-0.1899999976158142</v>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K241" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N241" t="n">
+        <v>63.51</v>
+      </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-20)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O241"/>
+  <dimension ref="A1:O261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15924,6 +15924,1266 @@
       <c r="O241" t="inlineStr">
         <is>
           <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E242" t="n">
+        <v>1413.6</v>
+      </c>
+      <c r="F242" t="n">
+        <v>1619.81</v>
+      </c>
+      <c r="G242" t="n">
+        <v>14.59</v>
+      </c>
+      <c r="H242" t="n">
+        <v>1525.449951171875</v>
+      </c>
+      <c r="I242" t="n">
+        <v>7.909999847412109</v>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K242" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N242" t="n">
+        <v>83.31999999999999</v>
+      </c>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E243" t="n">
+        <v>3163.6</v>
+      </c>
+      <c r="F243" t="n">
+        <v>3151.84</v>
+      </c>
+      <c r="G243" t="n">
+        <v>-0.37</v>
+      </c>
+      <c r="H243" t="n">
+        <v>3436.340087890625</v>
+      </c>
+      <c r="I243" t="n">
+        <v>8.619999885559082</v>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K243" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N243" t="n">
+        <v>63.44</v>
+      </c>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E244" t="n">
+        <v>1681.2</v>
+      </c>
+      <c r="F244" t="n">
+        <v>1622.25</v>
+      </c>
+      <c r="G244" t="n">
+        <v>-3.51</v>
+      </c>
+      <c r="H244" t="n">
+        <v>1417.469970703125</v>
+      </c>
+      <c r="I244" t="n">
+        <v>-15.6899995803833</v>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K244" t="n">
+        <v>0</v>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N244" t="n">
+        <v>44.74</v>
+      </c>
+      <c r="O244" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E245" t="n">
+        <v>927.9</v>
+      </c>
+      <c r="F245" t="n">
+        <v>921.26</v>
+      </c>
+      <c r="G245" t="n">
+        <v>-0.72</v>
+      </c>
+      <c r="H245" t="n">
+        <v>862.8599853515625</v>
+      </c>
+      <c r="I245" t="n">
+        <v>-7.010000228881836</v>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K245" t="n">
+        <v>-0.178</v>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N245" t="n">
+        <v>45.37</v>
+      </c>
+      <c r="O245" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E246" t="n">
+        <v>1380.6</v>
+      </c>
+      <c r="F246" t="n">
+        <v>1369.37</v>
+      </c>
+      <c r="G246" t="n">
+        <v>-0.8100000000000001</v>
+      </c>
+      <c r="H246" t="n">
+        <v>1352.900024414062</v>
+      </c>
+      <c r="I246" t="n">
+        <v>-2.009999990463257</v>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K246" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N246" t="n">
+        <v>64.34</v>
+      </c>
+      <c r="O246" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E247" t="n">
+        <v>1038.4</v>
+      </c>
+      <c r="F247" t="n">
+        <v>1023.79</v>
+      </c>
+      <c r="G247" t="n">
+        <v>-1.41</v>
+      </c>
+      <c r="H247" t="n">
+        <v>1282.199951171875</v>
+      </c>
+      <c r="I247" t="n">
+        <v>23.47999954223633</v>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K247" t="n">
+        <v>-0.421</v>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N247" t="n">
+        <v>39.47</v>
+      </c>
+      <c r="O247" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E248" t="n">
+        <v>2413.9</v>
+      </c>
+      <c r="F248" t="n">
+        <v>2310.42</v>
+      </c>
+      <c r="G248" t="n">
+        <v>-4.29</v>
+      </c>
+      <c r="H248" t="n">
+        <v>2387.75</v>
+      </c>
+      <c r="I248" t="n">
+        <v>-1.080000042915344</v>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K248" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N248" t="n">
+        <v>53.79</v>
+      </c>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E249" t="n">
+        <v>333.2</v>
+      </c>
+      <c r="F249" t="n">
+        <v>345.09</v>
+      </c>
+      <c r="G249" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="H249" t="n">
+        <v>381.4400024414062</v>
+      </c>
+      <c r="I249" t="n">
+        <v>14.47999954223633</v>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K249" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N249" t="n">
+        <v>73.34999999999999</v>
+      </c>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E250" t="n">
+        <v>3869.8</v>
+      </c>
+      <c r="F250" t="n">
+        <v>3869.27</v>
+      </c>
+      <c r="G250" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="H250" t="n">
+        <v>3518.3701171875</v>
+      </c>
+      <c r="I250" t="n">
+        <v>-9.079999923706055</v>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K250" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N250" t="n">
+        <v>63.18</v>
+      </c>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E251" t="n">
+        <v>969.45</v>
+      </c>
+      <c r="F251" t="n">
+        <v>1014.14</v>
+      </c>
+      <c r="G251" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="H251" t="n">
+        <v>782.7100219726562</v>
+      </c>
+      <c r="I251" t="n">
+        <v>-19.26000022888184</v>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K251" t="n">
+        <v>-0.273</v>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N251" t="n">
+        <v>51.46</v>
+      </c>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E252" t="n">
+        <v>2010</v>
+      </c>
+      <c r="F252" t="n">
+        <v>2161.93</v>
+      </c>
+      <c r="G252" t="n">
+        <v>7.56</v>
+      </c>
+      <c r="H252" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I252" t="n">
+        <v>0.699999988079071</v>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K252" t="n">
+        <v>-0.751</v>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N252" t="n">
+        <v>46.32</v>
+      </c>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E253" t="n">
+        <v>2754</v>
+      </c>
+      <c r="F253" t="n">
+        <v>2716.91</v>
+      </c>
+      <c r="G253" t="n">
+        <v>-1.35</v>
+      </c>
+      <c r="H253" t="n">
+        <v>3307.3701171875</v>
+      </c>
+      <c r="I253" t="n">
+        <v>20.09000015258789</v>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K253" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N253" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E254" t="n">
+        <v>1307.5</v>
+      </c>
+      <c r="F254" t="n">
+        <v>1235.07</v>
+      </c>
+      <c r="G254" t="n">
+        <v>-5.54</v>
+      </c>
+      <c r="H254" t="n">
+        <v>1269.300048828125</v>
+      </c>
+      <c r="I254" t="n">
+        <v>-2.920000076293945</v>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K254" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N254" t="n">
+        <v>57.25</v>
+      </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E255" t="n">
+        <v>16176</v>
+      </c>
+      <c r="F255" t="n">
+        <v>18318.32</v>
+      </c>
+      <c r="G255" t="n">
+        <v>13.24</v>
+      </c>
+      <c r="H255" t="n">
+        <v>14410.51953125</v>
+      </c>
+      <c r="I255" t="n">
+        <v>-10.90999984741211</v>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K255" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N255" t="n">
+        <v>82.87</v>
+      </c>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E256" t="n">
+        <v>1675.4</v>
+      </c>
+      <c r="F256" t="n">
+        <v>1784.09</v>
+      </c>
+      <c r="G256" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="H256" t="n">
+        <v>1646.06005859375</v>
+      </c>
+      <c r="I256" t="n">
+        <v>-1.75</v>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K256" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N256" t="n">
+        <v>72.73</v>
+      </c>
+      <c r="O256" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E257" t="n">
+        <v>245.95</v>
+      </c>
+      <c r="F257" t="n">
+        <v>273.16</v>
+      </c>
+      <c r="G257" t="n">
+        <v>11.06</v>
+      </c>
+      <c r="H257" t="n">
+        <v>286.8500061035156</v>
+      </c>
+      <c r="I257" t="n">
+        <v>16.6299991607666</v>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K257" t="n">
+        <v>-0.527</v>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N257" t="n">
+        <v>56.05</v>
+      </c>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E258" t="n">
+        <v>12297</v>
+      </c>
+      <c r="F258" t="n">
+        <v>11682.3</v>
+      </c>
+      <c r="G258" t="n">
+        <v>-5</v>
+      </c>
+      <c r="H258" t="n">
+        <v>13795.3896484375</v>
+      </c>
+      <c r="I258" t="n">
+        <v>12.18000030517578</v>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K258" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N258" t="n">
+        <v>53.64</v>
+      </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E259" t="n">
+        <v>343.35</v>
+      </c>
+      <c r="F259" t="n">
+        <v>334.91</v>
+      </c>
+      <c r="G259" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="H259" t="n">
+        <v>333.5199890136719</v>
+      </c>
+      <c r="I259" t="n">
+        <v>-2.859999895095825</v>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K259" t="n">
+        <v>0.852</v>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N259" t="n">
+        <v>63.35</v>
+      </c>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E260" t="n">
+        <v>257.65</v>
+      </c>
+      <c r="F260" t="n">
+        <v>254.14</v>
+      </c>
+      <c r="G260" t="n">
+        <v>-1.36</v>
+      </c>
+      <c r="H260" t="n">
+        <v>230.7599945068359</v>
+      </c>
+      <c r="I260" t="n">
+        <v>-10.4399995803833</v>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K260" t="n">
+        <v>0.791</v>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N260" t="n">
+        <v>63.78</v>
+      </c>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E261" t="n">
+        <v>4144.1</v>
+      </c>
+      <c r="F261" t="n">
+        <v>4034.34</v>
+      </c>
+      <c r="G261" t="n">
+        <v>-2.65</v>
+      </c>
+      <c r="H261" t="n">
+        <v>3711.840087890625</v>
+      </c>
+      <c r="I261" t="n">
+        <v>-10.43000030517578</v>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K261" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N261" t="n">
+        <v>61.95</v>
+      </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
         </is>
       </c>
     </row>
@@ -15938,7 +17198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O121"/>
+  <dimension ref="A1:O131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23715,6 +24975,636 @@
       <c r="O121" t="inlineStr">
         <is>
           <t>19 Jan 2026, 06:58:08 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>1413.25</v>
+      </c>
+      <c r="F122" t="n">
+        <v>1636.79</v>
+      </c>
+      <c r="G122" t="n">
+        <v>15.82</v>
+      </c>
+      <c r="H122" t="n">
+        <v>1335.319946289062</v>
+      </c>
+      <c r="I122" t="n">
+        <v>-5.510000228881836</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K122" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N122" t="n">
+        <v>85.17</v>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>3163</v>
+      </c>
+      <c r="F123" t="n">
+        <v>3198.47</v>
+      </c>
+      <c r="G123" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="H123" t="n">
+        <v>3315.300048828125</v>
+      </c>
+      <c r="I123" t="n">
+        <v>4.809999942779541</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K123" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N123" t="n">
+        <v>65.68000000000001</v>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>1680.35</v>
+      </c>
+      <c r="F124" t="n">
+        <v>1626.66</v>
+      </c>
+      <c r="G124" t="n">
+        <v>-3.2</v>
+      </c>
+      <c r="H124" t="n">
+        <v>1664.93994140625</v>
+      </c>
+      <c r="I124" t="n">
+        <v>-0.9200000166893005</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K124" t="n">
+        <v>0</v>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N124" t="n">
+        <v>45.21</v>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>927.6</v>
+      </c>
+      <c r="F125" t="n">
+        <v>922.97</v>
+      </c>
+      <c r="G125" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="H125" t="n">
+        <v>930.72998046875</v>
+      </c>
+      <c r="I125" t="n">
+        <v>0.3400000035762787</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K125" t="n">
+        <v>-0.421</v>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N125" t="n">
+        <v>40.83</v>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>1379.8</v>
+      </c>
+      <c r="F126" t="n">
+        <v>1372.99</v>
+      </c>
+      <c r="G126" t="n">
+        <v>-0.49</v>
+      </c>
+      <c r="H126" t="n">
+        <v>1309.890014648438</v>
+      </c>
+      <c r="I126" t="n">
+        <v>-5.070000171661377</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K126" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N126" t="n">
+        <v>64.81999999999999</v>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>1038.2</v>
+      </c>
+      <c r="F127" t="n">
+        <v>1029.59</v>
+      </c>
+      <c r="G127" t="n">
+        <v>-0.83</v>
+      </c>
+      <c r="H127" t="n">
+        <v>1095.75</v>
+      </c>
+      <c r="I127" t="n">
+        <v>5.539999961853027</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K127" t="n">
+        <v>-0.421</v>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N127" t="n">
+        <v>40.34</v>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>332.9</v>
+      </c>
+      <c r="F128" t="n">
+        <v>350.99</v>
+      </c>
+      <c r="G128" t="n">
+        <v>5.44</v>
+      </c>
+      <c r="H128" t="n">
+        <v>379.1600036621094</v>
+      </c>
+      <c r="I128" t="n">
+        <v>13.89000034332275</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K128" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N128" t="n">
+        <v>76.15000000000001</v>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>3867.4</v>
+      </c>
+      <c r="F129" t="n">
+        <v>3892.79</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="H129" t="n">
+        <v>3452.31005859375</v>
+      </c>
+      <c r="I129" t="n">
+        <v>-10.72999954223633</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K129" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N129" t="n">
+        <v>64.18000000000001</v>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>1307.55</v>
+      </c>
+      <c r="F130" t="n">
+        <v>1245.84</v>
+      </c>
+      <c r="G130" t="n">
+        <v>-4.72</v>
+      </c>
+      <c r="H130" t="n">
+        <v>1296.75</v>
+      </c>
+      <c r="I130" t="n">
+        <v>-0.8299999833106995</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K130" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N130" t="n">
+        <v>58.48</v>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>16179.75</v>
+      </c>
+      <c r="F131" t="n">
+        <v>18414.69</v>
+      </c>
+      <c r="G131" t="n">
+        <v>13.81</v>
+      </c>
+      <c r="H131" t="n">
+        <v>13841.2802734375</v>
+      </c>
+      <c r="I131" t="n">
+        <v>-14.44999980926514</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K131" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N131" t="n">
+        <v>83.72</v>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
         </is>
       </c>
     </row>
@@ -23729,7 +25619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O241"/>
+  <dimension ref="A1:O261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39209,6 +41099,1266 @@
         </is>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E242" t="n">
+        <v>255.53</v>
+      </c>
+      <c r="F242" t="n">
+        <v>283.69</v>
+      </c>
+      <c r="G242" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="H242" t="n">
+        <v>263.4200134277344</v>
+      </c>
+      <c r="I242" t="n">
+        <v>3.089999914169312</v>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K242" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N242" t="n">
+        <v>79.73</v>
+      </c>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E243" t="n">
+        <v>459.86</v>
+      </c>
+      <c r="F243" t="n">
+        <v>466.43</v>
+      </c>
+      <c r="G243" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="H243" t="n">
+        <v>452.989990234375</v>
+      </c>
+      <c r="I243" t="n">
+        <v>-1.490000009536743</v>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K243" t="n">
+        <v>0.637</v>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N243" t="n">
+        <v>64.88</v>
+      </c>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E244" t="n">
+        <v>330</v>
+      </c>
+      <c r="F244" t="n">
+        <v>356.79</v>
+      </c>
+      <c r="G244" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H244" t="n">
+        <v>348.8900146484375</v>
+      </c>
+      <c r="I244" t="n">
+        <v>5.71999979019165</v>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K244" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N244" t="n">
+        <v>75.38</v>
+      </c>
+      <c r="O244" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E245" t="n">
+        <v>239.12</v>
+      </c>
+      <c r="F245" t="n">
+        <v>251.08</v>
+      </c>
+      <c r="G245" t="n">
+        <v>5</v>
+      </c>
+      <c r="H245" t="n">
+        <v>253.9499969482422</v>
+      </c>
+      <c r="I245" t="n">
+        <v>6.199999809265137</v>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K245" t="n">
+        <v>0.751</v>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N245" t="n">
+        <v>72.52</v>
+      </c>
+      <c r="O245" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E246" t="n">
+        <v>620.25</v>
+      </c>
+      <c r="F246" t="n">
+        <v>712.46</v>
+      </c>
+      <c r="G246" t="n">
+        <v>14.87</v>
+      </c>
+      <c r="H246" t="n">
+        <v>673.1699829101562</v>
+      </c>
+      <c r="I246" t="n">
+        <v>8.529999732971191</v>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K246" t="n">
+        <v>-0.827</v>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N246" t="n">
+        <v>55.76</v>
+      </c>
+      <c r="O246" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E247" t="n">
+        <v>437.5</v>
+      </c>
+      <c r="F247" t="n">
+        <v>445.22</v>
+      </c>
+      <c r="G247" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="H247" t="n">
+        <v>319.8099975585938</v>
+      </c>
+      <c r="I247" t="n">
+        <v>-26.89999961853027</v>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K247" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N247" t="n">
+        <v>62.87</v>
+      </c>
+      <c r="O247" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E248" t="n">
+        <v>186.23</v>
+      </c>
+      <c r="F248" t="n">
+        <v>200.41</v>
+      </c>
+      <c r="G248" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="H248" t="n">
+        <v>206.2299957275391</v>
+      </c>
+      <c r="I248" t="n">
+        <v>10.73999977111816</v>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K248" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N248" t="n">
+        <v>74.42</v>
+      </c>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E249" t="n">
+        <v>312.47</v>
+      </c>
+      <c r="F249" t="n">
+        <v>341.12</v>
+      </c>
+      <c r="G249" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="H249" t="n">
+        <v>363.8800048828125</v>
+      </c>
+      <c r="I249" t="n">
+        <v>16.45000076293945</v>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K249" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N249" t="n">
+        <v>69.67</v>
+      </c>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E250" t="n">
+        <v>328.3</v>
+      </c>
+      <c r="F250" t="n">
+        <v>354.33</v>
+      </c>
+      <c r="G250" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="H250" t="n">
+        <v>336.0400085449219</v>
+      </c>
+      <c r="I250" t="n">
+        <v>2.359999895095825</v>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K250" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N250" t="n">
+        <v>75.09</v>
+      </c>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E251" t="n">
+        <v>218.66</v>
+      </c>
+      <c r="F251" t="n">
+        <v>222.72</v>
+      </c>
+      <c r="G251" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="H251" t="n">
+        <v>235.8399963378906</v>
+      </c>
+      <c r="I251" t="n">
+        <v>7.860000133514404</v>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K251" t="n">
+        <v>0</v>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N251" t="n">
+        <v>52.79</v>
+      </c>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E252" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="F252" t="n">
+        <v>120.54</v>
+      </c>
+      <c r="G252" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H252" t="n">
+        <v>114.120002746582</v>
+      </c>
+      <c r="I252" t="n">
+        <v>-4.659999847412109</v>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K252" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N252" t="n">
+        <v>64.26000000000001</v>
+      </c>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E253" t="n">
+        <v>144.53</v>
+      </c>
+      <c r="F253" t="n">
+        <v>144.13</v>
+      </c>
+      <c r="G253" t="n">
+        <v>-0.28</v>
+      </c>
+      <c r="H253" t="n">
+        <v>139.3999938964844</v>
+      </c>
+      <c r="I253" t="n">
+        <v>-3.549999952316284</v>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K253" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N253" t="n">
+        <v>66.19</v>
+      </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E254" t="n">
+        <v>539.49</v>
+      </c>
+      <c r="F254" t="n">
+        <v>579.1900000000001</v>
+      </c>
+      <c r="G254" t="n">
+        <v>7.36</v>
+      </c>
+      <c r="H254" t="n">
+        <v>552.3800048828125</v>
+      </c>
+      <c r="I254" t="n">
+        <v>2.390000104904175</v>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K254" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N254" t="n">
+        <v>74.23999999999999</v>
+      </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E255" t="n">
+        <v>331.02</v>
+      </c>
+      <c r="F255" t="n">
+        <v>319.01</v>
+      </c>
+      <c r="G255" t="n">
+        <v>-3.63</v>
+      </c>
+      <c r="H255" t="n">
+        <v>378.5899963378906</v>
+      </c>
+      <c r="I255" t="n">
+        <v>14.36999988555908</v>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K255" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N255" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E256" t="n">
+        <v>380.17</v>
+      </c>
+      <c r="F256" t="n">
+        <v>349.37</v>
+      </c>
+      <c r="G256" t="n">
+        <v>-8.1</v>
+      </c>
+      <c r="H256" t="n">
+        <v>376.4800109863281</v>
+      </c>
+      <c r="I256" t="n">
+        <v>-0.9700000286102295</v>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K256" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N256" t="n">
+        <v>51.05</v>
+      </c>
+      <c r="O256" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E257" t="n">
+        <v>52.97</v>
+      </c>
+      <c r="F257" t="n">
+        <v>56.73</v>
+      </c>
+      <c r="G257" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="H257" t="n">
+        <v>59.09000015258789</v>
+      </c>
+      <c r="I257" t="n">
+        <v>11.55000019073486</v>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K257" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N257" t="n">
+        <v>73.84</v>
+      </c>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E258" t="n">
+        <v>129.89</v>
+      </c>
+      <c r="F258" t="n">
+        <v>126.56</v>
+      </c>
+      <c r="G258" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="H258" t="n">
+        <v>130.9700012207031</v>
+      </c>
+      <c r="I258" t="n">
+        <v>0.8299999833106995</v>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K258" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N258" t="n">
+        <v>61.01</v>
+      </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E259" t="n">
+        <v>351.71</v>
+      </c>
+      <c r="F259" t="n">
+        <v>398.02</v>
+      </c>
+      <c r="G259" t="n">
+        <v>13.17</v>
+      </c>
+      <c r="H259" t="n">
+        <v>397.1300048828125</v>
+      </c>
+      <c r="I259" t="n">
+        <v>12.90999984741211</v>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K259" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N259" t="n">
+        <v>83.95</v>
+      </c>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E260" t="n">
+        <v>963.61</v>
+      </c>
+      <c r="F260" t="n">
+        <v>938.84</v>
+      </c>
+      <c r="G260" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="H260" t="n">
+        <v>953.280029296875</v>
+      </c>
+      <c r="I260" t="n">
+        <v>-1.070000052452087</v>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K260" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N260" t="n">
+        <v>59.34</v>
+      </c>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E261" t="n">
+        <v>146.32</v>
+      </c>
+      <c r="F261" t="n">
+        <v>148.18</v>
+      </c>
+      <c r="G261" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="H261" t="n">
+        <v>143.3899993896484</v>
+      </c>
+      <c r="I261" t="n">
+        <v>-2</v>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K261" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N261" t="n">
+        <v>63.35</v>
+      </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-21)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O261"/>
+  <dimension ref="A1:O281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17184,6 +17184,1266 @@
       <c r="O261" t="inlineStr">
         <is>
           <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E262" t="n">
+        <v>1394</v>
+      </c>
+      <c r="F262" t="n">
+        <v>1611.54</v>
+      </c>
+      <c r="G262" t="n">
+        <v>15.61</v>
+      </c>
+      <c r="H262" t="n">
+        <v>1510.339965820312</v>
+      </c>
+      <c r="I262" t="n">
+        <v>8.350000381469727</v>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K262" t="n">
+        <v>-0.542</v>
+      </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N262" t="n">
+        <v>62.57</v>
+      </c>
+      <c r="O262" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E263" t="n">
+        <v>3102.3</v>
+      </c>
+      <c r="F263" t="n">
+        <v>3129.24</v>
+      </c>
+      <c r="G263" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="H263" t="n">
+        <v>3151.8701171875</v>
+      </c>
+      <c r="I263" t="n">
+        <v>1.600000023841858</v>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K263" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N263" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E264" t="n">
+        <v>1658.9</v>
+      </c>
+      <c r="F264" t="n">
+        <v>1612.38</v>
+      </c>
+      <c r="G264" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="H264" t="n">
+        <v>1580.550048828125</v>
+      </c>
+      <c r="I264" t="n">
+        <v>-4.71999979019165</v>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K264" t="n">
+        <v>0.637</v>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N264" t="n">
+        <v>58.53</v>
+      </c>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E265" t="n">
+        <v>931.2</v>
+      </c>
+      <c r="F265" t="n">
+        <v>919.46</v>
+      </c>
+      <c r="G265" t="n">
+        <v>-1.26</v>
+      </c>
+      <c r="H265" t="n">
+        <v>891.8599853515625</v>
+      </c>
+      <c r="I265" t="n">
+        <v>-4.21999979019165</v>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K265" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N265" t="n">
+        <v>61.11</v>
+      </c>
+      <c r="O265" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E266" t="n">
+        <v>1375.8</v>
+      </c>
+      <c r="F266" t="n">
+        <v>1369.16</v>
+      </c>
+      <c r="G266" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="H266" t="n">
+        <v>1382.859985351562</v>
+      </c>
+      <c r="I266" t="n">
+        <v>0.5099999904632568</v>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K266" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N266" t="n">
+        <v>64.84</v>
+      </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E267" t="n">
+        <v>1036.4</v>
+      </c>
+      <c r="F267" t="n">
+        <v>1030.93</v>
+      </c>
+      <c r="G267" t="n">
+        <v>-0.53</v>
+      </c>
+      <c r="H267" t="n">
+        <v>1247.829956054688</v>
+      </c>
+      <c r="I267" t="n">
+        <v>20.39999961853027</v>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K267" t="n">
+        <v>-0.402</v>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N267" t="n">
+        <v>41.17</v>
+      </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E268" t="n">
+        <v>2379.1</v>
+      </c>
+      <c r="F268" t="n">
+        <v>2284.61</v>
+      </c>
+      <c r="G268" t="n">
+        <v>-3.97</v>
+      </c>
+      <c r="H268" t="n">
+        <v>3286.7900390625</v>
+      </c>
+      <c r="I268" t="n">
+        <v>38.15000152587891</v>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K268" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N268" t="n">
+        <v>54.26</v>
+      </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E269" t="n">
+        <v>326.3</v>
+      </c>
+      <c r="F269" t="n">
+        <v>340.64</v>
+      </c>
+      <c r="G269" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="H269" t="n">
+        <v>409.739990234375</v>
+      </c>
+      <c r="I269" t="n">
+        <v>25.56999969482422</v>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K269" t="n">
+        <v>0.832</v>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N269" t="n">
+        <v>73.23</v>
+      </c>
+      <c r="O269" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E270" t="n">
+        <v>3810.5</v>
+      </c>
+      <c r="F270" t="n">
+        <v>3868.78</v>
+      </c>
+      <c r="G270" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="H270" t="n">
+        <v>4327.3798828125</v>
+      </c>
+      <c r="I270" t="n">
+        <v>13.5600004196167</v>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K270" t="n">
+        <v>0</v>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N270" t="n">
+        <v>52.29</v>
+      </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E271" t="n">
+        <v>933.2</v>
+      </c>
+      <c r="F271" t="n">
+        <v>1010.64</v>
+      </c>
+      <c r="G271" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="H271" t="n">
+        <v>1056.47998046875</v>
+      </c>
+      <c r="I271" t="n">
+        <v>13.21000003814697</v>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K271" t="n">
+        <v>-0.273</v>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N271" t="n">
+        <v>56.99</v>
+      </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E272" t="n">
+        <v>1996</v>
+      </c>
+      <c r="F272" t="n">
+        <v>2157.26</v>
+      </c>
+      <c r="G272" t="n">
+        <v>8.08</v>
+      </c>
+      <c r="H272" t="n">
+        <v>2112.75</v>
+      </c>
+      <c r="I272" t="n">
+        <v>5.849999904632568</v>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K272" t="n">
+        <v>-0.361</v>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N272" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E273" t="n">
+        <v>2675.6</v>
+      </c>
+      <c r="F273" t="n">
+        <v>2678.66</v>
+      </c>
+      <c r="G273" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H273" t="n">
+        <v>2545.1201171875</v>
+      </c>
+      <c r="I273" t="n">
+        <v>-4.880000114440918</v>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K273" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N273" t="n">
+        <v>61.31</v>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E274" t="n">
+        <v>1293.5</v>
+      </c>
+      <c r="F274" t="n">
+        <v>1236.46</v>
+      </c>
+      <c r="G274" t="n">
+        <v>-4.41</v>
+      </c>
+      <c r="H274" t="n">
+        <v>1334.800048828125</v>
+      </c>
+      <c r="I274" t="n">
+        <v>3.190000057220459</v>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K274" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N274" t="n">
+        <v>52.93</v>
+      </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E275" t="n">
+        <v>15879</v>
+      </c>
+      <c r="F275" t="n">
+        <v>18236.73</v>
+      </c>
+      <c r="G275" t="n">
+        <v>14.85</v>
+      </c>
+      <c r="H275" t="n">
+        <v>13868.7900390625</v>
+      </c>
+      <c r="I275" t="n">
+        <v>-12.65999984741211</v>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K275" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N275" t="n">
+        <v>85.27</v>
+      </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E276" t="n">
+        <v>1613.8</v>
+      </c>
+      <c r="F276" t="n">
+        <v>1771.36</v>
+      </c>
+      <c r="G276" t="n">
+        <v>9.76</v>
+      </c>
+      <c r="H276" t="n">
+        <v>1827.800048828125</v>
+      </c>
+      <c r="I276" t="n">
+        <v>13.26000022888184</v>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K276" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N276" t="n">
+        <v>77.65000000000001</v>
+      </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E277" t="n">
+        <v>239.9</v>
+      </c>
+      <c r="F277" t="n">
+        <v>271.12</v>
+      </c>
+      <c r="G277" t="n">
+        <v>13.01</v>
+      </c>
+      <c r="H277" t="n">
+        <v>278.3800048828125</v>
+      </c>
+      <c r="I277" t="n">
+        <v>16.04000091552734</v>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K277" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N277" t="n">
+        <v>82.52</v>
+      </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E278" t="n">
+        <v>12059</v>
+      </c>
+      <c r="F278" t="n">
+        <v>11684.53</v>
+      </c>
+      <c r="G278" t="n">
+        <v>-3.11</v>
+      </c>
+      <c r="H278" t="n">
+        <v>11455.8701171875</v>
+      </c>
+      <c r="I278" t="n">
+        <v>-5</v>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K278" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N278" t="n">
+        <v>56.48</v>
+      </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E279" t="n">
+        <v>338.75</v>
+      </c>
+      <c r="F279" t="n">
+        <v>334.71</v>
+      </c>
+      <c r="G279" t="n">
+        <v>-1.19</v>
+      </c>
+      <c r="H279" t="n">
+        <v>369.9400024414062</v>
+      </c>
+      <c r="I279" t="n">
+        <v>9.210000038146973</v>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K279" t="n">
+        <v>0.852</v>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N279" t="n">
+        <v>65.25</v>
+      </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E280" t="n">
+        <v>254.05</v>
+      </c>
+      <c r="F280" t="n">
+        <v>254.18</v>
+      </c>
+      <c r="G280" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H280" t="n">
+        <v>279.3099975585938</v>
+      </c>
+      <c r="I280" t="n">
+        <v>9.939999580383301</v>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K280" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N280" t="n">
+        <v>60.29</v>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E281" t="n">
+        <v>4075.5</v>
+      </c>
+      <c r="F281" t="n">
+        <v>4043.76</v>
+      </c>
+      <c r="G281" t="n">
+        <v>-0.78</v>
+      </c>
+      <c r="H281" t="n">
+        <v>3393.169921875</v>
+      </c>
+      <c r="I281" t="n">
+        <v>-16.73999977111816</v>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K281" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N281" t="n">
+        <v>64.75</v>
+      </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
         </is>
       </c>
     </row>
@@ -17198,7 +18458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O131"/>
+  <dimension ref="A1:O141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25605,6 +26865,636 @@
       <c r="O131" t="inlineStr">
         <is>
           <t>20 Jan 2026, 06:58:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>1393.4</v>
+      </c>
+      <c r="F132" t="n">
+        <v>1619.6</v>
+      </c>
+      <c r="G132" t="n">
+        <v>16.23</v>
+      </c>
+      <c r="H132" t="n">
+        <v>1416.47998046875</v>
+      </c>
+      <c r="I132" t="n">
+        <v>1.659999966621399</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K132" t="n">
+        <v>-0.542</v>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N132" t="n">
+        <v>63.51</v>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>3108.05</v>
+      </c>
+      <c r="F133" t="n">
+        <v>3178.91</v>
+      </c>
+      <c r="G133" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="H133" t="n">
+        <v>3145.489990234375</v>
+      </c>
+      <c r="I133" t="n">
+        <v>1.200000047683716</v>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K133" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N133" t="n">
+        <v>67.42</v>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>1657.7</v>
+      </c>
+      <c r="F134" t="n">
+        <v>1626.74</v>
+      </c>
+      <c r="G134" t="n">
+        <v>-1.87</v>
+      </c>
+      <c r="H134" t="n">
+        <v>1627.130004882812</v>
+      </c>
+      <c r="I134" t="n">
+        <v>-1.840000033378601</v>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K134" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N134" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>931.15</v>
+      </c>
+      <c r="F135" t="n">
+        <v>922.6799999999999</v>
+      </c>
+      <c r="G135" t="n">
+        <v>-0.91</v>
+      </c>
+      <c r="H135" t="n">
+        <v>939.27001953125</v>
+      </c>
+      <c r="I135" t="n">
+        <v>0.8700000047683716</v>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K135" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N135" t="n">
+        <v>61.64</v>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>1375.35</v>
+      </c>
+      <c r="F136" t="n">
+        <v>1372.15</v>
+      </c>
+      <c r="G136" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="H136" t="n">
+        <v>1366.380004882812</v>
+      </c>
+      <c r="I136" t="n">
+        <v>-0.6499999761581421</v>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K136" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N136" t="n">
+        <v>61.63</v>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>1037.15</v>
+      </c>
+      <c r="F137" t="n">
+        <v>1036.14</v>
+      </c>
+      <c r="G137" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="H137" t="n">
+        <v>1215.489990234375</v>
+      </c>
+      <c r="I137" t="n">
+        <v>17.20000076293945</v>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K137" t="n">
+        <v>-0.402</v>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N137" t="n">
+        <v>41.81</v>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>326.4</v>
+      </c>
+      <c r="F138" t="n">
+        <v>347.12</v>
+      </c>
+      <c r="G138" t="n">
+        <v>6.35</v>
+      </c>
+      <c r="H138" t="n">
+        <v>382.5599975585938</v>
+      </c>
+      <c r="I138" t="n">
+        <v>17.20999908447266</v>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K138" t="n">
+        <v>0.832</v>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N138" t="n">
+        <v>76.16</v>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>3808</v>
+      </c>
+      <c r="F139" t="n">
+        <v>3887.2</v>
+      </c>
+      <c r="G139" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="H139" t="n">
+        <v>3812.659912109375</v>
+      </c>
+      <c r="I139" t="n">
+        <v>0.119999997317791</v>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K139" t="n">
+        <v>0</v>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N139" t="n">
+        <v>53.12</v>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>1293.1</v>
+      </c>
+      <c r="F140" t="n">
+        <v>1247.35</v>
+      </c>
+      <c r="G140" t="n">
+        <v>-3.54</v>
+      </c>
+      <c r="H140" t="n">
+        <v>1161.06005859375</v>
+      </c>
+      <c r="I140" t="n">
+        <v>-10.21000003814697</v>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K140" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N140" t="n">
+        <v>54.23</v>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>15881.1</v>
+      </c>
+      <c r="F141" t="n">
+        <v>18323.9</v>
+      </c>
+      <c r="G141" t="n">
+        <v>15.38</v>
+      </c>
+      <c r="H141" t="n">
+        <v>12896.6298828125</v>
+      </c>
+      <c r="I141" t="n">
+        <v>-18.79000091552734</v>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K141" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N141" t="n">
+        <v>86.06999999999999</v>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
         </is>
       </c>
     </row>
@@ -25619,7 +27509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O261"/>
+  <dimension ref="A1:O281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42359,6 +44249,1266 @@
         </is>
       </c>
     </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E262" t="n">
+        <v>246.7</v>
+      </c>
+      <c r="F262" t="n">
+        <v>280.31</v>
+      </c>
+      <c r="G262" t="n">
+        <v>13.62</v>
+      </c>
+      <c r="H262" t="n">
+        <v>251.3500061035156</v>
+      </c>
+      <c r="I262" t="n">
+        <v>1.879999995231628</v>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K262" t="n">
+        <v>0.361</v>
+      </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N262" t="n">
+        <v>77.66</v>
+      </c>
+      <c r="O262" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E263" t="n">
+        <v>454.52</v>
+      </c>
+      <c r="F263" t="n">
+        <v>461.41</v>
+      </c>
+      <c r="G263" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="H263" t="n">
+        <v>459.4500122070312</v>
+      </c>
+      <c r="I263" t="n">
+        <v>1.090000033378601</v>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K263" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N263" t="n">
+        <v>63.99</v>
+      </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E264" t="n">
+        <v>322</v>
+      </c>
+      <c r="F264" t="n">
+        <v>353.53</v>
+      </c>
+      <c r="G264" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="H264" t="n">
+        <v>421.6400146484375</v>
+      </c>
+      <c r="I264" t="n">
+        <v>30.95000076293945</v>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K264" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N264" t="n">
+        <v>77.89</v>
+      </c>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E265" t="n">
+        <v>231</v>
+      </c>
+      <c r="F265" t="n">
+        <v>251.45</v>
+      </c>
+      <c r="G265" t="n">
+        <v>8.85</v>
+      </c>
+      <c r="H265" t="n">
+        <v>212.7899932861328</v>
+      </c>
+      <c r="I265" t="n">
+        <v>-7.880000114440918</v>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K265" t="n">
+        <v>0.751</v>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N265" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="O265" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E266" t="n">
+        <v>604.12</v>
+      </c>
+      <c r="F266" t="n">
+        <v>703.0599999999999</v>
+      </c>
+      <c r="G266" t="n">
+        <v>16.38</v>
+      </c>
+      <c r="H266" t="n">
+        <v>654.7000122070312</v>
+      </c>
+      <c r="I266" t="n">
+        <v>8.369999885559082</v>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K266" t="n">
+        <v>-0.743</v>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N266" t="n">
+        <v>59.71</v>
+      </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E267" t="n">
+        <v>419.25</v>
+      </c>
+      <c r="F267" t="n">
+        <v>437.67</v>
+      </c>
+      <c r="G267" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="H267" t="n">
+        <v>488.1099853515625</v>
+      </c>
+      <c r="I267" t="n">
+        <v>16.42000007629395</v>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K267" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N267" t="n">
+        <v>67.13</v>
+      </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E268" t="n">
+        <v>178.07</v>
+      </c>
+      <c r="F268" t="n">
+        <v>202.49</v>
+      </c>
+      <c r="G268" t="n">
+        <v>13.71</v>
+      </c>
+      <c r="H268" t="n">
+        <v>173.6999969482422</v>
+      </c>
+      <c r="I268" t="n">
+        <v>-2.450000047683716</v>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K268" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N268" t="n">
+        <v>83.56999999999999</v>
+      </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E269" t="n">
+        <v>302.74</v>
+      </c>
+      <c r="F269" t="n">
+        <v>339.2</v>
+      </c>
+      <c r="G269" t="n">
+        <v>12.04</v>
+      </c>
+      <c r="H269" t="n">
+        <v>298.6900024414062</v>
+      </c>
+      <c r="I269" t="n">
+        <v>-1.340000033378601</v>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K269" t="n">
+        <v>0</v>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N269" t="n">
+        <v>68.06999999999999</v>
+      </c>
+      <c r="O269" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E270" t="n">
+        <v>325.82</v>
+      </c>
+      <c r="F270" t="n">
+        <v>351.67</v>
+      </c>
+      <c r="G270" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="H270" t="n">
+        <v>325.2999877929688</v>
+      </c>
+      <c r="I270" t="n">
+        <v>-0.1599999964237213</v>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K270" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N270" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E271" t="n">
+        <v>218.21</v>
+      </c>
+      <c r="F271" t="n">
+        <v>223.47</v>
+      </c>
+      <c r="G271" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="H271" t="n">
+        <v>214.5099945068359</v>
+      </c>
+      <c r="I271" t="n">
+        <v>-1.690000057220459</v>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K271" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N271" t="n">
+        <v>62.41</v>
+      </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E272" t="n">
+        <v>118.71</v>
+      </c>
+      <c r="F272" t="n">
+        <v>119.74</v>
+      </c>
+      <c r="G272" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="H272" t="n">
+        <v>124.7200012207031</v>
+      </c>
+      <c r="I272" t="n">
+        <v>5.059999942779541</v>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K272" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N272" t="n">
+        <v>57.66</v>
+      </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E273" t="n">
+        <v>147</v>
+      </c>
+      <c r="F273" t="n">
+        <v>143.6</v>
+      </c>
+      <c r="G273" t="n">
+        <v>-2.31</v>
+      </c>
+      <c r="H273" t="n">
+        <v>141.7100067138672</v>
+      </c>
+      <c r="I273" t="n">
+        <v>-3.599999904632568</v>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K273" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N273" t="n">
+        <v>52.45</v>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E274" t="n">
+        <v>531.74</v>
+      </c>
+      <c r="F274" t="n">
+        <v>578.15</v>
+      </c>
+      <c r="G274" t="n">
+        <v>8.73</v>
+      </c>
+      <c r="H274" t="n">
+        <v>517.9199829101562</v>
+      </c>
+      <c r="I274" t="n">
+        <v>-2.599999904632568</v>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K274" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N274" t="n">
+        <v>76.29000000000001</v>
+      </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E275" t="n">
+        <v>338.43</v>
+      </c>
+      <c r="F275" t="n">
+        <v>303.13</v>
+      </c>
+      <c r="G275" t="n">
+        <v>-10.43</v>
+      </c>
+      <c r="H275" t="n">
+        <v>370.4299926757812</v>
+      </c>
+      <c r="I275" t="n">
+        <v>9.460000038146973</v>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K275" t="n">
+        <v>0</v>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N275" t="n">
+        <v>34.35</v>
+      </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E276" t="n">
+        <v>375.11</v>
+      </c>
+      <c r="F276" t="n">
+        <v>346.65</v>
+      </c>
+      <c r="G276" t="n">
+        <v>-7.59</v>
+      </c>
+      <c r="H276" t="n">
+        <v>416.5700073242188</v>
+      </c>
+      <c r="I276" t="n">
+        <v>11.05000019073486</v>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K276" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N276" t="n">
+        <v>52.02</v>
+      </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E277" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="F277" t="n">
+        <v>56.26</v>
+      </c>
+      <c r="G277" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="H277" t="n">
+        <v>46.36999893188477</v>
+      </c>
+      <c r="I277" t="n">
+        <v>-10.98999977111816</v>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K277" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N277" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E278" t="n">
+        <v>130.46</v>
+      </c>
+      <c r="F278" t="n">
+        <v>127.45</v>
+      </c>
+      <c r="G278" t="n">
+        <v>-2.31</v>
+      </c>
+      <c r="H278" t="n">
+        <v>142.5200042724609</v>
+      </c>
+      <c r="I278" t="n">
+        <v>9.239999771118164</v>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K278" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N278" t="n">
+        <v>59.94</v>
+      </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E279" t="n">
+        <v>332.6</v>
+      </c>
+      <c r="F279" t="n">
+        <v>405.32</v>
+      </c>
+      <c r="G279" t="n">
+        <v>21.86</v>
+      </c>
+      <c r="H279" t="n">
+        <v>400.3099975585938</v>
+      </c>
+      <c r="I279" t="n">
+        <v>20.36000061035156</v>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K279" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N279" t="n">
+        <v>86.8</v>
+      </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E280" t="n">
+        <v>964.26</v>
+      </c>
+      <c r="F280" t="n">
+        <v>942.2</v>
+      </c>
+      <c r="G280" t="n">
+        <v>-2.29</v>
+      </c>
+      <c r="H280" t="n">
+        <v>920.6300048828125</v>
+      </c>
+      <c r="I280" t="n">
+        <v>-4.53000020980835</v>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K280" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N280" t="n">
+        <v>59.57</v>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E281" t="n">
+        <v>147.66</v>
+      </c>
+      <c r="F281" t="n">
+        <v>148.85</v>
+      </c>
+      <c r="G281" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="H281" t="n">
+        <v>153.5200042724609</v>
+      </c>
+      <c r="I281" t="n">
+        <v>3.970000028610229</v>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K281" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N281" t="n">
+        <v>61.09</v>
+      </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-22)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O281"/>
+  <dimension ref="A1:O301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18444,6 +18444,1266 @@
       <c r="O281" t="inlineStr">
         <is>
           <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E282" t="n">
+        <v>1404.6</v>
+      </c>
+      <c r="F282" t="n">
+        <v>1602.07</v>
+      </c>
+      <c r="G282" t="n">
+        <v>14.06</v>
+      </c>
+      <c r="H282" t="n">
+        <v>1396.599975585938</v>
+      </c>
+      <c r="I282" t="n">
+        <v>-0.5699999928474426</v>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K282" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N282" t="n">
+        <v>82.81</v>
+      </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E283" t="n">
+        <v>3122.6</v>
+      </c>
+      <c r="F283" t="n">
+        <v>3122.1</v>
+      </c>
+      <c r="G283" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="H283" t="n">
+        <v>3199.320068359375</v>
+      </c>
+      <c r="I283" t="n">
+        <v>2.460000038146973</v>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K283" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N283" t="n">
+        <v>63.98</v>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E284" t="n">
+        <v>1654.4</v>
+      </c>
+      <c r="F284" t="n">
+        <v>1619.68</v>
+      </c>
+      <c r="G284" t="n">
+        <v>-2.1</v>
+      </c>
+      <c r="H284" t="n">
+        <v>1572.97998046875</v>
+      </c>
+      <c r="I284" t="n">
+        <v>-4.920000076293945</v>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K284" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N284" t="n">
+        <v>50.89</v>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E285" t="n">
+        <v>920.35</v>
+      </c>
+      <c r="F285" t="n">
+        <v>916.41</v>
+      </c>
+      <c r="G285" t="n">
+        <v>-0.43</v>
+      </c>
+      <c r="H285" t="n">
+        <v>1014.030029296875</v>
+      </c>
+      <c r="I285" t="n">
+        <v>10.18000030517578</v>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K285" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N285" t="n">
+        <v>66.23999999999999</v>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E286" t="n">
+        <v>1349</v>
+      </c>
+      <c r="F286" t="n">
+        <v>1370.01</v>
+      </c>
+      <c r="G286" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="H286" t="n">
+        <v>1498.72998046875</v>
+      </c>
+      <c r="I286" t="n">
+        <v>11.10000038146973</v>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K286" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N286" t="n">
+        <v>61.14</v>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E287" t="n">
+        <v>1028.65</v>
+      </c>
+      <c r="F287" t="n">
+        <v>1036.97</v>
+      </c>
+      <c r="G287" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="H287" t="n">
+        <v>1055.369995117188</v>
+      </c>
+      <c r="I287" t="n">
+        <v>2.599999904632568</v>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K287" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N287" t="n">
+        <v>58.01</v>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E288" t="n">
+        <v>2368</v>
+      </c>
+      <c r="F288" t="n">
+        <v>2307.44</v>
+      </c>
+      <c r="G288" t="n">
+        <v>-2.56</v>
+      </c>
+      <c r="H288" t="n">
+        <v>2410.860107421875</v>
+      </c>
+      <c r="I288" t="n">
+        <v>1.809999942779541</v>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K288" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N288" t="n">
+        <v>59.16</v>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E289" t="n">
+        <v>324.75</v>
+      </c>
+      <c r="F289" t="n">
+        <v>334.96</v>
+      </c>
+      <c r="G289" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="H289" t="n">
+        <v>364.8200073242188</v>
+      </c>
+      <c r="I289" t="n">
+        <v>12.34000015258789</v>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K289" t="n">
+        <v>-0.273</v>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N289" t="n">
+        <v>49.26</v>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E290" t="n">
+        <v>3766.5</v>
+      </c>
+      <c r="F290" t="n">
+        <v>3858.56</v>
+      </c>
+      <c r="G290" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="H290" t="n">
+        <v>3603.659912109375</v>
+      </c>
+      <c r="I290" t="n">
+        <v>-4.320000171661377</v>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K290" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N290" t="n">
+        <v>58.19</v>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E291" t="n">
+        <v>936.25</v>
+      </c>
+      <c r="F291" t="n">
+        <v>1010.3</v>
+      </c>
+      <c r="G291" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="H291" t="n">
+        <v>801.010009765625</v>
+      </c>
+      <c r="I291" t="n">
+        <v>-14.4399995803833</v>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K291" t="n">
+        <v>-0.511</v>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N291" t="n">
+        <v>51.64</v>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E292" t="n">
+        <v>1996.1</v>
+      </c>
+      <c r="F292" t="n">
+        <v>2142.57</v>
+      </c>
+      <c r="G292" t="n">
+        <v>7.34</v>
+      </c>
+      <c r="H292" t="n">
+        <v>2036.0400390625</v>
+      </c>
+      <c r="I292" t="n">
+        <v>2</v>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K292" t="n">
+        <v>-0.178</v>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N292" t="n">
+        <v>57.45</v>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>2661.1</v>
+      </c>
+      <c r="F293" t="n">
+        <v>2687.82</v>
+      </c>
+      <c r="G293" t="n">
+        <v>1</v>
+      </c>
+      <c r="H293" t="n">
+        <v>2865.659912109375</v>
+      </c>
+      <c r="I293" t="n">
+        <v>7.690000057220459</v>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K293" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N293" t="n">
+        <v>58.31</v>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E294" t="n">
+        <v>1284.9</v>
+      </c>
+      <c r="F294" t="n">
+        <v>1242.75</v>
+      </c>
+      <c r="G294" t="n">
+        <v>-3.28</v>
+      </c>
+      <c r="H294" t="n">
+        <v>1340.359985351562</v>
+      </c>
+      <c r="I294" t="n">
+        <v>4.320000171661377</v>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K294" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N294" t="n">
+        <v>58.08</v>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>15770</v>
+      </c>
+      <c r="F295" t="n">
+        <v>18276.16</v>
+      </c>
+      <c r="G295" t="n">
+        <v>15.89</v>
+      </c>
+      <c r="H295" t="n">
+        <v>14784.33984375</v>
+      </c>
+      <c r="I295" t="n">
+        <v>-6.25</v>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K295" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N295" t="n">
+        <v>84.06</v>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E296" t="n">
+        <v>1612.9</v>
+      </c>
+      <c r="F296" t="n">
+        <v>1762.19</v>
+      </c>
+      <c r="G296" t="n">
+        <v>9.26</v>
+      </c>
+      <c r="H296" t="n">
+        <v>1751.869995117188</v>
+      </c>
+      <c r="I296" t="n">
+        <v>8.619999885559082</v>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K296" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N296" t="n">
+        <v>76.88</v>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E297" t="n">
+        <v>239.55</v>
+      </c>
+      <c r="F297" t="n">
+        <v>265.68</v>
+      </c>
+      <c r="G297" t="n">
+        <v>10.91</v>
+      </c>
+      <c r="H297" t="n">
+        <v>244.2100067138672</v>
+      </c>
+      <c r="I297" t="n">
+        <v>1.950000047683716</v>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K297" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N297" t="n">
+        <v>79.56</v>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E298" t="n">
+        <v>12231</v>
+      </c>
+      <c r="F298" t="n">
+        <v>11689.41</v>
+      </c>
+      <c r="G298" t="n">
+        <v>-4.43</v>
+      </c>
+      <c r="H298" t="n">
+        <v>11949.0498046875</v>
+      </c>
+      <c r="I298" t="n">
+        <v>-2.309999942779541</v>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K298" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N298" t="n">
+        <v>53.58</v>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E299" t="n">
+        <v>338.7</v>
+      </c>
+      <c r="F299" t="n">
+        <v>334.88</v>
+      </c>
+      <c r="G299" t="n">
+        <v>-1.13</v>
+      </c>
+      <c r="H299" t="n">
+        <v>351.9299926757812</v>
+      </c>
+      <c r="I299" t="n">
+        <v>3.910000085830688</v>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K299" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N299" t="n">
+        <v>62.51</v>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E300" t="n">
+        <v>255.8</v>
+      </c>
+      <c r="F300" t="n">
+        <v>253.69</v>
+      </c>
+      <c r="G300" t="n">
+        <v>-0.82</v>
+      </c>
+      <c r="H300" t="n">
+        <v>253.3099975585938</v>
+      </c>
+      <c r="I300" t="n">
+        <v>-0.9700000286102295</v>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K300" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N300" t="n">
+        <v>58.98</v>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E301" t="n">
+        <v>4079.2</v>
+      </c>
+      <c r="F301" t="n">
+        <v>4035.01</v>
+      </c>
+      <c r="G301" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="H301" t="n">
+        <v>3613.75</v>
+      </c>
+      <c r="I301" t="n">
+        <v>-11.40999984741211</v>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K301" t="n">
+        <v>0.765</v>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N301" t="n">
+        <v>63.68</v>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
         </is>
       </c>
     </row>
@@ -18458,7 +19718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O141"/>
+  <dimension ref="A1:O151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27495,6 +28755,636 @@
       <c r="O141" t="inlineStr">
         <is>
           <t>21 Jan 2026, 06:57:52 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>1403.9</v>
+      </c>
+      <c r="F142" t="n">
+        <v>1603.58</v>
+      </c>
+      <c r="G142" t="n">
+        <v>14.22</v>
+      </c>
+      <c r="H142" t="n">
+        <v>1396.43994140625</v>
+      </c>
+      <c r="I142" t="n">
+        <v>-0.5299999713897705</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K142" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N142" t="n">
+        <v>83.06</v>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>3121.3</v>
+      </c>
+      <c r="F143" t="n">
+        <v>3172.14</v>
+      </c>
+      <c r="G143" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="H143" t="n">
+        <v>3175.7900390625</v>
+      </c>
+      <c r="I143" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K143" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N143" t="n">
+        <v>61.62</v>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>1654.6</v>
+      </c>
+      <c r="F144" t="n">
+        <v>1614.47</v>
+      </c>
+      <c r="G144" t="n">
+        <v>-2.43</v>
+      </c>
+      <c r="H144" t="n">
+        <v>1557.510009765625</v>
+      </c>
+      <c r="I144" t="n">
+        <v>-5.869999885559082</v>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K144" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N144" t="n">
+        <v>52.72</v>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>920.15</v>
+      </c>
+      <c r="F145" t="n">
+        <v>920.76</v>
+      </c>
+      <c r="G145" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H145" t="n">
+        <v>1125.800048828125</v>
+      </c>
+      <c r="I145" t="n">
+        <v>22.35000038146973</v>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K145" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N145" t="n">
+        <v>66.98</v>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>1348.45</v>
+      </c>
+      <c r="F146" t="n">
+        <v>1369.17</v>
+      </c>
+      <c r="G146" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="H146" t="n">
+        <v>1281.949951171875</v>
+      </c>
+      <c r="I146" t="n">
+        <v>-4.929999828338623</v>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K146" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N146" t="n">
+        <v>61.11</v>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>1028.15</v>
+      </c>
+      <c r="F147" t="n">
+        <v>1045.03</v>
+      </c>
+      <c r="G147" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="H147" t="n">
+        <v>1083.109985351562</v>
+      </c>
+      <c r="I147" t="n">
+        <v>5.349999904632568</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K147" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N147" t="n">
+        <v>59.26</v>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>324.7</v>
+      </c>
+      <c r="F148" t="n">
+        <v>343.91</v>
+      </c>
+      <c r="G148" t="n">
+        <v>5.92</v>
+      </c>
+      <c r="H148" t="n">
+        <v>362.9500122070312</v>
+      </c>
+      <c r="I148" t="n">
+        <v>11.77999973297119</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K148" t="n">
+        <v>-0.317</v>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N148" t="n">
+        <v>52.54</v>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>3767.15</v>
+      </c>
+      <c r="F149" t="n">
+        <v>3880.8</v>
+      </c>
+      <c r="G149" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="H149" t="n">
+        <v>3409.320068359375</v>
+      </c>
+      <c r="I149" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K149" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N149" t="n">
+        <v>59.05</v>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>1284.35</v>
+      </c>
+      <c r="F150" t="n">
+        <v>1239.04</v>
+      </c>
+      <c r="G150" t="n">
+        <v>-3.53</v>
+      </c>
+      <c r="H150" t="n">
+        <v>1096.72998046875</v>
+      </c>
+      <c r="I150" t="n">
+        <v>-14.60999965667725</v>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K150" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N150" t="n">
+        <v>57.71</v>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>15769.1</v>
+      </c>
+      <c r="F151" t="n">
+        <v>18225.18</v>
+      </c>
+      <c r="G151" t="n">
+        <v>15.58</v>
+      </c>
+      <c r="H151" t="n">
+        <v>13418.1103515625</v>
+      </c>
+      <c r="I151" t="n">
+        <v>-14.90999984741211</v>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K151" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N151" t="n">
+        <v>83.58</v>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
         </is>
       </c>
     </row>
@@ -27509,7 +29399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O281"/>
+  <dimension ref="A1:O301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45509,6 +47399,1266 @@
         </is>
       </c>
     </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E282" t="n">
+        <v>247.65</v>
+      </c>
+      <c r="F282" t="n">
+        <v>276.89</v>
+      </c>
+      <c r="G282" t="n">
+        <v>11.81</v>
+      </c>
+      <c r="H282" t="n">
+        <v>254.9499969482422</v>
+      </c>
+      <c r="I282" t="n">
+        <v>2.950000047683716</v>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K282" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N282" t="n">
+        <v>77.59</v>
+      </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E283" t="n">
+        <v>444.11</v>
+      </c>
+      <c r="F283" t="n">
+        <v>456.66</v>
+      </c>
+      <c r="G283" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="H283" t="n">
+        <v>401.5299987792969</v>
+      </c>
+      <c r="I283" t="n">
+        <v>-9.590000152587891</v>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K283" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N283" t="n">
+        <v>60.16</v>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E284" t="n">
+        <v>328.38</v>
+      </c>
+      <c r="F284" t="n">
+        <v>352.78</v>
+      </c>
+      <c r="G284" t="n">
+        <v>7.43</v>
+      </c>
+      <c r="H284" t="n">
+        <v>283.2200012207031</v>
+      </c>
+      <c r="I284" t="n">
+        <v>-13.75</v>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K284" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N284" t="n">
+        <v>74.34</v>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E285" t="n">
+        <v>231.31</v>
+      </c>
+      <c r="F285" t="n">
+        <v>248.22</v>
+      </c>
+      <c r="G285" t="n">
+        <v>7.31</v>
+      </c>
+      <c r="H285" t="n">
+        <v>250.3600006103516</v>
+      </c>
+      <c r="I285" t="n">
+        <v>8.239999771118164</v>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K285" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N285" t="n">
+        <v>47.97</v>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E286" t="n">
+        <v>612.96</v>
+      </c>
+      <c r="F286" t="n">
+        <v>707.51</v>
+      </c>
+      <c r="G286" t="n">
+        <v>15.42</v>
+      </c>
+      <c r="H286" t="n">
+        <v>555</v>
+      </c>
+      <c r="I286" t="n">
+        <v>-9.460000038146973</v>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K286" t="n">
+        <v>-0.67</v>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N286" t="n">
+        <v>59.74</v>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E287" t="n">
+        <v>431.44</v>
+      </c>
+      <c r="F287" t="n">
+        <v>440.82</v>
+      </c>
+      <c r="G287" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="H287" t="n">
+        <v>549.0999755859375</v>
+      </c>
+      <c r="I287" t="n">
+        <v>27.27000045776367</v>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K287" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N287" t="n">
+        <v>63.14</v>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E288" t="n">
+        <v>183.32</v>
+      </c>
+      <c r="F288" t="n">
+        <v>202.42</v>
+      </c>
+      <c r="G288" t="n">
+        <v>10.42</v>
+      </c>
+      <c r="H288" t="n">
+        <v>198.9600067138672</v>
+      </c>
+      <c r="I288" t="n">
+        <v>8.529999732971191</v>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K288" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N288" t="n">
+        <v>78.63</v>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E289" t="n">
+        <v>302.04</v>
+      </c>
+      <c r="F289" t="n">
+        <v>336.35</v>
+      </c>
+      <c r="G289" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="H289" t="n">
+        <v>238.8600006103516</v>
+      </c>
+      <c r="I289" t="n">
+        <v>-20.92000007629395</v>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K289" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N289" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E290" t="n">
+        <v>325.28</v>
+      </c>
+      <c r="F290" t="n">
+        <v>350.94</v>
+      </c>
+      <c r="G290" t="n">
+        <v>7.89</v>
+      </c>
+      <c r="H290" t="n">
+        <v>341.9400024414062</v>
+      </c>
+      <c r="I290" t="n">
+        <v>5.119999885559082</v>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K290" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N290" t="n">
+        <v>75.03</v>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E291" t="n">
+        <v>218.01</v>
+      </c>
+      <c r="F291" t="n">
+        <v>224.35</v>
+      </c>
+      <c r="G291" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="H291" t="n">
+        <v>249.3699951171875</v>
+      </c>
+      <c r="I291" t="n">
+        <v>14.38000011444092</v>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K291" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N291" t="n">
+        <v>60.72</v>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E292" t="n">
+        <v>119.36</v>
+      </c>
+      <c r="F292" t="n">
+        <v>119.89</v>
+      </c>
+      <c r="G292" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="H292" t="n">
+        <v>103.629997253418</v>
+      </c>
+      <c r="I292" t="n">
+        <v>-13.18000030517578</v>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K292" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N292" t="n">
+        <v>63.86</v>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>146.06</v>
+      </c>
+      <c r="F293" t="n">
+        <v>143.71</v>
+      </c>
+      <c r="G293" t="n">
+        <v>-1.61</v>
+      </c>
+      <c r="H293" t="n">
+        <v>154.4700012207031</v>
+      </c>
+      <c r="I293" t="n">
+        <v>5.760000228881836</v>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K293" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N293" t="n">
+        <v>60.58</v>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E294" t="n">
+        <v>527.5700000000001</v>
+      </c>
+      <c r="F294" t="n">
+        <v>573.36</v>
+      </c>
+      <c r="G294" t="n">
+        <v>8.68</v>
+      </c>
+      <c r="H294" t="n">
+        <v>652.280029296875</v>
+      </c>
+      <c r="I294" t="n">
+        <v>23.63999938964844</v>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K294" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N294" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>347.75</v>
+      </c>
+      <c r="F295" t="n">
+        <v>306.09</v>
+      </c>
+      <c r="G295" t="n">
+        <v>-11.98</v>
+      </c>
+      <c r="H295" t="n">
+        <v>335.1900024414062</v>
+      </c>
+      <c r="I295" t="n">
+        <v>-3.609999895095825</v>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K295" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N295" t="n">
+        <v>45.23</v>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E296" t="n">
+        <v>384.64</v>
+      </c>
+      <c r="F296" t="n">
+        <v>347.14</v>
+      </c>
+      <c r="G296" t="n">
+        <v>-9.75</v>
+      </c>
+      <c r="H296" t="n">
+        <v>408.5199890136719</v>
+      </c>
+      <c r="I296" t="n">
+        <v>6.210000038146973</v>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K296" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N296" t="n">
+        <v>48.58</v>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E297" t="n">
+        <v>52.07</v>
+      </c>
+      <c r="F297" t="n">
+        <v>55.94</v>
+      </c>
+      <c r="G297" t="n">
+        <v>7.43</v>
+      </c>
+      <c r="H297" t="n">
+        <v>55.72000122070312</v>
+      </c>
+      <c r="I297" t="n">
+        <v>7.010000228881836</v>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K297" t="n">
+        <v>0.735</v>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N297" t="n">
+        <v>75.84</v>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E298" t="n">
+        <v>133.61</v>
+      </c>
+      <c r="F298" t="n">
+        <v>129.28</v>
+      </c>
+      <c r="G298" t="n">
+        <v>-3.24</v>
+      </c>
+      <c r="H298" t="n">
+        <v>103.5299987792969</v>
+      </c>
+      <c r="I298" t="n">
+        <v>-22.52000045776367</v>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K298" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N298" t="n">
+        <v>60</v>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E299" t="n">
+        <v>328.8</v>
+      </c>
+      <c r="F299" t="n">
+        <v>397.18</v>
+      </c>
+      <c r="G299" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="H299" t="n">
+        <v>335.3699951171875</v>
+      </c>
+      <c r="I299" t="n">
+        <v>2</v>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K299" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N299" t="n">
+        <v>93.81999999999999</v>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E300" t="n">
+        <v>982.86</v>
+      </c>
+      <c r="F300" t="n">
+        <v>944.64</v>
+      </c>
+      <c r="G300" t="n">
+        <v>-3.89</v>
+      </c>
+      <c r="H300" t="n">
+        <v>913.52001953125</v>
+      </c>
+      <c r="I300" t="n">
+        <v>-7.050000190734863</v>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K300" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N300" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E301" t="n">
+        <v>146.74</v>
+      </c>
+      <c r="F301" t="n">
+        <v>149.11</v>
+      </c>
+      <c r="G301" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="H301" t="n">
+        <v>140.25</v>
+      </c>
+      <c r="I301" t="n">
+        <v>-4.429999828338623</v>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K301" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N301" t="n">
+        <v>65.81999999999999</v>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-23)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O301"/>
+  <dimension ref="A1:O321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19704,6 +19704,1266 @@
       <c r="O301" t="inlineStr">
         <is>
           <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E302" t="n">
+        <v>1402.5</v>
+      </c>
+      <c r="F302" t="n">
+        <v>1614.19</v>
+      </c>
+      <c r="G302" t="n">
+        <v>15.09</v>
+      </c>
+      <c r="H302" t="n">
+        <v>1402.880004882812</v>
+      </c>
+      <c r="I302" t="n">
+        <v>0.02999999932944775</v>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K302" t="n">
+        <v>-0.511</v>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N302" t="n">
+        <v>62.42</v>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E303" t="n">
+        <v>3150.4</v>
+      </c>
+      <c r="F303" t="n">
+        <v>3121.75</v>
+      </c>
+      <c r="G303" t="n">
+        <v>-0.91</v>
+      </c>
+      <c r="H303" t="n">
+        <v>3062.3798828125</v>
+      </c>
+      <c r="I303" t="n">
+        <v>-2.789999961853027</v>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K303" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N303" t="n">
+        <v>57.44</v>
+      </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E304" t="n">
+        <v>1663.5</v>
+      </c>
+      <c r="F304" t="n">
+        <v>1569.8</v>
+      </c>
+      <c r="G304" t="n">
+        <v>-5.63</v>
+      </c>
+      <c r="H304" t="n">
+        <v>1627.719970703125</v>
+      </c>
+      <c r="I304" t="n">
+        <v>-2.150000095367432</v>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K304" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N304" t="n">
+        <v>49.19</v>
+      </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E305" t="n">
+        <v>918.7</v>
+      </c>
+      <c r="F305" t="n">
+        <v>915.25</v>
+      </c>
+      <c r="G305" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="H305" t="n">
+        <v>1043.099975585938</v>
+      </c>
+      <c r="I305" t="n">
+        <v>13.53999996185303</v>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K305" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N305" t="n">
+        <v>65</v>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E306" t="n">
+        <v>1345.5</v>
+      </c>
+      <c r="F306" t="n">
+        <v>1376.57</v>
+      </c>
+      <c r="G306" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="H306" t="n">
+        <v>1283.900024414062</v>
+      </c>
+      <c r="I306" t="n">
+        <v>-4.579999923706055</v>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K306" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N306" t="n">
+        <v>60.26</v>
+      </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E307" t="n">
+        <v>1048.35</v>
+      </c>
+      <c r="F307" t="n">
+        <v>1063.27</v>
+      </c>
+      <c r="G307" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="H307" t="n">
+        <v>1273.079956054688</v>
+      </c>
+      <c r="I307" t="n">
+        <v>21.44000053405762</v>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K307" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N307" t="n">
+        <v>39.13</v>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E308" t="n">
+        <v>2390.6</v>
+      </c>
+      <c r="F308" t="n">
+        <v>2451.68</v>
+      </c>
+      <c r="G308" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="H308" t="n">
+        <v>2246.02001953125</v>
+      </c>
+      <c r="I308" t="n">
+        <v>-6.050000190734863</v>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K308" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N308" t="n">
+        <v>66.83</v>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E309" t="n">
+        <v>324.85</v>
+      </c>
+      <c r="F309" t="n">
+        <v>359.05</v>
+      </c>
+      <c r="G309" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="H309" t="n">
+        <v>368.1199951171875</v>
+      </c>
+      <c r="I309" t="n">
+        <v>13.31999969482422</v>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K309" t="n">
+        <v>-0.273</v>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N309" t="n">
+        <v>60.33</v>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E310" t="n">
+        <v>3793.8</v>
+      </c>
+      <c r="F310" t="n">
+        <v>3877.76</v>
+      </c>
+      <c r="G310" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="H310" t="n">
+        <v>3894.179931640625</v>
+      </c>
+      <c r="I310" t="n">
+        <v>2.650000095367432</v>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K310" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N310" t="n">
+        <v>57.84</v>
+      </c>
+      <c r="O310" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E311" t="n">
+        <v>942.85</v>
+      </c>
+      <c r="F311" t="n">
+        <v>1025.37</v>
+      </c>
+      <c r="G311" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="H311" t="n">
+        <v>832.6199951171875</v>
+      </c>
+      <c r="I311" t="n">
+        <v>-11.6899995803833</v>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K311" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N311" t="n">
+        <v>72.31</v>
+      </c>
+      <c r="O311" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E312" t="n">
+        <v>2002.2</v>
+      </c>
+      <c r="F312" t="n">
+        <v>2102.95</v>
+      </c>
+      <c r="G312" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="H312" t="n">
+        <v>2223.64990234375</v>
+      </c>
+      <c r="I312" t="n">
+        <v>11.0600004196167</v>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K312" t="n">
+        <v>-0.361</v>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M312" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N312" t="n">
+        <v>50.33</v>
+      </c>
+      <c r="O312" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E313" t="n">
+        <v>2703.8</v>
+      </c>
+      <c r="F313" t="n">
+        <v>2829.16</v>
+      </c>
+      <c r="G313" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="H313" t="n">
+        <v>2546.239990234375</v>
+      </c>
+      <c r="I313" t="n">
+        <v>-5.829999923706055</v>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K313" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N313" t="n">
+        <v>68.09</v>
+      </c>
+      <c r="O313" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E314" t="n">
+        <v>1294.8</v>
+      </c>
+      <c r="F314" t="n">
+        <v>1252.42</v>
+      </c>
+      <c r="G314" t="n">
+        <v>-3.27</v>
+      </c>
+      <c r="H314" t="n">
+        <v>1425.239990234375</v>
+      </c>
+      <c r="I314" t="n">
+        <v>10.06999969482422</v>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K314" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N314" t="n">
+        <v>58.49</v>
+      </c>
+      <c r="O314" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E315" t="n">
+        <v>15765</v>
+      </c>
+      <c r="F315" t="n">
+        <v>19030.49</v>
+      </c>
+      <c r="G315" t="n">
+        <v>20.71</v>
+      </c>
+      <c r="H315" t="n">
+        <v>16036.0595703125</v>
+      </c>
+      <c r="I315" t="n">
+        <v>1.720000028610229</v>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K315" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N315" t="n">
+        <v>90.22</v>
+      </c>
+      <c r="O315" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E316" t="n">
+        <v>1634.2</v>
+      </c>
+      <c r="F316" t="n">
+        <v>1735.09</v>
+      </c>
+      <c r="G316" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="H316" t="n">
+        <v>1722.449951171875</v>
+      </c>
+      <c r="I316" t="n">
+        <v>5.400000095367432</v>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K316" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N316" t="n">
+        <v>72.26000000000001</v>
+      </c>
+      <c r="O316" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E317" t="n">
+        <v>240.65</v>
+      </c>
+      <c r="F317" t="n">
+        <v>271.46</v>
+      </c>
+      <c r="G317" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="H317" t="n">
+        <v>233.2700042724609</v>
+      </c>
+      <c r="I317" t="n">
+        <v>-3.069999933242798</v>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K317" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N317" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="O317" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E318" t="n">
+        <v>12364</v>
+      </c>
+      <c r="F318" t="n">
+        <v>11676.65</v>
+      </c>
+      <c r="G318" t="n">
+        <v>-5.56</v>
+      </c>
+      <c r="H318" t="n">
+        <v>11420.7197265625</v>
+      </c>
+      <c r="I318" t="n">
+        <v>-7.630000114440918</v>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K318" t="n">
+        <v>-0.318</v>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M318" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N318" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="O318" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E319" t="n">
+        <v>342.45</v>
+      </c>
+      <c r="F319" t="n">
+        <v>336.55</v>
+      </c>
+      <c r="G319" t="n">
+        <v>-1.72</v>
+      </c>
+      <c r="H319" t="n">
+        <v>358.3200073242188</v>
+      </c>
+      <c r="I319" t="n">
+        <v>4.630000114440918</v>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K319" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N319" t="n">
+        <v>60.42</v>
+      </c>
+      <c r="O319" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E320" t="n">
+        <v>259.25</v>
+      </c>
+      <c r="F320" t="n">
+        <v>254.11</v>
+      </c>
+      <c r="G320" t="n">
+        <v>-1.98</v>
+      </c>
+      <c r="H320" t="n">
+        <v>261.4299926757812</v>
+      </c>
+      <c r="I320" t="n">
+        <v>0.8399999737739563</v>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K320" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N320" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="O320" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E321" t="n">
+        <v>4018.6</v>
+      </c>
+      <c r="F321" t="n">
+        <v>4264.87</v>
+      </c>
+      <c r="G321" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="H321" t="n">
+        <v>4496.18017578125</v>
+      </c>
+      <c r="I321" t="n">
+        <v>11.88000011444092</v>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K321" t="n">
+        <v>0.765</v>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M321" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N321" t="n">
+        <v>74.48999999999999</v>
+      </c>
+      <c r="O321" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
         </is>
       </c>
     </row>
@@ -19718,7 +20978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O151"/>
+  <dimension ref="A1:O161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29385,6 +30645,636 @@
       <c r="O151" t="inlineStr">
         <is>
           <t>22 Jan 2026, 06:58:33 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>1401.8</v>
+      </c>
+      <c r="F152" t="n">
+        <v>1623.7</v>
+      </c>
+      <c r="G152" t="n">
+        <v>15.83</v>
+      </c>
+      <c r="H152" t="n">
+        <v>1497.43994140625</v>
+      </c>
+      <c r="I152" t="n">
+        <v>6.820000171661377</v>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K152" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N152" t="n">
+        <v>85.45999999999999</v>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>3151.25</v>
+      </c>
+      <c r="F153" t="n">
+        <v>3167.43</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="H153" t="n">
+        <v>3232.219970703125</v>
+      </c>
+      <c r="I153" t="n">
+        <v>2.569999933242798</v>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K153" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N153" t="n">
+        <v>59.57</v>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>1663.35</v>
+      </c>
+      <c r="F154" t="n">
+        <v>1589.1</v>
+      </c>
+      <c r="G154" t="n">
+        <v>-4.46</v>
+      </c>
+      <c r="H154" t="n">
+        <v>1978.760009765625</v>
+      </c>
+      <c r="I154" t="n">
+        <v>18.95999908447266</v>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K154" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N154" t="n">
+        <v>50.94</v>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>919.4</v>
+      </c>
+      <c r="F155" t="n">
+        <v>917.74</v>
+      </c>
+      <c r="G155" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="H155" t="n">
+        <v>1141.949951171875</v>
+      </c>
+      <c r="I155" t="n">
+        <v>24.20999908447266</v>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K155" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N155" t="n">
+        <v>65.29000000000001</v>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>1345.65</v>
+      </c>
+      <c r="F156" t="n">
+        <v>1378.51</v>
+      </c>
+      <c r="G156" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="H156" t="n">
+        <v>1448</v>
+      </c>
+      <c r="I156" t="n">
+        <v>7.610000133514404</v>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K156" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N156" t="n">
+        <v>60.46</v>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>1048.25</v>
+      </c>
+      <c r="F157" t="n">
+        <v>1069.96</v>
+      </c>
+      <c r="G157" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="H157" t="n">
+        <v>1245.97998046875</v>
+      </c>
+      <c r="I157" t="n">
+        <v>18.86000061035156</v>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K157" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N157" t="n">
+        <v>40.11</v>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>324.9</v>
+      </c>
+      <c r="F158" t="n">
+        <v>364.08</v>
+      </c>
+      <c r="G158" t="n">
+        <v>12.06</v>
+      </c>
+      <c r="H158" t="n">
+        <v>375.6700134277344</v>
+      </c>
+      <c r="I158" t="n">
+        <v>15.63000011444092</v>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K158" t="n">
+        <v>-0.273</v>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N158" t="n">
+        <v>62.63</v>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>3794.3</v>
+      </c>
+      <c r="F159" t="n">
+        <v>3890.73</v>
+      </c>
+      <c r="G159" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="H159" t="n">
+        <v>3601.5400390625</v>
+      </c>
+      <c r="I159" t="n">
+        <v>-5.079999923706055</v>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K159" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N159" t="n">
+        <v>58.33</v>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>1295.35</v>
+      </c>
+      <c r="F160" t="n">
+        <v>1256.77</v>
+      </c>
+      <c r="G160" t="n">
+        <v>-2.98</v>
+      </c>
+      <c r="H160" t="n">
+        <v>1101.410034179688</v>
+      </c>
+      <c r="I160" t="n">
+        <v>-14.97000026702881</v>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K160" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N160" t="n">
+        <v>58.93</v>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>15764</v>
+      </c>
+      <c r="F161" t="n">
+        <v>19008.1</v>
+      </c>
+      <c r="G161" t="n">
+        <v>20.58</v>
+      </c>
+      <c r="H161" t="n">
+        <v>14184.7998046875</v>
+      </c>
+      <c r="I161" t="n">
+        <v>-10.02000045776367</v>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K161" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N161" t="n">
+        <v>90.22</v>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
         </is>
       </c>
     </row>
@@ -29399,7 +31289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O301"/>
+  <dimension ref="A1:O321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48659,6 +50549,1266 @@
         </is>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E302" t="n">
+        <v>248.35</v>
+      </c>
+      <c r="F302" t="n">
+        <v>271.54</v>
+      </c>
+      <c r="G302" t="n">
+        <v>9.34</v>
+      </c>
+      <c r="H302" t="n">
+        <v>215.2899932861328</v>
+      </c>
+      <c r="I302" t="n">
+        <v>-13.3100004196167</v>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K302" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N302" t="n">
+        <v>74.23</v>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E303" t="n">
+        <v>451.14</v>
+      </c>
+      <c r="F303" t="n">
+        <v>454.05</v>
+      </c>
+      <c r="G303" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="H303" t="n">
+        <v>389.6600036621094</v>
+      </c>
+      <c r="I303" t="n">
+        <v>-13.63000011444092</v>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K303" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N303" t="n">
+        <v>62.41</v>
+      </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E304" t="n">
+        <v>330.54</v>
+      </c>
+      <c r="F304" t="n">
+        <v>352.27</v>
+      </c>
+      <c r="G304" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="H304" t="n">
+        <v>361.260009765625</v>
+      </c>
+      <c r="I304" t="n">
+        <v>9.300000190734863</v>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K304" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N304" t="n">
+        <v>46.86</v>
+      </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E305" t="n">
+        <v>234.34</v>
+      </c>
+      <c r="F305" t="n">
+        <v>245.82</v>
+      </c>
+      <c r="G305" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="H305" t="n">
+        <v>208.1600036621094</v>
+      </c>
+      <c r="I305" t="n">
+        <v>-11.17000007629395</v>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K305" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N305" t="n">
+        <v>44.35</v>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E306" t="n">
+        <v>647.63</v>
+      </c>
+      <c r="F306" t="n">
+        <v>697.51</v>
+      </c>
+      <c r="G306" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="H306" t="n">
+        <v>676.260009765625</v>
+      </c>
+      <c r="I306" t="n">
+        <v>4.420000076293945</v>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K306" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N306" t="n">
+        <v>76.98999999999999</v>
+      </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E307" t="n">
+        <v>449.36</v>
+      </c>
+      <c r="F307" t="n">
+        <v>436.16</v>
+      </c>
+      <c r="G307" t="n">
+        <v>-2.94</v>
+      </c>
+      <c r="H307" t="n">
+        <v>401.0700073242188</v>
+      </c>
+      <c r="I307" t="n">
+        <v>-10.75</v>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K307" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N307" t="n">
+        <v>58.99</v>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E308" t="n">
+        <v>184.84</v>
+      </c>
+      <c r="F308" t="n">
+        <v>198.95</v>
+      </c>
+      <c r="G308" t="n">
+        <v>7.63</v>
+      </c>
+      <c r="H308" t="n">
+        <v>201.6499938964844</v>
+      </c>
+      <c r="I308" t="n">
+        <v>9.100000381469727</v>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K308" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N308" t="n">
+        <v>71.33</v>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E309" t="n">
+        <v>303.63</v>
+      </c>
+      <c r="F309" t="n">
+        <v>333.89</v>
+      </c>
+      <c r="G309" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="H309" t="n">
+        <v>296.5199890136719</v>
+      </c>
+      <c r="I309" t="n">
+        <v>-2.339999914169312</v>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K309" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N309" t="n">
+        <v>58.15</v>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E310" t="n">
+        <v>326.36</v>
+      </c>
+      <c r="F310" t="n">
+        <v>348.19</v>
+      </c>
+      <c r="G310" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="H310" t="n">
+        <v>323.989990234375</v>
+      </c>
+      <c r="I310" t="n">
+        <v>-0.7300000190734863</v>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K310" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N310" t="n">
+        <v>71.47</v>
+      </c>
+      <c r="O310" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E311" t="n">
+        <v>218.49</v>
+      </c>
+      <c r="F311" t="n">
+        <v>225.77</v>
+      </c>
+      <c r="G311" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="H311" t="n">
+        <v>263.2000122070312</v>
+      </c>
+      <c r="I311" t="n">
+        <v>20.45999908447266</v>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K311" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N311" t="n">
+        <v>68</v>
+      </c>
+      <c r="O311" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E312" t="n">
+        <v>117.83</v>
+      </c>
+      <c r="F312" t="n">
+        <v>120.65</v>
+      </c>
+      <c r="G312" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="H312" t="n">
+        <v>114.9700012207031</v>
+      </c>
+      <c r="I312" t="n">
+        <v>-2.430000066757202</v>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K312" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M312" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N312" t="n">
+        <v>66.79000000000001</v>
+      </c>
+      <c r="O312" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E313" t="n">
+        <v>149.93</v>
+      </c>
+      <c r="F313" t="n">
+        <v>144.27</v>
+      </c>
+      <c r="G313" t="n">
+        <v>-3.77</v>
+      </c>
+      <c r="H313" t="n">
+        <v>155.4600067138672</v>
+      </c>
+      <c r="I313" t="n">
+        <v>3.690000057220459</v>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K313" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N313" t="n">
+        <v>57.34</v>
+      </c>
+      <c r="O313" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E314" t="n">
+        <v>532.86</v>
+      </c>
+      <c r="F314" t="n">
+        <v>566.29</v>
+      </c>
+      <c r="G314" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="H314" t="n">
+        <v>542.8099975585938</v>
+      </c>
+      <c r="I314" t="n">
+        <v>1.870000004768372</v>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K314" t="n">
+        <v>0.637</v>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N314" t="n">
+        <v>72.15000000000001</v>
+      </c>
+      <c r="O314" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E315" t="n">
+        <v>354.47</v>
+      </c>
+      <c r="F315" t="n">
+        <v>313.99</v>
+      </c>
+      <c r="G315" t="n">
+        <v>-11.42</v>
+      </c>
+      <c r="H315" t="n">
+        <v>342.0599975585938</v>
+      </c>
+      <c r="I315" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K315" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N315" t="n">
+        <v>44.31</v>
+      </c>
+      <c r="O315" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E316" t="n">
+        <v>381.03</v>
+      </c>
+      <c r="F316" t="n">
+        <v>345.87</v>
+      </c>
+      <c r="G316" t="n">
+        <v>-9.23</v>
+      </c>
+      <c r="H316" t="n">
+        <v>383.5400085449219</v>
+      </c>
+      <c r="I316" t="n">
+        <v>0.6600000262260437</v>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K316" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N316" t="n">
+        <v>45.34</v>
+      </c>
+      <c r="O316" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E317" t="n">
+        <v>52.45</v>
+      </c>
+      <c r="F317" t="n">
+        <v>55.64</v>
+      </c>
+      <c r="G317" t="n">
+        <v>6.09</v>
+      </c>
+      <c r="H317" t="n">
+        <v>40.52000045776367</v>
+      </c>
+      <c r="I317" t="n">
+        <v>-22.75</v>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K317" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N317" t="n">
+        <v>72.33</v>
+      </c>
+      <c r="O317" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E318" t="n">
+        <v>133.64</v>
+      </c>
+      <c r="F318" t="n">
+        <v>129.1</v>
+      </c>
+      <c r="G318" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="H318" t="n">
+        <v>192.4900054931641</v>
+      </c>
+      <c r="I318" t="n">
+        <v>44.02999877929688</v>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K318" t="n">
+        <v>0.735</v>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M318" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N318" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="O318" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E319" t="n">
+        <v>325.49</v>
+      </c>
+      <c r="F319" t="n">
+        <v>393.73</v>
+      </c>
+      <c r="G319" t="n">
+        <v>20.97</v>
+      </c>
+      <c r="H319" t="n">
+        <v>357.6199951171875</v>
+      </c>
+      <c r="I319" t="n">
+        <v>9.869999885559082</v>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K319" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N319" t="n">
+        <v>93.81999999999999</v>
+      </c>
+      <c r="O319" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E320" t="n">
+        <v>976.17</v>
+      </c>
+      <c r="F320" t="n">
+        <v>945.26</v>
+      </c>
+      <c r="G320" t="n">
+        <v>-3.17</v>
+      </c>
+      <c r="H320" t="n">
+        <v>825.1500244140625</v>
+      </c>
+      <c r="I320" t="n">
+        <v>-15.47000026702881</v>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K320" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N320" t="n">
+        <v>58.25</v>
+      </c>
+      <c r="O320" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E321" t="n">
+        <v>144.4</v>
+      </c>
+      <c r="F321" t="n">
+        <v>149.26</v>
+      </c>
+      <c r="G321" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="H321" t="n">
+        <v>144.8699951171875</v>
+      </c>
+      <c r="I321" t="n">
+        <v>0.3300000131130219</v>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K321" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M321" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N321" t="n">
+        <v>68.25</v>
+      </c>
+      <c r="O321" t="inlineStr">
+        <is>
+          <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-24)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O321"/>
+  <dimension ref="A1:O341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20964,6 +20964,1266 @@
       <c r="O321" t="inlineStr">
         <is>
           <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E322" t="n">
+        <v>1386.1</v>
+      </c>
+      <c r="F322" t="n">
+        <v>1565.35</v>
+      </c>
+      <c r="G322" t="n">
+        <v>12.93</v>
+      </c>
+      <c r="H322" t="n">
+        <v>1430.150024414062</v>
+      </c>
+      <c r="I322" t="n">
+        <v>3.180000066757202</v>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K322" t="n">
+        <v>0.834</v>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M322" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N322" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="O322" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E323" t="n">
+        <v>3162.5</v>
+      </c>
+      <c r="F323" t="n">
+        <v>3121.67</v>
+      </c>
+      <c r="G323" t="n">
+        <v>-1.29</v>
+      </c>
+      <c r="H323" t="n">
+        <v>3172.830078125</v>
+      </c>
+      <c r="I323" t="n">
+        <v>0.3300000131130219</v>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K323" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N323" t="n">
+        <v>54.86</v>
+      </c>
+      <c r="O323" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E324" t="n">
+        <v>1670.8</v>
+      </c>
+      <c r="F324" t="n">
+        <v>1625.29</v>
+      </c>
+      <c r="G324" t="n">
+        <v>-2.72</v>
+      </c>
+      <c r="H324" t="n">
+        <v>1816.670043945312</v>
+      </c>
+      <c r="I324" t="n">
+        <v>8.729999542236328</v>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K324" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L324" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M324" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N324" t="n">
+        <v>52.71</v>
+      </c>
+      <c r="O324" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E325" t="n">
+        <v>916.1</v>
+      </c>
+      <c r="F325" t="n">
+        <v>913.09</v>
+      </c>
+      <c r="G325" t="n">
+        <v>-0.33</v>
+      </c>
+      <c r="H325" t="n">
+        <v>922.1900024414062</v>
+      </c>
+      <c r="I325" t="n">
+        <v>0.6700000166893005</v>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K325" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N325" t="n">
+        <v>65.06999999999999</v>
+      </c>
+      <c r="O325" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E326" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="F326" t="n">
+        <v>1363.56</v>
+      </c>
+      <c r="G326" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H326" t="n">
+        <v>1404.56005859375</v>
+      </c>
+      <c r="I326" t="n">
+        <v>4.550000190734863</v>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K326" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N326" t="n">
+        <v>47.73</v>
+      </c>
+      <c r="O326" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E327" t="n">
+        <v>1029.5</v>
+      </c>
+      <c r="F327" t="n">
+        <v>1050.77</v>
+      </c>
+      <c r="G327" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="H327" t="n">
+        <v>1271.199951171875</v>
+      </c>
+      <c r="I327" t="n">
+        <v>23.47999954223633</v>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K327" t="n">
+        <v>0.649</v>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M327" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N327" t="n">
+        <v>66.08</v>
+      </c>
+      <c r="O327" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E328" t="n">
+        <v>2409.5</v>
+      </c>
+      <c r="F328" t="n">
+        <v>2314.92</v>
+      </c>
+      <c r="G328" t="n">
+        <v>-3.93</v>
+      </c>
+      <c r="H328" t="n">
+        <v>2449.39990234375</v>
+      </c>
+      <c r="I328" t="n">
+        <v>1.659999966621399</v>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K328" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M328" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N328" t="n">
+        <v>57.11</v>
+      </c>
+      <c r="O328" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E329" t="n">
+        <v>323.4</v>
+      </c>
+      <c r="F329" t="n">
+        <v>333.27</v>
+      </c>
+      <c r="G329" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="H329" t="n">
+        <v>380.5700073242188</v>
+      </c>
+      <c r="I329" t="n">
+        <v>17.68000030517578</v>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K329" t="n">
+        <v>0.493</v>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N329" t="n">
+        <v>64.44</v>
+      </c>
+      <c r="O329" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E330" t="n">
+        <v>3743.8</v>
+      </c>
+      <c r="F330" t="n">
+        <v>3841.03</v>
+      </c>
+      <c r="G330" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H330" t="n">
+        <v>3763.090087890625</v>
+      </c>
+      <c r="I330" t="n">
+        <v>0.5199999809265137</v>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K330" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M330" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N330" t="n">
+        <v>58.42</v>
+      </c>
+      <c r="O330" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E331" t="n">
+        <v>927.85</v>
+      </c>
+      <c r="F331" t="n">
+        <v>1010.33</v>
+      </c>
+      <c r="G331" t="n">
+        <v>8.890000000000001</v>
+      </c>
+      <c r="H331" t="n">
+        <v>844.72998046875</v>
+      </c>
+      <c r="I331" t="n">
+        <v>-8.960000038146973</v>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K331" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L331" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M331" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N331" t="n">
+        <v>72.51000000000001</v>
+      </c>
+      <c r="O331" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E332" t="n">
+        <v>1984.7</v>
+      </c>
+      <c r="F332" t="n">
+        <v>2116.97</v>
+      </c>
+      <c r="G332" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="H332" t="n">
+        <v>2059.10009765625</v>
+      </c>
+      <c r="I332" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K332" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M332" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N332" t="n">
+        <v>69.18000000000001</v>
+      </c>
+      <c r="O332" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E333" t="n">
+        <v>2703.7</v>
+      </c>
+      <c r="F333" t="n">
+        <v>2749.45</v>
+      </c>
+      <c r="G333" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="H333" t="n">
+        <v>3037.739990234375</v>
+      </c>
+      <c r="I333" t="n">
+        <v>12.35000038146973</v>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K333" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M333" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N333" t="n">
+        <v>60.58</v>
+      </c>
+      <c r="O333" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E334" t="n">
+        <v>1258</v>
+      </c>
+      <c r="F334" t="n">
+        <v>1256.4</v>
+      </c>
+      <c r="G334" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="H334" t="n">
+        <v>1338.72998046875</v>
+      </c>
+      <c r="I334" t="n">
+        <v>6.420000076293945</v>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K334" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M334" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N334" t="n">
+        <v>63.21</v>
+      </c>
+      <c r="O334" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E335" t="n">
+        <v>15469</v>
+      </c>
+      <c r="F335" t="n">
+        <v>18091.32</v>
+      </c>
+      <c r="G335" t="n">
+        <v>16.95</v>
+      </c>
+      <c r="H335" t="n">
+        <v>12976.8701171875</v>
+      </c>
+      <c r="I335" t="n">
+        <v>-16.11000061035156</v>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K335" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L335" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M335" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N335" t="n">
+        <v>84.23</v>
+      </c>
+      <c r="O335" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E336" t="n">
+        <v>1631.9</v>
+      </c>
+      <c r="F336" t="n">
+        <v>1725.29</v>
+      </c>
+      <c r="G336" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="H336" t="n">
+        <v>1605.72998046875</v>
+      </c>
+      <c r="I336" t="n">
+        <v>-1.600000023841858</v>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K336" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M336" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N336" t="n">
+        <v>71.58</v>
+      </c>
+      <c r="O336" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E337" t="n">
+        <v>238.4</v>
+      </c>
+      <c r="F337" t="n">
+        <v>267.09</v>
+      </c>
+      <c r="G337" t="n">
+        <v>12.04</v>
+      </c>
+      <c r="H337" t="n">
+        <v>246.9700012207031</v>
+      </c>
+      <c r="I337" t="n">
+        <v>3.599999904632568</v>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K337" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="L337" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M337" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N337" t="n">
+        <v>83.73</v>
+      </c>
+      <c r="O337" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E338" t="n">
+        <v>12369</v>
+      </c>
+      <c r="F338" t="n">
+        <v>11685.29</v>
+      </c>
+      <c r="G338" t="n">
+        <v>-5.53</v>
+      </c>
+      <c r="H338" t="n">
+        <v>12668.98046875</v>
+      </c>
+      <c r="I338" t="n">
+        <v>2.430000066757202</v>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K338" t="n">
+        <v>0.735</v>
+      </c>
+      <c r="L338" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M338" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N338" t="n">
+        <v>56.41</v>
+      </c>
+      <c r="O338" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E339" t="n">
+        <v>336.7</v>
+      </c>
+      <c r="F339" t="n">
+        <v>336.68</v>
+      </c>
+      <c r="G339" t="n">
+        <v>0</v>
+      </c>
+      <c r="H339" t="n">
+        <v>346.1499938964844</v>
+      </c>
+      <c r="I339" t="n">
+        <v>2.809999942779541</v>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K339" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L339" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M339" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N339" t="n">
+        <v>62.99</v>
+      </c>
+      <c r="O339" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E340" t="n">
+        <v>254.15</v>
+      </c>
+      <c r="F340" t="n">
+        <v>252.73</v>
+      </c>
+      <c r="G340" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="H340" t="n">
+        <v>273.1900024414062</v>
+      </c>
+      <c r="I340" t="n">
+        <v>7.489999771118164</v>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K340" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="L340" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M340" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N340" t="n">
+        <v>61.14</v>
+      </c>
+      <c r="O340" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E341" t="n">
+        <v>4021.8</v>
+      </c>
+      <c r="F341" t="n">
+        <v>4094.69</v>
+      </c>
+      <c r="G341" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="H341" t="n">
+        <v>3992.669921875</v>
+      </c>
+      <c r="I341" t="n">
+        <v>-0.7200000286102295</v>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K341" t="n">
+        <v>0.765</v>
+      </c>
+      <c r="L341" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M341" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N341" t="n">
+        <v>68.02</v>
+      </c>
+      <c r="O341" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
         </is>
       </c>
     </row>
@@ -20978,7 +22238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O161"/>
+  <dimension ref="A1:O171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31275,6 +32535,636 @@
       <c r="O161" t="inlineStr">
         <is>
           <t>23 Jan 2026, 06:56:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>1385.95</v>
+      </c>
+      <c r="F162" t="n">
+        <v>1582.18</v>
+      </c>
+      <c r="G162" t="n">
+        <v>14.16</v>
+      </c>
+      <c r="H162" t="n">
+        <v>1223.569946289062</v>
+      </c>
+      <c r="I162" t="n">
+        <v>-11.72000026702881</v>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K162" t="n">
+        <v>0.834</v>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N162" t="n">
+        <v>87.92</v>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>3160.85</v>
+      </c>
+      <c r="F163" t="n">
+        <v>3134.6</v>
+      </c>
+      <c r="G163" t="n">
+        <v>-0.83</v>
+      </c>
+      <c r="H163" t="n">
+        <v>3344.2099609375</v>
+      </c>
+      <c r="I163" t="n">
+        <v>5.800000190734863</v>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K163" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N163" t="n">
+        <v>55.55</v>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>1670.6</v>
+      </c>
+      <c r="F164" t="n">
+        <v>1639.61</v>
+      </c>
+      <c r="G164" t="n">
+        <v>-1.86</v>
+      </c>
+      <c r="H164" t="n">
+        <v>1539.339965820312</v>
+      </c>
+      <c r="I164" t="n">
+        <v>-7.860000133514404</v>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K164" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N164" t="n">
+        <v>54.02</v>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>916.25</v>
+      </c>
+      <c r="F165" t="n">
+        <v>916.0599999999999</v>
+      </c>
+      <c r="G165" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="H165" t="n">
+        <v>950.6099853515625</v>
+      </c>
+      <c r="I165" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K165" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N165" t="n">
+        <v>65.53</v>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>1343.35</v>
+      </c>
+      <c r="F166" t="n">
+        <v>1365.4</v>
+      </c>
+      <c r="G166" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="H166" t="n">
+        <v>1396.150024414062</v>
+      </c>
+      <c r="I166" t="n">
+        <v>3.930000066757202</v>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K166" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N166" t="n">
+        <v>47.94</v>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>1029.4</v>
+      </c>
+      <c r="F167" t="n">
+        <v>1058.89</v>
+      </c>
+      <c r="G167" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="H167" t="n">
+        <v>1036.400024414062</v>
+      </c>
+      <c r="I167" t="n">
+        <v>0.6800000071525574</v>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K167" t="n">
+        <v>0.649</v>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N167" t="n">
+        <v>67.28</v>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>323.45</v>
+      </c>
+      <c r="F168" t="n">
+        <v>338.97</v>
+      </c>
+      <c r="G168" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H168" t="n">
+        <v>369.3099975585938</v>
+      </c>
+      <c r="I168" t="n">
+        <v>14.18000030517578</v>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K168" t="n">
+        <v>0.493</v>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N168" t="n">
+        <v>67.06</v>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>3745.05</v>
+      </c>
+      <c r="F169" t="n">
+        <v>3865.47</v>
+      </c>
+      <c r="G169" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="H169" t="n">
+        <v>3906.070068359375</v>
+      </c>
+      <c r="I169" t="n">
+        <v>4.300000190734863</v>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K169" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N169" t="n">
+        <v>59.34</v>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>1260.1</v>
+      </c>
+      <c r="F170" t="n">
+        <v>1255.15</v>
+      </c>
+      <c r="G170" t="n">
+        <v>-0.39</v>
+      </c>
+      <c r="H170" t="n">
+        <v>1092.089965820312</v>
+      </c>
+      <c r="I170" t="n">
+        <v>-13.32999992370605</v>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K170" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N170" t="n">
+        <v>62.81</v>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>15469.6</v>
+      </c>
+      <c r="F171" t="n">
+        <v>18101.6</v>
+      </c>
+      <c r="G171" t="n">
+        <v>17.01</v>
+      </c>
+      <c r="H171" t="n">
+        <v>16409.720703125</v>
+      </c>
+      <c r="I171" t="n">
+        <v>6.079999923706055</v>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K171" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N171" t="n">
+        <v>84.31999999999999</v>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
         </is>
       </c>
     </row>
@@ -31289,7 +33179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O321"/>
+  <dimension ref="A1:O341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51809,6 +53699,1266 @@
         </is>
       </c>
     </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E322" t="n">
+        <v>248.04</v>
+      </c>
+      <c r="F322" t="n">
+        <v>267.81</v>
+      </c>
+      <c r="G322" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="H322" t="n">
+        <v>253.0700073242188</v>
+      </c>
+      <c r="I322" t="n">
+        <v>2.029999971389771</v>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K322" t="n">
+        <v>0.361</v>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M322" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N322" t="n">
+        <v>69.18000000000001</v>
+      </c>
+      <c r="O322" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E323" t="n">
+        <v>465.95</v>
+      </c>
+      <c r="F323" t="n">
+        <v>452.75</v>
+      </c>
+      <c r="G323" t="n">
+        <v>-2.83</v>
+      </c>
+      <c r="H323" t="n">
+        <v>433.0799865722656</v>
+      </c>
+      <c r="I323" t="n">
+        <v>-7.059999942779541</v>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K323" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N323" t="n">
+        <v>59.75</v>
+      </c>
+      <c r="O323" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E324" t="n">
+        <v>327.93</v>
+      </c>
+      <c r="F324" t="n">
+        <v>351.24</v>
+      </c>
+      <c r="G324" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="H324" t="n">
+        <v>445.2000122070312</v>
+      </c>
+      <c r="I324" t="n">
+        <v>35.7599983215332</v>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K324" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L324" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M324" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N324" t="n">
+        <v>73.86</v>
+      </c>
+      <c r="O324" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E325" t="n">
+        <v>239.16</v>
+      </c>
+      <c r="F325" t="n">
+        <v>246</v>
+      </c>
+      <c r="G325" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="H325" t="n">
+        <v>250.3200073242188</v>
+      </c>
+      <c r="I325" t="n">
+        <v>4.670000076293945</v>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K325" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N325" t="n">
+        <v>41.29</v>
+      </c>
+      <c r="O325" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E326" t="n">
+        <v>658.76</v>
+      </c>
+      <c r="F326" t="n">
+        <v>696.39</v>
+      </c>
+      <c r="G326" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="H326" t="n">
+        <v>717.260009765625</v>
+      </c>
+      <c r="I326" t="n">
+        <v>8.880000114440918</v>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K326" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N326" t="n">
+        <v>71.77</v>
+      </c>
+      <c r="O326" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E327" t="n">
+        <v>449.06</v>
+      </c>
+      <c r="F327" t="n">
+        <v>434.17</v>
+      </c>
+      <c r="G327" t="n">
+        <v>-3.32</v>
+      </c>
+      <c r="H327" t="n">
+        <v>313.5299987792969</v>
+      </c>
+      <c r="I327" t="n">
+        <v>-30.18000030517578</v>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K327" t="n">
+        <v>0.727</v>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M327" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N327" t="n">
+        <v>59.57</v>
+      </c>
+      <c r="O327" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E328" t="n">
+        <v>187.67</v>
+      </c>
+      <c r="F328" t="n">
+        <v>199.19</v>
+      </c>
+      <c r="G328" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="H328" t="n">
+        <v>147.1900024414062</v>
+      </c>
+      <c r="I328" t="n">
+        <v>-21.56999969482422</v>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K328" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M328" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N328" t="n">
+        <v>74.36</v>
+      </c>
+      <c r="O328" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E329" t="n">
+        <v>297.72</v>
+      </c>
+      <c r="F329" t="n">
+        <v>333.17</v>
+      </c>
+      <c r="G329" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="H329" t="n">
+        <v>327.260009765625</v>
+      </c>
+      <c r="I329" t="n">
+        <v>9.920000076293945</v>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K329" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N329" t="n">
+        <v>61.06</v>
+      </c>
+      <c r="O329" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E330" t="n">
+        <v>326.18</v>
+      </c>
+      <c r="F330" t="n">
+        <v>346.98</v>
+      </c>
+      <c r="G330" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="H330" t="n">
+        <v>363.8099975585938</v>
+      </c>
+      <c r="I330" t="n">
+        <v>11.53999996185303</v>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K330" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M330" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N330" t="n">
+        <v>71.01000000000001</v>
+      </c>
+      <c r="O330" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E331" t="n">
+        <v>220.14</v>
+      </c>
+      <c r="F331" t="n">
+        <v>226.54</v>
+      </c>
+      <c r="G331" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="H331" t="n">
+        <v>203.2400054931641</v>
+      </c>
+      <c r="I331" t="n">
+        <v>-7.679999828338623</v>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K331" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L331" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M331" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N331" t="n">
+        <v>63.16</v>
+      </c>
+      <c r="O331" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E332" t="n">
+        <v>117.73</v>
+      </c>
+      <c r="F332" t="n">
+        <v>120.39</v>
+      </c>
+      <c r="G332" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="H332" t="n">
+        <v>115.25</v>
+      </c>
+      <c r="I332" t="n">
+        <v>-2.109999895095825</v>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K332" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M332" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N332" t="n">
+        <v>59.31</v>
+      </c>
+      <c r="O332" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E333" t="n">
+        <v>150.15</v>
+      </c>
+      <c r="F333" t="n">
+        <v>143.8</v>
+      </c>
+      <c r="G333" t="n">
+        <v>-4.23</v>
+      </c>
+      <c r="H333" t="n">
+        <v>147.0200042724609</v>
+      </c>
+      <c r="I333" t="n">
+        <v>-2.079999923706055</v>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K333" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M333" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N333" t="n">
+        <v>56.65</v>
+      </c>
+      <c r="O333" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E334" t="n">
+        <v>524.74</v>
+      </c>
+      <c r="F334" t="n">
+        <v>563.4299999999999</v>
+      </c>
+      <c r="G334" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="H334" t="n">
+        <v>533.8099975585938</v>
+      </c>
+      <c r="I334" t="n">
+        <v>1.730000019073486</v>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K334" t="n">
+        <v>0.637</v>
+      </c>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M334" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N334" t="n">
+        <v>73.8</v>
+      </c>
+      <c r="O334" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E335" t="n">
+        <v>356.26</v>
+      </c>
+      <c r="F335" t="n">
+        <v>315.25</v>
+      </c>
+      <c r="G335" t="n">
+        <v>-11.51</v>
+      </c>
+      <c r="H335" t="n">
+        <v>344.5700073242188</v>
+      </c>
+      <c r="I335" t="n">
+        <v>-3.279999971389771</v>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K335" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L335" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M335" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N335" t="n">
+        <v>19.73</v>
+      </c>
+      <c r="O335" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E336" t="n">
+        <v>383.77</v>
+      </c>
+      <c r="F336" t="n">
+        <v>346.84</v>
+      </c>
+      <c r="G336" t="n">
+        <v>-9.619999999999999</v>
+      </c>
+      <c r="H336" t="n">
+        <v>441.6300048828125</v>
+      </c>
+      <c r="I336" t="n">
+        <v>15.07999992370605</v>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K336" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M336" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N336" t="n">
+        <v>48.77</v>
+      </c>
+      <c r="O336" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E337" t="n">
+        <v>51.72</v>
+      </c>
+      <c r="F337" t="n">
+        <v>55.35</v>
+      </c>
+      <c r="G337" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="H337" t="n">
+        <v>50.95999908447266</v>
+      </c>
+      <c r="I337" t="n">
+        <v>-1.470000028610229</v>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K337" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L337" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M337" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N337" t="n">
+        <v>71.97</v>
+      </c>
+      <c r="O337" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E338" t="n">
+        <v>134.97</v>
+      </c>
+      <c r="F338" t="n">
+        <v>129.98</v>
+      </c>
+      <c r="G338" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="H338" t="n">
+        <v>204</v>
+      </c>
+      <c r="I338" t="n">
+        <v>51.15000152587891</v>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K338" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L338" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M338" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N338" t="n">
+        <v>54.33</v>
+      </c>
+      <c r="O338" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E339" t="n">
+        <v>320.05</v>
+      </c>
+      <c r="F339" t="n">
+        <v>384.44</v>
+      </c>
+      <c r="G339" t="n">
+        <v>20.12</v>
+      </c>
+      <c r="H339" t="n">
+        <v>394.4100036621094</v>
+      </c>
+      <c r="I339" t="n">
+        <v>23.22999954223633</v>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K339" t="n">
+        <v>0.827</v>
+      </c>
+      <c r="L339" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M339" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N339" t="n">
+        <v>96.54000000000001</v>
+      </c>
+      <c r="O339" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E340" t="n">
+        <v>983.25</v>
+      </c>
+      <c r="F340" t="n">
+        <v>948.02</v>
+      </c>
+      <c r="G340" t="n">
+        <v>-3.58</v>
+      </c>
+      <c r="H340" t="n">
+        <v>934.52001953125</v>
+      </c>
+      <c r="I340" t="n">
+        <v>-4.960000038146973</v>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K340" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L340" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M340" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N340" t="n">
+        <v>54.84</v>
+      </c>
+      <c r="O340" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E341" t="n">
+        <v>144.58</v>
+      </c>
+      <c r="F341" t="n">
+        <v>149.29</v>
+      </c>
+      <c r="G341" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="H341" t="n">
+        <v>148.1199951171875</v>
+      </c>
+      <c r="I341" t="n">
+        <v>2.450000047683716</v>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K341" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L341" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M341" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N341" t="n">
+        <v>68.28</v>
+      </c>
+      <c r="O341" t="inlineStr">
+        <is>
+          <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-25)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O341"/>
+  <dimension ref="A1:O361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22224,6 +22224,1266 @@
       <c r="O341" t="inlineStr">
         <is>
           <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E342" t="n">
+        <v>1386.1</v>
+      </c>
+      <c r="F342" t="n">
+        <v>1565.35</v>
+      </c>
+      <c r="G342" t="n">
+        <v>12.93</v>
+      </c>
+      <c r="H342" t="n">
+        <v>1323.119995117188</v>
+      </c>
+      <c r="I342" t="n">
+        <v>-4.539999961853027</v>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K342" t="n">
+        <v>0.834</v>
+      </c>
+      <c r="L342" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M342" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N342" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="O342" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E343" t="n">
+        <v>3162.5</v>
+      </c>
+      <c r="F343" t="n">
+        <v>3116.36</v>
+      </c>
+      <c r="G343" t="n">
+        <v>-1.46</v>
+      </c>
+      <c r="H343" t="n">
+        <v>3231.8701171875</v>
+      </c>
+      <c r="I343" t="n">
+        <v>2.190000057220459</v>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K343" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L343" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M343" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N343" t="n">
+        <v>58.95</v>
+      </c>
+      <c r="O343" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E344" t="n">
+        <v>1670.8</v>
+      </c>
+      <c r="F344" t="n">
+        <v>1616.87</v>
+      </c>
+      <c r="G344" t="n">
+        <v>-3.23</v>
+      </c>
+      <c r="H344" t="n">
+        <v>1501.239990234375</v>
+      </c>
+      <c r="I344" t="n">
+        <v>-10.14999961853027</v>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K344" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="L344" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M344" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N344" t="n">
+        <v>45.68</v>
+      </c>
+      <c r="O344" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E345" t="n">
+        <v>916.1</v>
+      </c>
+      <c r="F345" t="n">
+        <v>911.03</v>
+      </c>
+      <c r="G345" t="n">
+        <v>-0.55</v>
+      </c>
+      <c r="H345" t="n">
+        <v>845.8099975585938</v>
+      </c>
+      <c r="I345" t="n">
+        <v>-7.670000076293945</v>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K345" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L345" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M345" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N345" t="n">
+        <v>64.73</v>
+      </c>
+      <c r="O345" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E346" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="F346" t="n">
+        <v>1359.6</v>
+      </c>
+      <c r="G346" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="H346" t="n">
+        <v>1300.099975585938</v>
+      </c>
+      <c r="I346" t="n">
+        <v>-3.220000028610229</v>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K346" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="L346" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M346" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N346" t="n">
+        <v>47.29</v>
+      </c>
+      <c r="O346" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E347" t="n">
+        <v>1029.5</v>
+      </c>
+      <c r="F347" t="n">
+        <v>1049.35</v>
+      </c>
+      <c r="G347" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="H347" t="n">
+        <v>1030.449951171875</v>
+      </c>
+      <c r="I347" t="n">
+        <v>0.09000000357627869</v>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K347" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L347" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M347" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N347" t="n">
+        <v>39.89</v>
+      </c>
+      <c r="O347" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E348" t="n">
+        <v>2409.5</v>
+      </c>
+      <c r="F348" t="n">
+        <v>2312.72</v>
+      </c>
+      <c r="G348" t="n">
+        <v>-4.02</v>
+      </c>
+      <c r="H348" t="n">
+        <v>2456.639892578125</v>
+      </c>
+      <c r="I348" t="n">
+        <v>1.960000038146973</v>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K348" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L348" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M348" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N348" t="n">
+        <v>57.97</v>
+      </c>
+      <c r="O348" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E349" t="n">
+        <v>323.4</v>
+      </c>
+      <c r="F349" t="n">
+        <v>334.52</v>
+      </c>
+      <c r="G349" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="H349" t="n">
+        <v>374.3099975585938</v>
+      </c>
+      <c r="I349" t="n">
+        <v>15.73999977111816</v>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K349" t="n">
+        <v>-0.44</v>
+      </c>
+      <c r="L349" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M349" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N349" t="n">
+        <v>46.36</v>
+      </c>
+      <c r="O349" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E350" t="n">
+        <v>3743.8</v>
+      </c>
+      <c r="F350" t="n">
+        <v>3844.56</v>
+      </c>
+      <c r="G350" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="H350" t="n">
+        <v>3706.780029296875</v>
+      </c>
+      <c r="I350" t="n">
+        <v>-0.9900000095367432</v>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K350" t="n">
+        <v>0</v>
+      </c>
+      <c r="L350" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M350" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N350" t="n">
+        <v>54.04</v>
+      </c>
+      <c r="O350" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E351" t="n">
+        <v>927.85</v>
+      </c>
+      <c r="F351" t="n">
+        <v>1010.33</v>
+      </c>
+      <c r="G351" t="n">
+        <v>8.890000000000001</v>
+      </c>
+      <c r="H351" t="n">
+        <v>988.1099853515625</v>
+      </c>
+      <c r="I351" t="n">
+        <v>6.489999771118164</v>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K351" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M351" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N351" t="n">
+        <v>72.51000000000001</v>
+      </c>
+      <c r="O351" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E352" t="n">
+        <v>1984.7</v>
+      </c>
+      <c r="F352" t="n">
+        <v>2119.02</v>
+      </c>
+      <c r="G352" t="n">
+        <v>6.77</v>
+      </c>
+      <c r="H352" t="n">
+        <v>1923.2900390625</v>
+      </c>
+      <c r="I352" t="n">
+        <v>-3.089999914169312</v>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K352" t="n">
+        <v>0</v>
+      </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M352" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N352" t="n">
+        <v>60.15</v>
+      </c>
+      <c r="O352" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E353" t="n">
+        <v>2703.7</v>
+      </c>
+      <c r="F353" t="n">
+        <v>2724.8</v>
+      </c>
+      <c r="G353" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="H353" t="n">
+        <v>2812.35009765625</v>
+      </c>
+      <c r="I353" t="n">
+        <v>4.019999980926514</v>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K353" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M353" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N353" t="n">
+        <v>61.39</v>
+      </c>
+      <c r="O353" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E354" t="n">
+        <v>1258</v>
+      </c>
+      <c r="F354" t="n">
+        <v>1255.69</v>
+      </c>
+      <c r="G354" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="H354" t="n">
+        <v>1440.050048828125</v>
+      </c>
+      <c r="I354" t="n">
+        <v>14.47000026702881</v>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K354" t="n">
+        <v>-0.296</v>
+      </c>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M354" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N354" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="O354" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E355" t="n">
+        <v>15469</v>
+      </c>
+      <c r="F355" t="n">
+        <v>18067.57</v>
+      </c>
+      <c r="G355" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="H355" t="n">
+        <v>16768.5</v>
+      </c>
+      <c r="I355" t="n">
+        <v>8.399999618530273</v>
+      </c>
+      <c r="J355" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K355" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L355" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M355" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N355" t="n">
+        <v>84</v>
+      </c>
+      <c r="O355" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E356" t="n">
+        <v>1631.9</v>
+      </c>
+      <c r="F356" t="n">
+        <v>1738.38</v>
+      </c>
+      <c r="G356" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="H356" t="n">
+        <v>1533.02001953125</v>
+      </c>
+      <c r="I356" t="n">
+        <v>-6.059999942779541</v>
+      </c>
+      <c r="J356" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K356" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L356" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M356" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N356" t="n">
+        <v>72.79000000000001</v>
+      </c>
+      <c r="O356" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E357" t="n">
+        <v>238.4</v>
+      </c>
+      <c r="F357" t="n">
+        <v>267</v>
+      </c>
+      <c r="G357" t="n">
+        <v>12</v>
+      </c>
+      <c r="H357" t="n">
+        <v>288.6600036621094</v>
+      </c>
+      <c r="I357" t="n">
+        <v>21.07999992370605</v>
+      </c>
+      <c r="J357" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K357" t="n">
+        <v>-0.625</v>
+      </c>
+      <c r="L357" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M357" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N357" t="n">
+        <v>55.49</v>
+      </c>
+      <c r="O357" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E358" t="n">
+        <v>12369</v>
+      </c>
+      <c r="F358" t="n">
+        <v>11677.97</v>
+      </c>
+      <c r="G358" t="n">
+        <v>-5.59</v>
+      </c>
+      <c r="H358" t="n">
+        <v>10445.1201171875</v>
+      </c>
+      <c r="I358" t="n">
+        <v>-15.55000019073486</v>
+      </c>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K358" t="n">
+        <v>0.735</v>
+      </c>
+      <c r="L358" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M358" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N358" t="n">
+        <v>56.32</v>
+      </c>
+      <c r="O358" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E359" t="n">
+        <v>336.7</v>
+      </c>
+      <c r="F359" t="n">
+        <v>337.38</v>
+      </c>
+      <c r="G359" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H359" t="n">
+        <v>391.2300109863281</v>
+      </c>
+      <c r="I359" t="n">
+        <v>16.20000076293945</v>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K359" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L359" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M359" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N359" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="O359" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E360" t="n">
+        <v>254.15</v>
+      </c>
+      <c r="F360" t="n">
+        <v>253.42</v>
+      </c>
+      <c r="G360" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="H360" t="n">
+        <v>260.5899963378906</v>
+      </c>
+      <c r="I360" t="n">
+        <v>2.529999971389771</v>
+      </c>
+      <c r="J360" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K360" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="L360" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M360" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N360" t="n">
+        <v>61.55</v>
+      </c>
+      <c r="O360" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E361" t="n">
+        <v>4021.8</v>
+      </c>
+      <c r="F361" t="n">
+        <v>4087.02</v>
+      </c>
+      <c r="G361" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="H361" t="n">
+        <v>3801.25</v>
+      </c>
+      <c r="I361" t="n">
+        <v>-5.480000019073486</v>
+      </c>
+      <c r="J361" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K361" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L361" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M361" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N361" t="n">
+        <v>65.83</v>
+      </c>
+      <c r="O361" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
         </is>
       </c>
     </row>
@@ -22238,7 +23498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O171"/>
+  <dimension ref="A1:O181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33165,6 +34425,636 @@
       <c r="O171" t="inlineStr">
         <is>
           <t>24 Jan 2026, 06:39:42 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>1385.95</v>
+      </c>
+      <c r="F172" t="n">
+        <v>1582.05</v>
+      </c>
+      <c r="G172" t="n">
+        <v>14.15</v>
+      </c>
+      <c r="H172" t="n">
+        <v>1429.75</v>
+      </c>
+      <c r="I172" t="n">
+        <v>3.160000085830688</v>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K172" t="n">
+        <v>0.834</v>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N172" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>3160.85</v>
+      </c>
+      <c r="F173" t="n">
+        <v>3152.64</v>
+      </c>
+      <c r="G173" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="H173" t="n">
+        <v>3239.659912109375</v>
+      </c>
+      <c r="I173" t="n">
+        <v>2.490000009536743</v>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K173" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N173" t="n">
+        <v>60.75</v>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>1670.6</v>
+      </c>
+      <c r="F174" t="n">
+        <v>1648.05</v>
+      </c>
+      <c r="G174" t="n">
+        <v>-1.35</v>
+      </c>
+      <c r="H174" t="n">
+        <v>1590.02001953125</v>
+      </c>
+      <c r="I174" t="n">
+        <v>-4.820000171661377</v>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K174" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N174" t="n">
+        <v>54.34</v>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>916.25</v>
+      </c>
+      <c r="F175" t="n">
+        <v>915.04</v>
+      </c>
+      <c r="G175" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="H175" t="n">
+        <v>1050.989990234375</v>
+      </c>
+      <c r="I175" t="n">
+        <v>14.71000003814697</v>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K175" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N175" t="n">
+        <v>65.36</v>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>1343.35</v>
+      </c>
+      <c r="F176" t="n">
+        <v>1365.4</v>
+      </c>
+      <c r="G176" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="H176" t="n">
+        <v>1434.050048828125</v>
+      </c>
+      <c r="I176" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K176" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N176" t="n">
+        <v>47.94</v>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>1029.4</v>
+      </c>
+      <c r="F177" t="n">
+        <v>1060.07</v>
+      </c>
+      <c r="G177" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="H177" t="n">
+        <v>1180.199951171875</v>
+      </c>
+      <c r="I177" t="n">
+        <v>14.64999961853027</v>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K177" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N177" t="n">
+        <v>41.47</v>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>323.45</v>
+      </c>
+      <c r="F178" t="n">
+        <v>338.97</v>
+      </c>
+      <c r="G178" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H178" t="n">
+        <v>358.6300048828125</v>
+      </c>
+      <c r="I178" t="n">
+        <v>10.88000011444092</v>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K178" t="n">
+        <v>-0.44</v>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N178" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E179" t="n">
+        <v>3745.05</v>
+      </c>
+      <c r="F179" t="n">
+        <v>3865.47</v>
+      </c>
+      <c r="G179" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="H179" t="n">
+        <v>3618.27001953125</v>
+      </c>
+      <c r="I179" t="n">
+        <v>-3.390000104904175</v>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K179" t="n">
+        <v>0</v>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N179" t="n">
+        <v>54.82</v>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
+        <v>1260.1</v>
+      </c>
+      <c r="F180" t="n">
+        <v>1252.05</v>
+      </c>
+      <c r="G180" t="n">
+        <v>-0.64</v>
+      </c>
+      <c r="H180" t="n">
+        <v>1167.869995117188</v>
+      </c>
+      <c r="I180" t="n">
+        <v>-7.320000171661377</v>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K180" t="n">
+        <v>-0.511</v>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N180" t="n">
+        <v>38.82</v>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E181" t="n">
+        <v>15469.6</v>
+      </c>
+      <c r="F181" t="n">
+        <v>18101.6</v>
+      </c>
+      <c r="G181" t="n">
+        <v>17.01</v>
+      </c>
+      <c r="H181" t="n">
+        <v>12662.51953125</v>
+      </c>
+      <c r="I181" t="n">
+        <v>-18.14999961853027</v>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K181" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N181" t="n">
+        <v>84.31999999999999</v>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
         </is>
       </c>
     </row>
@@ -33179,7 +35069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O341"/>
+  <dimension ref="A1:O361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54959,6 +56849,1266 @@
         </is>
       </c>
     </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E342" t="n">
+        <v>248.04</v>
+      </c>
+      <c r="F342" t="n">
+        <v>271.29</v>
+      </c>
+      <c r="G342" t="n">
+        <v>9.369999999999999</v>
+      </c>
+      <c r="H342" t="n">
+        <v>240.1699981689453</v>
+      </c>
+      <c r="I342" t="n">
+        <v>-3.170000076293945</v>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K342" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L342" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M342" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N342" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="O342" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E343" t="n">
+        <v>465.95</v>
+      </c>
+      <c r="F343" t="n">
+        <v>451.25</v>
+      </c>
+      <c r="G343" t="n">
+        <v>-3.15</v>
+      </c>
+      <c r="H343" t="n">
+        <v>440.010009765625</v>
+      </c>
+      <c r="I343" t="n">
+        <v>-5.570000171661377</v>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K343" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L343" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M343" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N343" t="n">
+        <v>56.71</v>
+      </c>
+      <c r="O343" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E344" t="n">
+        <v>327.93</v>
+      </c>
+      <c r="F344" t="n">
+        <v>351.34</v>
+      </c>
+      <c r="G344" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="H344" t="n">
+        <v>299.739990234375</v>
+      </c>
+      <c r="I344" t="n">
+        <v>-8.590000152587891</v>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K344" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="L344" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M344" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N344" t="n">
+        <v>71.25</v>
+      </c>
+      <c r="O344" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E345" t="n">
+        <v>239.16</v>
+      </c>
+      <c r="F345" t="n">
+        <v>246</v>
+      </c>
+      <c r="G345" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="H345" t="n">
+        <v>241.3500061035156</v>
+      </c>
+      <c r="I345" t="n">
+        <v>0.9200000166893005</v>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K345" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L345" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M345" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N345" t="n">
+        <v>65.73</v>
+      </c>
+      <c r="O345" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E346" t="n">
+        <v>658.76</v>
+      </c>
+      <c r="F346" t="n">
+        <v>698.54</v>
+      </c>
+      <c r="G346" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="H346" t="n">
+        <v>542.4099731445312</v>
+      </c>
+      <c r="I346" t="n">
+        <v>-17.65999984741211</v>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K346" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L346" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M346" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N346" t="n">
+        <v>46.06</v>
+      </c>
+      <c r="O346" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E347" t="n">
+        <v>449.06</v>
+      </c>
+      <c r="F347" t="n">
+        <v>434.17</v>
+      </c>
+      <c r="G347" t="n">
+        <v>-3.32</v>
+      </c>
+      <c r="H347" t="n">
+        <v>402.2200012207031</v>
+      </c>
+      <c r="I347" t="n">
+        <v>-10.43000030517578</v>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K347" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L347" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M347" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N347" t="n">
+        <v>56.47</v>
+      </c>
+      <c r="O347" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E348" t="n">
+        <v>187.67</v>
+      </c>
+      <c r="F348" t="n">
+        <v>198.53</v>
+      </c>
+      <c r="G348" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="H348" t="n">
+        <v>119.9899978637695</v>
+      </c>
+      <c r="I348" t="n">
+        <v>-36.06000137329102</v>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K348" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L348" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M348" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N348" t="n">
+        <v>72.08</v>
+      </c>
+      <c r="O348" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E349" t="n">
+        <v>297.72</v>
+      </c>
+      <c r="F349" t="n">
+        <v>333.14</v>
+      </c>
+      <c r="G349" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="H349" t="n">
+        <v>282.8800048828125</v>
+      </c>
+      <c r="I349" t="n">
+        <v>-4.980000019073486</v>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K349" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L349" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M349" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N349" t="n">
+        <v>54.84</v>
+      </c>
+      <c r="O349" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E350" t="n">
+        <v>326.18</v>
+      </c>
+      <c r="F350" t="n">
+        <v>347.08</v>
+      </c>
+      <c r="G350" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="H350" t="n">
+        <v>336.1000061035156</v>
+      </c>
+      <c r="I350" t="n">
+        <v>3.039999961853027</v>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K350" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L350" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M350" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N350" t="n">
+        <v>72.81</v>
+      </c>
+      <c r="O350" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E351" t="n">
+        <v>220.14</v>
+      </c>
+      <c r="F351" t="n">
+        <v>226.34</v>
+      </c>
+      <c r="G351" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="H351" t="n">
+        <v>215.8899993896484</v>
+      </c>
+      <c r="I351" t="n">
+        <v>-1.929999947547913</v>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K351" t="n">
+        <v>0</v>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M351" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N351" t="n">
+        <v>54.23</v>
+      </c>
+      <c r="O351" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E352" t="n">
+        <v>117.73</v>
+      </c>
+      <c r="F352" t="n">
+        <v>120.28</v>
+      </c>
+      <c r="G352" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="H352" t="n">
+        <v>142.8699951171875</v>
+      </c>
+      <c r="I352" t="n">
+        <v>21.36000061035156</v>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K352" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M352" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N352" t="n">
+        <v>59.17</v>
+      </c>
+      <c r="O352" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E353" t="n">
+        <v>150.15</v>
+      </c>
+      <c r="F353" t="n">
+        <v>143.59</v>
+      </c>
+      <c r="G353" t="n">
+        <v>-4.37</v>
+      </c>
+      <c r="H353" t="n">
+        <v>149.1399993896484</v>
+      </c>
+      <c r="I353" t="n">
+        <v>-0.6700000166893005</v>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K353" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M353" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N353" t="n">
+        <v>56.45</v>
+      </c>
+      <c r="O353" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E354" t="n">
+        <v>524.74</v>
+      </c>
+      <c r="F354" t="n">
+        <v>564.02</v>
+      </c>
+      <c r="G354" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="H354" t="n">
+        <v>526.6599731445312</v>
+      </c>
+      <c r="I354" t="n">
+        <v>0.3700000047683716</v>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K354" t="n">
+        <v>0.637</v>
+      </c>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M354" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N354" t="n">
+        <v>73.97</v>
+      </c>
+      <c r="O354" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E355" t="n">
+        <v>356.26</v>
+      </c>
+      <c r="F355" t="n">
+        <v>311.48</v>
+      </c>
+      <c r="G355" t="n">
+        <v>-12.57</v>
+      </c>
+      <c r="H355" t="n">
+        <v>384.5400085449219</v>
+      </c>
+      <c r="I355" t="n">
+        <v>7.940000057220459</v>
+      </c>
+      <c r="J355" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K355" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L355" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M355" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N355" t="n">
+        <v>44.54</v>
+      </c>
+      <c r="O355" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E356" t="n">
+        <v>383.77</v>
+      </c>
+      <c r="F356" t="n">
+        <v>346.65</v>
+      </c>
+      <c r="G356" t="n">
+        <v>-9.67</v>
+      </c>
+      <c r="H356" t="n">
+        <v>392.4299926757812</v>
+      </c>
+      <c r="I356" t="n">
+        <v>2.259999990463257</v>
+      </c>
+      <c r="J356" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K356" t="n">
+        <v>0</v>
+      </c>
+      <c r="L356" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M356" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N356" t="n">
+        <v>35.49</v>
+      </c>
+      <c r="O356" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E357" t="n">
+        <v>51.72</v>
+      </c>
+      <c r="F357" t="n">
+        <v>55.31</v>
+      </c>
+      <c r="G357" t="n">
+        <v>6.94</v>
+      </c>
+      <c r="H357" t="n">
+        <v>47.02999877929688</v>
+      </c>
+      <c r="I357" t="n">
+        <v>-9.060000419616699</v>
+      </c>
+      <c r="J357" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K357" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L357" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M357" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N357" t="n">
+        <v>73.61</v>
+      </c>
+      <c r="O357" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E358" t="n">
+        <v>134.97</v>
+      </c>
+      <c r="F358" t="n">
+        <v>130.07</v>
+      </c>
+      <c r="G358" t="n">
+        <v>-3.63</v>
+      </c>
+      <c r="H358" t="n">
+        <v>160.4100036621094</v>
+      </c>
+      <c r="I358" t="n">
+        <v>18.85000038146973</v>
+      </c>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K358" t="n">
+        <v>0.361</v>
+      </c>
+      <c r="L358" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M358" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N358" t="n">
+        <v>51.77</v>
+      </c>
+      <c r="O358" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E359" t="n">
+        <v>320.05</v>
+      </c>
+      <c r="F359" t="n">
+        <v>391.81</v>
+      </c>
+      <c r="G359" t="n">
+        <v>22.42</v>
+      </c>
+      <c r="H359" t="n">
+        <v>399.7000122070312</v>
+      </c>
+      <c r="I359" t="n">
+        <v>24.88999938964844</v>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K359" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L359" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M359" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N359" t="n">
+        <v>93.2</v>
+      </c>
+      <c r="O359" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E360" t="n">
+        <v>983.25</v>
+      </c>
+      <c r="F360" t="n">
+        <v>947.75</v>
+      </c>
+      <c r="G360" t="n">
+        <v>-3.61</v>
+      </c>
+      <c r="H360" t="n">
+        <v>921.4600219726562</v>
+      </c>
+      <c r="I360" t="n">
+        <v>-6.28000020980835</v>
+      </c>
+      <c r="J360" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K360" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L360" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M360" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N360" t="n">
+        <v>57.98</v>
+      </c>
+      <c r="O360" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E361" t="n">
+        <v>144.58</v>
+      </c>
+      <c r="F361" t="n">
+        <v>149.04</v>
+      </c>
+      <c r="G361" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="H361" t="n">
+        <v>142.0399932861328</v>
+      </c>
+      <c r="I361" t="n">
+        <v>-1.759999990463257</v>
+      </c>
+      <c r="J361" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K361" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L361" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M361" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N361" t="n">
+        <v>66.06999999999999</v>
+      </c>
+      <c r="O361" t="inlineStr">
+        <is>
+          <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-26)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O361"/>
+  <dimension ref="A1:O381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23484,6 +23484,1266 @@
       <c r="O361" t="inlineStr">
         <is>
           <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E362" t="n">
+        <v>1386.1</v>
+      </c>
+      <c r="F362" t="n">
+        <v>1586.61</v>
+      </c>
+      <c r="G362" t="n">
+        <v>14.47</v>
+      </c>
+      <c r="H362" t="n">
+        <v>1483.329956054688</v>
+      </c>
+      <c r="I362" t="n">
+        <v>7.010000228881836</v>
+      </c>
+      <c r="J362" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K362" t="n">
+        <v>0.834</v>
+      </c>
+      <c r="L362" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M362" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N362" t="n">
+        <v>88.38</v>
+      </c>
+      <c r="O362" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E363" t="n">
+        <v>3162.5</v>
+      </c>
+      <c r="F363" t="n">
+        <v>3114.17</v>
+      </c>
+      <c r="G363" t="n">
+        <v>-1.53</v>
+      </c>
+      <c r="H363" t="n">
+        <v>3192.800048828125</v>
+      </c>
+      <c r="I363" t="n">
+        <v>0.9599999785423279</v>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K363" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L363" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M363" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N363" t="n">
+        <v>54.51</v>
+      </c>
+      <c r="O363" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E364" t="n">
+        <v>1670.8</v>
+      </c>
+      <c r="F364" t="n">
+        <v>1622.33</v>
+      </c>
+      <c r="G364" t="n">
+        <v>-2.9</v>
+      </c>
+      <c r="H364" t="n">
+        <v>2417.300048828125</v>
+      </c>
+      <c r="I364" t="n">
+        <v>44.68000030517578</v>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K364" t="n">
+        <v>0</v>
+      </c>
+      <c r="L364" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M364" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N364" t="n">
+        <v>45.65</v>
+      </c>
+      <c r="O364" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E365" t="n">
+        <v>916.1</v>
+      </c>
+      <c r="F365" t="n">
+        <v>913.01</v>
+      </c>
+      <c r="G365" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="H365" t="n">
+        <v>876.1699829101562</v>
+      </c>
+      <c r="I365" t="n">
+        <v>-4.360000133514404</v>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K365" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L365" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M365" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N365" t="n">
+        <v>62.69</v>
+      </c>
+      <c r="O365" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E366" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="F366" t="n">
+        <v>1359.6</v>
+      </c>
+      <c r="G366" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="H366" t="n">
+        <v>1578.630004882812</v>
+      </c>
+      <c r="I366" t="n">
+        <v>17.51000022888184</v>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K366" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L366" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M366" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N366" t="n">
+        <v>62.03</v>
+      </c>
+      <c r="O366" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E367" t="n">
+        <v>1029.5</v>
+      </c>
+      <c r="F367" t="n">
+        <v>1049.35</v>
+      </c>
+      <c r="G367" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="H367" t="n">
+        <v>1011.200012207031</v>
+      </c>
+      <c r="I367" t="n">
+        <v>-1.779999971389771</v>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K367" t="n">
+        <v>0.649</v>
+      </c>
+      <c r="L367" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M367" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N367" t="n">
+        <v>65.87</v>
+      </c>
+      <c r="O367" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E368" t="n">
+        <v>2409.5</v>
+      </c>
+      <c r="F368" t="n">
+        <v>2301.99</v>
+      </c>
+      <c r="G368" t="n">
+        <v>-4.46</v>
+      </c>
+      <c r="H368" t="n">
+        <v>2421.800048828125</v>
+      </c>
+      <c r="I368" t="n">
+        <v>0.5099999904632568</v>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K368" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="L368" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M368" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N368" t="n">
+        <v>53.85</v>
+      </c>
+      <c r="O368" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E369" t="n">
+        <v>323.4</v>
+      </c>
+      <c r="F369" t="n">
+        <v>333.51</v>
+      </c>
+      <c r="G369" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="H369" t="n">
+        <v>363.5599975585938</v>
+      </c>
+      <c r="I369" t="n">
+        <v>12.42000007629395</v>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K369" t="n">
+        <v>0.493</v>
+      </c>
+      <c r="L369" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M369" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N369" t="n">
+        <v>64.55</v>
+      </c>
+      <c r="O369" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E370" t="n">
+        <v>3743.8</v>
+      </c>
+      <c r="F370" t="n">
+        <v>3846.47</v>
+      </c>
+      <c r="G370" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="H370" t="n">
+        <v>3571.570068359375</v>
+      </c>
+      <c r="I370" t="n">
+        <v>-4.599999904632568</v>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K370" t="n">
+        <v>0</v>
+      </c>
+      <c r="L370" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M370" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N370" t="n">
+        <v>54.11</v>
+      </c>
+      <c r="O370" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E371" t="n">
+        <v>927.85</v>
+      </c>
+      <c r="F371" t="n">
+        <v>1008.51</v>
+      </c>
+      <c r="G371" t="n">
+        <v>8.69</v>
+      </c>
+      <c r="H371" t="n">
+        <v>845.0999755859375</v>
+      </c>
+      <c r="I371" t="n">
+        <v>-8.920000076293945</v>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K371" t="n">
+        <v>0.852</v>
+      </c>
+      <c r="L371" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M371" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N371" t="n">
+        <v>80.08</v>
+      </c>
+      <c r="O371" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E372" t="n">
+        <v>1984.7</v>
+      </c>
+      <c r="F372" t="n">
+        <v>2115.65</v>
+      </c>
+      <c r="G372" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="H372" t="n">
+        <v>2117.139892578125</v>
+      </c>
+      <c r="I372" t="n">
+        <v>6.670000076293945</v>
+      </c>
+      <c r="J372" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K372" t="n">
+        <v>0</v>
+      </c>
+      <c r="L372" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M372" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N372" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="O372" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E373" t="n">
+        <v>2703.7</v>
+      </c>
+      <c r="F373" t="n">
+        <v>2740.04</v>
+      </c>
+      <c r="G373" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="H373" t="n">
+        <v>2607.199951171875</v>
+      </c>
+      <c r="I373" t="n">
+        <v>-3.569999933242798</v>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K373" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="L373" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M373" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N373" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="O373" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E374" t="n">
+        <v>1258</v>
+      </c>
+      <c r="F374" t="n">
+        <v>1256.4</v>
+      </c>
+      <c r="G374" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="H374" t="n">
+        <v>1114.859985351562</v>
+      </c>
+      <c r="I374" t="n">
+        <v>-11.38000011444092</v>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K374" t="n">
+        <v>0.852</v>
+      </c>
+      <c r="L374" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M374" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N374" t="n">
+        <v>66.84999999999999</v>
+      </c>
+      <c r="O374" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E375" t="n">
+        <v>15469</v>
+      </c>
+      <c r="F375" t="n">
+        <v>18118.48</v>
+      </c>
+      <c r="G375" t="n">
+        <v>17.13</v>
+      </c>
+      <c r="H375" t="n">
+        <v>14713.51953125</v>
+      </c>
+      <c r="I375" t="n">
+        <v>-4.880000114440918</v>
+      </c>
+      <c r="J375" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K375" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L375" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M375" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N375" t="n">
+        <v>84.48999999999999</v>
+      </c>
+      <c r="O375" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E376" t="n">
+        <v>1631.9</v>
+      </c>
+      <c r="F376" t="n">
+        <v>1735.68</v>
+      </c>
+      <c r="G376" t="n">
+        <v>6.36</v>
+      </c>
+      <c r="H376" t="n">
+        <v>1620.97998046875</v>
+      </c>
+      <c r="I376" t="n">
+        <v>-0.6700000166893005</v>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K376" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L376" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M376" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N376" t="n">
+        <v>72.54000000000001</v>
+      </c>
+      <c r="O376" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E377" t="n">
+        <v>238.4</v>
+      </c>
+      <c r="F377" t="n">
+        <v>267.9</v>
+      </c>
+      <c r="G377" t="n">
+        <v>12.37</v>
+      </c>
+      <c r="H377" t="n">
+        <v>238.7700042724609</v>
+      </c>
+      <c r="I377" t="n">
+        <v>0.1599999964237213</v>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K377" t="n">
+        <v>-0.625</v>
+      </c>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N377" t="n">
+        <v>56.06</v>
+      </c>
+      <c r="O377" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E378" t="n">
+        <v>12369</v>
+      </c>
+      <c r="F378" t="n">
+        <v>11664.3</v>
+      </c>
+      <c r="G378" t="n">
+        <v>-5.7</v>
+      </c>
+      <c r="H378" t="n">
+        <v>10775.3095703125</v>
+      </c>
+      <c r="I378" t="n">
+        <v>-12.88000011444092</v>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K378" t="n">
+        <v>0.735</v>
+      </c>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M378" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N378" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="O378" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E379" t="n">
+        <v>336.7</v>
+      </c>
+      <c r="F379" t="n">
+        <v>336.86</v>
+      </c>
+      <c r="G379" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H379" t="n">
+        <v>322.3900146484375</v>
+      </c>
+      <c r="I379" t="n">
+        <v>-4.25</v>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K379" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L379" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M379" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N379" t="n">
+        <v>63.07</v>
+      </c>
+      <c r="O379" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E380" t="n">
+        <v>254.15</v>
+      </c>
+      <c r="F380" t="n">
+        <v>252.82</v>
+      </c>
+      <c r="G380" t="n">
+        <v>-0.52</v>
+      </c>
+      <c r="H380" t="n">
+        <v>282.3500061035156</v>
+      </c>
+      <c r="I380" t="n">
+        <v>11.10000038146973</v>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K380" t="n">
+        <v>0.542</v>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N380" t="n">
+        <v>60.05</v>
+      </c>
+      <c r="O380" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E381" t="n">
+        <v>4021.8</v>
+      </c>
+      <c r="F381" t="n">
+        <v>4087.02</v>
+      </c>
+      <c r="G381" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="H381" t="n">
+        <v>3943.050048828125</v>
+      </c>
+      <c r="I381" t="n">
+        <v>-1.960000038146973</v>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K381" t="n">
+        <v>0.727</v>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N381" t="n">
+        <v>66.97</v>
+      </c>
+      <c r="O381" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
         </is>
       </c>
     </row>
@@ -23498,7 +24758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O181"/>
+  <dimension ref="A1:O191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35055,6 +36315,636 @@
       <c r="O181" t="inlineStr">
         <is>
           <t>25 Jan 2026, 06:41:05 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>1385.95</v>
+      </c>
+      <c r="F182" t="n">
+        <v>1566.63</v>
+      </c>
+      <c r="G182" t="n">
+        <v>13.04</v>
+      </c>
+      <c r="H182" t="n">
+        <v>1328.069946289062</v>
+      </c>
+      <c r="I182" t="n">
+        <v>-4.179999828338623</v>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K182" t="n">
+        <v>0.834</v>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N182" t="n">
+        <v>86.23999999999999</v>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E183" t="n">
+        <v>3160.85</v>
+      </c>
+      <c r="F183" t="n">
+        <v>3153.45</v>
+      </c>
+      <c r="G183" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="H183" t="n">
+        <v>3209.010009765625</v>
+      </c>
+      <c r="I183" t="n">
+        <v>1.519999980926514</v>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K183" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N183" t="n">
+        <v>56.45</v>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E184" t="n">
+        <v>1670.6</v>
+      </c>
+      <c r="F184" t="n">
+        <v>1638.28</v>
+      </c>
+      <c r="G184" t="n">
+        <v>-1.93</v>
+      </c>
+      <c r="H184" t="n">
+        <v>1350.760009765625</v>
+      </c>
+      <c r="I184" t="n">
+        <v>-19.14999961853027</v>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K184" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N184" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E185" t="n">
+        <v>916.25</v>
+      </c>
+      <c r="F185" t="n">
+        <v>917.15</v>
+      </c>
+      <c r="G185" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H185" t="n">
+        <v>988.3200073242188</v>
+      </c>
+      <c r="I185" t="n">
+        <v>7.869999885559082</v>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K185" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N185" t="n">
+        <v>63.35</v>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>1343.35</v>
+      </c>
+      <c r="F186" t="n">
+        <v>1362.01</v>
+      </c>
+      <c r="G186" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="H186" t="n">
+        <v>1330.510009765625</v>
+      </c>
+      <c r="I186" t="n">
+        <v>-0.9599999785423279</v>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K186" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N186" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E187" t="n">
+        <v>1029.4</v>
+      </c>
+      <c r="F187" t="n">
+        <v>1058.79</v>
+      </c>
+      <c r="G187" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="H187" t="n">
+        <v>1277.489990234375</v>
+      </c>
+      <c r="I187" t="n">
+        <v>24.10000038146973</v>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K187" t="n">
+        <v>0.649</v>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N187" t="n">
+        <v>67.26000000000001</v>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E188" t="n">
+        <v>323.45</v>
+      </c>
+      <c r="F188" t="n">
+        <v>338.22</v>
+      </c>
+      <c r="G188" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="H188" t="n">
+        <v>355.75</v>
+      </c>
+      <c r="I188" t="n">
+        <v>9.989999771118164</v>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K188" t="n">
+        <v>-0.44</v>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N188" t="n">
+        <v>48.05</v>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E189" t="n">
+        <v>3745.05</v>
+      </c>
+      <c r="F189" t="n">
+        <v>3863.82</v>
+      </c>
+      <c r="G189" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="H189" t="n">
+        <v>3650.409912109375</v>
+      </c>
+      <c r="I189" t="n">
+        <v>-2.529999971389771</v>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K189" t="n">
+        <v>0</v>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N189" t="n">
+        <v>54.76</v>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E190" t="n">
+        <v>1260.1</v>
+      </c>
+      <c r="F190" t="n">
+        <v>1252.05</v>
+      </c>
+      <c r="G190" t="n">
+        <v>-0.64</v>
+      </c>
+      <c r="H190" t="n">
+        <v>1279.300048828125</v>
+      </c>
+      <c r="I190" t="n">
+        <v>1.519999980926514</v>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K190" t="n">
+        <v>0.852</v>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N190" t="n">
+        <v>66.08</v>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E191" t="n">
+        <v>15469.6</v>
+      </c>
+      <c r="F191" t="n">
+        <v>18101.6</v>
+      </c>
+      <c r="G191" t="n">
+        <v>17.01</v>
+      </c>
+      <c r="H191" t="n">
+        <v>13778.4599609375</v>
+      </c>
+      <c r="I191" t="n">
+        <v>-10.93000030517578</v>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K191" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N191" t="n">
+        <v>84.31999999999999</v>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
         </is>
       </c>
     </row>
@@ -35069,7 +36959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O361"/>
+  <dimension ref="A1:O381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58109,6 +59999,1266 @@
         </is>
       </c>
     </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E362" t="n">
+        <v>248.04</v>
+      </c>
+      <c r="F362" t="n">
+        <v>271.67</v>
+      </c>
+      <c r="G362" t="n">
+        <v>9.529999999999999</v>
+      </c>
+      <c r="H362" t="n">
+        <v>240.3000030517578</v>
+      </c>
+      <c r="I362" t="n">
+        <v>-3.119999885559082</v>
+      </c>
+      <c r="J362" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K362" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L362" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M362" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N362" t="n">
+        <v>74.17</v>
+      </c>
+      <c r="O362" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E363" t="n">
+        <v>465.95</v>
+      </c>
+      <c r="F363" t="n">
+        <v>450.39</v>
+      </c>
+      <c r="G363" t="n">
+        <v>-3.34</v>
+      </c>
+      <c r="H363" t="n">
+        <v>468.7900085449219</v>
+      </c>
+      <c r="I363" t="n">
+        <v>0.6100000143051147</v>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K363" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L363" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M363" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N363" t="n">
+        <v>54.17</v>
+      </c>
+      <c r="O363" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E364" t="n">
+        <v>327.93</v>
+      </c>
+      <c r="F364" t="n">
+        <v>351.24</v>
+      </c>
+      <c r="G364" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="H364" t="n">
+        <v>375.5499877929688</v>
+      </c>
+      <c r="I364" t="n">
+        <v>14.52000045776367</v>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K364" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="L364" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M364" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N364" t="n">
+        <v>75.81999999999999</v>
+      </c>
+      <c r="O364" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E365" t="n">
+        <v>239.16</v>
+      </c>
+      <c r="F365" t="n">
+        <v>246</v>
+      </c>
+      <c r="G365" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="H365" t="n">
+        <v>219.6600036621094</v>
+      </c>
+      <c r="I365" t="n">
+        <v>-8.149999618530273</v>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K365" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L365" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M365" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N365" t="n">
+        <v>41.29</v>
+      </c>
+      <c r="O365" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E366" t="n">
+        <v>658.76</v>
+      </c>
+      <c r="F366" t="n">
+        <v>697.5599999999999</v>
+      </c>
+      <c r="G366" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="H366" t="n">
+        <v>608.9099731445312</v>
+      </c>
+      <c r="I366" t="n">
+        <v>-7.570000171661377</v>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K366" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L366" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M366" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N366" t="n">
+        <v>45.83</v>
+      </c>
+      <c r="O366" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E367" t="n">
+        <v>449.06</v>
+      </c>
+      <c r="F367" t="n">
+        <v>434.17</v>
+      </c>
+      <c r="G367" t="n">
+        <v>-3.32</v>
+      </c>
+      <c r="H367" t="n">
+        <v>385.0799865722656</v>
+      </c>
+      <c r="I367" t="n">
+        <v>-14.25</v>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K367" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L367" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M367" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N367" t="n">
+        <v>54.91</v>
+      </c>
+      <c r="O367" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E368" t="n">
+        <v>187.67</v>
+      </c>
+      <c r="F368" t="n">
+        <v>198.69</v>
+      </c>
+      <c r="G368" t="n">
+        <v>5.87</v>
+      </c>
+      <c r="H368" t="n">
+        <v>139.0500030517578</v>
+      </c>
+      <c r="I368" t="n">
+        <v>-25.90999984741211</v>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K368" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L368" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M368" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N368" t="n">
+        <v>64.73</v>
+      </c>
+      <c r="O368" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E369" t="n">
+        <v>297.72</v>
+      </c>
+      <c r="F369" t="n">
+        <v>332.36</v>
+      </c>
+      <c r="G369" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="H369" t="n">
+        <v>342.760009765625</v>
+      </c>
+      <c r="I369" t="n">
+        <v>15.13000011444092</v>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K369" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L369" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M369" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N369" t="n">
+        <v>54.45</v>
+      </c>
+      <c r="O369" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E370" t="n">
+        <v>326.18</v>
+      </c>
+      <c r="F370" t="n">
+        <v>347.15</v>
+      </c>
+      <c r="G370" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="H370" t="n">
+        <v>350.0299987792969</v>
+      </c>
+      <c r="I370" t="n">
+        <v>7.309999942779541</v>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K370" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L370" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M370" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N370" t="n">
+        <v>72.84</v>
+      </c>
+      <c r="O370" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E371" t="n">
+        <v>220.14</v>
+      </c>
+      <c r="F371" t="n">
+        <v>226.83</v>
+      </c>
+      <c r="G371" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="H371" t="n">
+        <v>271.510009765625</v>
+      </c>
+      <c r="I371" t="n">
+        <v>23.32999992370605</v>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K371" t="n">
+        <v>0</v>
+      </c>
+      <c r="L371" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M371" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N371" t="n">
+        <v>54.56</v>
+      </c>
+      <c r="O371" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E372" t="n">
+        <v>117.73</v>
+      </c>
+      <c r="F372" t="n">
+        <v>120.36</v>
+      </c>
+      <c r="G372" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="H372" t="n">
+        <v>109.1900024414062</v>
+      </c>
+      <c r="I372" t="n">
+        <v>-7.25</v>
+      </c>
+      <c r="J372" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K372" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L372" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M372" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N372" t="n">
+        <v>59.27</v>
+      </c>
+      <c r="O372" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E373" t="n">
+        <v>150.15</v>
+      </c>
+      <c r="F373" t="n">
+        <v>143.5</v>
+      </c>
+      <c r="G373" t="n">
+        <v>-4.43</v>
+      </c>
+      <c r="H373" t="n">
+        <v>151.7100067138672</v>
+      </c>
+      <c r="I373" t="n">
+        <v>1.039999961853027</v>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K373" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L373" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M373" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N373" t="n">
+        <v>56.36</v>
+      </c>
+      <c r="O373" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E374" t="n">
+        <v>524.74</v>
+      </c>
+      <c r="F374" t="n">
+        <v>566.09</v>
+      </c>
+      <c r="G374" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="H374" t="n">
+        <v>570.469970703125</v>
+      </c>
+      <c r="I374" t="n">
+        <v>8.710000038146973</v>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K374" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L374" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M374" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N374" t="n">
+        <v>71.36</v>
+      </c>
+      <c r="O374" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E375" t="n">
+        <v>356.26</v>
+      </c>
+      <c r="F375" t="n">
+        <v>312.88</v>
+      </c>
+      <c r="G375" t="n">
+        <v>-12.18</v>
+      </c>
+      <c r="H375" t="n">
+        <v>372.3099975585938</v>
+      </c>
+      <c r="I375" t="n">
+        <v>4.510000228881836</v>
+      </c>
+      <c r="J375" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K375" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L375" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M375" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N375" t="n">
+        <v>45.14</v>
+      </c>
+      <c r="O375" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E376" t="n">
+        <v>383.77</v>
+      </c>
+      <c r="F376" t="n">
+        <v>346.15</v>
+      </c>
+      <c r="G376" t="n">
+        <v>-9.800000000000001</v>
+      </c>
+      <c r="H376" t="n">
+        <v>388.3399963378906</v>
+      </c>
+      <c r="I376" t="n">
+        <v>1.190000057220459</v>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K376" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L376" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M376" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N376" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="O376" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E377" t="n">
+        <v>51.72</v>
+      </c>
+      <c r="F377" t="n">
+        <v>55.31</v>
+      </c>
+      <c r="G377" t="n">
+        <v>6.93</v>
+      </c>
+      <c r="H377" t="n">
+        <v>58.66999816894531</v>
+      </c>
+      <c r="I377" t="n">
+        <v>13.4399995803833</v>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K377" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N377" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="O377" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E378" t="n">
+        <v>134.97</v>
+      </c>
+      <c r="F378" t="n">
+        <v>129.97</v>
+      </c>
+      <c r="G378" t="n">
+        <v>-3.71</v>
+      </c>
+      <c r="H378" t="n">
+        <v>140.9499969482422</v>
+      </c>
+      <c r="I378" t="n">
+        <v>4.429999828338623</v>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K378" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M378" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N378" t="n">
+        <v>55.88</v>
+      </c>
+      <c r="O378" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E379" t="n">
+        <v>320.05</v>
+      </c>
+      <c r="F379" t="n">
+        <v>392.48</v>
+      </c>
+      <c r="G379" t="n">
+        <v>22.63</v>
+      </c>
+      <c r="H379" t="n">
+        <v>350.3500061035156</v>
+      </c>
+      <c r="I379" t="n">
+        <v>9.470000267028809</v>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K379" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L379" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M379" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N379" t="n">
+        <v>93.40000000000001</v>
+      </c>
+      <c r="O379" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E380" t="n">
+        <v>983.25</v>
+      </c>
+      <c r="F380" t="n">
+        <v>945.58</v>
+      </c>
+      <c r="G380" t="n">
+        <v>-3.83</v>
+      </c>
+      <c r="H380" t="n">
+        <v>897</v>
+      </c>
+      <c r="I380" t="n">
+        <v>-8.770000457763672</v>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K380" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N380" t="n">
+        <v>57.65</v>
+      </c>
+      <c r="O380" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E381" t="n">
+        <v>144.58</v>
+      </c>
+      <c r="F381" t="n">
+        <v>149.15</v>
+      </c>
+      <c r="G381" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="H381" t="n">
+        <v>139.5899963378906</v>
+      </c>
+      <c r="I381" t="n">
+        <v>-3.450000047683716</v>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K381" t="n">
+        <v>0.894</v>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N381" t="n">
+        <v>72.63</v>
+      </c>
+      <c r="O381" t="inlineStr">
+        <is>
+          <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-27)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O381"/>
+  <dimension ref="A1:O401"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24744,6 +24744,1266 @@
       <c r="O381" t="inlineStr">
         <is>
           <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E382" t="n">
+        <v>1386.1</v>
+      </c>
+      <c r="F382" t="n">
+        <v>1587.81</v>
+      </c>
+      <c r="G382" t="n">
+        <v>14.55</v>
+      </c>
+      <c r="H382" t="n">
+        <v>1270.380004882812</v>
+      </c>
+      <c r="I382" t="n">
+        <v>-8.350000381469727</v>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K382" t="n">
+        <v>0.921</v>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N382" t="n">
+        <v>90.25</v>
+      </c>
+      <c r="O382" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E383" t="n">
+        <v>3162.5</v>
+      </c>
+      <c r="F383" t="n">
+        <v>3109.65</v>
+      </c>
+      <c r="G383" t="n">
+        <v>-1.67</v>
+      </c>
+      <c r="H383" t="n">
+        <v>3158.93994140625</v>
+      </c>
+      <c r="I383" t="n">
+        <v>-0.1099999994039536</v>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K383" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N383" t="n">
+        <v>54.29</v>
+      </c>
+      <c r="O383" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E384" t="n">
+        <v>1670.8</v>
+      </c>
+      <c r="F384" t="n">
+        <v>1616.57</v>
+      </c>
+      <c r="G384" t="n">
+        <v>-3.25</v>
+      </c>
+      <c r="H384" t="n">
+        <v>1709.449951171875</v>
+      </c>
+      <c r="I384" t="n">
+        <v>2.309999942779541</v>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K384" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N384" t="n">
+        <v>60.69</v>
+      </c>
+      <c r="O384" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E385" t="n">
+        <v>916.1</v>
+      </c>
+      <c r="F385" t="n">
+        <v>913.09</v>
+      </c>
+      <c r="G385" t="n">
+        <v>-0.33</v>
+      </c>
+      <c r="H385" t="n">
+        <v>964.3099975585938</v>
+      </c>
+      <c r="I385" t="n">
+        <v>5.260000228881836</v>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K385" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N385" t="n">
+        <v>60.65</v>
+      </c>
+      <c r="O385" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E386" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="F386" t="n">
+        <v>1363.91</v>
+      </c>
+      <c r="G386" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="H386" t="n">
+        <v>1325.43994140625</v>
+      </c>
+      <c r="I386" t="n">
+        <v>-1.340000033378601</v>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K386" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M386" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N386" t="n">
+        <v>62.51</v>
+      </c>
+      <c r="O386" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E387" t="n">
+        <v>1029.5</v>
+      </c>
+      <c r="F387" t="n">
+        <v>1050.77</v>
+      </c>
+      <c r="G387" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="H387" t="n">
+        <v>1065.530029296875</v>
+      </c>
+      <c r="I387" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K387" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N387" t="n">
+        <v>66.09999999999999</v>
+      </c>
+      <c r="O387" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E388" t="n">
+        <v>2409.5</v>
+      </c>
+      <c r="F388" t="n">
+        <v>2312.9</v>
+      </c>
+      <c r="G388" t="n">
+        <v>-4.01</v>
+      </c>
+      <c r="H388" t="n">
+        <v>2279.56005859375</v>
+      </c>
+      <c r="I388" t="n">
+        <v>-5.389999866485596</v>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K388" t="n">
+        <v>0.836</v>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N388" t="n">
+        <v>60.71</v>
+      </c>
+      <c r="O388" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E389" t="n">
+        <v>323.4</v>
+      </c>
+      <c r="F389" t="n">
+        <v>333.45</v>
+      </c>
+      <c r="G389" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="H389" t="n">
+        <v>395.3200073242188</v>
+      </c>
+      <c r="I389" t="n">
+        <v>22.23999977111816</v>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K389" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N389" t="n">
+        <v>67.66</v>
+      </c>
+      <c r="O389" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E390" t="n">
+        <v>3743.8</v>
+      </c>
+      <c r="F390" t="n">
+        <v>3844.12</v>
+      </c>
+      <c r="G390" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="H390" t="n">
+        <v>3300.820068359375</v>
+      </c>
+      <c r="I390" t="n">
+        <v>-11.82999992370605</v>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K390" t="n">
+        <v>0</v>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N390" t="n">
+        <v>54.02</v>
+      </c>
+      <c r="O390" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E391" t="n">
+        <v>927.85</v>
+      </c>
+      <c r="F391" t="n">
+        <v>1009.06</v>
+      </c>
+      <c r="G391" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="H391" t="n">
+        <v>1315.449951171875</v>
+      </c>
+      <c r="I391" t="n">
+        <v>41.77000045776367</v>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K391" t="n">
+        <v>0.836</v>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N391" t="n">
+        <v>79.84999999999999</v>
+      </c>
+      <c r="O391" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E392" t="n">
+        <v>1984.7</v>
+      </c>
+      <c r="F392" t="n">
+        <v>2119.02</v>
+      </c>
+      <c r="G392" t="n">
+        <v>6.77</v>
+      </c>
+      <c r="H392" t="n">
+        <v>2106.860107421875</v>
+      </c>
+      <c r="I392" t="n">
+        <v>6.159999847412109</v>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K392" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N392" t="n">
+        <v>71.87</v>
+      </c>
+      <c r="O392" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E393" t="n">
+        <v>2703.7</v>
+      </c>
+      <c r="F393" t="n">
+        <v>2741.12</v>
+      </c>
+      <c r="G393" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="H393" t="n">
+        <v>3010.02001953125</v>
+      </c>
+      <c r="I393" t="n">
+        <v>11.32999992370605</v>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K393" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N393" t="n">
+        <v>66.08</v>
+      </c>
+      <c r="O393" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E394" t="n">
+        <v>1258</v>
+      </c>
+      <c r="F394" t="n">
+        <v>1253.31</v>
+      </c>
+      <c r="G394" t="n">
+        <v>-0.37</v>
+      </c>
+      <c r="H394" t="n">
+        <v>1209.2900390625</v>
+      </c>
+      <c r="I394" t="n">
+        <v>-3.869999885559082</v>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K394" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N394" t="n">
+        <v>60.88</v>
+      </c>
+      <c r="O394" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E395" t="n">
+        <v>15469</v>
+      </c>
+      <c r="F395" t="n">
+        <v>18058.41</v>
+      </c>
+      <c r="G395" t="n">
+        <v>16.74</v>
+      </c>
+      <c r="H395" t="n">
+        <v>12282.5302734375</v>
+      </c>
+      <c r="I395" t="n">
+        <v>-20.60000038146973</v>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K395" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N395" t="n">
+        <v>85.65000000000001</v>
+      </c>
+      <c r="O395" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E396" t="n">
+        <v>1631.9</v>
+      </c>
+      <c r="F396" t="n">
+        <v>1741</v>
+      </c>
+      <c r="G396" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="H396" t="n">
+        <v>1622.140014648438</v>
+      </c>
+      <c r="I396" t="n">
+        <v>-0.6000000238418579</v>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K396" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N396" t="n">
+        <v>69.20999999999999</v>
+      </c>
+      <c r="O396" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E397" t="n">
+        <v>238.4</v>
+      </c>
+      <c r="F397" t="n">
+        <v>267.13</v>
+      </c>
+      <c r="G397" t="n">
+        <v>12.05</v>
+      </c>
+      <c r="H397" t="n">
+        <v>219.5899963378906</v>
+      </c>
+      <c r="I397" t="n">
+        <v>-7.889999866485596</v>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K397" t="n">
+        <v>0.421</v>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N397" t="n">
+        <v>76.5</v>
+      </c>
+      <c r="O397" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E398" t="n">
+        <v>12369</v>
+      </c>
+      <c r="F398" t="n">
+        <v>11664.45</v>
+      </c>
+      <c r="G398" t="n">
+        <v>-5.7</v>
+      </c>
+      <c r="H398" t="n">
+        <v>12244.330078125</v>
+      </c>
+      <c r="I398" t="n">
+        <v>-1.009999990463257</v>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K398" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M398" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N398" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="O398" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E399" t="n">
+        <v>336.7</v>
+      </c>
+      <c r="F399" t="n">
+        <v>335.28</v>
+      </c>
+      <c r="G399" t="n">
+        <v>-0.42</v>
+      </c>
+      <c r="H399" t="n">
+        <v>327.4500122070312</v>
+      </c>
+      <c r="I399" t="n">
+        <v>-2.75</v>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K399" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N399" t="n">
+        <v>62.37</v>
+      </c>
+      <c r="O399" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E400" t="n">
+        <v>254.15</v>
+      </c>
+      <c r="F400" t="n">
+        <v>252.87</v>
+      </c>
+      <c r="G400" t="n">
+        <v>-0.51</v>
+      </c>
+      <c r="H400" t="n">
+        <v>242.3200073242188</v>
+      </c>
+      <c r="I400" t="n">
+        <v>-4.650000095367432</v>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K400" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N400" t="n">
+        <v>60.68</v>
+      </c>
+      <c r="O400" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E401" t="n">
+        <v>4021.8</v>
+      </c>
+      <c r="F401" t="n">
+        <v>4090.23</v>
+      </c>
+      <c r="G401" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H401" t="n">
+        <v>3659.669921875</v>
+      </c>
+      <c r="I401" t="n">
+        <v>-9</v>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K401" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N401" t="n">
+        <v>65.55</v>
+      </c>
+      <c r="O401" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
         </is>
       </c>
     </row>
@@ -24758,7 +26018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O191"/>
+  <dimension ref="A1:O201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36945,6 +38205,636 @@
       <c r="O191" t="inlineStr">
         <is>
           <t>26 Jan 2026, 06:57:29 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E192" t="n">
+        <v>1385.95</v>
+      </c>
+      <c r="F192" t="n">
+        <v>1567.94</v>
+      </c>
+      <c r="G192" t="n">
+        <v>13.13</v>
+      </c>
+      <c r="H192" t="n">
+        <v>1498.869995117188</v>
+      </c>
+      <c r="I192" t="n">
+        <v>8.149999618530273</v>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K192" t="n">
+        <v>0.921</v>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N192" t="n">
+        <v>88.12</v>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E193" t="n">
+        <v>3160.85</v>
+      </c>
+      <c r="F193" t="n">
+        <v>3144.77</v>
+      </c>
+      <c r="G193" t="n">
+        <v>-0.51</v>
+      </c>
+      <c r="H193" t="n">
+        <v>3257.47998046875</v>
+      </c>
+      <c r="I193" t="n">
+        <v>3.059999942779541</v>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K193" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N193" t="n">
+        <v>56.04</v>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>1670.6</v>
+      </c>
+      <c r="F194" t="n">
+        <v>1636.09</v>
+      </c>
+      <c r="G194" t="n">
+        <v>-2.07</v>
+      </c>
+      <c r="H194" t="n">
+        <v>1595.109985351562</v>
+      </c>
+      <c r="I194" t="n">
+        <v>-4.519999980926514</v>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K194" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N194" t="n">
+        <v>62.46</v>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E195" t="n">
+        <v>916.25</v>
+      </c>
+      <c r="F195" t="n">
+        <v>915.23</v>
+      </c>
+      <c r="G195" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="H195" t="n">
+        <v>987.1099853515625</v>
+      </c>
+      <c r="I195" t="n">
+        <v>7.730000019073486</v>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K195" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N195" t="n">
+        <v>60.97</v>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>1343.35</v>
+      </c>
+      <c r="F196" t="n">
+        <v>1366.02</v>
+      </c>
+      <c r="G196" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="H196" t="n">
+        <v>1295.650024414062</v>
+      </c>
+      <c r="I196" t="n">
+        <v>-3.549999952316284</v>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K196" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N196" t="n">
+        <v>62.75</v>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E197" t="n">
+        <v>1029.4</v>
+      </c>
+      <c r="F197" t="n">
+        <v>1060.07</v>
+      </c>
+      <c r="G197" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="H197" t="n">
+        <v>1157.56005859375</v>
+      </c>
+      <c r="I197" t="n">
+        <v>12.44999980926514</v>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K197" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N197" t="n">
+        <v>67.47</v>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>323.45</v>
+      </c>
+      <c r="F198" t="n">
+        <v>339.05</v>
+      </c>
+      <c r="G198" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="H198" t="n">
+        <v>351.4100036621094</v>
+      </c>
+      <c r="I198" t="n">
+        <v>8.649999618530273</v>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K198" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N198" t="n">
+        <v>70.23</v>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E199" t="n">
+        <v>3745.05</v>
+      </c>
+      <c r="F199" t="n">
+        <v>3865.47</v>
+      </c>
+      <c r="G199" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="H199" t="n">
+        <v>3500.18994140625</v>
+      </c>
+      <c r="I199" t="n">
+        <v>-6.539999961853027</v>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K199" t="n">
+        <v>0</v>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N199" t="n">
+        <v>54.82</v>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>1260.1</v>
+      </c>
+      <c r="F200" t="n">
+        <v>1255.15</v>
+      </c>
+      <c r="G200" t="n">
+        <v>-0.39</v>
+      </c>
+      <c r="H200" t="n">
+        <v>1186.170043945312</v>
+      </c>
+      <c r="I200" t="n">
+        <v>-5.869999885559082</v>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K200" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N200" t="n">
+        <v>60.85</v>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E201" t="n">
+        <v>15469.6</v>
+      </c>
+      <c r="F201" t="n">
+        <v>18112.86</v>
+      </c>
+      <c r="G201" t="n">
+        <v>17.09</v>
+      </c>
+      <c r="H201" t="n">
+        <v>15793.1796875</v>
+      </c>
+      <c r="I201" t="n">
+        <v>2.089999914169312</v>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K201" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N201" t="n">
+        <v>87.34999999999999</v>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
         </is>
       </c>
     </row>
@@ -36959,7 +38849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O381"/>
+  <dimension ref="A1:O401"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61259,6 +63149,1266 @@
         </is>
       </c>
     </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E382" t="n">
+        <v>255.41</v>
+      </c>
+      <c r="F382" t="n">
+        <v>265.66</v>
+      </c>
+      <c r="G382" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="H382" t="n">
+        <v>275.7000122070312</v>
+      </c>
+      <c r="I382" t="n">
+        <v>7.940000057220459</v>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K382" t="n">
+        <v>0.361</v>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N382" t="n">
+        <v>63.24</v>
+      </c>
+      <c r="O382" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E383" t="n">
+        <v>470.28</v>
+      </c>
+      <c r="F383" t="n">
+        <v>447.41</v>
+      </c>
+      <c r="G383" t="n">
+        <v>-4.86</v>
+      </c>
+      <c r="H383" t="n">
+        <v>548.1199951171875</v>
+      </c>
+      <c r="I383" t="n">
+        <v>16.54999923706055</v>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K383" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N383" t="n">
+        <v>57.87</v>
+      </c>
+      <c r="O383" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E384" t="n">
+        <v>333.26</v>
+      </c>
+      <c r="F384" t="n">
+        <v>348.78</v>
+      </c>
+      <c r="G384" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="H384" t="n">
+        <v>351.0400085449219</v>
+      </c>
+      <c r="I384" t="n">
+        <v>5.340000152587891</v>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K384" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N384" t="n">
+        <v>43.99</v>
+      </c>
+      <c r="O384" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E385" t="n">
+        <v>238.42</v>
+      </c>
+      <c r="F385" t="n">
+        <v>245.6</v>
+      </c>
+      <c r="G385" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="H385" t="n">
+        <v>196.8800048828125</v>
+      </c>
+      <c r="I385" t="n">
+        <v>-17.42000007629395</v>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K385" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N385" t="n">
+        <v>41.51</v>
+      </c>
+      <c r="O385" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E386" t="n">
+        <v>672.36</v>
+      </c>
+      <c r="F386" t="n">
+        <v>694.59</v>
+      </c>
+      <c r="G386" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="H386" t="n">
+        <v>753.6300048828125</v>
+      </c>
+      <c r="I386" t="n">
+        <v>12.09000015258789</v>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K386" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M386" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N386" t="n">
+        <v>68.36</v>
+      </c>
+      <c r="O386" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E387" t="n">
+        <v>435.2</v>
+      </c>
+      <c r="F387" t="n">
+        <v>427.64</v>
+      </c>
+      <c r="G387" t="n">
+        <v>-1.74</v>
+      </c>
+      <c r="H387" t="n">
+        <v>535.9199829101562</v>
+      </c>
+      <c r="I387" t="n">
+        <v>23.13999938964844</v>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K387" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N387" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="O387" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E388" t="n">
+        <v>186.47</v>
+      </c>
+      <c r="F388" t="n">
+        <v>200.12</v>
+      </c>
+      <c r="G388" t="n">
+        <v>7.32</v>
+      </c>
+      <c r="H388" t="n">
+        <v>162.9900054931641</v>
+      </c>
+      <c r="I388" t="n">
+        <v>-12.59000015258789</v>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K388" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N388" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="O388" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E389" t="n">
+        <v>301.04</v>
+      </c>
+      <c r="F389" t="n">
+        <v>330.41</v>
+      </c>
+      <c r="G389" t="n">
+        <v>9.76</v>
+      </c>
+      <c r="H389" t="n">
+        <v>353.3800048828125</v>
+      </c>
+      <c r="I389" t="n">
+        <v>17.38999938964844</v>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K389" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N389" t="n">
+        <v>51.63</v>
+      </c>
+      <c r="O389" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E390" t="n">
+        <v>328.49</v>
+      </c>
+      <c r="F390" t="n">
+        <v>344.75</v>
+      </c>
+      <c r="G390" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="H390" t="n">
+        <v>310.9599914550781</v>
+      </c>
+      <c r="I390" t="n">
+        <v>-5.340000152587891</v>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K390" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N390" t="n">
+        <v>70.42</v>
+      </c>
+      <c r="O390" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E391" t="n">
+        <v>221.49</v>
+      </c>
+      <c r="F391" t="n">
+        <v>227.91</v>
+      </c>
+      <c r="G391" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="H391" t="n">
+        <v>212.4600067138672</v>
+      </c>
+      <c r="I391" t="n">
+        <v>-4.079999923706055</v>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K391" t="n">
+        <v>0</v>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N391" t="n">
+        <v>54.35</v>
+      </c>
+      <c r="O391" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E392" t="n">
+        <v>117.64</v>
+      </c>
+      <c r="F392" t="n">
+        <v>119.32</v>
+      </c>
+      <c r="G392" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="H392" t="n">
+        <v>118.4800033569336</v>
+      </c>
+      <c r="I392" t="n">
+        <v>0.7099999785423279</v>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K392" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N392" t="n">
+        <v>65.34</v>
+      </c>
+      <c r="O392" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E393" t="n">
+        <v>149.49</v>
+      </c>
+      <c r="F393" t="n">
+        <v>143.91</v>
+      </c>
+      <c r="G393" t="n">
+        <v>-3.73</v>
+      </c>
+      <c r="H393" t="n">
+        <v>149.1600036621094</v>
+      </c>
+      <c r="I393" t="n">
+        <v>-0.2199999988079071</v>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K393" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N393" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="O393" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E394" t="n">
+        <v>527.36</v>
+      </c>
+      <c r="F394" t="n">
+        <v>561.65</v>
+      </c>
+      <c r="G394" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H394" t="n">
+        <v>554.7999877929688</v>
+      </c>
+      <c r="I394" t="n">
+        <v>5.199999809265137</v>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K394" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N394" t="n">
+        <v>69.97</v>
+      </c>
+      <c r="O394" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E395" t="n">
+        <v>351.64</v>
+      </c>
+      <c r="F395" t="n">
+        <v>303.72</v>
+      </c>
+      <c r="G395" t="n">
+        <v>-13.63</v>
+      </c>
+      <c r="H395" t="n">
+        <v>377.2999877929688</v>
+      </c>
+      <c r="I395" t="n">
+        <v>7.300000190734863</v>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K395" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N395" t="n">
+        <v>42.76</v>
+      </c>
+      <c r="O395" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E396" t="n">
+        <v>386.53</v>
+      </c>
+      <c r="F396" t="n">
+        <v>344.43</v>
+      </c>
+      <c r="G396" t="n">
+        <v>-10.89</v>
+      </c>
+      <c r="H396" t="n">
+        <v>359.5899963378906</v>
+      </c>
+      <c r="I396" t="n">
+        <v>-6.96999979019165</v>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K396" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N396" t="n">
+        <v>46.86</v>
+      </c>
+      <c r="O396" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E397" t="n">
+        <v>52.02</v>
+      </c>
+      <c r="F397" t="n">
+        <v>54.91</v>
+      </c>
+      <c r="G397" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="H397" t="n">
+        <v>56.0099983215332</v>
+      </c>
+      <c r="I397" t="n">
+        <v>7.679999828338623</v>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K397" t="n">
+        <v>-0.527</v>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N397" t="n">
+        <v>47.78</v>
+      </c>
+      <c r="O397" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E398" t="n">
+        <v>134.84</v>
+      </c>
+      <c r="F398" t="n">
+        <v>131.64</v>
+      </c>
+      <c r="G398" t="n">
+        <v>-2.37</v>
+      </c>
+      <c r="H398" t="n">
+        <v>165.0500030517578</v>
+      </c>
+      <c r="I398" t="n">
+        <v>22.39999961853027</v>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K398" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M398" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N398" t="n">
+        <v>33.44</v>
+      </c>
+      <c r="O398" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E399" t="n">
+        <v>324.85</v>
+      </c>
+      <c r="F399" t="n">
+        <v>391.2</v>
+      </c>
+      <c r="G399" t="n">
+        <v>20.42</v>
+      </c>
+      <c r="H399" t="n">
+        <v>345.5700073242188</v>
+      </c>
+      <c r="I399" t="n">
+        <v>6.380000114440918</v>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K399" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N399" t="n">
+        <v>93.40000000000001</v>
+      </c>
+      <c r="O399" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E400" t="n">
+        <v>977.67</v>
+      </c>
+      <c r="F400" t="n">
+        <v>947.24</v>
+      </c>
+      <c r="G400" t="n">
+        <v>-3.11</v>
+      </c>
+      <c r="H400" t="n">
+        <v>947.1699829101562</v>
+      </c>
+      <c r="I400" t="n">
+        <v>-3.119999885559082</v>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K400" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N400" t="n">
+        <v>58.73</v>
+      </c>
+      <c r="O400" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E401" t="n">
+        <v>145.87</v>
+      </c>
+      <c r="F401" t="n">
+        <v>149.34</v>
+      </c>
+      <c r="G401" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="H401" t="n">
+        <v>142.1600036621094</v>
+      </c>
+      <c r="I401" t="n">
+        <v>-2.549999952316284</v>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K401" t="n">
+        <v>0.894</v>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N401" t="n">
+        <v>71.45</v>
+      </c>
+      <c r="O401" t="inlineStr">
+        <is>
+          <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-28)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O401"/>
+  <dimension ref="A1:O421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26004,6 +26004,1266 @@
       <c r="O401" t="inlineStr">
         <is>
           <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E402" t="n">
+        <v>1380.5</v>
+      </c>
+      <c r="F402" t="n">
+        <v>1564.58</v>
+      </c>
+      <c r="G402" t="n">
+        <v>13.33</v>
+      </c>
+      <c r="H402" t="n">
+        <v>1318.969970703125</v>
+      </c>
+      <c r="I402" t="n">
+        <v>-4.460000038146973</v>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K402" t="n">
+        <v>0.921</v>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N402" t="n">
+        <v>88.42</v>
+      </c>
+      <c r="O402" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E403" t="n">
+        <v>3158</v>
+      </c>
+      <c r="F403" t="n">
+        <v>3052.69</v>
+      </c>
+      <c r="G403" t="n">
+        <v>-3.33</v>
+      </c>
+      <c r="H403" t="n">
+        <v>3264.5400390625</v>
+      </c>
+      <c r="I403" t="n">
+        <v>3.369999885559082</v>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K403" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N403" t="n">
+        <v>55.22</v>
+      </c>
+      <c r="O403" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E404" t="n">
+        <v>1682.7</v>
+      </c>
+      <c r="F404" t="n">
+        <v>1578.71</v>
+      </c>
+      <c r="G404" t="n">
+        <v>-6.18</v>
+      </c>
+      <c r="H404" t="n">
+        <v>1597.27001953125</v>
+      </c>
+      <c r="I404" t="n">
+        <v>-5.079999923706055</v>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K404" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N404" t="n">
+        <v>53.73</v>
+      </c>
+      <c r="O404" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E405" t="n">
+        <v>926.4</v>
+      </c>
+      <c r="F405" t="n">
+        <v>913.11</v>
+      </c>
+      <c r="G405" t="n">
+        <v>-1.43</v>
+      </c>
+      <c r="H405" t="n">
+        <v>806.02001953125</v>
+      </c>
+      <c r="I405" t="n">
+        <v>-12.98999977111816</v>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K405" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N405" t="n">
+        <v>59.57</v>
+      </c>
+      <c r="O405" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E406" t="n">
+        <v>1361.4</v>
+      </c>
+      <c r="F406" t="n">
+        <v>1361.48</v>
+      </c>
+      <c r="G406" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H406" t="n">
+        <v>1300.550048828125</v>
+      </c>
+      <c r="I406" t="n">
+        <v>-4.46999979019165</v>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K406" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N406" t="n">
+        <v>61.73</v>
+      </c>
+      <c r="O406" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E407" t="n">
+        <v>1053.15</v>
+      </c>
+      <c r="F407" t="n">
+        <v>1057.99</v>
+      </c>
+      <c r="G407" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="H407" t="n">
+        <v>1129.670043945312</v>
+      </c>
+      <c r="I407" t="n">
+        <v>7.269999980926514</v>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K407" t="n">
+        <v>-0.382</v>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M407" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N407" t="n">
+        <v>43.05</v>
+      </c>
+      <c r="O407" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E408" t="n">
+        <v>2400.9</v>
+      </c>
+      <c r="F408" t="n">
+        <v>2280.02</v>
+      </c>
+      <c r="G408" t="n">
+        <v>-5.03</v>
+      </c>
+      <c r="H408" t="n">
+        <v>2352.300048828125</v>
+      </c>
+      <c r="I408" t="n">
+        <v>-2.019999980926514</v>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K408" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M408" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N408" t="n">
+        <v>53.59</v>
+      </c>
+      <c r="O408" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E409" t="n">
+        <v>318.65</v>
+      </c>
+      <c r="F409" t="n">
+        <v>319.09</v>
+      </c>
+      <c r="G409" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H409" t="n">
+        <v>370.760009765625</v>
+      </c>
+      <c r="I409" t="n">
+        <v>16.35000038146973</v>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K409" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N409" t="n">
+        <v>63.21</v>
+      </c>
+      <c r="O409" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E410" t="n">
+        <v>3787.8</v>
+      </c>
+      <c r="F410" t="n">
+        <v>3841.3</v>
+      </c>
+      <c r="G410" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="H410" t="n">
+        <v>3868.27001953125</v>
+      </c>
+      <c r="I410" t="n">
+        <v>2.119999885559082</v>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K410" t="n">
+        <v>0.493</v>
+      </c>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N410" t="n">
+        <v>61.98</v>
+      </c>
+      <c r="O410" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E411" t="n">
+        <v>914.7</v>
+      </c>
+      <c r="F411" t="n">
+        <v>991.17</v>
+      </c>
+      <c r="G411" t="n">
+        <v>8.359999999999999</v>
+      </c>
+      <c r="H411" t="n">
+        <v>840.3400268554688</v>
+      </c>
+      <c r="I411" t="n">
+        <v>-8.130000114440918</v>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K411" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L411" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M411" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N411" t="n">
+        <v>74.26000000000001</v>
+      </c>
+      <c r="O411" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E412" t="n">
+        <v>1973.4</v>
+      </c>
+      <c r="F412" t="n">
+        <v>2102.61</v>
+      </c>
+      <c r="G412" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="H412" t="n">
+        <v>2188.81005859375</v>
+      </c>
+      <c r="I412" t="n">
+        <v>10.92000007629395</v>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K412" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M412" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N412" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="O412" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E413" t="n">
+        <v>2622.8</v>
+      </c>
+      <c r="F413" t="n">
+        <v>2644.65</v>
+      </c>
+      <c r="G413" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="H413" t="n">
+        <v>2578.02001953125</v>
+      </c>
+      <c r="I413" t="n">
+        <v>-1.710000038146973</v>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K413" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="L413" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N413" t="n">
+        <v>63.49</v>
+      </c>
+      <c r="O413" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E414" t="n">
+        <v>1315.8</v>
+      </c>
+      <c r="F414" t="n">
+        <v>1256.15</v>
+      </c>
+      <c r="G414" t="n">
+        <v>-4.53</v>
+      </c>
+      <c r="H414" t="n">
+        <v>1139.7900390625</v>
+      </c>
+      <c r="I414" t="n">
+        <v>-13.38000011444092</v>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K414" t="n">
+        <v>0.8070000000000001</v>
+      </c>
+      <c r="L414" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M414" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N414" t="n">
+        <v>59.34</v>
+      </c>
+      <c r="O414" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E415" t="n">
+        <v>15245</v>
+      </c>
+      <c r="F415" t="n">
+        <v>17809.87</v>
+      </c>
+      <c r="G415" t="n">
+        <v>16.82</v>
+      </c>
+      <c r="H415" t="n">
+        <v>15451.3701171875</v>
+      </c>
+      <c r="I415" t="n">
+        <v>1.350000023841858</v>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K415" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="L415" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M415" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N415" t="n">
+        <v>87.48</v>
+      </c>
+      <c r="O415" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E416" t="n">
+        <v>1638.9</v>
+      </c>
+      <c r="F416" t="n">
+        <v>1716.58</v>
+      </c>
+      <c r="G416" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="H416" t="n">
+        <v>1686.369995117188</v>
+      </c>
+      <c r="I416" t="n">
+        <v>2.900000095367432</v>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K416" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="L416" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M416" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N416" t="n">
+        <v>69.09</v>
+      </c>
+      <c r="O416" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E417" t="n">
+        <v>234.8</v>
+      </c>
+      <c r="F417" t="n">
+        <v>252.17</v>
+      </c>
+      <c r="G417" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="H417" t="n">
+        <v>263.8099975585938</v>
+      </c>
+      <c r="I417" t="n">
+        <v>12.35000038146973</v>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K417" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L417" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M417" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N417" t="n">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="O417" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E418" t="n">
+        <v>12589</v>
+      </c>
+      <c r="F418" t="n">
+        <v>11648.5</v>
+      </c>
+      <c r="G418" t="n">
+        <v>-7.47</v>
+      </c>
+      <c r="H418" t="n">
+        <v>11010.2900390625</v>
+      </c>
+      <c r="I418" t="n">
+        <v>-12.53999996185303</v>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K418" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L418" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M418" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N418" t="n">
+        <v>45.59</v>
+      </c>
+      <c r="O418" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E419" t="n">
+        <v>344.7</v>
+      </c>
+      <c r="F419" t="n">
+        <v>337.82</v>
+      </c>
+      <c r="G419" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H419" t="n">
+        <v>312.25</v>
+      </c>
+      <c r="I419" t="n">
+        <v>-9.420000076293945</v>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K419" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="L419" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M419" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N419" t="n">
+        <v>57.54</v>
+      </c>
+      <c r="O419" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E420" t="n">
+        <v>254.35</v>
+      </c>
+      <c r="F420" t="n">
+        <v>253.54</v>
+      </c>
+      <c r="G420" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="H420" t="n">
+        <v>312.3900146484375</v>
+      </c>
+      <c r="I420" t="n">
+        <v>22.81999969482422</v>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K420" t="n">
+        <v>0.542</v>
+      </c>
+      <c r="L420" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M420" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N420" t="n">
+        <v>60.36</v>
+      </c>
+      <c r="O420" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E421" t="n">
+        <v>3997</v>
+      </c>
+      <c r="F421" t="n">
+        <v>3995.49</v>
+      </c>
+      <c r="G421" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="H421" t="n">
+        <v>4207.56005859375</v>
+      </c>
+      <c r="I421" t="n">
+        <v>5.269999980926514</v>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K421" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L421" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M421" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N421" t="n">
+        <v>62.94</v>
+      </c>
+      <c r="O421" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
         </is>
       </c>
     </row>
@@ -26018,7 +27278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O201"/>
+  <dimension ref="A1:O211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38835,6 +40095,636 @@
       <c r="O201" t="inlineStr">
         <is>
           <t>27 Jan 2026, 06:59:32 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E202" t="n">
+        <v>1381.05</v>
+      </c>
+      <c r="F202" t="n">
+        <v>1533.21</v>
+      </c>
+      <c r="G202" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="H202" t="n">
+        <v>1332.030029296875</v>
+      </c>
+      <c r="I202" t="n">
+        <v>-3.549999952316284</v>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K202" t="n">
+        <v>0.802</v>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N202" t="n">
+        <v>82.56999999999999</v>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E203" t="n">
+        <v>3158.4</v>
+      </c>
+      <c r="F203" t="n">
+        <v>3089.85</v>
+      </c>
+      <c r="G203" t="n">
+        <v>-2.17</v>
+      </c>
+      <c r="H203" t="n">
+        <v>3274.75</v>
+      </c>
+      <c r="I203" t="n">
+        <v>3.680000066757202</v>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K203" t="n">
+        <v>-0.077</v>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N203" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E204" t="n">
+        <v>1683.4</v>
+      </c>
+      <c r="F204" t="n">
+        <v>1604.43</v>
+      </c>
+      <c r="G204" t="n">
+        <v>-4.69</v>
+      </c>
+      <c r="H204" t="n">
+        <v>1722.239990234375</v>
+      </c>
+      <c r="I204" t="n">
+        <v>2.309999942779541</v>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K204" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N204" t="n">
+        <v>58.52</v>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E205" t="n">
+        <v>926.85</v>
+      </c>
+      <c r="F205" t="n">
+        <v>916.3</v>
+      </c>
+      <c r="G205" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="H205" t="n">
+        <v>984.8699951171875</v>
+      </c>
+      <c r="I205" t="n">
+        <v>6.260000228881836</v>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K205" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N205" t="n">
+        <v>60.01</v>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E206" t="n">
+        <v>1363.35</v>
+      </c>
+      <c r="F206" t="n">
+        <v>1358.49</v>
+      </c>
+      <c r="G206" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="H206" t="n">
+        <v>1430.81005859375</v>
+      </c>
+      <c r="I206" t="n">
+        <v>4.949999809265137</v>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K206" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N206" t="n">
+        <v>61.19</v>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E207" t="n">
+        <v>1052.9</v>
+      </c>
+      <c r="F207" t="n">
+        <v>1065.75</v>
+      </c>
+      <c r="G207" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="H207" t="n">
+        <v>1128.670043945312</v>
+      </c>
+      <c r="I207" t="n">
+        <v>7.199999809265137</v>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K207" t="n">
+        <v>-0.382</v>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N207" t="n">
+        <v>44.19</v>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>318.8</v>
+      </c>
+      <c r="F208" t="n">
+        <v>330.44</v>
+      </c>
+      <c r="G208" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="H208" t="n">
+        <v>379.9200134277344</v>
+      </c>
+      <c r="I208" t="n">
+        <v>19.17000007629395</v>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K208" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N208" t="n">
+        <v>68.48</v>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E209" t="n">
+        <v>3790</v>
+      </c>
+      <c r="F209" t="n">
+        <v>3856.28</v>
+      </c>
+      <c r="G209" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H209" t="n">
+        <v>3777.260009765625</v>
+      </c>
+      <c r="I209" t="n">
+        <v>-0.3400000035762787</v>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K209" t="n">
+        <v>0.493</v>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N209" t="n">
+        <v>62.48</v>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>1314.45</v>
+      </c>
+      <c r="F210" t="n">
+        <v>1253.94</v>
+      </c>
+      <c r="G210" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="H210" t="n">
+        <v>1283.839965820312</v>
+      </c>
+      <c r="I210" t="n">
+        <v>-2.329999923706055</v>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K210" t="n">
+        <v>0.8070000000000001</v>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N210" t="n">
+        <v>59.23</v>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>15240.95</v>
+      </c>
+      <c r="F211" t="n">
+        <v>17898</v>
+      </c>
+      <c r="G211" t="n">
+        <v>17.43</v>
+      </c>
+      <c r="H211" t="n">
+        <v>17704.900390625</v>
+      </c>
+      <c r="I211" t="n">
+        <v>16.17000007629395</v>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K211" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N211" t="n">
+        <v>88.39</v>
+      </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
         </is>
       </c>
     </row>
@@ -38849,7 +40739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O401"/>
+  <dimension ref="A1:O421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64409,6 +66299,1266 @@
         </is>
       </c>
     </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E402" t="n">
+        <v>258.27</v>
+      </c>
+      <c r="F402" t="n">
+        <v>267.51</v>
+      </c>
+      <c r="G402" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="H402" t="n">
+        <v>216.1199951171875</v>
+      </c>
+      <c r="I402" t="n">
+        <v>-16.31999969482422</v>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K402" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N402" t="n">
+        <v>65.59</v>
+      </c>
+      <c r="O402" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E403" t="n">
+        <v>480.58</v>
+      </c>
+      <c r="F403" t="n">
+        <v>448.73</v>
+      </c>
+      <c r="G403" t="n">
+        <v>-6.63</v>
+      </c>
+      <c r="H403" t="n">
+        <v>484.7699890136719</v>
+      </c>
+      <c r="I403" t="n">
+        <v>0.8700000047683716</v>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K403" t="n">
+        <v>0</v>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N403" t="n">
+        <v>40.06</v>
+      </c>
+      <c r="O403" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E404" t="n">
+        <v>334.55</v>
+      </c>
+      <c r="F404" t="n">
+        <v>348.96</v>
+      </c>
+      <c r="G404" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="H404" t="n">
+        <v>384.5</v>
+      </c>
+      <c r="I404" t="n">
+        <v>14.93000030517578</v>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K404" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N404" t="n">
+        <v>69.86</v>
+      </c>
+      <c r="O404" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E405" t="n">
+        <v>244.68</v>
+      </c>
+      <c r="F405" t="n">
+        <v>244.19</v>
+      </c>
+      <c r="G405" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="H405" t="n">
+        <v>235.8300018310547</v>
+      </c>
+      <c r="I405" t="n">
+        <v>-3.619999885559082</v>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K405" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N405" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="O405" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E406" t="n">
+        <v>672.97</v>
+      </c>
+      <c r="F406" t="n">
+        <v>688.58</v>
+      </c>
+      <c r="G406" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="H406" t="n">
+        <v>716.3900146484375</v>
+      </c>
+      <c r="I406" t="n">
+        <v>6.449999809265137</v>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K406" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N406" t="n">
+        <v>66.68000000000001</v>
+      </c>
+      <c r="O406" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E407" t="n">
+        <v>430.9</v>
+      </c>
+      <c r="F407" t="n">
+        <v>424.31</v>
+      </c>
+      <c r="G407" t="n">
+        <v>-1.53</v>
+      </c>
+      <c r="H407" t="n">
+        <v>571.219970703125</v>
+      </c>
+      <c r="I407" t="n">
+        <v>32.56000137329102</v>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K407" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M407" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N407" t="n">
+        <v>60.91</v>
+      </c>
+      <c r="O407" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E408" t="n">
+        <v>188.52</v>
+      </c>
+      <c r="F408" t="n">
+        <v>200.52</v>
+      </c>
+      <c r="G408" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="H408" t="n">
+        <v>157.3800048828125</v>
+      </c>
+      <c r="I408" t="n">
+        <v>-16.52000045776367</v>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K408" t="n">
+        <v>0</v>
+      </c>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M408" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N408" t="n">
+        <v>59.55</v>
+      </c>
+      <c r="O408" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E409" t="n">
+        <v>300.31</v>
+      </c>
+      <c r="F409" t="n">
+        <v>328.16</v>
+      </c>
+      <c r="G409" t="n">
+        <v>9.27</v>
+      </c>
+      <c r="H409" t="n">
+        <v>316.2300109863281</v>
+      </c>
+      <c r="I409" t="n">
+        <v>5.300000190734863</v>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K409" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N409" t="n">
+        <v>50.91</v>
+      </c>
+      <c r="O409" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E410" t="n">
+        <v>325.26</v>
+      </c>
+      <c r="F410" t="n">
+        <v>343.26</v>
+      </c>
+      <c r="G410" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="H410" t="n">
+        <v>338.0299987792969</v>
+      </c>
+      <c r="I410" t="n">
+        <v>3.930000066757202</v>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K410" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N410" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="O410" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E411" t="n">
+        <v>224.44</v>
+      </c>
+      <c r="F411" t="n">
+        <v>228.16</v>
+      </c>
+      <c r="G411" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="H411" t="n">
+        <v>299.7999877929688</v>
+      </c>
+      <c r="I411" t="n">
+        <v>33.58000183105469</v>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K411" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L411" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M411" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N411" t="n">
+        <v>59.28</v>
+      </c>
+      <c r="O411" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E412" t="n">
+        <v>116.94</v>
+      </c>
+      <c r="F412" t="n">
+        <v>119.13</v>
+      </c>
+      <c r="G412" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="H412" t="n">
+        <v>96.83999633789062</v>
+      </c>
+      <c r="I412" t="n">
+        <v>-17.19000053405762</v>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K412" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M412" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N412" t="n">
+        <v>64.53</v>
+      </c>
+      <c r="O412" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E413" t="n">
+        <v>148.34</v>
+      </c>
+      <c r="F413" t="n">
+        <v>144.16</v>
+      </c>
+      <c r="G413" t="n">
+        <v>-2.82</v>
+      </c>
+      <c r="H413" t="n">
+        <v>138.8200073242188</v>
+      </c>
+      <c r="I413" t="n">
+        <v>-6.420000076293945</v>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K413" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L413" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N413" t="n">
+        <v>58.77</v>
+      </c>
+      <c r="O413" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E414" t="n">
+        <v>520.41</v>
+      </c>
+      <c r="F414" t="n">
+        <v>556.5700000000001</v>
+      </c>
+      <c r="G414" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="H414" t="n">
+        <v>516.6099853515625</v>
+      </c>
+      <c r="I414" t="n">
+        <v>-0.7300000190734863</v>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K414" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L414" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M414" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N414" t="n">
+        <v>70.64</v>
+      </c>
+      <c r="O414" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E415" t="n">
+        <v>282.7</v>
+      </c>
+      <c r="F415" t="n">
+        <v>296.95</v>
+      </c>
+      <c r="G415" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="H415" t="n">
+        <v>334.0799865722656</v>
+      </c>
+      <c r="I415" t="n">
+        <v>18.18000030517578</v>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K415" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L415" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M415" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N415" t="n">
+        <v>67.44</v>
+      </c>
+      <c r="O415" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E416" t="n">
+        <v>380.36</v>
+      </c>
+      <c r="F416" t="n">
+        <v>344.46</v>
+      </c>
+      <c r="G416" t="n">
+        <v>-9.44</v>
+      </c>
+      <c r="H416" t="n">
+        <v>410.7900085449219</v>
+      </c>
+      <c r="I416" t="n">
+        <v>8</v>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K416" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L416" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M416" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N416" t="n">
+        <v>49.04</v>
+      </c>
+      <c r="O416" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E417" t="n">
+        <v>52.17</v>
+      </c>
+      <c r="F417" t="n">
+        <v>54.38</v>
+      </c>
+      <c r="G417" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="H417" t="n">
+        <v>56.47999954223633</v>
+      </c>
+      <c r="I417" t="n">
+        <v>8.270000457763672</v>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K417" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L417" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M417" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N417" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="O417" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E418" t="n">
+        <v>136.83</v>
+      </c>
+      <c r="F418" t="n">
+        <v>133.66</v>
+      </c>
+      <c r="G418" t="n">
+        <v>-2.32</v>
+      </c>
+      <c r="H418" t="n">
+        <v>279.1799926757812</v>
+      </c>
+      <c r="I418" t="n">
+        <v>104.0400009155273</v>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K418" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L418" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M418" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N418" t="n">
+        <v>33.52</v>
+      </c>
+      <c r="O418" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E419" t="n">
+        <v>332.79</v>
+      </c>
+      <c r="F419" t="n">
+        <v>388.39</v>
+      </c>
+      <c r="G419" t="n">
+        <v>16.71</v>
+      </c>
+      <c r="H419" t="n">
+        <v>307.1600036621094</v>
+      </c>
+      <c r="I419" t="n">
+        <v>-7.699999809265137</v>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K419" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L419" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M419" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N419" t="n">
+        <v>88.26000000000001</v>
+      </c>
+      <c r="O419" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E420" t="n">
+        <v>970.28</v>
+      </c>
+      <c r="F420" t="n">
+        <v>945.6799999999999</v>
+      </c>
+      <c r="G420" t="n">
+        <v>-2.54</v>
+      </c>
+      <c r="H420" t="n">
+        <v>990.97998046875</v>
+      </c>
+      <c r="I420" t="n">
+        <v>2.130000114440918</v>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K420" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L420" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M420" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N420" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="O420" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E421" t="n">
+        <v>148.78</v>
+      </c>
+      <c r="F421" t="n">
+        <v>149.79</v>
+      </c>
+      <c r="G421" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="H421" t="n">
+        <v>148.4299926757812</v>
+      </c>
+      <c r="I421" t="n">
+        <v>-0.239999994635582</v>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K421" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L421" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M421" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N421" t="n">
+        <v>59.82</v>
+      </c>
+      <c r="O421" t="inlineStr">
+        <is>
+          <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-29)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O421"/>
+  <dimension ref="A1:O441"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27264,6 +27264,1266 @@
       <c r="O421" t="inlineStr">
         <is>
           <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E422" t="n">
+        <v>1396.7</v>
+      </c>
+      <c r="F422" t="n">
+        <v>1552.03</v>
+      </c>
+      <c r="G422" t="n">
+        <v>11.12</v>
+      </c>
+      <c r="H422" t="n">
+        <v>1311.869995117188</v>
+      </c>
+      <c r="I422" t="n">
+        <v>-6.070000171661377</v>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K422" t="n">
+        <v>0.921</v>
+      </c>
+      <c r="L422" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M422" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N422" t="n">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="O422" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E423" t="n">
+        <v>3200.1</v>
+      </c>
+      <c r="F423" t="n">
+        <v>3049.85</v>
+      </c>
+      <c r="G423" t="n">
+        <v>-4.7</v>
+      </c>
+      <c r="H423" t="n">
+        <v>3234.39990234375</v>
+      </c>
+      <c r="I423" t="n">
+        <v>1.070000052452087</v>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K423" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="L423" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M423" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N423" t="n">
+        <v>38.44</v>
+      </c>
+      <c r="O423" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E424" t="n">
+        <v>1666.5</v>
+      </c>
+      <c r="F424" t="n">
+        <v>1581.76</v>
+      </c>
+      <c r="G424" t="n">
+        <v>-5.08</v>
+      </c>
+      <c r="H424" t="n">
+        <v>1766.630004882812</v>
+      </c>
+      <c r="I424" t="n">
+        <v>6.010000228881836</v>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K424" t="n">
+        <v>0</v>
+      </c>
+      <c r="L424" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N424" t="n">
+        <v>42.37</v>
+      </c>
+      <c r="O424" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E425" t="n">
+        <v>932.7</v>
+      </c>
+      <c r="F425" t="n">
+        <v>910.59</v>
+      </c>
+      <c r="G425" t="n">
+        <v>-2.37</v>
+      </c>
+      <c r="H425" t="n">
+        <v>861.3800048828125</v>
+      </c>
+      <c r="I425" t="n">
+        <v>-7.650000095367432</v>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K425" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L425" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M425" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N425" t="n">
+        <v>58.16</v>
+      </c>
+      <c r="O425" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E426" t="n">
+        <v>1367.7</v>
+      </c>
+      <c r="F426" t="n">
+        <v>1352.44</v>
+      </c>
+      <c r="G426" t="n">
+        <v>-1.12</v>
+      </c>
+      <c r="H426" t="n">
+        <v>1331.260009765625</v>
+      </c>
+      <c r="I426" t="n">
+        <v>-2.660000085830688</v>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K426" t="n">
+        <v>-0.459</v>
+      </c>
+      <c r="L426" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M426" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N426" t="n">
+        <v>39.15</v>
+      </c>
+      <c r="O426" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E427" t="n">
+        <v>1063.5</v>
+      </c>
+      <c r="F427" t="n">
+        <v>1066.12</v>
+      </c>
+      <c r="G427" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H427" t="n">
+        <v>944.8400268554688</v>
+      </c>
+      <c r="I427" t="n">
+        <v>-11.15999984741211</v>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K427" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M427" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N427" t="n">
+        <v>58.41</v>
+      </c>
+      <c r="O427" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E428" t="n">
+        <v>2378.4</v>
+      </c>
+      <c r="F428" t="n">
+        <v>2290.25</v>
+      </c>
+      <c r="G428" t="n">
+        <v>-3.71</v>
+      </c>
+      <c r="H428" t="n">
+        <v>2454.7099609375</v>
+      </c>
+      <c r="I428" t="n">
+        <v>3.210000038146973</v>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K428" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N428" t="n">
+        <v>53.62</v>
+      </c>
+      <c r="O428" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E429" t="n">
+        <v>321.15</v>
+      </c>
+      <c r="F429" t="n">
+        <v>321.08</v>
+      </c>
+      <c r="G429" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="H429" t="n">
+        <v>356.3599853515625</v>
+      </c>
+      <c r="I429" t="n">
+        <v>10.96000003814697</v>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K429" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L429" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M429" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N429" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="O429" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E430" t="n">
+        <v>3794</v>
+      </c>
+      <c r="F430" t="n">
+        <v>3835.16</v>
+      </c>
+      <c r="G430" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="H430" t="n">
+        <v>4054.010009765625</v>
+      </c>
+      <c r="I430" t="n">
+        <v>6.849999904632568</v>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K430" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L430" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N430" t="n">
+        <v>61.85</v>
+      </c>
+      <c r="O430" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E431" t="n">
+        <v>935.15</v>
+      </c>
+      <c r="F431" t="n">
+        <v>985.84</v>
+      </c>
+      <c r="G431" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="H431" t="n">
+        <v>1024.81005859375</v>
+      </c>
+      <c r="I431" t="n">
+        <v>9.590000152587891</v>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K431" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N431" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="O431" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E432" t="n">
+        <v>1957.7</v>
+      </c>
+      <c r="F432" t="n">
+        <v>2088.41</v>
+      </c>
+      <c r="G432" t="n">
+        <v>6.68</v>
+      </c>
+      <c r="H432" t="n">
+        <v>2046.239990234375</v>
+      </c>
+      <c r="I432" t="n">
+        <v>4.519999980926514</v>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K432" t="n">
+        <v>0</v>
+      </c>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M432" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N432" t="n">
+        <v>60.02</v>
+      </c>
+      <c r="O432" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E433" t="n">
+        <v>2511.8</v>
+      </c>
+      <c r="F433" t="n">
+        <v>2634.13</v>
+      </c>
+      <c r="G433" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="H433" t="n">
+        <v>2794.02001953125</v>
+      </c>
+      <c r="I433" t="n">
+        <v>11.23999977111816</v>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K433" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N433" t="n">
+        <v>66.11</v>
+      </c>
+      <c r="O433" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E434" t="n">
+        <v>1319.8</v>
+      </c>
+      <c r="F434" t="n">
+        <v>1257.51</v>
+      </c>
+      <c r="G434" t="n">
+        <v>-4.72</v>
+      </c>
+      <c r="H434" t="n">
+        <v>1217.109985351562</v>
+      </c>
+      <c r="I434" t="n">
+        <v>-7.78000020980835</v>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K434" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L434" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M434" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N434" t="n">
+        <v>49.72</v>
+      </c>
+      <c r="O434" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E435" t="n">
+        <v>14877</v>
+      </c>
+      <c r="F435" t="n">
+        <v>17707.19</v>
+      </c>
+      <c r="G435" t="n">
+        <v>19.02</v>
+      </c>
+      <c r="H435" t="n">
+        <v>14334.400390625</v>
+      </c>
+      <c r="I435" t="n">
+        <v>-3.650000095367432</v>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K435" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L435" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M435" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N435" t="n">
+        <v>89.98</v>
+      </c>
+      <c r="O435" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E436" t="n">
+        <v>1610.6</v>
+      </c>
+      <c r="F436" t="n">
+        <v>1700.89</v>
+      </c>
+      <c r="G436" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="H436" t="n">
+        <v>1796.81005859375</v>
+      </c>
+      <c r="I436" t="n">
+        <v>11.5600004196167</v>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K436" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L436" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M436" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N436" t="n">
+        <v>67.59</v>
+      </c>
+      <c r="O436" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E437" t="n">
+        <v>237.35</v>
+      </c>
+      <c r="F437" t="n">
+        <v>249.07</v>
+      </c>
+      <c r="G437" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="H437" t="n">
+        <v>247.5899963378906</v>
+      </c>
+      <c r="I437" t="n">
+        <v>4.309999942779541</v>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K437" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L437" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N437" t="n">
+        <v>70.41</v>
+      </c>
+      <c r="O437" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E438" t="n">
+        <v>12767</v>
+      </c>
+      <c r="F438" t="n">
+        <v>11630.01</v>
+      </c>
+      <c r="G438" t="n">
+        <v>-8.91</v>
+      </c>
+      <c r="H438" t="n">
+        <v>11447.6904296875</v>
+      </c>
+      <c r="I438" t="n">
+        <v>-10.32999992370605</v>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K438" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L438" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N438" t="n">
+        <v>43.44</v>
+      </c>
+      <c r="O438" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E439" t="n">
+        <v>348.05</v>
+      </c>
+      <c r="F439" t="n">
+        <v>339.32</v>
+      </c>
+      <c r="G439" t="n">
+        <v>-2.51</v>
+      </c>
+      <c r="H439" t="n">
+        <v>359.3399963378906</v>
+      </c>
+      <c r="I439" t="n">
+        <v>3.240000009536743</v>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K439" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L439" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M439" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N439" t="n">
+        <v>58.74</v>
+      </c>
+      <c r="O439" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E440" t="n">
+        <v>259.8</v>
+      </c>
+      <c r="F440" t="n">
+        <v>253.36</v>
+      </c>
+      <c r="G440" t="n">
+        <v>-2.48</v>
+      </c>
+      <c r="H440" t="n">
+        <v>319.8999938964844</v>
+      </c>
+      <c r="I440" t="n">
+        <v>23.1299991607666</v>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K440" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L440" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M440" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N440" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="O440" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E441" t="n">
+        <v>3975.2</v>
+      </c>
+      <c r="F441" t="n">
+        <v>3999.93</v>
+      </c>
+      <c r="G441" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="H441" t="n">
+        <v>4221.509765625</v>
+      </c>
+      <c r="I441" t="n">
+        <v>6.199999809265137</v>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K441" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L441" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M441" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N441" t="n">
+        <v>37.93</v>
+      </c>
+      <c r="O441" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
         </is>
       </c>
     </row>
@@ -27278,7 +28538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O211"/>
+  <dimension ref="A1:O221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40725,6 +41985,636 @@
       <c r="O211" t="inlineStr">
         <is>
           <t>28 Jan 2026, 07:00:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>1397.05</v>
+      </c>
+      <c r="F212" t="n">
+        <v>1547.54</v>
+      </c>
+      <c r="G212" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="H212" t="n">
+        <v>1457.93994140625</v>
+      </c>
+      <c r="I212" t="n">
+        <v>4.360000133514404</v>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K212" t="n">
+        <v>0.921</v>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N212" t="n">
+        <v>84.58</v>
+      </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E213" t="n">
+        <v>3199.85</v>
+      </c>
+      <c r="F213" t="n">
+        <v>3081.84</v>
+      </c>
+      <c r="G213" t="n">
+        <v>-3.69</v>
+      </c>
+      <c r="H213" t="n">
+        <v>3041.47998046875</v>
+      </c>
+      <c r="I213" t="n">
+        <v>-4.949999809265137</v>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K213" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N213" t="n">
+        <v>56.45</v>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>1666.4</v>
+      </c>
+      <c r="F214" t="n">
+        <v>1594.37</v>
+      </c>
+      <c r="G214" t="n">
+        <v>-4.32</v>
+      </c>
+      <c r="H214" t="n">
+        <v>1755.380004882812</v>
+      </c>
+      <c r="I214" t="n">
+        <v>5.340000152587891</v>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K214" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N214" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E215" t="n">
+        <v>932.65</v>
+      </c>
+      <c r="F215" t="n">
+        <v>915.7</v>
+      </c>
+      <c r="G215" t="n">
+        <v>-1.82</v>
+      </c>
+      <c r="H215" t="n">
+        <v>822.239990234375</v>
+      </c>
+      <c r="I215" t="n">
+        <v>-11.84000015258789</v>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K215" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N215" t="n">
+        <v>58.99</v>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E216" t="n">
+        <v>1367.4</v>
+      </c>
+      <c r="F216" t="n">
+        <v>1358.33</v>
+      </c>
+      <c r="G216" t="n">
+        <v>-0.66</v>
+      </c>
+      <c r="H216" t="n">
+        <v>1331.859985351562</v>
+      </c>
+      <c r="I216" t="n">
+        <v>-2.599999904632568</v>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K216" t="n">
+        <v>-0.459</v>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N216" t="n">
+        <v>39.82</v>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E217" t="n">
+        <v>1062.8</v>
+      </c>
+      <c r="F217" t="n">
+        <v>1080.15</v>
+      </c>
+      <c r="G217" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="H217" t="n">
+        <v>1203.420043945312</v>
+      </c>
+      <c r="I217" t="n">
+        <v>13.22999954223633</v>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K217" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N217" t="n">
+        <v>60.49</v>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E218" t="n">
+        <v>321.25</v>
+      </c>
+      <c r="F218" t="n">
+        <v>330.11</v>
+      </c>
+      <c r="G218" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="H218" t="n">
+        <v>384.5400085449219</v>
+      </c>
+      <c r="I218" t="n">
+        <v>19.70000076293945</v>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K218" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N218" t="n">
+        <v>63.68</v>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E219" t="n">
+        <v>3793.65</v>
+      </c>
+      <c r="F219" t="n">
+        <v>3851.68</v>
+      </c>
+      <c r="G219" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="H219" t="n">
+        <v>3690.6298828125</v>
+      </c>
+      <c r="I219" t="n">
+        <v>-2.720000028610229</v>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K219" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N219" t="n">
+        <v>62.51</v>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E220" t="n">
+        <v>1320.5</v>
+      </c>
+      <c r="F220" t="n">
+        <v>1255.42</v>
+      </c>
+      <c r="G220" t="n">
+        <v>-4.93</v>
+      </c>
+      <c r="H220" t="n">
+        <v>1486.380004882812</v>
+      </c>
+      <c r="I220" t="n">
+        <v>12.5600004196167</v>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K220" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N220" t="n">
+        <v>52.83</v>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E221" t="n">
+        <v>14876.8</v>
+      </c>
+      <c r="F221" t="n">
+        <v>17797.2</v>
+      </c>
+      <c r="G221" t="n">
+        <v>19.63</v>
+      </c>
+      <c r="H221" t="n">
+        <v>16075.490234375</v>
+      </c>
+      <c r="I221" t="n">
+        <v>8.060000419616699</v>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K221" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N221" t="n">
+        <v>90.89</v>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
         </is>
       </c>
     </row>
@@ -40739,7 +42629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O421"/>
+  <dimension ref="A1:O441"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -67559,6 +69449,1266 @@
         </is>
       </c>
     </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E422" t="n">
+        <v>256.44</v>
+      </c>
+      <c r="F422" t="n">
+        <v>264.37</v>
+      </c>
+      <c r="G422" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="H422" t="n">
+        <v>247.3899993896484</v>
+      </c>
+      <c r="I422" t="n">
+        <v>-3.529999971389771</v>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K422" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L422" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M422" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N422" t="n">
+        <v>67.84</v>
+      </c>
+      <c r="O422" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E423" t="n">
+        <v>481.63</v>
+      </c>
+      <c r="F423" t="n">
+        <v>444.99</v>
+      </c>
+      <c r="G423" t="n">
+        <v>-7.61</v>
+      </c>
+      <c r="H423" t="n">
+        <v>469.0700073242188</v>
+      </c>
+      <c r="I423" t="n">
+        <v>-2.609999895095825</v>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K423" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L423" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M423" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N423" t="n">
+        <v>48.47</v>
+      </c>
+      <c r="O423" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E424" t="n">
+        <v>336.01</v>
+      </c>
+      <c r="F424" t="n">
+        <v>347.96</v>
+      </c>
+      <c r="G424" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="H424" t="n">
+        <v>350.8999938964844</v>
+      </c>
+      <c r="I424" t="n">
+        <v>4.429999828338623</v>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K424" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L424" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N424" t="n">
+        <v>68.53</v>
+      </c>
+      <c r="O424" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E425" t="n">
+        <v>243.01</v>
+      </c>
+      <c r="F425" t="n">
+        <v>243.77</v>
+      </c>
+      <c r="G425" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="H425" t="n">
+        <v>264.6199951171875</v>
+      </c>
+      <c r="I425" t="n">
+        <v>8.890000343322754</v>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K425" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L425" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M425" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N425" t="n">
+        <v>63.47</v>
+      </c>
+      <c r="O425" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E426" t="n">
+        <v>668.73</v>
+      </c>
+      <c r="F426" t="n">
+        <v>684.76</v>
+      </c>
+      <c r="G426" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H426" t="n">
+        <v>668.47998046875</v>
+      </c>
+      <c r="I426" t="n">
+        <v>-0.03999999910593033</v>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K426" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="L426" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M426" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N426" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="O426" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E427" t="n">
+        <v>431.46</v>
+      </c>
+      <c r="F427" t="n">
+        <v>425.73</v>
+      </c>
+      <c r="G427" t="n">
+        <v>-1.33</v>
+      </c>
+      <c r="H427" t="n">
+        <v>321.3699951171875</v>
+      </c>
+      <c r="I427" t="n">
+        <v>-25.52000045776367</v>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K427" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M427" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N427" t="n">
+        <v>56.81</v>
+      </c>
+      <c r="O427" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E428" t="n">
+        <v>191.52</v>
+      </c>
+      <c r="F428" t="n">
+        <v>199.64</v>
+      </c>
+      <c r="G428" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="H428" t="n">
+        <v>187.25</v>
+      </c>
+      <c r="I428" t="n">
+        <v>-2.230000019073486</v>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K428" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N428" t="n">
+        <v>69.36</v>
+      </c>
+      <c r="O428" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E429" t="n">
+        <v>300.77</v>
+      </c>
+      <c r="F429" t="n">
+        <v>325.97</v>
+      </c>
+      <c r="G429" t="n">
+        <v>8.380000000000001</v>
+      </c>
+      <c r="H429" t="n">
+        <v>300.9500122070312</v>
+      </c>
+      <c r="I429" t="n">
+        <v>0.05999999865889549</v>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K429" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L429" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M429" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N429" t="n">
+        <v>49.57</v>
+      </c>
+      <c r="O429" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E430" t="n">
+        <v>326.98</v>
+      </c>
+      <c r="F430" t="n">
+        <v>341.32</v>
+      </c>
+      <c r="G430" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="H430" t="n">
+        <v>353.8800048828125</v>
+      </c>
+      <c r="I430" t="n">
+        <v>8.229999542236328</v>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K430" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L430" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N430" t="n">
+        <v>68.02</v>
+      </c>
+      <c r="O430" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E431" t="n">
+        <v>227.72</v>
+      </c>
+      <c r="F431" t="n">
+        <v>230.74</v>
+      </c>
+      <c r="G431" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="H431" t="n">
+        <v>293.2099914550781</v>
+      </c>
+      <c r="I431" t="n">
+        <v>28.76000022888184</v>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K431" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N431" t="n">
+        <v>58.79</v>
+      </c>
+      <c r="O431" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E432" t="n">
+        <v>116.57</v>
+      </c>
+      <c r="F432" t="n">
+        <v>118.81</v>
+      </c>
+      <c r="G432" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="H432" t="n">
+        <v>107.9199981689453</v>
+      </c>
+      <c r="I432" t="n">
+        <v>-7.420000076293945</v>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K432" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M432" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N432" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="O432" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E433" t="n">
+        <v>147.34</v>
+      </c>
+      <c r="F433" t="n">
+        <v>144.76</v>
+      </c>
+      <c r="G433" t="n">
+        <v>-1.75</v>
+      </c>
+      <c r="H433" t="n">
+        <v>148.3300018310547</v>
+      </c>
+      <c r="I433" t="n">
+        <v>0.6700000166893005</v>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K433" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N433" t="n">
+        <v>60.38</v>
+      </c>
+      <c r="O433" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E434" t="n">
+        <v>521.37</v>
+      </c>
+      <c r="F434" t="n">
+        <v>556.29</v>
+      </c>
+      <c r="G434" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="H434" t="n">
+        <v>506.1799926757812</v>
+      </c>
+      <c r="I434" t="n">
+        <v>-2.910000085830688</v>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K434" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="L434" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M434" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N434" t="n">
+        <v>74.91</v>
+      </c>
+      <c r="O434" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E435" t="n">
+        <v>294.02</v>
+      </c>
+      <c r="F435" t="n">
+        <v>293.61</v>
+      </c>
+      <c r="G435" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="H435" t="n">
+        <v>317.8599853515625</v>
+      </c>
+      <c r="I435" t="n">
+        <v>8.109999656677246</v>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K435" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L435" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M435" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N435" t="n">
+        <v>58.59</v>
+      </c>
+      <c r="O435" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E436" t="n">
+        <v>375.3</v>
+      </c>
+      <c r="F436" t="n">
+        <v>343.99</v>
+      </c>
+      <c r="G436" t="n">
+        <v>-8.34</v>
+      </c>
+      <c r="H436" t="n">
+        <v>367.8500061035156</v>
+      </c>
+      <c r="I436" t="n">
+        <v>-1.990000009536743</v>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K436" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L436" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M436" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N436" t="n">
+        <v>47.37</v>
+      </c>
+      <c r="O436" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E437" t="n">
+        <v>51.81</v>
+      </c>
+      <c r="F437" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="G437" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="H437" t="n">
+        <v>50.38000106811523</v>
+      </c>
+      <c r="I437" t="n">
+        <v>-2.75</v>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K437" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L437" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N437" t="n">
+        <v>70.41</v>
+      </c>
+      <c r="O437" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E438" t="n">
+        <v>137.58</v>
+      </c>
+      <c r="F438" t="n">
+        <v>134.47</v>
+      </c>
+      <c r="G438" t="n">
+        <v>-2.26</v>
+      </c>
+      <c r="H438" t="n">
+        <v>258.5599975585938</v>
+      </c>
+      <c r="I438" t="n">
+        <v>87.93000030517578</v>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K438" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L438" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N438" t="n">
+        <v>33.61</v>
+      </c>
+      <c r="O438" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E439" t="n">
+        <v>333.24</v>
+      </c>
+      <c r="F439" t="n">
+        <v>379.2</v>
+      </c>
+      <c r="G439" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="H439" t="n">
+        <v>341.1099853515625</v>
+      </c>
+      <c r="I439" t="n">
+        <v>2.359999895095825</v>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K439" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L439" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M439" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N439" t="n">
+        <v>79.87</v>
+      </c>
+      <c r="O439" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E440" t="n">
+        <v>960.78</v>
+      </c>
+      <c r="F440" t="n">
+        <v>945.09</v>
+      </c>
+      <c r="G440" t="n">
+        <v>-1.63</v>
+      </c>
+      <c r="H440" t="n">
+        <v>810.25</v>
+      </c>
+      <c r="I440" t="n">
+        <v>-15.67000007629395</v>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K440" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L440" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M440" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N440" t="n">
+        <v>34.55</v>
+      </c>
+      <c r="O440" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E441" t="n">
+        <v>148.5</v>
+      </c>
+      <c r="F441" t="n">
+        <v>150.46</v>
+      </c>
+      <c r="G441" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="H441" t="n">
+        <v>149.9499969482422</v>
+      </c>
+      <c r="I441" t="n">
+        <v>0.9800000190734863</v>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K441" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L441" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M441" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N441" t="n">
+        <v>63.42</v>
+      </c>
+      <c r="O441" t="inlineStr">
+        <is>
+          <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-30)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O441"/>
+  <dimension ref="A1:O461"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28524,6 +28524,1266 @@
       <c r="O441" t="inlineStr">
         <is>
           <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E442" t="n">
+        <v>1391</v>
+      </c>
+      <c r="F442" t="n">
+        <v>1587.51</v>
+      </c>
+      <c r="G442" t="n">
+        <v>14.13</v>
+      </c>
+      <c r="H442" t="n">
+        <v>1371.5400390625</v>
+      </c>
+      <c r="I442" t="n">
+        <v>-1.399999976158142</v>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K442" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L442" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M442" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N442" t="n">
+        <v>84.39</v>
+      </c>
+      <c r="O442" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E443" t="n">
+        <v>3144.4</v>
+      </c>
+      <c r="F443" t="n">
+        <v>3043.11</v>
+      </c>
+      <c r="G443" t="n">
+        <v>-3.22</v>
+      </c>
+      <c r="H443" t="n">
+        <v>3131.590087890625</v>
+      </c>
+      <c r="I443" t="n">
+        <v>-0.4099999964237213</v>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K443" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="L443" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M443" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N443" t="n">
+        <v>40.65</v>
+      </c>
+      <c r="O443" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E444" t="n">
+        <v>1659.5</v>
+      </c>
+      <c r="F444" t="n">
+        <v>1534.99</v>
+      </c>
+      <c r="G444" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="H444" t="n">
+        <v>1627.150024414062</v>
+      </c>
+      <c r="I444" t="n">
+        <v>-1.950000047683716</v>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K444" t="n">
+        <v>-0.645</v>
+      </c>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M444" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N444" t="n">
+        <v>25.85</v>
+      </c>
+      <c r="O444" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E445" t="n">
+        <v>935.5</v>
+      </c>
+      <c r="F445" t="n">
+        <v>913.72</v>
+      </c>
+      <c r="G445" t="n">
+        <v>-2.33</v>
+      </c>
+      <c r="H445" t="n">
+        <v>918.0900268554688</v>
+      </c>
+      <c r="I445" t="n">
+        <v>-1.860000014305115</v>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K445" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="L445" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M445" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N445" t="n">
+        <v>60.33</v>
+      </c>
+      <c r="O445" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E446" t="n">
+        <v>1383.6</v>
+      </c>
+      <c r="F446" t="n">
+        <v>1371.97</v>
+      </c>
+      <c r="G446" t="n">
+        <v>-0.84</v>
+      </c>
+      <c r="H446" t="n">
+        <v>1256.449951171875</v>
+      </c>
+      <c r="I446" t="n">
+        <v>-9.189999580383301</v>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K446" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="L446" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M446" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N446" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="O446" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E447" t="n">
+        <v>1066.2</v>
+      </c>
+      <c r="F447" t="n">
+        <v>1088.21</v>
+      </c>
+      <c r="G447" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="H447" t="n">
+        <v>1269.630004882812</v>
+      </c>
+      <c r="I447" t="n">
+        <v>19.07999992370605</v>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K447" t="n">
+        <v>-0.382</v>
+      </c>
+      <c r="L447" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M447" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N447" t="n">
+        <v>45.46</v>
+      </c>
+      <c r="O447" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E448" t="n">
+        <v>2352.6</v>
+      </c>
+      <c r="F448" t="n">
+        <v>2436.5</v>
+      </c>
+      <c r="G448" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="H448" t="n">
+        <v>2408.9599609375</v>
+      </c>
+      <c r="I448" t="n">
+        <v>2.400000095367432</v>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K448" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="L448" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M448" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N448" t="n">
+        <v>69.17</v>
+      </c>
+      <c r="O448" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E449" t="n">
+        <v>318.6</v>
+      </c>
+      <c r="F449" t="n">
+        <v>331.62</v>
+      </c>
+      <c r="G449" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="H449" t="n">
+        <v>371.8299865722656</v>
+      </c>
+      <c r="I449" t="n">
+        <v>16.70999908447266</v>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K449" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L449" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M449" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N449" t="n">
+        <v>64.93000000000001</v>
+      </c>
+      <c r="O449" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E450" t="n">
+        <v>3932.9</v>
+      </c>
+      <c r="F450" t="n">
+        <v>3876.55</v>
+      </c>
+      <c r="G450" t="n">
+        <v>-1.43</v>
+      </c>
+      <c r="H450" t="n">
+        <v>4256.31005859375</v>
+      </c>
+      <c r="I450" t="n">
+        <v>8.220000267028809</v>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K450" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M450" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N450" t="n">
+        <v>56.65</v>
+      </c>
+      <c r="O450" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E451" t="n">
+        <v>935.15</v>
+      </c>
+      <c r="F451" t="n">
+        <v>1008.83</v>
+      </c>
+      <c r="G451" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="H451" t="n">
+        <v>986.0700073242188</v>
+      </c>
+      <c r="I451" t="n">
+        <v>5.440000057220459</v>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K451" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L451" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M451" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N451" t="n">
+        <v>48.82</v>
+      </c>
+      <c r="O451" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E452" t="n">
+        <v>1967.9</v>
+      </c>
+      <c r="F452" t="n">
+        <v>2059.57</v>
+      </c>
+      <c r="G452" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="H452" t="n">
+        <v>1949.640014648438</v>
+      </c>
+      <c r="I452" t="n">
+        <v>-0.9300000071525574</v>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K452" t="n">
+        <v>-0.44</v>
+      </c>
+      <c r="L452" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M452" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N452" t="n">
+        <v>48.19</v>
+      </c>
+      <c r="O452" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E453" t="n">
+        <v>2416</v>
+      </c>
+      <c r="F453" t="n">
+        <v>2782.81</v>
+      </c>
+      <c r="G453" t="n">
+        <v>15.18</v>
+      </c>
+      <c r="H453" t="n">
+        <v>2718.159912109375</v>
+      </c>
+      <c r="I453" t="n">
+        <v>12.51000022888184</v>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K453" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L453" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M453" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N453" t="n">
+        <v>81.56999999999999</v>
+      </c>
+      <c r="O453" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E454" t="n">
+        <v>1363.7</v>
+      </c>
+      <c r="F454" t="n">
+        <v>1275.49</v>
+      </c>
+      <c r="G454" t="n">
+        <v>-6.47</v>
+      </c>
+      <c r="H454" t="n">
+        <v>1414.900024414062</v>
+      </c>
+      <c r="I454" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K454" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L454" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M454" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N454" t="n">
+        <v>48.34</v>
+      </c>
+      <c r="O454" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E455" t="n">
+        <v>14502</v>
+      </c>
+      <c r="F455" t="n">
+        <v>18536.92</v>
+      </c>
+      <c r="G455" t="n">
+        <v>27.82</v>
+      </c>
+      <c r="H455" t="n">
+        <v>13667.8701171875</v>
+      </c>
+      <c r="I455" t="n">
+        <v>-5.75</v>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K455" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L455" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M455" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N455" t="n">
+        <v>93.40000000000001</v>
+      </c>
+      <c r="O455" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E456" t="n">
+        <v>1589.3</v>
+      </c>
+      <c r="F456" t="n">
+        <v>1665.16</v>
+      </c>
+      <c r="G456" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="H456" t="n">
+        <v>1742.22998046875</v>
+      </c>
+      <c r="I456" t="n">
+        <v>9.619999885559082</v>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K456" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L456" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M456" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N456" t="n">
+        <v>70.56</v>
+      </c>
+      <c r="O456" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E457" t="n">
+        <v>239.8</v>
+      </c>
+      <c r="F457" t="n">
+        <v>251.12</v>
+      </c>
+      <c r="G457" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="H457" t="n">
+        <v>226.2599945068359</v>
+      </c>
+      <c r="I457" t="n">
+        <v>-5.650000095367432</v>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K457" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L457" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M457" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N457" t="n">
+        <v>70.08</v>
+      </c>
+      <c r="O457" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E458" t="n">
+        <v>12717</v>
+      </c>
+      <c r="F458" t="n">
+        <v>11557.74</v>
+      </c>
+      <c r="G458" t="n">
+        <v>-9.119999999999999</v>
+      </c>
+      <c r="H458" t="n">
+        <v>13001.66015625</v>
+      </c>
+      <c r="I458" t="n">
+        <v>2.240000009536743</v>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K458" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="L458" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M458" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N458" t="n">
+        <v>40.85</v>
+      </c>
+      <c r="O458" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E459" t="n">
+        <v>358.15</v>
+      </c>
+      <c r="F459" t="n">
+        <v>342.46</v>
+      </c>
+      <c r="G459" t="n">
+        <v>-4.38</v>
+      </c>
+      <c r="H459" t="n">
+        <v>355.3800048828125</v>
+      </c>
+      <c r="I459" t="n">
+        <v>-0.7699999809265137</v>
+      </c>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K459" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L459" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M459" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N459" t="n">
+        <v>56.43</v>
+      </c>
+      <c r="O459" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E460" t="n">
+        <v>260.5</v>
+      </c>
+      <c r="F460" t="n">
+        <v>252.57</v>
+      </c>
+      <c r="G460" t="n">
+        <v>-3.04</v>
+      </c>
+      <c r="H460" t="n">
+        <v>290.6000061035156</v>
+      </c>
+      <c r="I460" t="n">
+        <v>11.55000019073486</v>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K460" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L460" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M460" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N460" t="n">
+        <v>54.24</v>
+      </c>
+      <c r="O460" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E461" t="n">
+        <v>3939.7</v>
+      </c>
+      <c r="F461" t="n">
+        <v>4239.07</v>
+      </c>
+      <c r="G461" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="H461" t="n">
+        <v>3236.780029296875</v>
+      </c>
+      <c r="I461" t="n">
+        <v>-17.84000015258789</v>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K461" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L461" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M461" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N461" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="O461" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
         </is>
       </c>
     </row>
@@ -28538,7 +29798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O221"/>
+  <dimension ref="A1:O231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42615,6 +43875,636 @@
       <c r="O221" t="inlineStr">
         <is>
           <t>29 Jan 2026, 07:10:34 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E222" t="n">
+        <v>1391.9</v>
+      </c>
+      <c r="F222" t="n">
+        <v>1565.46</v>
+      </c>
+      <c r="G222" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="H222" t="n">
+        <v>1305.900024414062</v>
+      </c>
+      <c r="I222" t="n">
+        <v>-6.179999828338623</v>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K222" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N222" t="n">
+        <v>81.90000000000001</v>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E223" t="n">
+        <v>3146.1</v>
+      </c>
+      <c r="F223" t="n">
+        <v>3074.49</v>
+      </c>
+      <c r="G223" t="n">
+        <v>-2.28</v>
+      </c>
+      <c r="H223" t="n">
+        <v>3252.06005859375</v>
+      </c>
+      <c r="I223" t="n">
+        <v>3.369999885559082</v>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K223" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N223" t="n">
+        <v>42.07</v>
+      </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E224" t="n">
+        <v>1657.7</v>
+      </c>
+      <c r="F224" t="n">
+        <v>1561.51</v>
+      </c>
+      <c r="G224" t="n">
+        <v>-5.8</v>
+      </c>
+      <c r="H224" t="n">
+        <v>1742.599975585938</v>
+      </c>
+      <c r="I224" t="n">
+        <v>5.119999885559082</v>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K224" t="n">
+        <v>-0.645</v>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N224" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E225" t="n">
+        <v>935.65</v>
+      </c>
+      <c r="F225" t="n">
+        <v>915.86</v>
+      </c>
+      <c r="G225" t="n">
+        <v>-2.11</v>
+      </c>
+      <c r="H225" t="n">
+        <v>887.1400146484375</v>
+      </c>
+      <c r="I225" t="n">
+        <v>-5.179999828338623</v>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K225" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N225" t="n">
+        <v>60.65</v>
+      </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E226" t="n">
+        <v>1384.1</v>
+      </c>
+      <c r="F226" t="n">
+        <v>1370.34</v>
+      </c>
+      <c r="G226" t="n">
+        <v>-0.99</v>
+      </c>
+      <c r="H226" t="n">
+        <v>1491.599975585938</v>
+      </c>
+      <c r="I226" t="n">
+        <v>7.769999980926514</v>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K226" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N226" t="n">
+        <v>51.07</v>
+      </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E227" t="n">
+        <v>1064.5</v>
+      </c>
+      <c r="F227" t="n">
+        <v>1100.36</v>
+      </c>
+      <c r="G227" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="H227" t="n">
+        <v>1091.349975585938</v>
+      </c>
+      <c r="I227" t="n">
+        <v>2.519999980926514</v>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K227" t="n">
+        <v>-0.382</v>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N227" t="n">
+        <v>47.41</v>
+      </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E228" t="n">
+        <v>318.65</v>
+      </c>
+      <c r="F228" t="n">
+        <v>351.17</v>
+      </c>
+      <c r="G228" t="n">
+        <v>10.21</v>
+      </c>
+      <c r="H228" t="n">
+        <v>377.0899963378906</v>
+      </c>
+      <c r="I228" t="n">
+        <v>18.34000015258789</v>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K228" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N228" t="n">
+        <v>74.11</v>
+      </c>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E229" t="n">
+        <v>3932.45</v>
+      </c>
+      <c r="F229" t="n">
+        <v>3895.51</v>
+      </c>
+      <c r="G229" t="n">
+        <v>-0.9399999999999999</v>
+      </c>
+      <c r="H229" t="n">
+        <v>3416.9599609375</v>
+      </c>
+      <c r="I229" t="n">
+        <v>-13.10999965667725</v>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K229" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N229" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E230" t="n">
+        <v>1364.35</v>
+      </c>
+      <c r="F230" t="n">
+        <v>1257.24</v>
+      </c>
+      <c r="G230" t="n">
+        <v>-7.85</v>
+      </c>
+      <c r="H230" t="n">
+        <v>1287.400024414062</v>
+      </c>
+      <c r="I230" t="n">
+        <v>-5.639999866485596</v>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K230" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N230" t="n">
+        <v>48.44</v>
+      </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E231" t="n">
+        <v>14499.5</v>
+      </c>
+      <c r="F231" t="n">
+        <v>18535.64</v>
+      </c>
+      <c r="G231" t="n">
+        <v>27.84</v>
+      </c>
+      <c r="H231" t="n">
+        <v>15542.2998046875</v>
+      </c>
+      <c r="I231" t="n">
+        <v>7.190000057220459</v>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K231" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N231" t="n">
+        <v>93.40000000000001</v>
+      </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
         </is>
       </c>
     </row>
@@ -42629,7 +44519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O441"/>
+  <dimension ref="A1:O461"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -70709,6 +72599,1266 @@
         </is>
       </c>
     </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E442" t="n">
+        <v>258.28</v>
+      </c>
+      <c r="F442" t="n">
+        <v>263.2</v>
+      </c>
+      <c r="G442" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="H442" t="n">
+        <v>273.3500061035156</v>
+      </c>
+      <c r="I442" t="n">
+        <v>5.829999923706055</v>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K442" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L442" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M442" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N442" t="n">
+        <v>66.06</v>
+      </c>
+      <c r="O442" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E443" t="n">
+        <v>433.5</v>
+      </c>
+      <c r="F443" t="n">
+        <v>444.09</v>
+      </c>
+      <c r="G443" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="H443" t="n">
+        <v>451.489990234375</v>
+      </c>
+      <c r="I443" t="n">
+        <v>4.150000095367432</v>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K443" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L443" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M443" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N443" t="n">
+        <v>40.66</v>
+      </c>
+      <c r="O443" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E444" t="n">
+        <v>338.25</v>
+      </c>
+      <c r="F444" t="n">
+        <v>347.91</v>
+      </c>
+      <c r="G444" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="H444" t="n">
+        <v>291.8900146484375</v>
+      </c>
+      <c r="I444" t="n">
+        <v>-13.69999980926514</v>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K444" t="n">
+        <v>-0.572</v>
+      </c>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M444" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N444" t="n">
+        <v>42.84</v>
+      </c>
+      <c r="O444" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E445" t="n">
+        <v>241.73</v>
+      </c>
+      <c r="F445" t="n">
+        <v>241.46</v>
+      </c>
+      <c r="G445" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="H445" t="n">
+        <v>204.5700073242188</v>
+      </c>
+      <c r="I445" t="n">
+        <v>-15.36999988555908</v>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K445" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L445" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M445" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N445" t="n">
+        <v>62.83</v>
+      </c>
+      <c r="O445" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E446" t="n">
+        <v>738.3099999999999</v>
+      </c>
+      <c r="F446" t="n">
+        <v>685.17</v>
+      </c>
+      <c r="G446" t="n">
+        <v>-7.2</v>
+      </c>
+      <c r="H446" t="n">
+        <v>673.6400146484375</v>
+      </c>
+      <c r="I446" t="n">
+        <v>-8.760000228881836</v>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K446" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="L446" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M446" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N446" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="O446" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E447" t="n">
+        <v>416.56</v>
+      </c>
+      <c r="F447" t="n">
+        <v>418.4</v>
+      </c>
+      <c r="G447" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="H447" t="n">
+        <v>298.0199890136719</v>
+      </c>
+      <c r="I447" t="n">
+        <v>-28.45999908447266</v>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K447" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="L447" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M447" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N447" t="n">
+        <v>65.52</v>
+      </c>
+      <c r="O447" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E448" t="n">
+        <v>192.51</v>
+      </c>
+      <c r="F448" t="n">
+        <v>199.07</v>
+      </c>
+      <c r="G448" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="H448" t="n">
+        <v>221.3600006103516</v>
+      </c>
+      <c r="I448" t="n">
+        <v>14.98999977111816</v>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K448" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L448" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M448" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N448" t="n">
+        <v>68.31</v>
+      </c>
+      <c r="O448" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E449" t="n">
+        <v>306.42</v>
+      </c>
+      <c r="F449" t="n">
+        <v>324.4</v>
+      </c>
+      <c r="G449" t="n">
+        <v>5.87</v>
+      </c>
+      <c r="H449" t="n">
+        <v>290.1600036621094</v>
+      </c>
+      <c r="I449" t="n">
+        <v>-5.309999942779541</v>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K449" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L449" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M449" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N449" t="n">
+        <v>71.3</v>
+      </c>
+      <c r="O449" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E450" t="n">
+        <v>331.8</v>
+      </c>
+      <c r="F450" t="n">
+        <v>339.34</v>
+      </c>
+      <c r="G450" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="H450" t="n">
+        <v>337.2200012207031</v>
+      </c>
+      <c r="I450" t="n">
+        <v>1.629999995231628</v>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K450" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M450" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N450" t="n">
+        <v>66.41</v>
+      </c>
+      <c r="O450" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E451" t="n">
+        <v>227.29</v>
+      </c>
+      <c r="F451" t="n">
+        <v>232.31</v>
+      </c>
+      <c r="G451" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="H451" t="n">
+        <v>239.0200042724609</v>
+      </c>
+      <c r="I451" t="n">
+        <v>5.159999847412109</v>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K451" t="n">
+        <v>0</v>
+      </c>
+      <c r="L451" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M451" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N451" t="n">
+        <v>53.32</v>
+      </c>
+      <c r="O451" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E452" t="n">
+        <v>117.41</v>
+      </c>
+      <c r="F452" t="n">
+        <v>119.24</v>
+      </c>
+      <c r="G452" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="H452" t="n">
+        <v>100.3300018310547</v>
+      </c>
+      <c r="I452" t="n">
+        <v>-14.55000019073486</v>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K452" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L452" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M452" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N452" t="n">
+        <v>58.25</v>
+      </c>
+      <c r="O452" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E453" t="n">
+        <v>149.9</v>
+      </c>
+      <c r="F453" t="n">
+        <v>145.69</v>
+      </c>
+      <c r="G453" t="n">
+        <v>-2.81</v>
+      </c>
+      <c r="H453" t="n">
+        <v>145.3999938964844</v>
+      </c>
+      <c r="I453" t="n">
+        <v>-3</v>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K453" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L453" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M453" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N453" t="n">
+        <v>58.79</v>
+      </c>
+      <c r="O453" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E454" t="n">
+        <v>543.73</v>
+      </c>
+      <c r="F454" t="n">
+        <v>549.8</v>
+      </c>
+      <c r="G454" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="H454" t="n">
+        <v>533.0900268554688</v>
+      </c>
+      <c r="I454" t="n">
+        <v>-1.960000038146973</v>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K454" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L454" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M454" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N454" t="n">
+        <v>61.89</v>
+      </c>
+      <c r="O454" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E455" t="n">
+        <v>292.29</v>
+      </c>
+      <c r="F455" t="n">
+        <v>298.41</v>
+      </c>
+      <c r="G455" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="H455" t="n">
+        <v>285.5799865722656</v>
+      </c>
+      <c r="I455" t="n">
+        <v>-2.299999952316284</v>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K455" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L455" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M455" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N455" t="n">
+        <v>66.34</v>
+      </c>
+      <c r="O455" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E456" t="n">
+        <v>371.81</v>
+      </c>
+      <c r="F456" t="n">
+        <v>343.03</v>
+      </c>
+      <c r="G456" t="n">
+        <v>-7.74</v>
+      </c>
+      <c r="H456" t="n">
+        <v>367.5899963378906</v>
+      </c>
+      <c r="I456" t="n">
+        <v>-1.139999985694885</v>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K456" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L456" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M456" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N456" t="n">
+        <v>44.31</v>
+      </c>
+      <c r="O456" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E457" t="n">
+        <v>53.08</v>
+      </c>
+      <c r="F457" t="n">
+        <v>53.86</v>
+      </c>
+      <c r="G457" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="H457" t="n">
+        <v>50.40999984741211</v>
+      </c>
+      <c r="I457" t="n">
+        <v>-5.019999980926514</v>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K457" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L457" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M457" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N457" t="n">
+        <v>65.40000000000001</v>
+      </c>
+      <c r="O457" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E458" t="n">
+        <v>140.51</v>
+      </c>
+      <c r="F458" t="n">
+        <v>133.9</v>
+      </c>
+      <c r="G458" t="n">
+        <v>-4.71</v>
+      </c>
+      <c r="H458" t="n">
+        <v>313.760009765625</v>
+      </c>
+      <c r="I458" t="n">
+        <v>123.3000030517578</v>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K458" t="n">
+        <v>0.681</v>
+      </c>
+      <c r="L458" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M458" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N458" t="n">
+        <v>56.56</v>
+      </c>
+      <c r="O458" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E459" t="n">
+        <v>330.73</v>
+      </c>
+      <c r="F459" t="n">
+        <v>380.42</v>
+      </c>
+      <c r="G459" t="n">
+        <v>15.02</v>
+      </c>
+      <c r="H459" t="n">
+        <v>260.75</v>
+      </c>
+      <c r="I459" t="n">
+        <v>-21.15999984741211</v>
+      </c>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K459" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L459" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M459" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N459" t="n">
+        <v>82.08</v>
+      </c>
+      <c r="O459" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E460" t="n">
+        <v>952.89</v>
+      </c>
+      <c r="F460" t="n">
+        <v>940.59</v>
+      </c>
+      <c r="G460" t="n">
+        <v>-1.29</v>
+      </c>
+      <c r="H460" t="n">
+        <v>880.0599975585938</v>
+      </c>
+      <c r="I460" t="n">
+        <v>-7.639999866485596</v>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K460" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L460" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M460" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N460" t="n">
+        <v>35.06</v>
+      </c>
+      <c r="O460" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E461" t="n">
+        <v>148.69</v>
+      </c>
+      <c r="F461" t="n">
+        <v>150.81</v>
+      </c>
+      <c r="G461" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="H461" t="n">
+        <v>161.5899963378906</v>
+      </c>
+      <c r="I461" t="n">
+        <v>8.670000076293945</v>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K461" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L461" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M461" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N461" t="n">
+        <v>63.58</v>
+      </c>
+      <c r="O461" t="inlineStr">
+        <is>
+          <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-01-31)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O461"/>
+  <dimension ref="A1:O481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29784,6 +29784,1266 @@
       <c r="O461" t="inlineStr">
         <is>
           <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E462" t="n">
+        <v>1395.4</v>
+      </c>
+      <c r="F462" t="n">
+        <v>1537.09</v>
+      </c>
+      <c r="G462" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="H462" t="n">
+        <v>1416.119995117188</v>
+      </c>
+      <c r="I462" t="n">
+        <v>1.490000009536743</v>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K462" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L462" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M462" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N462" t="n">
+        <v>78.43000000000001</v>
+      </c>
+      <c r="O462" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E463" t="n">
+        <v>3123.9</v>
+      </c>
+      <c r="F463" t="n">
+        <v>3031.66</v>
+      </c>
+      <c r="G463" t="n">
+        <v>-2.95</v>
+      </c>
+      <c r="H463" t="n">
+        <v>3515.090087890625</v>
+      </c>
+      <c r="I463" t="n">
+        <v>12.52000045776367</v>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K463" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="L463" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N463" t="n">
+        <v>41.05</v>
+      </c>
+      <c r="O463" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E464" t="n">
+        <v>1641</v>
+      </c>
+      <c r="F464" t="n">
+        <v>1576.64</v>
+      </c>
+      <c r="G464" t="n">
+        <v>-3.92</v>
+      </c>
+      <c r="H464" t="n">
+        <v>1658.7099609375</v>
+      </c>
+      <c r="I464" t="n">
+        <v>1.080000042915344</v>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K464" t="n">
+        <v>0</v>
+      </c>
+      <c r="L464" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M464" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N464" t="n">
+        <v>44.12</v>
+      </c>
+      <c r="O464" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E465" t="n">
+        <v>929.25</v>
+      </c>
+      <c r="F465" t="n">
+        <v>910.59</v>
+      </c>
+      <c r="G465" t="n">
+        <v>-2.01</v>
+      </c>
+      <c r="H465" t="n">
+        <v>1115.969970703125</v>
+      </c>
+      <c r="I465" t="n">
+        <v>20.09000015258789</v>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K465" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L465" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M465" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N465" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="O465" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E466" t="n">
+        <v>1355</v>
+      </c>
+      <c r="F466" t="n">
+        <v>1357.07</v>
+      </c>
+      <c r="G466" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H466" t="n">
+        <v>1377.880004882812</v>
+      </c>
+      <c r="I466" t="n">
+        <v>1.690000057220459</v>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K466" t="n">
+        <v>0</v>
+      </c>
+      <c r="L466" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M466" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N466" t="n">
+        <v>50.23</v>
+      </c>
+      <c r="O466" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E467" t="n">
+        <v>1077.15</v>
+      </c>
+      <c r="F467" t="n">
+        <v>1078.08</v>
+      </c>
+      <c r="G467" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H467" t="n">
+        <v>1240.780029296875</v>
+      </c>
+      <c r="I467" t="n">
+        <v>15.1899995803833</v>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K467" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L467" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M467" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N467" t="n">
+        <v>57.77</v>
+      </c>
+      <c r="O467" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E468" t="n">
+        <v>2373</v>
+      </c>
+      <c r="F468" t="n">
+        <v>2288.04</v>
+      </c>
+      <c r="G468" t="n">
+        <v>-3.58</v>
+      </c>
+      <c r="H468" t="n">
+        <v>2313.68994140625</v>
+      </c>
+      <c r="I468" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K468" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="L468" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M468" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N468" t="n">
+        <v>59.49</v>
+      </c>
+      <c r="O468" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E469" t="n">
+        <v>322.15</v>
+      </c>
+      <c r="F469" t="n">
+        <v>312.66</v>
+      </c>
+      <c r="G469" t="n">
+        <v>-2.95</v>
+      </c>
+      <c r="H469" t="n">
+        <v>377.1700134277344</v>
+      </c>
+      <c r="I469" t="n">
+        <v>17.07999992370605</v>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K469" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L469" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M469" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N469" t="n">
+        <v>55.12</v>
+      </c>
+      <c r="O469" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E470" t="n">
+        <v>3932.3</v>
+      </c>
+      <c r="F470" t="n">
+        <v>3848.87</v>
+      </c>
+      <c r="G470" t="n">
+        <v>-2.12</v>
+      </c>
+      <c r="H470" t="n">
+        <v>3984.949951171875</v>
+      </c>
+      <c r="I470" t="n">
+        <v>1.340000033378601</v>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K470" t="n">
+        <v>-0.477</v>
+      </c>
+      <c r="L470" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M470" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N470" t="n">
+        <v>37.28</v>
+      </c>
+      <c r="O470" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E471" t="n">
+        <v>929.85</v>
+      </c>
+      <c r="F471" t="n">
+        <v>984.4</v>
+      </c>
+      <c r="G471" t="n">
+        <v>5.87</v>
+      </c>
+      <c r="H471" t="n">
+        <v>806.5499877929688</v>
+      </c>
+      <c r="I471" t="n">
+        <v>-13.26000022888184</v>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K471" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M471" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N471" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="O471" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E472" t="n">
+        <v>1968.7</v>
+      </c>
+      <c r="F472" t="n">
+        <v>2069.53</v>
+      </c>
+      <c r="G472" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="H472" t="n">
+        <v>1831.5400390625</v>
+      </c>
+      <c r="I472" t="n">
+        <v>-6.96999979019165</v>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K472" t="n">
+        <v>0</v>
+      </c>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M472" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N472" t="n">
+        <v>57.68</v>
+      </c>
+      <c r="O472" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E473" t="n">
+        <v>2428.3</v>
+      </c>
+      <c r="F473" t="n">
+        <v>2677.32</v>
+      </c>
+      <c r="G473" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="H473" t="n">
+        <v>2397.02001953125</v>
+      </c>
+      <c r="I473" t="n">
+        <v>-1.289999961853027</v>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K473" t="n">
+        <v>-0.44</v>
+      </c>
+      <c r="L473" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M473" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N473" t="n">
+        <v>56.58</v>
+      </c>
+      <c r="O473" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E474" t="n">
+        <v>1370.4</v>
+      </c>
+      <c r="F474" t="n">
+        <v>1281.76</v>
+      </c>
+      <c r="G474" t="n">
+        <v>-6.47</v>
+      </c>
+      <c r="H474" t="n">
+        <v>1303.02001953125</v>
+      </c>
+      <c r="I474" t="n">
+        <v>-4.920000076293945</v>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K474" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L474" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M474" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N474" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="O474" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E475" t="n">
+        <v>14599</v>
+      </c>
+      <c r="F475" t="n">
+        <v>17485.03</v>
+      </c>
+      <c r="G475" t="n">
+        <v>19.77</v>
+      </c>
+      <c r="H475" t="n">
+        <v>15510.099609375</v>
+      </c>
+      <c r="I475" t="n">
+        <v>6.239999771118164</v>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K475" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L475" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M475" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N475" t="n">
+        <v>93.05</v>
+      </c>
+      <c r="O475" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E476" t="n">
+        <v>1595.3</v>
+      </c>
+      <c r="F476" t="n">
+        <v>1662.86</v>
+      </c>
+      <c r="G476" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="H476" t="n">
+        <v>1844.239990234375</v>
+      </c>
+      <c r="I476" t="n">
+        <v>15.60000038146973</v>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K476" t="n">
+        <v>0.832</v>
+      </c>
+      <c r="L476" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M476" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N476" t="n">
+        <v>72.98999999999999</v>
+      </c>
+      <c r="O476" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E477" t="n">
+        <v>236.9</v>
+      </c>
+      <c r="F477" t="n">
+        <v>246.6</v>
+      </c>
+      <c r="G477" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="H477" t="n">
+        <v>215.5099945068359</v>
+      </c>
+      <c r="I477" t="n">
+        <v>-9.029999732971191</v>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K477" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="L477" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M477" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N477" t="n">
+        <v>72.06</v>
+      </c>
+      <c r="O477" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E478" t="n">
+        <v>12694</v>
+      </c>
+      <c r="F478" t="n">
+        <v>11633.03</v>
+      </c>
+      <c r="G478" t="n">
+        <v>-8.359999999999999</v>
+      </c>
+      <c r="H478" t="n">
+        <v>12273.4296875</v>
+      </c>
+      <c r="I478" t="n">
+        <v>-3.309999942779541</v>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K478" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="L478" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M478" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N478" t="n">
+        <v>41.98</v>
+      </c>
+      <c r="O478" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E479" t="n">
+        <v>356</v>
+      </c>
+      <c r="F479" t="n">
+        <v>344.1</v>
+      </c>
+      <c r="G479" t="n">
+        <v>-3.34</v>
+      </c>
+      <c r="H479" t="n">
+        <v>331.3299865722656</v>
+      </c>
+      <c r="I479" t="n">
+        <v>-6.929999828338623</v>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K479" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L479" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M479" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N479" t="n">
+        <v>57.99</v>
+      </c>
+      <c r="O479" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E480" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="F480" t="n">
+        <v>251.78</v>
+      </c>
+      <c r="G480" t="n">
+        <v>-1.84</v>
+      </c>
+      <c r="H480" t="n">
+        <v>253.5299987792969</v>
+      </c>
+      <c r="I480" t="n">
+        <v>-1.159999966621399</v>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K480" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L480" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M480" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N480" t="n">
+        <v>56.04</v>
+      </c>
+      <c r="O480" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E481" t="n">
+        <v>3977.4</v>
+      </c>
+      <c r="F481" t="n">
+        <v>4054.08</v>
+      </c>
+      <c r="G481" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="H481" t="n">
+        <v>3788.89990234375</v>
+      </c>
+      <c r="I481" t="n">
+        <v>-4.739999771118164</v>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K481" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L481" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M481" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N481" t="n">
+        <v>39.89</v>
+      </c>
+      <c r="O481" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
         </is>
       </c>
     </row>
@@ -29798,7 +31058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O231"/>
+  <dimension ref="A1:O241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44505,6 +45765,636 @@
       <c r="O231" t="inlineStr">
         <is>
           <t>30 Jan 2026, 07:07:06 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E232" t="n">
+        <v>1395.9</v>
+      </c>
+      <c r="F232" t="n">
+        <v>1501.22</v>
+      </c>
+      <c r="G232" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="H232" t="n">
+        <v>1348.93994140625</v>
+      </c>
+      <c r="I232" t="n">
+        <v>-3.359999895095825</v>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K232" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N232" t="n">
+        <v>74.52</v>
+      </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E233" t="n">
+        <v>3125.05</v>
+      </c>
+      <c r="F233" t="n">
+        <v>3064.94</v>
+      </c>
+      <c r="G233" t="n">
+        <v>-1.92</v>
+      </c>
+      <c r="H233" t="n">
+        <v>3327.6201171875</v>
+      </c>
+      <c r="I233" t="n">
+        <v>6.480000019073486</v>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K233" t="n">
+        <v>-0.226</v>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N233" t="n">
+        <v>42.59</v>
+      </c>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E234" t="n">
+        <v>1640.45</v>
+      </c>
+      <c r="F234" t="n">
+        <v>1594.75</v>
+      </c>
+      <c r="G234" t="n">
+        <v>-2.79</v>
+      </c>
+      <c r="H234" t="n">
+        <v>1665.079956054688</v>
+      </c>
+      <c r="I234" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K234" t="n">
+        <v>0</v>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N234" t="n">
+        <v>45.82</v>
+      </c>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E235" t="n">
+        <v>929.35</v>
+      </c>
+      <c r="F235" t="n">
+        <v>913.4400000000001</v>
+      </c>
+      <c r="G235" t="n">
+        <v>-1.71</v>
+      </c>
+      <c r="H235" t="n">
+        <v>880.5800170898438</v>
+      </c>
+      <c r="I235" t="n">
+        <v>-5.25</v>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K235" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N235" t="n">
+        <v>60.43</v>
+      </c>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E236" t="n">
+        <v>1355.05</v>
+      </c>
+      <c r="F236" t="n">
+        <v>1361.3</v>
+      </c>
+      <c r="G236" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="H236" t="n">
+        <v>1428.640014648438</v>
+      </c>
+      <c r="I236" t="n">
+        <v>5.429999828338623</v>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K236" t="n">
+        <v>0</v>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N236" t="n">
+        <v>50.69</v>
+      </c>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E237" t="n">
+        <v>1077.55</v>
+      </c>
+      <c r="F237" t="n">
+        <v>1091.54</v>
+      </c>
+      <c r="G237" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H237" t="n">
+        <v>972.8499755859375</v>
+      </c>
+      <c r="I237" t="n">
+        <v>-9.720000267028809</v>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K237" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N237" t="n">
+        <v>59.59</v>
+      </c>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E238" t="n">
+        <v>322.2</v>
+      </c>
+      <c r="F238" t="n">
+        <v>316.27</v>
+      </c>
+      <c r="G238" t="n">
+        <v>-1.84</v>
+      </c>
+      <c r="H238" t="n">
+        <v>359.5799865722656</v>
+      </c>
+      <c r="I238" t="n">
+        <v>11.60000038146973</v>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K238" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N238" t="n">
+        <v>56.78</v>
+      </c>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E239" t="n">
+        <v>3933.45</v>
+      </c>
+      <c r="F239" t="n">
+        <v>3865.17</v>
+      </c>
+      <c r="G239" t="n">
+        <v>-1.74</v>
+      </c>
+      <c r="H239" t="n">
+        <v>3680.860107421875</v>
+      </c>
+      <c r="I239" t="n">
+        <v>-6.420000076293945</v>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K239" t="n">
+        <v>-0.477</v>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N239" t="n">
+        <v>37.86</v>
+      </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E240" t="n">
+        <v>1370.25</v>
+      </c>
+      <c r="F240" t="n">
+        <v>1275.57</v>
+      </c>
+      <c r="G240" t="n">
+        <v>-6.91</v>
+      </c>
+      <c r="H240" t="n">
+        <v>1394.4599609375</v>
+      </c>
+      <c r="I240" t="n">
+        <v>1.769999980926514</v>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K240" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N240" t="n">
+        <v>26.64</v>
+      </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E241" t="n">
+        <v>14601.55</v>
+      </c>
+      <c r="F241" t="n">
+        <v>17523.7</v>
+      </c>
+      <c r="G241" t="n">
+        <v>20.01</v>
+      </c>
+      <c r="H241" t="n">
+        <v>14144.580078125</v>
+      </c>
+      <c r="I241" t="n">
+        <v>-3.130000114440918</v>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K241" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N241" t="n">
+        <v>93.40000000000001</v>
+      </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
         </is>
       </c>
     </row>
@@ -44519,7 +46409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O461"/>
+  <dimension ref="A1:O481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -73859,6 +75749,1266 @@
         </is>
       </c>
     </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E462" t="n">
+        <v>259.48</v>
+      </c>
+      <c r="F462" t="n">
+        <v>261.41</v>
+      </c>
+      <c r="G462" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="H462" t="n">
+        <v>269.9800109863281</v>
+      </c>
+      <c r="I462" t="n">
+        <v>4.050000190734863</v>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K462" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L462" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M462" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N462" t="n">
+        <v>38.11</v>
+      </c>
+      <c r="O462" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E463" t="n">
+        <v>430.29</v>
+      </c>
+      <c r="F463" t="n">
+        <v>438.58</v>
+      </c>
+      <c r="G463" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="H463" t="n">
+        <v>466.4800109863281</v>
+      </c>
+      <c r="I463" t="n">
+        <v>8.409999847412109</v>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K463" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L463" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N463" t="n">
+        <v>39.89</v>
+      </c>
+      <c r="O463" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E464" t="n">
+        <v>338</v>
+      </c>
+      <c r="F464" t="n">
+        <v>348.11</v>
+      </c>
+      <c r="G464" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="H464" t="n">
+        <v>348.4500122070312</v>
+      </c>
+      <c r="I464" t="n">
+        <v>3.089999914169312</v>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K464" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L464" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M464" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N464" t="n">
+        <v>67.69</v>
+      </c>
+      <c r="O464" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E465" t="n">
+        <v>239.3</v>
+      </c>
+      <c r="F465" t="n">
+        <v>242.38</v>
+      </c>
+      <c r="G465" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="H465" t="n">
+        <v>239.6900024414062</v>
+      </c>
+      <c r="I465" t="n">
+        <v>0.1599999964237213</v>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K465" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L465" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M465" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N465" t="n">
+        <v>38.93</v>
+      </c>
+      <c r="O465" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E466" t="n">
+        <v>716.5</v>
+      </c>
+      <c r="F466" t="n">
+        <v>685.03</v>
+      </c>
+      <c r="G466" t="n">
+        <v>-4.39</v>
+      </c>
+      <c r="H466" t="n">
+        <v>740.3099975585938</v>
+      </c>
+      <c r="I466" t="n">
+        <v>3.319999933242798</v>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K466" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L466" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M466" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N466" t="n">
+        <v>58.97</v>
+      </c>
+      <c r="O466" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E467" t="n">
+        <v>430.41</v>
+      </c>
+      <c r="F467" t="n">
+        <v>417.39</v>
+      </c>
+      <c r="G467" t="n">
+        <v>-3.03</v>
+      </c>
+      <c r="H467" t="n">
+        <v>402.2699890136719</v>
+      </c>
+      <c r="I467" t="n">
+        <v>-6.539999961853027</v>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K467" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L467" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M467" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N467" t="n">
+        <v>54.26</v>
+      </c>
+      <c r="O467" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E468" t="n">
+        <v>191.13</v>
+      </c>
+      <c r="F468" t="n">
+        <v>198.54</v>
+      </c>
+      <c r="G468" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="H468" t="n">
+        <v>191.2299957275391</v>
+      </c>
+      <c r="I468" t="n">
+        <v>0.05000000074505806</v>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K468" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L468" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M468" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N468" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="O468" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E469" t="n">
+        <v>305.89</v>
+      </c>
+      <c r="F469" t="n">
+        <v>321.92</v>
+      </c>
+      <c r="G469" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="H469" t="n">
+        <v>294.6499938964844</v>
+      </c>
+      <c r="I469" t="n">
+        <v>-3.670000076293945</v>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K469" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L469" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M469" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N469" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="O469" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E470" t="n">
+        <v>321.83</v>
+      </c>
+      <c r="F470" t="n">
+        <v>337.82</v>
+      </c>
+      <c r="G470" t="n">
+        <v>4.97</v>
+      </c>
+      <c r="H470" t="n">
+        <v>341.4599914550781</v>
+      </c>
+      <c r="I470" t="n">
+        <v>6.099999904632568</v>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K470" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L470" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M470" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N470" t="n">
+        <v>70.45</v>
+      </c>
+      <c r="O470" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E471" t="n">
+        <v>227.25</v>
+      </c>
+      <c r="F471" t="n">
+        <v>233.2</v>
+      </c>
+      <c r="G471" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="H471" t="n">
+        <v>203.5899963378906</v>
+      </c>
+      <c r="I471" t="n">
+        <v>-10.40999984741211</v>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K471" t="n">
+        <v>-0.637</v>
+      </c>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M471" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N471" t="n">
+        <v>41.19</v>
+      </c>
+      <c r="O471" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E472" t="n">
+        <v>119.14</v>
+      </c>
+      <c r="F472" t="n">
+        <v>119.07</v>
+      </c>
+      <c r="G472" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="H472" t="n">
+        <v>113.8300018310547</v>
+      </c>
+      <c r="I472" t="n">
+        <v>-4.449999809265137</v>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K472" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M472" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N472" t="n">
+        <v>55.83</v>
+      </c>
+      <c r="O472" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E473" t="n">
+        <v>151.77</v>
+      </c>
+      <c r="F473" t="n">
+        <v>145.73</v>
+      </c>
+      <c r="G473" t="n">
+        <v>-3.98</v>
+      </c>
+      <c r="H473" t="n">
+        <v>154.3300018310547</v>
+      </c>
+      <c r="I473" t="n">
+        <v>1.690000057220459</v>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K473" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L473" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M473" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N473" t="n">
+        <v>57.03</v>
+      </c>
+      <c r="O473" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E474" t="n">
+        <v>538.79</v>
+      </c>
+      <c r="F474" t="n">
+        <v>546.45</v>
+      </c>
+      <c r="G474" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="H474" t="n">
+        <v>541.969970703125</v>
+      </c>
+      <c r="I474" t="n">
+        <v>0.5899999737739563</v>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K474" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L474" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M474" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N474" t="n">
+        <v>62.35</v>
+      </c>
+      <c r="O474" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E475" t="n">
+        <v>286.93</v>
+      </c>
+      <c r="F475" t="n">
+        <v>295.23</v>
+      </c>
+      <c r="G475" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="H475" t="n">
+        <v>332.8399963378906</v>
+      </c>
+      <c r="I475" t="n">
+        <v>16</v>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K475" t="n">
+        <v>0</v>
+      </c>
+      <c r="L475" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M475" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N475" t="n">
+        <v>54.34</v>
+      </c>
+      <c r="O475" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E476" t="n">
+        <v>374.59</v>
+      </c>
+      <c r="F476" t="n">
+        <v>342.76</v>
+      </c>
+      <c r="G476" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="H476" t="n">
+        <v>355.3299865722656</v>
+      </c>
+      <c r="I476" t="n">
+        <v>-5.139999866485596</v>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K476" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L476" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M476" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N476" t="n">
+        <v>43.17</v>
+      </c>
+      <c r="O476" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E477" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="F477" t="n">
+        <v>53.78</v>
+      </c>
+      <c r="G477" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="H477" t="n">
+        <v>51.47999954223633</v>
+      </c>
+      <c r="I477" t="n">
+        <v>-3.230000019073486</v>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K477" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L477" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M477" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N477" t="n">
+        <v>64.84</v>
+      </c>
+      <c r="O477" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E478" t="n">
+        <v>141.4</v>
+      </c>
+      <c r="F478" t="n">
+        <v>134.55</v>
+      </c>
+      <c r="G478" t="n">
+        <v>-4.84</v>
+      </c>
+      <c r="H478" t="n">
+        <v>308.0400085449219</v>
+      </c>
+      <c r="I478" t="n">
+        <v>117.8499984741211</v>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K478" t="n">
+        <v>-0.703</v>
+      </c>
+      <c r="L478" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M478" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N478" t="n">
+        <v>28.67</v>
+      </c>
+      <c r="O478" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E479" t="n">
+        <v>331.3</v>
+      </c>
+      <c r="F479" t="n">
+        <v>375.23</v>
+      </c>
+      <c r="G479" t="n">
+        <v>13.26</v>
+      </c>
+      <c r="H479" t="n">
+        <v>340.8399963378906</v>
+      </c>
+      <c r="I479" t="n">
+        <v>2.880000114440918</v>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K479" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="L479" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M479" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N479" t="n">
+        <v>84.09</v>
+      </c>
+      <c r="O479" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E480" t="n">
+        <v>940.25</v>
+      </c>
+      <c r="F480" t="n">
+        <v>936.85</v>
+      </c>
+      <c r="G480" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="H480" t="n">
+        <v>956.2899780273438</v>
+      </c>
+      <c r="I480" t="n">
+        <v>1.710000038146973</v>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K480" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L480" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M480" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N480" t="n">
+        <v>36.46</v>
+      </c>
+      <c r="O480" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E481" t="n">
+        <v>153.63</v>
+      </c>
+      <c r="F481" t="n">
+        <v>151.24</v>
+      </c>
+      <c r="G481" t="n">
+        <v>-1.55</v>
+      </c>
+      <c r="H481" t="n">
+        <v>166.9299926757812</v>
+      </c>
+      <c r="I481" t="n">
+        <v>8.659999847412109</v>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K481" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L481" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M481" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N481" t="n">
+        <v>57.55</v>
+      </c>
+      <c r="O481" t="inlineStr">
+        <is>
+          <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-02-01)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O481"/>
+  <dimension ref="A1:O501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31044,6 +31044,1266 @@
       <c r="O481" t="inlineStr">
         <is>
           <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E482" t="n">
+        <v>1395.4</v>
+      </c>
+      <c r="F482" t="n">
+        <v>1541.29</v>
+      </c>
+      <c r="G482" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="H482" t="n">
+        <v>1301.140014648438</v>
+      </c>
+      <c r="I482" t="n">
+        <v>-6.760000228881836</v>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K482" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L482" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M482" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N482" t="n">
+        <v>78.88</v>
+      </c>
+      <c r="O482" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E483" t="n">
+        <v>3123.9</v>
+      </c>
+      <c r="F483" t="n">
+        <v>3025.51</v>
+      </c>
+      <c r="G483" t="n">
+        <v>-3.15</v>
+      </c>
+      <c r="H483" t="n">
+        <v>3008.580078125</v>
+      </c>
+      <c r="I483" t="n">
+        <v>-3.690000057220459</v>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K483" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L483" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M483" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N483" t="n">
+        <v>53.32</v>
+      </c>
+      <c r="O483" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E484" t="n">
+        <v>1641</v>
+      </c>
+      <c r="F484" t="n">
+        <v>1578.38</v>
+      </c>
+      <c r="G484" t="n">
+        <v>-3.82</v>
+      </c>
+      <c r="H484" t="n">
+        <v>1901.72998046875</v>
+      </c>
+      <c r="I484" t="n">
+        <v>15.89000034332275</v>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K484" t="n">
+        <v>-0.71</v>
+      </c>
+      <c r="L484" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M484" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N484" t="n">
+        <v>30.08</v>
+      </c>
+      <c r="O484" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E485" t="n">
+        <v>929.25</v>
+      </c>
+      <c r="F485" t="n">
+        <v>909.98</v>
+      </c>
+      <c r="G485" t="n">
+        <v>-2.07</v>
+      </c>
+      <c r="H485" t="n">
+        <v>923.4500122070312</v>
+      </c>
+      <c r="I485" t="n">
+        <v>-0.6200000047683716</v>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K485" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L485" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M485" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N485" t="n">
+        <v>59.89</v>
+      </c>
+      <c r="O485" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E486" t="n">
+        <v>1355</v>
+      </c>
+      <c r="F486" t="n">
+        <v>1363.01</v>
+      </c>
+      <c r="G486" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="H486" t="n">
+        <v>1421.010009765625</v>
+      </c>
+      <c r="I486" t="n">
+        <v>4.869999885559082</v>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K486" t="n">
+        <v>0</v>
+      </c>
+      <c r="L486" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M486" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N486" t="n">
+        <v>50.89</v>
+      </c>
+      <c r="O486" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E487" t="n">
+        <v>1077.15</v>
+      </c>
+      <c r="F487" t="n">
+        <v>1078.22</v>
+      </c>
+      <c r="G487" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H487" t="n">
+        <v>1253.160034179688</v>
+      </c>
+      <c r="I487" t="n">
+        <v>16.34000015258789</v>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K487" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="L487" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M487" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N487" t="n">
+        <v>62.39</v>
+      </c>
+      <c r="O487" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E488" t="n">
+        <v>2373</v>
+      </c>
+      <c r="F488" t="n">
+        <v>2294.26</v>
+      </c>
+      <c r="G488" t="n">
+        <v>-3.32</v>
+      </c>
+      <c r="H488" t="n">
+        <v>2485.18994140625</v>
+      </c>
+      <c r="I488" t="n">
+        <v>4.730000019073486</v>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K488" t="n">
+        <v>0.751</v>
+      </c>
+      <c r="L488" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M488" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N488" t="n">
+        <v>60.04</v>
+      </c>
+      <c r="O488" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E489" t="n">
+        <v>322.15</v>
+      </c>
+      <c r="F489" t="n">
+        <v>310.34</v>
+      </c>
+      <c r="G489" t="n">
+        <v>-3.67</v>
+      </c>
+      <c r="H489" t="n">
+        <v>372.489990234375</v>
+      </c>
+      <c r="I489" t="n">
+        <v>15.61999988555908</v>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K489" t="n">
+        <v>-0.636</v>
+      </c>
+      <c r="L489" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M489" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N489" t="n">
+        <v>31.78</v>
+      </c>
+      <c r="O489" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E490" t="n">
+        <v>3932.3</v>
+      </c>
+      <c r="F490" t="n">
+        <v>3844.35</v>
+      </c>
+      <c r="G490" t="n">
+        <v>-2.24</v>
+      </c>
+      <c r="H490" t="n">
+        <v>3421.81005859375</v>
+      </c>
+      <c r="I490" t="n">
+        <v>-12.97999954223633</v>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K490" t="n">
+        <v>-0.511</v>
+      </c>
+      <c r="L490" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M490" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N490" t="n">
+        <v>36.42</v>
+      </c>
+      <c r="O490" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E491" t="n">
+        <v>929.85</v>
+      </c>
+      <c r="F491" t="n">
+        <v>987.12</v>
+      </c>
+      <c r="G491" t="n">
+        <v>6.16</v>
+      </c>
+      <c r="H491" t="n">
+        <v>939.3099975585938</v>
+      </c>
+      <c r="I491" t="n">
+        <v>1.019999980926514</v>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K491" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L491" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M491" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N491" t="n">
+        <v>68.04000000000001</v>
+      </c>
+      <c r="O491" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E492" t="n">
+        <v>1968.7</v>
+      </c>
+      <c r="F492" t="n">
+        <v>2070.56</v>
+      </c>
+      <c r="G492" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="H492" t="n">
+        <v>2001.160034179688</v>
+      </c>
+      <c r="I492" t="n">
+        <v>1.649999976158142</v>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K492" t="n">
+        <v>0</v>
+      </c>
+      <c r="L492" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M492" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N492" t="n">
+        <v>57.76</v>
+      </c>
+      <c r="O492" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E493" t="n">
+        <v>2428.3</v>
+      </c>
+      <c r="F493" t="n">
+        <v>2690.52</v>
+      </c>
+      <c r="G493" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H493" t="n">
+        <v>2381.52001953125</v>
+      </c>
+      <c r="I493" t="n">
+        <v>-1.929999947547913</v>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K493" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L493" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M493" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N493" t="n">
+        <v>74.23999999999999</v>
+      </c>
+      <c r="O493" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E494" t="n">
+        <v>1370.4</v>
+      </c>
+      <c r="F494" t="n">
+        <v>1281.76</v>
+      </c>
+      <c r="G494" t="n">
+        <v>-6.47</v>
+      </c>
+      <c r="H494" t="n">
+        <v>1408.140014648438</v>
+      </c>
+      <c r="I494" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K494" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L494" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M494" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N494" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="O494" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E495" t="n">
+        <v>14599</v>
+      </c>
+      <c r="F495" t="n">
+        <v>17498.2</v>
+      </c>
+      <c r="G495" t="n">
+        <v>19.86</v>
+      </c>
+      <c r="H495" t="n">
+        <v>14597.3701171875</v>
+      </c>
+      <c r="I495" t="n">
+        <v>-0.009999999776482582</v>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K495" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L495" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M495" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N495" t="n">
+        <v>93.19</v>
+      </c>
+      <c r="O495" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E496" t="n">
+        <v>1589.3</v>
+      </c>
+      <c r="F496" t="n">
+        <v>1686.9</v>
+      </c>
+      <c r="G496" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="H496" t="n">
+        <v>1728.630004882812</v>
+      </c>
+      <c r="I496" t="n">
+        <v>8.770000457763672</v>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K496" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L496" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M496" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N496" t="n">
+        <v>71.70999999999999</v>
+      </c>
+      <c r="O496" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E497" t="n">
+        <v>236.9</v>
+      </c>
+      <c r="F497" t="n">
+        <v>245.81</v>
+      </c>
+      <c r="G497" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="H497" t="n">
+        <v>240.1799926757812</v>
+      </c>
+      <c r="I497" t="n">
+        <v>1.379999995231628</v>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K497" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L497" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M497" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N497" t="n">
+        <v>68.64</v>
+      </c>
+      <c r="O497" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E498" t="n">
+        <v>12717</v>
+      </c>
+      <c r="F498" t="n">
+        <v>11579.03</v>
+      </c>
+      <c r="G498" t="n">
+        <v>-8.949999999999999</v>
+      </c>
+      <c r="H498" t="n">
+        <v>11771.01953125</v>
+      </c>
+      <c r="I498" t="n">
+        <v>-7.440000057220459</v>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K498" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L498" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M498" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N498" t="n">
+        <v>49.58</v>
+      </c>
+      <c r="O498" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E499" t="n">
+        <v>356</v>
+      </c>
+      <c r="F499" t="n">
+        <v>343.81</v>
+      </c>
+      <c r="G499" t="n">
+        <v>-3.43</v>
+      </c>
+      <c r="H499" t="n">
+        <v>354.4500122070312</v>
+      </c>
+      <c r="I499" t="n">
+        <v>-0.4300000071525574</v>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K499" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L499" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M499" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N499" t="n">
+        <v>57.86</v>
+      </c>
+      <c r="O499" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E500" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="F500" t="n">
+        <v>252.22</v>
+      </c>
+      <c r="G500" t="n">
+        <v>-1.67</v>
+      </c>
+      <c r="H500" t="n">
+        <v>289.0599975585938</v>
+      </c>
+      <c r="I500" t="n">
+        <v>12.6899995803833</v>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K500" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L500" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M500" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N500" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="O500" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E501" t="n">
+        <v>3977.4</v>
+      </c>
+      <c r="F501" t="n">
+        <v>4051.64</v>
+      </c>
+      <c r="G501" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="H501" t="n">
+        <v>3486.39990234375</v>
+      </c>
+      <c r="I501" t="n">
+        <v>-12.34000015258789</v>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K501" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M501" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N501" t="n">
+        <v>63.34</v>
+      </c>
+      <c r="O501" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
         </is>
       </c>
     </row>
@@ -31058,7 +32318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O241"/>
+  <dimension ref="A1:O251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46395,6 +47655,636 @@
       <c r="O241" t="inlineStr">
         <is>
           <t>31 Jan 2026, 06:54:57 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E242" t="n">
+        <v>1395.9</v>
+      </c>
+      <c r="F242" t="n">
+        <v>1507.59</v>
+      </c>
+      <c r="G242" t="n">
+        <v>8</v>
+      </c>
+      <c r="H242" t="n">
+        <v>1317.170043945312</v>
+      </c>
+      <c r="I242" t="n">
+        <v>-5.639999866485596</v>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K242" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N242" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E243" t="n">
+        <v>3125.05</v>
+      </c>
+      <c r="F243" t="n">
+        <v>3055.76</v>
+      </c>
+      <c r="G243" t="n">
+        <v>-2.22</v>
+      </c>
+      <c r="H243" t="n">
+        <v>3183.64990234375</v>
+      </c>
+      <c r="I243" t="n">
+        <v>1.879999995231628</v>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K243" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N243" t="n">
+        <v>54.71</v>
+      </c>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E244" t="n">
+        <v>1640.45</v>
+      </c>
+      <c r="F244" t="n">
+        <v>1595.34</v>
+      </c>
+      <c r="G244" t="n">
+        <v>-2.75</v>
+      </c>
+      <c r="H244" t="n">
+        <v>1782.43994140625</v>
+      </c>
+      <c r="I244" t="n">
+        <v>8.659999847412109</v>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K244" t="n">
+        <v>-0.71</v>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N244" t="n">
+        <v>31.67</v>
+      </c>
+      <c r="O244" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E245" t="n">
+        <v>929.35</v>
+      </c>
+      <c r="F245" t="n">
+        <v>913.4400000000001</v>
+      </c>
+      <c r="G245" t="n">
+        <v>-1.71</v>
+      </c>
+      <c r="H245" t="n">
+        <v>995.760009765625</v>
+      </c>
+      <c r="I245" t="n">
+        <v>7.150000095367432</v>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K245" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N245" t="n">
+        <v>60.43</v>
+      </c>
+      <c r="O245" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E246" t="n">
+        <v>1355.05</v>
+      </c>
+      <c r="F246" t="n">
+        <v>1361.22</v>
+      </c>
+      <c r="G246" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="H246" t="n">
+        <v>1581.0400390625</v>
+      </c>
+      <c r="I246" t="n">
+        <v>16.68000030517578</v>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K246" t="n">
+        <v>0</v>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N246" t="n">
+        <v>50.68</v>
+      </c>
+      <c r="O246" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E247" t="n">
+        <v>1077.55</v>
+      </c>
+      <c r="F247" t="n">
+        <v>1091.88</v>
+      </c>
+      <c r="G247" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="H247" t="n">
+        <v>1306.050048828125</v>
+      </c>
+      <c r="I247" t="n">
+        <v>21.20999908447266</v>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K247" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N247" t="n">
+        <v>64.23</v>
+      </c>
+      <c r="O247" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E248" t="n">
+        <v>322.2</v>
+      </c>
+      <c r="F248" t="n">
+        <v>323.54</v>
+      </c>
+      <c r="G248" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="H248" t="n">
+        <v>365.7799987792969</v>
+      </c>
+      <c r="I248" t="n">
+        <v>13.52999973297119</v>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K248" t="n">
+        <v>-0.636</v>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N248" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E249" t="n">
+        <v>3933.45</v>
+      </c>
+      <c r="F249" t="n">
+        <v>3864.74</v>
+      </c>
+      <c r="G249" t="n">
+        <v>-1.75</v>
+      </c>
+      <c r="H249" t="n">
+        <v>3575.9599609375</v>
+      </c>
+      <c r="I249" t="n">
+        <v>-9.090000152587891</v>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K249" t="n">
+        <v>-0.511</v>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N249" t="n">
+        <v>37.16</v>
+      </c>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E250" t="n">
+        <v>1370.25</v>
+      </c>
+      <c r="F250" t="n">
+        <v>1273.07</v>
+      </c>
+      <c r="G250" t="n">
+        <v>-7.09</v>
+      </c>
+      <c r="H250" t="n">
+        <v>1141.589965820312</v>
+      </c>
+      <c r="I250" t="n">
+        <v>-16.69000053405762</v>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K250" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N250" t="n">
+        <v>26.36</v>
+      </c>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E251" t="n">
+        <v>14601.55</v>
+      </c>
+      <c r="F251" t="n">
+        <v>17523.7</v>
+      </c>
+      <c r="G251" t="n">
+        <v>20.01</v>
+      </c>
+      <c r="H251" t="n">
+        <v>15159.3896484375</v>
+      </c>
+      <c r="I251" t="n">
+        <v>3.819999933242798</v>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K251" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N251" t="n">
+        <v>93.40000000000001</v>
+      </c>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
         </is>
       </c>
     </row>
@@ -46409,7 +48299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O481"/>
+  <dimension ref="A1:O501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77009,6 +78899,1266 @@
         </is>
       </c>
     </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E482" t="n">
+        <v>259.48</v>
+      </c>
+      <c r="F482" t="n">
+        <v>261.57</v>
+      </c>
+      <c r="G482" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="H482" t="n">
+        <v>325.760009765625</v>
+      </c>
+      <c r="I482" t="n">
+        <v>25.54000091552734</v>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K482" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L482" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M482" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N482" t="n">
+        <v>64.41</v>
+      </c>
+      <c r="O482" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E483" t="n">
+        <v>430.29</v>
+      </c>
+      <c r="F483" t="n">
+        <v>438.34</v>
+      </c>
+      <c r="G483" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="H483" t="n">
+        <v>441.1300048828125</v>
+      </c>
+      <c r="I483" t="n">
+        <v>2.519999980926514</v>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K483" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L483" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M483" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N483" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="O483" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E484" t="n">
+        <v>338</v>
+      </c>
+      <c r="F484" t="n">
+        <v>348.1</v>
+      </c>
+      <c r="G484" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="H484" t="n">
+        <v>436.3299865722656</v>
+      </c>
+      <c r="I484" t="n">
+        <v>29.09000015258789</v>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K484" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L484" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M484" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N484" t="n">
+        <v>67.88</v>
+      </c>
+      <c r="O484" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E485" t="n">
+        <v>239.3</v>
+      </c>
+      <c r="F485" t="n">
+        <v>242.38</v>
+      </c>
+      <c r="G485" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="H485" t="n">
+        <v>228.5700073242188</v>
+      </c>
+      <c r="I485" t="n">
+        <v>-4.480000019073486</v>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K485" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L485" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M485" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N485" t="n">
+        <v>38.93</v>
+      </c>
+      <c r="O485" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E486" t="n">
+        <v>716.5</v>
+      </c>
+      <c r="F486" t="n">
+        <v>686.0700000000001</v>
+      </c>
+      <c r="G486" t="n">
+        <v>-4.25</v>
+      </c>
+      <c r="H486" t="n">
+        <v>701.1699829101562</v>
+      </c>
+      <c r="I486" t="n">
+        <v>-2.140000104904175</v>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K486" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L486" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M486" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N486" t="n">
+        <v>56.83</v>
+      </c>
+      <c r="O486" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E487" t="n">
+        <v>430.41</v>
+      </c>
+      <c r="F487" t="n">
+        <v>417.39</v>
+      </c>
+      <c r="G487" t="n">
+        <v>-3.03</v>
+      </c>
+      <c r="H487" t="n">
+        <v>335.8099975585938</v>
+      </c>
+      <c r="I487" t="n">
+        <v>-21.97999954223633</v>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K487" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L487" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M487" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N487" t="n">
+        <v>58.66</v>
+      </c>
+      <c r="O487" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E488" t="n">
+        <v>191.13</v>
+      </c>
+      <c r="F488" t="n">
+        <v>198.35</v>
+      </c>
+      <c r="G488" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="H488" t="n">
+        <v>178.7799987792969</v>
+      </c>
+      <c r="I488" t="n">
+        <v>-6.460000038146973</v>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K488" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L488" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M488" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N488" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="O488" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E489" t="n">
+        <v>305.89</v>
+      </c>
+      <c r="F489" t="n">
+        <v>322.19</v>
+      </c>
+      <c r="G489" t="n">
+        <v>5.33</v>
+      </c>
+      <c r="H489" t="n">
+        <v>310.9400024414062</v>
+      </c>
+      <c r="I489" t="n">
+        <v>1.649999976158142</v>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K489" t="n">
+        <v>-0.361</v>
+      </c>
+      <c r="L489" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M489" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N489" t="n">
+        <v>50.78</v>
+      </c>
+      <c r="O489" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E490" t="n">
+        <v>321.83</v>
+      </c>
+      <c r="F490" t="n">
+        <v>337.99</v>
+      </c>
+      <c r="G490" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="H490" t="n">
+        <v>331.010009765625</v>
+      </c>
+      <c r="I490" t="n">
+        <v>2.849999904632568</v>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K490" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L490" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M490" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N490" t="n">
+        <v>70.53</v>
+      </c>
+      <c r="O490" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E491" t="n">
+        <v>227.25</v>
+      </c>
+      <c r="F491" t="n">
+        <v>233.06</v>
+      </c>
+      <c r="G491" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="H491" t="n">
+        <v>229.9700012207031</v>
+      </c>
+      <c r="I491" t="n">
+        <v>1.200000047683716</v>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K491" t="n">
+        <v>0</v>
+      </c>
+      <c r="L491" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M491" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N491" t="n">
+        <v>53.84</v>
+      </c>
+      <c r="O491" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E492" t="n">
+        <v>119.14</v>
+      </c>
+      <c r="F492" t="n">
+        <v>119</v>
+      </c>
+      <c r="G492" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="H492" t="n">
+        <v>107.8300018310547</v>
+      </c>
+      <c r="I492" t="n">
+        <v>-9.489999771118164</v>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K492" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L492" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M492" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N492" t="n">
+        <v>55.75</v>
+      </c>
+      <c r="O492" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E493" t="n">
+        <v>151.77</v>
+      </c>
+      <c r="F493" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="G493" t="n">
+        <v>-3.97</v>
+      </c>
+      <c r="H493" t="n">
+        <v>152.7799987792969</v>
+      </c>
+      <c r="I493" t="n">
+        <v>0.6700000166893005</v>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K493" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L493" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M493" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N493" t="n">
+        <v>57.04</v>
+      </c>
+      <c r="O493" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E494" t="n">
+        <v>538.79</v>
+      </c>
+      <c r="F494" t="n">
+        <v>547.72</v>
+      </c>
+      <c r="G494" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="H494" t="n">
+        <v>591.6400146484375</v>
+      </c>
+      <c r="I494" t="n">
+        <v>9.810000419616699</v>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K494" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L494" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M494" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N494" t="n">
+        <v>62.71</v>
+      </c>
+      <c r="O494" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E495" t="n">
+        <v>286.93</v>
+      </c>
+      <c r="F495" t="n">
+        <v>296.96</v>
+      </c>
+      <c r="G495" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H495" t="n">
+        <v>326.239990234375</v>
+      </c>
+      <c r="I495" t="n">
+        <v>13.69999980926514</v>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K495" t="n">
+        <v>-0.637</v>
+      </c>
+      <c r="L495" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M495" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N495" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="O495" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E496" t="n">
+        <v>374.59</v>
+      </c>
+      <c r="F496" t="n">
+        <v>342.74</v>
+      </c>
+      <c r="G496" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="H496" t="n">
+        <v>363.0499877929688</v>
+      </c>
+      <c r="I496" t="n">
+        <v>-3.079999923706055</v>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K496" t="n">
+        <v>0.832</v>
+      </c>
+      <c r="L496" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M496" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N496" t="n">
+        <v>53.89</v>
+      </c>
+      <c r="O496" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E497" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="F497" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="G497" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="H497" t="n">
+        <v>53.31999969482422</v>
+      </c>
+      <c r="I497" t="n">
+        <v>0.2199999988079071</v>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K497" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L497" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M497" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N497" t="n">
+        <v>57.32</v>
+      </c>
+      <c r="O497" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E498" t="n">
+        <v>141.4</v>
+      </c>
+      <c r="F498" t="n">
+        <v>134.26</v>
+      </c>
+      <c r="G498" t="n">
+        <v>-5.05</v>
+      </c>
+      <c r="H498" t="n">
+        <v>315.1600036621094</v>
+      </c>
+      <c r="I498" t="n">
+        <v>122.8899993896484</v>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K498" t="n">
+        <v>-0.703</v>
+      </c>
+      <c r="L498" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M498" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N498" t="n">
+        <v>28.36</v>
+      </c>
+      <c r="O498" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E499" t="n">
+        <v>331.3</v>
+      </c>
+      <c r="F499" t="n">
+        <v>368.25</v>
+      </c>
+      <c r="G499" t="n">
+        <v>11.15</v>
+      </c>
+      <c r="H499" t="n">
+        <v>284.0599975585938</v>
+      </c>
+      <c r="I499" t="n">
+        <v>-14.26000022888184</v>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K499" t="n">
+        <v>0.765</v>
+      </c>
+      <c r="L499" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M499" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N499" t="n">
+        <v>82.03</v>
+      </c>
+      <c r="O499" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E500" t="n">
+        <v>940.25</v>
+      </c>
+      <c r="F500" t="n">
+        <v>935.88</v>
+      </c>
+      <c r="G500" t="n">
+        <v>-0.46</v>
+      </c>
+      <c r="H500" t="n">
+        <v>977.8599853515625</v>
+      </c>
+      <c r="I500" t="n">
+        <v>4</v>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K500" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L500" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M500" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N500" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="O500" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E501" t="n">
+        <v>153.63</v>
+      </c>
+      <c r="F501" t="n">
+        <v>151.41</v>
+      </c>
+      <c r="G501" t="n">
+        <v>-1.45</v>
+      </c>
+      <c r="H501" t="n">
+        <v>150.2799987792969</v>
+      </c>
+      <c r="I501" t="n">
+        <v>-2.180000066757202</v>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K501" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M501" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N501" t="n">
+        <v>54.63</v>
+      </c>
+      <c r="O501" t="inlineStr">
+        <is>
+          <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-02-02)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O501"/>
+  <dimension ref="A1:O521"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32304,6 +32304,1266 @@
       <c r="O501" t="inlineStr">
         <is>
           <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E502" t="n">
+        <v>1395.4</v>
+      </c>
+      <c r="F502" t="n">
+        <v>1537.09</v>
+      </c>
+      <c r="G502" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="H502" t="n">
+        <v>1430.7900390625</v>
+      </c>
+      <c r="I502" t="n">
+        <v>2.539999961853027</v>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K502" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M502" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N502" t="n">
+        <v>80.09</v>
+      </c>
+      <c r="O502" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E503" t="n">
+        <v>3123.9</v>
+      </c>
+      <c r="F503" t="n">
+        <v>3033.54</v>
+      </c>
+      <c r="G503" t="n">
+        <v>-2.89</v>
+      </c>
+      <c r="H503" t="n">
+        <v>3210.39990234375</v>
+      </c>
+      <c r="I503" t="n">
+        <v>2.769999980926514</v>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K503" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M503" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N503" t="n">
+        <v>57.64</v>
+      </c>
+      <c r="O503" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E504" t="n">
+        <v>1641</v>
+      </c>
+      <c r="F504" t="n">
+        <v>1582.6</v>
+      </c>
+      <c r="G504" t="n">
+        <v>-3.56</v>
+      </c>
+      <c r="H504" t="n">
+        <v>1537.829956054688</v>
+      </c>
+      <c r="I504" t="n">
+        <v>-6.289999961853027</v>
+      </c>
+      <c r="J504" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K504" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L504" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M504" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N504" t="n">
+        <v>57.66</v>
+      </c>
+      <c r="O504" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E505" t="n">
+        <v>929.25</v>
+      </c>
+      <c r="F505" t="n">
+        <v>908.65</v>
+      </c>
+      <c r="G505" t="n">
+        <v>-2.22</v>
+      </c>
+      <c r="H505" t="n">
+        <v>932.6699829101562</v>
+      </c>
+      <c r="I505" t="n">
+        <v>0.3700000047683716</v>
+      </c>
+      <c r="J505" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K505" t="n">
+        <v>-0.296</v>
+      </c>
+      <c r="L505" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M505" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N505" t="n">
+        <v>40.76</v>
+      </c>
+      <c r="O505" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E506" t="n">
+        <v>1355</v>
+      </c>
+      <c r="F506" t="n">
+        <v>1363.46</v>
+      </c>
+      <c r="G506" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="H506" t="n">
+        <v>1434.260009765625</v>
+      </c>
+      <c r="I506" t="n">
+        <v>5.849999904632568</v>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K506" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L506" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M506" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N506" t="n">
+        <v>62.66</v>
+      </c>
+      <c r="O506" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E507" t="n">
+        <v>1077.15</v>
+      </c>
+      <c r="F507" t="n">
+        <v>1076.02</v>
+      </c>
+      <c r="G507" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="H507" t="n">
+        <v>1361.9599609375</v>
+      </c>
+      <c r="I507" t="n">
+        <v>26.44000053405762</v>
+      </c>
+      <c r="J507" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K507" t="n">
+        <v>0.532</v>
+      </c>
+      <c r="L507" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M507" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N507" t="n">
+        <v>60.48</v>
+      </c>
+      <c r="O507" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E508" t="n">
+        <v>2373</v>
+      </c>
+      <c r="F508" t="n">
+        <v>2271.35</v>
+      </c>
+      <c r="G508" t="n">
+        <v>-4.28</v>
+      </c>
+      <c r="H508" t="n">
+        <v>2243.97998046875</v>
+      </c>
+      <c r="I508" t="n">
+        <v>-5.440000057220459</v>
+      </c>
+      <c r="J508" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K508" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L508" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M508" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N508" t="n">
+        <v>52.37</v>
+      </c>
+      <c r="O508" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E509" t="n">
+        <v>322.15</v>
+      </c>
+      <c r="F509" t="n">
+        <v>311.07</v>
+      </c>
+      <c r="G509" t="n">
+        <v>-3.44</v>
+      </c>
+      <c r="H509" t="n">
+        <v>361.0400085449219</v>
+      </c>
+      <c r="I509" t="n">
+        <v>12.06999969482422</v>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K509" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L509" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M509" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N509" t="n">
+        <v>54.02</v>
+      </c>
+      <c r="O509" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E510" t="n">
+        <v>3932.3</v>
+      </c>
+      <c r="F510" t="n">
+        <v>3843.78</v>
+      </c>
+      <c r="G510" t="n">
+        <v>-2.25</v>
+      </c>
+      <c r="H510" t="n">
+        <v>3930.64990234375</v>
+      </c>
+      <c r="I510" t="n">
+        <v>-0.03999999910593033</v>
+      </c>
+      <c r="J510" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K510" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L510" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M510" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N510" t="n">
+        <v>56.84</v>
+      </c>
+      <c r="O510" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E511" t="n">
+        <v>929.85</v>
+      </c>
+      <c r="F511" t="n">
+        <v>983.6</v>
+      </c>
+      <c r="G511" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="H511" t="n">
+        <v>925.0399780273438</v>
+      </c>
+      <c r="I511" t="n">
+        <v>-0.5199999809265137</v>
+      </c>
+      <c r="J511" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K511" t="n">
+        <v>0.542</v>
+      </c>
+      <c r="L511" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M511" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N511" t="n">
+        <v>69.51000000000001</v>
+      </c>
+      <c r="O511" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E512" t="n">
+        <v>1968.7</v>
+      </c>
+      <c r="F512" t="n">
+        <v>2070.56</v>
+      </c>
+      <c r="G512" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="H512" t="n">
+        <v>2126.830078125</v>
+      </c>
+      <c r="I512" t="n">
+        <v>8.029999732971191</v>
+      </c>
+      <c r="J512" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K512" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L512" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M512" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N512" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="O512" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E513" t="n">
+        <v>2428.3</v>
+      </c>
+      <c r="F513" t="n">
+        <v>2650.01</v>
+      </c>
+      <c r="G513" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="H513" t="n">
+        <v>2384.3701171875</v>
+      </c>
+      <c r="I513" t="n">
+        <v>-1.809999942779541</v>
+      </c>
+      <c r="J513" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K513" t="n">
+        <v>-0.273</v>
+      </c>
+      <c r="L513" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M513" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N513" t="n">
+        <v>58.24</v>
+      </c>
+      <c r="O513" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E514" t="n">
+        <v>1370.4</v>
+      </c>
+      <c r="F514" t="n">
+        <v>1282.05</v>
+      </c>
+      <c r="G514" t="n">
+        <v>-6.45</v>
+      </c>
+      <c r="H514" t="n">
+        <v>1302.180053710938</v>
+      </c>
+      <c r="I514" t="n">
+        <v>-4.980000019073486</v>
+      </c>
+      <c r="J514" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K514" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="L514" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M514" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N514" t="n">
+        <v>52.31</v>
+      </c>
+      <c r="O514" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E515" t="n">
+        <v>14599</v>
+      </c>
+      <c r="F515" t="n">
+        <v>17491.7</v>
+      </c>
+      <c r="G515" t="n">
+        <v>19.81</v>
+      </c>
+      <c r="H515" t="n">
+        <v>15445.1201171875</v>
+      </c>
+      <c r="I515" t="n">
+        <v>5.800000190734863</v>
+      </c>
+      <c r="J515" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K515" t="n">
+        <v>0</v>
+      </c>
+      <c r="L515" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M515" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N515" t="n">
+        <v>79.72</v>
+      </c>
+      <c r="O515" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E516" t="n">
+        <v>1589.3</v>
+      </c>
+      <c r="F516" t="n">
+        <v>1652.34</v>
+      </c>
+      <c r="G516" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="H516" t="n">
+        <v>1485.359985351562</v>
+      </c>
+      <c r="I516" t="n">
+        <v>-6.539999961853027</v>
+      </c>
+      <c r="J516" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K516" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L516" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M516" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N516" t="n">
+        <v>69.34999999999999</v>
+      </c>
+      <c r="O516" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E517" t="n">
+        <v>236.9</v>
+      </c>
+      <c r="F517" t="n">
+        <v>247.53</v>
+      </c>
+      <c r="G517" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="H517" t="n">
+        <v>241.9400024414062</v>
+      </c>
+      <c r="I517" t="n">
+        <v>2.130000114440918</v>
+      </c>
+      <c r="J517" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K517" t="n">
+        <v>0.802</v>
+      </c>
+      <c r="L517" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M517" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N517" t="n">
+        <v>72.77</v>
+      </c>
+      <c r="O517" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E518" t="n">
+        <v>12717</v>
+      </c>
+      <c r="F518" t="n">
+        <v>11579.03</v>
+      </c>
+      <c r="G518" t="n">
+        <v>-8.949999999999999</v>
+      </c>
+      <c r="H518" t="n">
+        <v>11276.83984375</v>
+      </c>
+      <c r="I518" t="n">
+        <v>-11.31999969482422</v>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K518" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L518" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M518" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N518" t="n">
+        <v>44.62</v>
+      </c>
+      <c r="O518" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E519" t="n">
+        <v>356</v>
+      </c>
+      <c r="F519" t="n">
+        <v>344.39</v>
+      </c>
+      <c r="G519" t="n">
+        <v>-3.26</v>
+      </c>
+      <c r="H519" t="n">
+        <v>320.4200134277344</v>
+      </c>
+      <c r="I519" t="n">
+        <v>-9.989999771118164</v>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K519" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L519" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M519" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N519" t="n">
+        <v>58.11</v>
+      </c>
+      <c r="O519" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E520" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="F520" t="n">
+        <v>252.08</v>
+      </c>
+      <c r="G520" t="n">
+        <v>-1.72</v>
+      </c>
+      <c r="H520" t="n">
+        <v>280.7200012207031</v>
+      </c>
+      <c r="I520" t="n">
+        <v>9.439999580383301</v>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K520" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L520" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M520" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N520" t="n">
+        <v>60.42</v>
+      </c>
+      <c r="O520" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E521" t="n">
+        <v>3977.4</v>
+      </c>
+      <c r="F521" t="n">
+        <v>4054.08</v>
+      </c>
+      <c r="G521" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="H521" t="n">
+        <v>3497.1298828125</v>
+      </c>
+      <c r="I521" t="n">
+        <v>-12.06999969482422</v>
+      </c>
+      <c r="J521" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K521" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L521" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M521" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N521" t="n">
+        <v>65.39</v>
+      </c>
+      <c r="O521" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
         </is>
       </c>
     </row>
@@ -32318,7 +33578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O251"/>
+  <dimension ref="A1:O261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48285,6 +49545,636 @@
       <c r="O251" t="inlineStr">
         <is>
           <t>01 Feb 2026, 06:56:39 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E252" t="n">
+        <v>1395.9</v>
+      </c>
+      <c r="F252" t="n">
+        <v>1507.59</v>
+      </c>
+      <c r="G252" t="n">
+        <v>8</v>
+      </c>
+      <c r="H252" t="n">
+        <v>1463.2900390625</v>
+      </c>
+      <c r="I252" t="n">
+        <v>4.829999923706055</v>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K252" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N252" t="n">
+        <v>76.86</v>
+      </c>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E253" t="n">
+        <v>3125.05</v>
+      </c>
+      <c r="F253" t="n">
+        <v>3061.85</v>
+      </c>
+      <c r="G253" t="n">
+        <v>-2.02</v>
+      </c>
+      <c r="H253" t="n">
+        <v>3053.820068359375</v>
+      </c>
+      <c r="I253" t="n">
+        <v>-2.279999971389771</v>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K253" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N253" t="n">
+        <v>58.95</v>
+      </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E254" t="n">
+        <v>1640.45</v>
+      </c>
+      <c r="F254" t="n">
+        <v>1597.4</v>
+      </c>
+      <c r="G254" t="n">
+        <v>-2.62</v>
+      </c>
+      <c r="H254" t="n">
+        <v>1684.589965820312</v>
+      </c>
+      <c r="I254" t="n">
+        <v>2.690000057220459</v>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K254" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N254" t="n">
+        <v>59.06</v>
+      </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E255" t="n">
+        <v>929.35</v>
+      </c>
+      <c r="F255" t="n">
+        <v>915.33</v>
+      </c>
+      <c r="G255" t="n">
+        <v>-1.51</v>
+      </c>
+      <c r="H255" t="n">
+        <v>951.5999755859375</v>
+      </c>
+      <c r="I255" t="n">
+        <v>2.390000104904175</v>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K255" t="n">
+        <v>-0.296</v>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N255" t="n">
+        <v>41.82</v>
+      </c>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E256" t="n">
+        <v>1355.05</v>
+      </c>
+      <c r="F256" t="n">
+        <v>1359.81</v>
+      </c>
+      <c r="G256" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="H256" t="n">
+        <v>1317.469970703125</v>
+      </c>
+      <c r="I256" t="n">
+        <v>-2.769999980926514</v>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K256" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N256" t="n">
+        <v>62.25</v>
+      </c>
+      <c r="O256" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E257" t="n">
+        <v>1077.55</v>
+      </c>
+      <c r="F257" t="n">
+        <v>1090.74</v>
+      </c>
+      <c r="G257" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="H257" t="n">
+        <v>985.25</v>
+      </c>
+      <c r="I257" t="n">
+        <v>-8.569999694824219</v>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K257" t="n">
+        <v>0.532</v>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N257" t="n">
+        <v>62.48</v>
+      </c>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E258" t="n">
+        <v>322.2</v>
+      </c>
+      <c r="F258" t="n">
+        <v>325.91</v>
+      </c>
+      <c r="G258" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="H258" t="n">
+        <v>353.8599853515625</v>
+      </c>
+      <c r="I258" t="n">
+        <v>9.819999694824219</v>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K258" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N258" t="n">
+        <v>60.91</v>
+      </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E259" t="n">
+        <v>3933.45</v>
+      </c>
+      <c r="F259" t="n">
+        <v>3864.74</v>
+      </c>
+      <c r="G259" t="n">
+        <v>-1.75</v>
+      </c>
+      <c r="H259" t="n">
+        <v>3769.429931640625</v>
+      </c>
+      <c r="I259" t="n">
+        <v>-4.170000076293945</v>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K259" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N259" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E260" t="n">
+        <v>1370.25</v>
+      </c>
+      <c r="F260" t="n">
+        <v>1273.07</v>
+      </c>
+      <c r="G260" t="n">
+        <v>-7.09</v>
+      </c>
+      <c r="H260" t="n">
+        <v>1211.97998046875</v>
+      </c>
+      <c r="I260" t="n">
+        <v>-11.55000019073486</v>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K260" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N260" t="n">
+        <v>51.34</v>
+      </c>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E261" t="n">
+        <v>14601.55</v>
+      </c>
+      <c r="F261" t="n">
+        <v>17560.54</v>
+      </c>
+      <c r="G261" t="n">
+        <v>20.26</v>
+      </c>
+      <c r="H261" t="n">
+        <v>14007.2802734375</v>
+      </c>
+      <c r="I261" t="n">
+        <v>-4.070000171661377</v>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K261" t="n">
+        <v>0</v>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N261" t="n">
+        <v>80</v>
+      </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
         </is>
       </c>
     </row>
@@ -48299,7 +50189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O501"/>
+  <dimension ref="A1:O521"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -80159,6 +82049,1266 @@
         </is>
       </c>
     </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E502" t="n">
+        <v>259.48</v>
+      </c>
+      <c r="F502" t="n">
+        <v>262.58</v>
+      </c>
+      <c r="G502" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H502" t="n">
+        <v>245.0399932861328</v>
+      </c>
+      <c r="I502" t="n">
+        <v>-5.570000171661377</v>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K502" t="n">
+        <v>0.421</v>
+      </c>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M502" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N502" t="n">
+        <v>60.21</v>
+      </c>
+      <c r="O502" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E503" t="n">
+        <v>430.29</v>
+      </c>
+      <c r="F503" t="n">
+        <v>438.47</v>
+      </c>
+      <c r="G503" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H503" t="n">
+        <v>452.0400085449219</v>
+      </c>
+      <c r="I503" t="n">
+        <v>5.059999942779541</v>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K503" t="n">
+        <v>0.361</v>
+      </c>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M503" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N503" t="n">
+        <v>60.07</v>
+      </c>
+      <c r="O503" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E504" t="n">
+        <v>338</v>
+      </c>
+      <c r="F504" t="n">
+        <v>348</v>
+      </c>
+      <c r="G504" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="H504" t="n">
+        <v>418.4500122070312</v>
+      </c>
+      <c r="I504" t="n">
+        <v>23.79999923706055</v>
+      </c>
+      <c r="J504" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K504" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L504" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M504" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N504" t="n">
+        <v>67.84</v>
+      </c>
+      <c r="O504" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E505" t="n">
+        <v>239.3</v>
+      </c>
+      <c r="F505" t="n">
+        <v>242.38</v>
+      </c>
+      <c r="G505" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="H505" t="n">
+        <v>194.2400054931641</v>
+      </c>
+      <c r="I505" t="n">
+        <v>-18.82999992370605</v>
+      </c>
+      <c r="J505" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K505" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L505" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M505" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N505" t="n">
+        <v>59.57</v>
+      </c>
+      <c r="O505" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E506" t="n">
+        <v>716.5</v>
+      </c>
+      <c r="F506" t="n">
+        <v>684.99</v>
+      </c>
+      <c r="G506" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="H506" t="n">
+        <v>604.0800170898438</v>
+      </c>
+      <c r="I506" t="n">
+        <v>-15.6899995803833</v>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K506" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L506" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M506" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N506" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="O506" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E507" t="n">
+        <v>430.41</v>
+      </c>
+      <c r="F507" t="n">
+        <v>417.39</v>
+      </c>
+      <c r="G507" t="n">
+        <v>-3.03</v>
+      </c>
+      <c r="H507" t="n">
+        <v>484.8900146484375</v>
+      </c>
+      <c r="I507" t="n">
+        <v>12.65999984741211</v>
+      </c>
+      <c r="J507" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K507" t="n">
+        <v>0</v>
+      </c>
+      <c r="L507" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M507" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N507" t="n">
+        <v>45.46</v>
+      </c>
+      <c r="O507" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E508" t="n">
+        <v>191.13</v>
+      </c>
+      <c r="F508" t="n">
+        <v>198.11</v>
+      </c>
+      <c r="G508" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="H508" t="n">
+        <v>210.0700073242188</v>
+      </c>
+      <c r="I508" t="n">
+        <v>9.909999847412109</v>
+      </c>
+      <c r="J508" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K508" t="n">
+        <v>0.493</v>
+      </c>
+      <c r="L508" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M508" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N508" t="n">
+        <v>65.34</v>
+      </c>
+      <c r="O508" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E509" t="n">
+        <v>305.89</v>
+      </c>
+      <c r="F509" t="n">
+        <v>322.3</v>
+      </c>
+      <c r="G509" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="H509" t="n">
+        <v>345.9200134277344</v>
+      </c>
+      <c r="I509" t="n">
+        <v>13.09000015258789</v>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K509" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L509" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M509" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N509" t="n">
+        <v>66.84999999999999</v>
+      </c>
+      <c r="O509" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E510" t="n">
+        <v>321.83</v>
+      </c>
+      <c r="F510" t="n">
+        <v>337.74</v>
+      </c>
+      <c r="G510" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="H510" t="n">
+        <v>345.989990234375</v>
+      </c>
+      <c r="I510" t="n">
+        <v>7.510000228881836</v>
+      </c>
+      <c r="J510" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K510" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L510" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M510" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N510" t="n">
+        <v>65.05</v>
+      </c>
+      <c r="O510" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E511" t="n">
+        <v>227.25</v>
+      </c>
+      <c r="F511" t="n">
+        <v>233.39</v>
+      </c>
+      <c r="G511" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H511" t="n">
+        <v>292.7799987792969</v>
+      </c>
+      <c r="I511" t="n">
+        <v>28.82999992370605</v>
+      </c>
+      <c r="J511" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K511" t="n">
+        <v>-0.273</v>
+      </c>
+      <c r="L511" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M511" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N511" t="n">
+        <v>48.59</v>
+      </c>
+      <c r="O511" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E512" t="n">
+        <v>119.14</v>
+      </c>
+      <c r="F512" t="n">
+        <v>119.16</v>
+      </c>
+      <c r="G512" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H512" t="n">
+        <v>117.1699981689453</v>
+      </c>
+      <c r="I512" t="n">
+        <v>-1.659999966621399</v>
+      </c>
+      <c r="J512" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K512" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L512" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M512" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N512" t="n">
+        <v>55.95</v>
+      </c>
+      <c r="O512" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E513" t="n">
+        <v>151.77</v>
+      </c>
+      <c r="F513" t="n">
+        <v>146.13</v>
+      </c>
+      <c r="G513" t="n">
+        <v>-3.71</v>
+      </c>
+      <c r="H513" t="n">
+        <v>149.0899963378906</v>
+      </c>
+      <c r="I513" t="n">
+        <v>-1.759999990463257</v>
+      </c>
+      <c r="J513" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K513" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L513" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M513" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N513" t="n">
+        <v>57.43</v>
+      </c>
+      <c r="O513" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E514" t="n">
+        <v>538.79</v>
+      </c>
+      <c r="F514" t="n">
+        <v>549.0599999999999</v>
+      </c>
+      <c r="G514" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="H514" t="n">
+        <v>529.4600219726562</v>
+      </c>
+      <c r="I514" t="n">
+        <v>-1.730000019073486</v>
+      </c>
+      <c r="J514" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K514" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L514" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M514" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N514" t="n">
+        <v>58.78</v>
+      </c>
+      <c r="O514" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E515" t="n">
+        <v>286.93</v>
+      </c>
+      <c r="F515" t="n">
+        <v>299.74</v>
+      </c>
+      <c r="G515" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="H515" t="n">
+        <v>283.3900146484375</v>
+      </c>
+      <c r="I515" t="n">
+        <v>-1.230000019073486</v>
+      </c>
+      <c r="J515" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K515" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L515" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M515" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N515" t="n">
+        <v>68.14</v>
+      </c>
+      <c r="O515" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E516" t="n">
+        <v>374.59</v>
+      </c>
+      <c r="F516" t="n">
+        <v>342.35</v>
+      </c>
+      <c r="G516" t="n">
+        <v>-8.609999999999999</v>
+      </c>
+      <c r="H516" t="n">
+        <v>453.0799865722656</v>
+      </c>
+      <c r="I516" t="n">
+        <v>20.95000076293945</v>
+      </c>
+      <c r="J516" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K516" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L516" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M516" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N516" t="n">
+        <v>50.09</v>
+      </c>
+      <c r="O516" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E517" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="F517" t="n">
+        <v>53.81</v>
+      </c>
+      <c r="G517" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="H517" t="n">
+        <v>59.31000137329102</v>
+      </c>
+      <c r="I517" t="n">
+        <v>11.48999977111816</v>
+      </c>
+      <c r="J517" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K517" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="L517" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M517" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N517" t="n">
+        <v>62.27</v>
+      </c>
+      <c r="O517" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E518" t="n">
+        <v>141.4</v>
+      </c>
+      <c r="F518" t="n">
+        <v>134.53</v>
+      </c>
+      <c r="G518" t="n">
+        <v>-4.86</v>
+      </c>
+      <c r="H518" t="n">
+        <v>308.6499938964844</v>
+      </c>
+      <c r="I518" t="n">
+        <v>118.2799987792969</v>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K518" t="n">
+        <v>-0.703</v>
+      </c>
+      <c r="L518" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M518" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N518" t="n">
+        <v>28.66</v>
+      </c>
+      <c r="O518" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E519" t="n">
+        <v>331.3</v>
+      </c>
+      <c r="F519" t="n">
+        <v>374.34</v>
+      </c>
+      <c r="G519" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="H519" t="n">
+        <v>341.6099853515625</v>
+      </c>
+      <c r="I519" t="n">
+        <v>3.109999895095825</v>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K519" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L519" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M519" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N519" t="n">
+        <v>80.93000000000001</v>
+      </c>
+      <c r="O519" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E520" t="n">
+        <v>940.25</v>
+      </c>
+      <c r="F520" t="n">
+        <v>935.84</v>
+      </c>
+      <c r="G520" t="n">
+        <v>-0.47</v>
+      </c>
+      <c r="H520" t="n">
+        <v>885.0900268554688</v>
+      </c>
+      <c r="I520" t="n">
+        <v>-5.869999885559082</v>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K520" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L520" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M520" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N520" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="O520" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E521" t="n">
+        <v>153.63</v>
+      </c>
+      <c r="F521" t="n">
+        <v>151.45</v>
+      </c>
+      <c r="G521" t="n">
+        <v>-1.42</v>
+      </c>
+      <c r="H521" t="n">
+        <v>149.6100006103516</v>
+      </c>
+      <c r="I521" t="n">
+        <v>-2.619999885559082</v>
+      </c>
+      <c r="J521" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K521" t="n">
+        <v>0.361</v>
+      </c>
+      <c r="L521" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M521" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N521" t="n">
+        <v>55.09</v>
+      </c>
+      <c r="O521" t="inlineStr">
+        <is>
+          <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-02-03)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O521"/>
+  <dimension ref="A1:O541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33564,6 +33564,1266 @@
       <c r="O521" t="inlineStr">
         <is>
           <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E522" t="n">
+        <v>1390.4</v>
+      </c>
+      <c r="F522" t="n">
+        <v>1517.31</v>
+      </c>
+      <c r="G522" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="H522" t="n">
+        <v>1302.069946289062</v>
+      </c>
+      <c r="I522" t="n">
+        <v>-6.349999904632568</v>
+      </c>
+      <c r="J522" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K522" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L522" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M522" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N522" t="n">
+        <v>76.69</v>
+      </c>
+      <c r="O522" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E523" t="n">
+        <v>3169.6</v>
+      </c>
+      <c r="F523" t="n">
+        <v>2974.76</v>
+      </c>
+      <c r="G523" t="n">
+        <v>-6.15</v>
+      </c>
+      <c r="H523" t="n">
+        <v>3170.989990234375</v>
+      </c>
+      <c r="I523" t="n">
+        <v>0.03999999910593033</v>
+      </c>
+      <c r="J523" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K523" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L523" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M523" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N523" t="n">
+        <v>54.78</v>
+      </c>
+      <c r="O523" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E524" t="n">
+        <v>1629.4</v>
+      </c>
+      <c r="F524" t="n">
+        <v>1539.04</v>
+      </c>
+      <c r="G524" t="n">
+        <v>-5.55</v>
+      </c>
+      <c r="H524" t="n">
+        <v>1668.150024414062</v>
+      </c>
+      <c r="I524" t="n">
+        <v>2.380000114440918</v>
+      </c>
+      <c r="J524" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K524" t="n">
+        <v>0.488</v>
+      </c>
+      <c r="L524" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M524" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N524" t="n">
+        <v>51.44</v>
+      </c>
+      <c r="O524" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E525" t="n">
+        <v>928.1</v>
+      </c>
+      <c r="F525" t="n">
+        <v>917.03</v>
+      </c>
+      <c r="G525" t="n">
+        <v>-1.19</v>
+      </c>
+      <c r="H525" t="n">
+        <v>1002.429992675781</v>
+      </c>
+      <c r="I525" t="n">
+        <v>8.010000228881836</v>
+      </c>
+      <c r="J525" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K525" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L525" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M525" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N525" t="n">
+        <v>59.93</v>
+      </c>
+      <c r="O525" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E526" t="n">
+        <v>1352.8</v>
+      </c>
+      <c r="F526" t="n">
+        <v>1360.6</v>
+      </c>
+      <c r="G526" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="H526" t="n">
+        <v>1392.06005859375</v>
+      </c>
+      <c r="I526" t="n">
+        <v>2.900000095367432</v>
+      </c>
+      <c r="J526" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K526" t="n">
+        <v>-0.44</v>
+      </c>
+      <c r="L526" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M526" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N526" t="n">
+        <v>42.06</v>
+      </c>
+      <c r="O526" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E527" t="n">
+        <v>1028.7</v>
+      </c>
+      <c r="F527" t="n">
+        <v>1091.31</v>
+      </c>
+      <c r="G527" t="n">
+        <v>6.09</v>
+      </c>
+      <c r="H527" t="n">
+        <v>1518.469970703125</v>
+      </c>
+      <c r="I527" t="n">
+        <v>47.61000061035156</v>
+      </c>
+      <c r="J527" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K527" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="L527" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M527" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N527" t="n">
+        <v>74.81</v>
+      </c>
+      <c r="O527" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E528" t="n">
+        <v>2357.3</v>
+      </c>
+      <c r="F528" t="n">
+        <v>2281.52</v>
+      </c>
+      <c r="G528" t="n">
+        <v>-3.21</v>
+      </c>
+      <c r="H528" t="n">
+        <v>2425.070068359375</v>
+      </c>
+      <c r="I528" t="n">
+        <v>2.869999885559082</v>
+      </c>
+      <c r="J528" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K528" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L528" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M528" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N528" t="n">
+        <v>53.98</v>
+      </c>
+      <c r="O528" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E529" t="n">
+        <v>314.7</v>
+      </c>
+      <c r="F529" t="n">
+        <v>299.17</v>
+      </c>
+      <c r="G529" t="n">
+        <v>-4.93</v>
+      </c>
+      <c r="H529" t="n">
+        <v>369.6000061035156</v>
+      </c>
+      <c r="I529" t="n">
+        <v>17.44000053405762</v>
+      </c>
+      <c r="J529" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K529" t="n">
+        <v>-0.636</v>
+      </c>
+      <c r="L529" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M529" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N529" t="n">
+        <v>29.88</v>
+      </c>
+      <c r="O529" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E530" t="n">
+        <v>3921.3</v>
+      </c>
+      <c r="F530" t="n">
+        <v>3853.18</v>
+      </c>
+      <c r="G530" t="n">
+        <v>-1.74</v>
+      </c>
+      <c r="H530" t="n">
+        <v>4077.739990234375</v>
+      </c>
+      <c r="I530" t="n">
+        <v>3.990000009536743</v>
+      </c>
+      <c r="J530" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K530" t="n">
+        <v>0</v>
+      </c>
+      <c r="L530" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M530" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N530" t="n">
+        <v>47.39</v>
+      </c>
+      <c r="O530" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E531" t="n">
+        <v>903.7</v>
+      </c>
+      <c r="F531" t="n">
+        <v>958</v>
+      </c>
+      <c r="G531" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="H531" t="n">
+        <v>906.3599853515625</v>
+      </c>
+      <c r="I531" t="n">
+        <v>0.2899999916553497</v>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K531" t="n">
+        <v>0.751</v>
+      </c>
+      <c r="L531" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M531" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N531" t="n">
+        <v>74.03</v>
+      </c>
+      <c r="O531" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E532" t="n">
+        <v>1965.4</v>
+      </c>
+      <c r="F532" t="n">
+        <v>2067.95</v>
+      </c>
+      <c r="G532" t="n">
+        <v>5.22</v>
+      </c>
+      <c r="H532" t="n">
+        <v>1984.949951171875</v>
+      </c>
+      <c r="I532" t="n">
+        <v>0.9900000095367432</v>
+      </c>
+      <c r="J532" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K532" t="n">
+        <v>0</v>
+      </c>
+      <c r="L532" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M532" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N532" t="n">
+        <v>57.83</v>
+      </c>
+      <c r="O532" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E533" t="n">
+        <v>2402</v>
+      </c>
+      <c r="F533" t="n">
+        <v>2590.99</v>
+      </c>
+      <c r="G533" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="H533" t="n">
+        <v>2405.64990234375</v>
+      </c>
+      <c r="I533" t="n">
+        <v>0.1500000059604645</v>
+      </c>
+      <c r="J533" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K533" t="n">
+        <v>0.8070000000000001</v>
+      </c>
+      <c r="L533" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M533" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N533" t="n">
+        <v>77.94</v>
+      </c>
+      <c r="O533" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E534" t="n">
+        <v>1311.5</v>
+      </c>
+      <c r="F534" t="n">
+        <v>1279.32</v>
+      </c>
+      <c r="G534" t="n">
+        <v>-2.45</v>
+      </c>
+      <c r="H534" t="n">
+        <v>1518.420043945312</v>
+      </c>
+      <c r="I534" t="n">
+        <v>15.77999973297119</v>
+      </c>
+      <c r="J534" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K534" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L534" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M534" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N534" t="n">
+        <v>61.88</v>
+      </c>
+      <c r="O534" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E535" t="n">
+        <v>14384</v>
+      </c>
+      <c r="F535" t="n">
+        <v>17206.29</v>
+      </c>
+      <c r="G535" t="n">
+        <v>19.62</v>
+      </c>
+      <c r="H535" t="n">
+        <v>18337.220703125</v>
+      </c>
+      <c r="I535" t="n">
+        <v>27.47999954223633</v>
+      </c>
+      <c r="J535" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K535" t="n">
+        <v>-0.637</v>
+      </c>
+      <c r="L535" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M535" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N535" t="n">
+        <v>66.69</v>
+      </c>
+      <c r="O535" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E536" t="n">
+        <v>1627.9</v>
+      </c>
+      <c r="F536" t="n">
+        <v>1649.68</v>
+      </c>
+      <c r="G536" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="H536" t="n">
+        <v>1756.489990234375</v>
+      </c>
+      <c r="I536" t="n">
+        <v>7.900000095367432</v>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K536" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L536" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M536" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N536" t="n">
+        <v>65.41</v>
+      </c>
+      <c r="O536" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E537" t="n">
+        <v>242.3</v>
+      </c>
+      <c r="F537" t="n">
+        <v>239.15</v>
+      </c>
+      <c r="G537" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="H537" t="n">
+        <v>241.2599945068359</v>
+      </c>
+      <c r="I537" t="n">
+        <v>-0.4300000071525574</v>
+      </c>
+      <c r="J537" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K537" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L537" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M537" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N537" t="n">
+        <v>63.61</v>
+      </c>
+      <c r="O537" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E538" t="n">
+        <v>12535</v>
+      </c>
+      <c r="F538" t="n">
+        <v>11605.98</v>
+      </c>
+      <c r="G538" t="n">
+        <v>-7.41</v>
+      </c>
+      <c r="H538" t="n">
+        <v>13001.3701171875</v>
+      </c>
+      <c r="I538" t="n">
+        <v>3.720000028610229</v>
+      </c>
+      <c r="J538" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K538" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="L538" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M538" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N538" t="n">
+        <v>50.86</v>
+      </c>
+      <c r="O538" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E539" t="n">
+        <v>350.35</v>
+      </c>
+      <c r="F539" t="n">
+        <v>343.71</v>
+      </c>
+      <c r="G539" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="H539" t="n">
+        <v>368.4500122070312</v>
+      </c>
+      <c r="I539" t="n">
+        <v>5.170000076293945</v>
+      </c>
+      <c r="J539" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K539" t="n">
+        <v>0.649</v>
+      </c>
+      <c r="L539" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M539" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N539" t="n">
+        <v>60.14</v>
+      </c>
+      <c r="O539" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E540" t="n">
+        <v>270.4</v>
+      </c>
+      <c r="F540" t="n">
+        <v>255.23</v>
+      </c>
+      <c r="G540" t="n">
+        <v>-5.61</v>
+      </c>
+      <c r="H540" t="n">
+        <v>285.2999877929688</v>
+      </c>
+      <c r="I540" t="n">
+        <v>5.510000228881836</v>
+      </c>
+      <c r="J540" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K540" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L540" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M540" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N540" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="O540" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E541" t="n">
+        <v>3953.2</v>
+      </c>
+      <c r="F541" t="n">
+        <v>3964.94</v>
+      </c>
+      <c r="G541" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H541" t="n">
+        <v>3805.080078125</v>
+      </c>
+      <c r="I541" t="n">
+        <v>-3.75</v>
+      </c>
+      <c r="J541" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K541" t="n">
+        <v>0.8179999999999999</v>
+      </c>
+      <c r="L541" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M541" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N541" t="n">
+        <v>66.81</v>
+      </c>
+      <c r="O541" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
         </is>
       </c>
     </row>
@@ -33578,7 +34838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O261"/>
+  <dimension ref="A1:O271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50175,6 +51435,636 @@
       <c r="O261" t="inlineStr">
         <is>
           <t>02 Feb 2026, 07:13:23 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E262" t="n">
+        <v>1390.15</v>
+      </c>
+      <c r="F262" t="n">
+        <v>1479.77</v>
+      </c>
+      <c r="G262" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="H262" t="n">
+        <v>1457.640014648438</v>
+      </c>
+      <c r="I262" t="n">
+        <v>4.849999904632568</v>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K262" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N262" t="n">
+        <v>72.67</v>
+      </c>
+      <c r="O262" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E263" t="n">
+        <v>3169.3</v>
+      </c>
+      <c r="F263" t="n">
+        <v>3020.49</v>
+      </c>
+      <c r="G263" t="n">
+        <v>-4.7</v>
+      </c>
+      <c r="H263" t="n">
+        <v>3369</v>
+      </c>
+      <c r="I263" t="n">
+        <v>6.300000190734863</v>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K263" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N263" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E264" t="n">
+        <v>1629</v>
+      </c>
+      <c r="F264" t="n">
+        <v>1560.54</v>
+      </c>
+      <c r="G264" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="H264" t="n">
+        <v>1629.910034179688</v>
+      </c>
+      <c r="I264" t="n">
+        <v>0.05999999865889549</v>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K264" t="n">
+        <v>0.488</v>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N264" t="n">
+        <v>53.46</v>
+      </c>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E265" t="n">
+        <v>927.3</v>
+      </c>
+      <c r="F265" t="n">
+        <v>920.9299999999999</v>
+      </c>
+      <c r="G265" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+      <c r="H265" t="n">
+        <v>973.4400024414062</v>
+      </c>
+      <c r="I265" t="n">
+        <v>4.980000019073486</v>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K265" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N265" t="n">
+        <v>60.69</v>
+      </c>
+      <c r="O265" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E266" t="n">
+        <v>1352.2</v>
+      </c>
+      <c r="F266" t="n">
+        <v>1357.55</v>
+      </c>
+      <c r="G266" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H266" t="n">
+        <v>1334.150024414062</v>
+      </c>
+      <c r="I266" t="n">
+        <v>-1.340000033378601</v>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K266" t="n">
+        <v>0.537</v>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N266" t="n">
+        <v>61.33</v>
+      </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E267" t="n">
+        <v>1028.45</v>
+      </c>
+      <c r="F267" t="n">
+        <v>1092.96</v>
+      </c>
+      <c r="G267" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="H267" t="n">
+        <v>1007.52001953125</v>
+      </c>
+      <c r="I267" t="n">
+        <v>-2.029999971389771</v>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K267" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N267" t="n">
+        <v>75.09</v>
+      </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E268" t="n">
+        <v>314.8</v>
+      </c>
+      <c r="F268" t="n">
+        <v>317.89</v>
+      </c>
+      <c r="G268" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="H268" t="n">
+        <v>374.25</v>
+      </c>
+      <c r="I268" t="n">
+        <v>18.8799991607666</v>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K268" t="n">
+        <v>-0.636</v>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N268" t="n">
+        <v>38.75</v>
+      </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E269" t="n">
+        <v>3922</v>
+      </c>
+      <c r="F269" t="n">
+        <v>3869.26</v>
+      </c>
+      <c r="G269" t="n">
+        <v>-1.34</v>
+      </c>
+      <c r="H269" t="n">
+        <v>3996.4599609375</v>
+      </c>
+      <c r="I269" t="n">
+        <v>1.899999976158142</v>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K269" t="n">
+        <v>0</v>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N269" t="n">
+        <v>47.98</v>
+      </c>
+      <c r="O269" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E270" t="n">
+        <v>1317.85</v>
+      </c>
+      <c r="F270" t="n">
+        <v>1269.13</v>
+      </c>
+      <c r="G270" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="H270" t="n">
+        <v>1330.430053710938</v>
+      </c>
+      <c r="I270" t="n">
+        <v>0.949999988079071</v>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K270" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N270" t="n">
+        <v>60.01</v>
+      </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E271" t="n">
+        <v>14387.05</v>
+      </c>
+      <c r="F271" t="n">
+        <v>17212.98</v>
+      </c>
+      <c r="G271" t="n">
+        <v>19.64</v>
+      </c>
+      <c r="H271" t="n">
+        <v>13461.2099609375</v>
+      </c>
+      <c r="I271" t="n">
+        <v>-6.440000057220459</v>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K271" t="n">
+        <v>-0.637</v>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N271" t="n">
+        <v>66.72</v>
+      </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
         </is>
       </c>
     </row>
@@ -50189,7 +52079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O521"/>
+  <dimension ref="A1:O541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83309,6 +85199,1266 @@
         </is>
       </c>
     </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E522" t="n">
+        <v>270.01</v>
+      </c>
+      <c r="F522" t="n">
+        <v>257.62</v>
+      </c>
+      <c r="G522" t="n">
+        <v>-4.59</v>
+      </c>
+      <c r="H522" t="n">
+        <v>224.7200012207031</v>
+      </c>
+      <c r="I522" t="n">
+        <v>-16.77000045776367</v>
+      </c>
+      <c r="J522" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K522" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L522" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M522" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N522" t="n">
+        <v>56.12</v>
+      </c>
+      <c r="O522" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E523" t="n">
+        <v>423.37</v>
+      </c>
+      <c r="F523" t="n">
+        <v>432.87</v>
+      </c>
+      <c r="G523" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="H523" t="n">
+        <v>418.0299987792969</v>
+      </c>
+      <c r="I523" t="n">
+        <v>-1.259999990463257</v>
+      </c>
+      <c r="J523" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K523" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L523" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M523" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N523" t="n">
+        <v>59.29</v>
+      </c>
+      <c r="O523" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E524" t="n">
+        <v>343.69</v>
+      </c>
+      <c r="F524" t="n">
+        <v>348.93</v>
+      </c>
+      <c r="G524" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="H524" t="n">
+        <v>353.9100036621094</v>
+      </c>
+      <c r="I524" t="n">
+        <v>2.970000028610229</v>
+      </c>
+      <c r="J524" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K524" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L524" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M524" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N524" t="n">
+        <v>65.48999999999999</v>
+      </c>
+      <c r="O524" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E525" t="n">
+        <v>242.96</v>
+      </c>
+      <c r="F525" t="n">
+        <v>240.39</v>
+      </c>
+      <c r="G525" t="n">
+        <v>-1.06</v>
+      </c>
+      <c r="H525" t="n">
+        <v>235.2599945068359</v>
+      </c>
+      <c r="I525" t="n">
+        <v>-3.170000076293945</v>
+      </c>
+      <c r="J525" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K525" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L525" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M525" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N525" t="n">
+        <v>57.95</v>
+      </c>
+      <c r="O525" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E526" t="n">
+        <v>706.41</v>
+      </c>
+      <c r="F526" t="n">
+        <v>684.84</v>
+      </c>
+      <c r="G526" t="n">
+        <v>-3.05</v>
+      </c>
+      <c r="H526" t="n">
+        <v>663.4099731445312</v>
+      </c>
+      <c r="I526" t="n">
+        <v>-6.090000152587891</v>
+      </c>
+      <c r="J526" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K526" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="L526" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M526" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N526" t="n">
+        <v>60.58</v>
+      </c>
+      <c r="O526" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E527" t="n">
+        <v>421.81</v>
+      </c>
+      <c r="F527" t="n">
+        <v>408.66</v>
+      </c>
+      <c r="G527" t="n">
+        <v>-3.12</v>
+      </c>
+      <c r="H527" t="n">
+        <v>272.6199951171875</v>
+      </c>
+      <c r="I527" t="n">
+        <v>-35.36999893188477</v>
+      </c>
+      <c r="J527" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K527" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L527" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M527" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N527" t="n">
+        <v>51.25</v>
+      </c>
+      <c r="O527" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E528" t="n">
+        <v>185.61</v>
+      </c>
+      <c r="F528" t="n">
+        <v>199.38</v>
+      </c>
+      <c r="G528" t="n">
+        <v>7.42</v>
+      </c>
+      <c r="H528" t="n">
+        <v>205.2599945068359</v>
+      </c>
+      <c r="I528" t="n">
+        <v>10.59000015258789</v>
+      </c>
+      <c r="J528" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K528" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L528" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M528" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N528" t="n">
+        <v>74.13</v>
+      </c>
+      <c r="O528" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E529" t="n">
+        <v>308.14</v>
+      </c>
+      <c r="F529" t="n">
+        <v>319.59</v>
+      </c>
+      <c r="G529" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="H529" t="n">
+        <v>294.3500061035156</v>
+      </c>
+      <c r="I529" t="n">
+        <v>-4.480000019073486</v>
+      </c>
+      <c r="J529" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K529" t="n">
+        <v>0</v>
+      </c>
+      <c r="L529" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M529" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N529" t="n">
+        <v>55.58</v>
+      </c>
+      <c r="O529" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E530" t="n">
+        <v>333.84</v>
+      </c>
+      <c r="F530" t="n">
+        <v>336.33</v>
+      </c>
+      <c r="G530" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H530" t="n">
+        <v>325.7699890136719</v>
+      </c>
+      <c r="I530" t="n">
+        <v>-2.420000076293945</v>
+      </c>
+      <c r="J530" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K530" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L530" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M530" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N530" t="n">
+        <v>61</v>
+      </c>
+      <c r="O530" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E531" t="n">
+        <v>230.75</v>
+      </c>
+      <c r="F531" t="n">
+        <v>235.4</v>
+      </c>
+      <c r="G531" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="H531" t="n">
+        <v>373.25</v>
+      </c>
+      <c r="I531" t="n">
+        <v>61.75</v>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K531" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L531" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M531" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N531" t="n">
+        <v>62.91</v>
+      </c>
+      <c r="O531" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E532" t="n">
+        <v>124.06</v>
+      </c>
+      <c r="F532" t="n">
+        <v>118.1</v>
+      </c>
+      <c r="G532" t="n">
+        <v>-4.81</v>
+      </c>
+      <c r="H532" t="n">
+        <v>124.2699966430664</v>
+      </c>
+      <c r="I532" t="n">
+        <v>0.1700000017881393</v>
+      </c>
+      <c r="J532" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K532" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L532" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M532" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N532" t="n">
+        <v>48.71</v>
+      </c>
+      <c r="O532" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E533" t="n">
+        <v>153.19</v>
+      </c>
+      <c r="F533" t="n">
+        <v>146.64</v>
+      </c>
+      <c r="G533" t="n">
+        <v>-4.28</v>
+      </c>
+      <c r="H533" t="n">
+        <v>144.6300048828125</v>
+      </c>
+      <c r="I533" t="n">
+        <v>-5.590000152587891</v>
+      </c>
+      <c r="J533" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K533" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L533" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M533" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N533" t="n">
+        <v>56.59</v>
+      </c>
+      <c r="O533" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E534" t="n">
+        <v>555.37</v>
+      </c>
+      <c r="F534" t="n">
+        <v>545.71</v>
+      </c>
+      <c r="G534" t="n">
+        <v>-1.74</v>
+      </c>
+      <c r="H534" t="n">
+        <v>575.77001953125</v>
+      </c>
+      <c r="I534" t="n">
+        <v>3.670000076293945</v>
+      </c>
+      <c r="J534" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K534" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L534" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M534" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N534" t="n">
+        <v>58.53</v>
+      </c>
+      <c r="O534" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E535" t="n">
+        <v>285.59</v>
+      </c>
+      <c r="F535" t="n">
+        <v>284</v>
+      </c>
+      <c r="G535" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="H535" t="n">
+        <v>287.9500122070312</v>
+      </c>
+      <c r="I535" t="n">
+        <v>0.8299999833106995</v>
+      </c>
+      <c r="J535" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K535" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L535" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M535" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N535" t="n">
+        <v>60.61</v>
+      </c>
+      <c r="O535" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E536" t="n">
+        <v>378.12</v>
+      </c>
+      <c r="F536" t="n">
+        <v>339.21</v>
+      </c>
+      <c r="G536" t="n">
+        <v>-10.29</v>
+      </c>
+      <c r="H536" t="n">
+        <v>384.3800048828125</v>
+      </c>
+      <c r="I536" t="n">
+        <v>1.659999966621399</v>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K536" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L536" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M536" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N536" t="n">
+        <v>47.76</v>
+      </c>
+      <c r="O536" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E537" t="n">
+        <v>54.03</v>
+      </c>
+      <c r="F537" t="n">
+        <v>53.62</v>
+      </c>
+      <c r="G537" t="n">
+        <v>-0.76</v>
+      </c>
+      <c r="H537" t="n">
+        <v>52.83000183105469</v>
+      </c>
+      <c r="I537" t="n">
+        <v>-2.210000038146973</v>
+      </c>
+      <c r="J537" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K537" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L537" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M537" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N537" t="n">
+        <v>61.86</v>
+      </c>
+      <c r="O537" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E538" t="n">
+        <v>138.4</v>
+      </c>
+      <c r="F538" t="n">
+        <v>136.59</v>
+      </c>
+      <c r="G538" t="n">
+        <v>-1.31</v>
+      </c>
+      <c r="H538" t="n">
+        <v>233.6600036621094</v>
+      </c>
+      <c r="I538" t="n">
+        <v>68.83000183105469</v>
+      </c>
+      <c r="J538" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K538" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L538" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M538" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N538" t="n">
+        <v>57.92</v>
+      </c>
+      <c r="O538" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E539" t="n">
+        <v>331.11</v>
+      </c>
+      <c r="F539" t="n">
+        <v>363.85</v>
+      </c>
+      <c r="G539" t="n">
+        <v>9.890000000000001</v>
+      </c>
+      <c r="H539" t="n">
+        <v>322.1099853515625</v>
+      </c>
+      <c r="I539" t="n">
+        <v>-2.720000028610229</v>
+      </c>
+      <c r="J539" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K539" t="n">
+        <v>0.765</v>
+      </c>
+      <c r="L539" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M539" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N539" t="n">
+        <v>80.13</v>
+      </c>
+      <c r="O539" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E540" t="n">
+        <v>968.36</v>
+      </c>
+      <c r="F540" t="n">
+        <v>928.46</v>
+      </c>
+      <c r="G540" t="n">
+        <v>-4.12</v>
+      </c>
+      <c r="H540" t="n">
+        <v>863.4500122070312</v>
+      </c>
+      <c r="I540" t="n">
+        <v>-10.82999992370605</v>
+      </c>
+      <c r="J540" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K540" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L540" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M540" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N540" t="n">
+        <v>30.82</v>
+      </c>
+      <c r="O540" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E541" t="n">
+        <v>155.2</v>
+      </c>
+      <c r="F541" t="n">
+        <v>152.46</v>
+      </c>
+      <c r="G541" t="n">
+        <v>-1.76</v>
+      </c>
+      <c r="H541" t="n">
+        <v>156.0500030517578</v>
+      </c>
+      <c r="I541" t="n">
+        <v>0.550000011920929</v>
+      </c>
+      <c r="J541" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K541" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="L541" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M541" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N541" t="n">
+        <v>62.79</v>
+      </c>
+      <c r="O541" t="inlineStr">
+        <is>
+          <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-02-04)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O541"/>
+  <dimension ref="A1:O561"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34824,6 +34824,1266 @@
       <c r="O541" t="inlineStr">
         <is>
           <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E542" t="n">
+        <v>1437.1</v>
+      </c>
+      <c r="F542" t="n">
+        <v>1511.47</v>
+      </c>
+      <c r="G542" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="H542" t="n">
+        <v>1391.199951171875</v>
+      </c>
+      <c r="I542" t="n">
+        <v>-3.190000057220459</v>
+      </c>
+      <c r="J542" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K542" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L542" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M542" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N542" t="n">
+        <v>70.76000000000001</v>
+      </c>
+      <c r="O542" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E543" t="n">
+        <v>3225.3</v>
+      </c>
+      <c r="F543" t="n">
+        <v>2967.54</v>
+      </c>
+      <c r="G543" t="n">
+        <v>-7.99</v>
+      </c>
+      <c r="H543" t="n">
+        <v>3309.469970703125</v>
+      </c>
+      <c r="I543" t="n">
+        <v>2.609999895095825</v>
+      </c>
+      <c r="J543" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K543" t="n">
+        <v>-0.542</v>
+      </c>
+      <c r="L543" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M543" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N543" t="n">
+        <v>27.17</v>
+      </c>
+      <c r="O543" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E544" t="n">
+        <v>1656</v>
+      </c>
+      <c r="F544" t="n">
+        <v>1520.39</v>
+      </c>
+      <c r="G544" t="n">
+        <v>-8.19</v>
+      </c>
+      <c r="H544" t="n">
+        <v>1609.949951171875</v>
+      </c>
+      <c r="I544" t="n">
+        <v>-2.779999971389771</v>
+      </c>
+      <c r="J544" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K544" t="n">
+        <v>-0.493</v>
+      </c>
+      <c r="L544" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M544" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N544" t="n">
+        <v>27.86</v>
+      </c>
+      <c r="O544" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E545" t="n">
+        <v>948.7</v>
+      </c>
+      <c r="F545" t="n">
+        <v>917.46</v>
+      </c>
+      <c r="G545" t="n">
+        <v>-3.29</v>
+      </c>
+      <c r="H545" t="n">
+        <v>834.0700073242188</v>
+      </c>
+      <c r="I545" t="n">
+        <v>-12.07999992370605</v>
+      </c>
+      <c r="J545" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K545" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="L545" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M545" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N545" t="n">
+        <v>62.02</v>
+      </c>
+      <c r="O545" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E546" t="n">
+        <v>1389.7</v>
+      </c>
+      <c r="F546" t="n">
+        <v>1363.38</v>
+      </c>
+      <c r="G546" t="n">
+        <v>-1.89</v>
+      </c>
+      <c r="H546" t="n">
+        <v>1396</v>
+      </c>
+      <c r="I546" t="n">
+        <v>0.449999988079071</v>
+      </c>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K546" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L546" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M546" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N546" t="n">
+        <v>57.38</v>
+      </c>
+      <c r="O546" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E547" t="n">
+        <v>1064.2</v>
+      </c>
+      <c r="F547" t="n">
+        <v>1089.81</v>
+      </c>
+      <c r="G547" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="H547" t="n">
+        <v>1086.569946289062</v>
+      </c>
+      <c r="I547" t="n">
+        <v>2.099999904632568</v>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K547" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L547" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M547" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N547" t="n">
+        <v>66.61</v>
+      </c>
+      <c r="O547" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E548" t="n">
+        <v>2368.6</v>
+      </c>
+      <c r="F548" t="n">
+        <v>2248.33</v>
+      </c>
+      <c r="G548" t="n">
+        <v>-5.08</v>
+      </c>
+      <c r="H548" t="n">
+        <v>2273.360107421875</v>
+      </c>
+      <c r="I548" t="n">
+        <v>-4.019999980926514</v>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K548" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L548" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M548" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N548" t="n">
+        <v>29.38</v>
+      </c>
+      <c r="O548" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E549" t="n">
+        <v>310.15</v>
+      </c>
+      <c r="F549" t="n">
+        <v>289.15</v>
+      </c>
+      <c r="G549" t="n">
+        <v>-6.77</v>
+      </c>
+      <c r="H549" t="n">
+        <v>358.9299926757812</v>
+      </c>
+      <c r="I549" t="n">
+        <v>15.72999954223633</v>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K549" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L549" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M549" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N549" t="n">
+        <v>52.34</v>
+      </c>
+      <c r="O549" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E550" t="n">
+        <v>4038.8</v>
+      </c>
+      <c r="F550" t="n">
+        <v>3859.76</v>
+      </c>
+      <c r="G550" t="n">
+        <v>-4.43</v>
+      </c>
+      <c r="H550" t="n">
+        <v>4092.75</v>
+      </c>
+      <c r="I550" t="n">
+        <v>1.340000033378601</v>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K550" t="n">
+        <v>0</v>
+      </c>
+      <c r="L550" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M550" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N550" t="n">
+        <v>43.35</v>
+      </c>
+      <c r="O550" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E551" t="n">
+        <v>964.4</v>
+      </c>
+      <c r="F551" t="n">
+        <v>958.55</v>
+      </c>
+      <c r="G551" t="n">
+        <v>-0.61</v>
+      </c>
+      <c r="H551" t="n">
+        <v>811.010009765625</v>
+      </c>
+      <c r="I551" t="n">
+        <v>-15.90999984741211</v>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K551" t="n">
+        <v>0.827</v>
+      </c>
+      <c r="L551" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M551" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N551" t="n">
+        <v>65.63</v>
+      </c>
+      <c r="O551" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E552" t="n">
+        <v>1997.3</v>
+      </c>
+      <c r="F552" t="n">
+        <v>2051.53</v>
+      </c>
+      <c r="G552" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="H552" t="n">
+        <v>2061.949951171875</v>
+      </c>
+      <c r="I552" t="n">
+        <v>3.240000009536743</v>
+      </c>
+      <c r="J552" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K552" t="n">
+        <v>0.832</v>
+      </c>
+      <c r="L552" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M552" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N552" t="n">
+        <v>70.70999999999999</v>
+      </c>
+      <c r="O552" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E553" t="n">
+        <v>2426</v>
+      </c>
+      <c r="F553" t="n">
+        <v>2529.05</v>
+      </c>
+      <c r="G553" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="H553" t="n">
+        <v>2361.02001953125</v>
+      </c>
+      <c r="I553" t="n">
+        <v>-2.680000066757202</v>
+      </c>
+      <c r="J553" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K553" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L553" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M553" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N553" t="n">
+        <v>65.17</v>
+      </c>
+      <c r="O553" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E554" t="n">
+        <v>1356.2</v>
+      </c>
+      <c r="F554" t="n">
+        <v>1284.54</v>
+      </c>
+      <c r="G554" t="n">
+        <v>-5.28</v>
+      </c>
+      <c r="H554" t="n">
+        <v>1240.989990234375</v>
+      </c>
+      <c r="I554" t="n">
+        <v>-8.489999771118164</v>
+      </c>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K554" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L554" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M554" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N554" t="n">
+        <v>53.21</v>
+      </c>
+      <c r="O554" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E555" t="n">
+        <v>14782</v>
+      </c>
+      <c r="F555" t="n">
+        <v>17064.73</v>
+      </c>
+      <c r="G555" t="n">
+        <v>15.44</v>
+      </c>
+      <c r="H555" t="n">
+        <v>16576.150390625</v>
+      </c>
+      <c r="I555" t="n">
+        <v>12.14000034332275</v>
+      </c>
+      <c r="J555" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K555" t="n">
+        <v>-0.637</v>
+      </c>
+      <c r="L555" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M555" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N555" t="n">
+        <v>60.42</v>
+      </c>
+      <c r="O555" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E556" t="n">
+        <v>1702.1</v>
+      </c>
+      <c r="F556" t="n">
+        <v>1646.65</v>
+      </c>
+      <c r="G556" t="n">
+        <v>-3.26</v>
+      </c>
+      <c r="H556" t="n">
+        <v>1657.349975585938</v>
+      </c>
+      <c r="I556" t="n">
+        <v>-2.630000114440918</v>
+      </c>
+      <c r="J556" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K556" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L556" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M556" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N556" t="n">
+        <v>57.61</v>
+      </c>
+      <c r="O556" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E557" t="n">
+        <v>242.69</v>
+      </c>
+      <c r="F557" t="n">
+        <v>237.44</v>
+      </c>
+      <c r="G557" t="n">
+        <v>-2.16</v>
+      </c>
+      <c r="H557" t="n">
+        <v>225.2200012207031</v>
+      </c>
+      <c r="I557" t="n">
+        <v>-7.199999809265137</v>
+      </c>
+      <c r="J557" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K557" t="n">
+        <v>-0.8070000000000001</v>
+      </c>
+      <c r="L557" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M557" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N557" t="n">
+        <v>30.61</v>
+      </c>
+      <c r="O557" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E558" t="n">
+        <v>12590</v>
+      </c>
+      <c r="F558" t="n">
+        <v>11681.77</v>
+      </c>
+      <c r="G558" t="n">
+        <v>-7.21</v>
+      </c>
+      <c r="H558" t="n">
+        <v>12951.740234375</v>
+      </c>
+      <c r="I558" t="n">
+        <v>2.869999885559082</v>
+      </c>
+      <c r="J558" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K558" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="L558" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M558" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N558" t="n">
+        <v>51.16</v>
+      </c>
+      <c r="O558" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E559" t="n">
+        <v>358.55</v>
+      </c>
+      <c r="F559" t="n">
+        <v>345.36</v>
+      </c>
+      <c r="G559" t="n">
+        <v>-3.68</v>
+      </c>
+      <c r="H559" t="n">
+        <v>341.5299987792969</v>
+      </c>
+      <c r="I559" t="n">
+        <v>-4.75</v>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K559" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L559" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M559" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N559" t="n">
+        <v>57.48</v>
+      </c>
+      <c r="O559" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E560" t="n">
+        <v>283.2</v>
+      </c>
+      <c r="F560" t="n">
+        <v>257.4</v>
+      </c>
+      <c r="G560" t="n">
+        <v>-9.109999999999999</v>
+      </c>
+      <c r="H560" t="n">
+        <v>277.9100036621094</v>
+      </c>
+      <c r="I560" t="n">
+        <v>-1.870000004768372</v>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K560" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L560" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M560" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N560" t="n">
+        <v>46.56</v>
+      </c>
+      <c r="O560" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E561" t="n">
+        <v>4068.6</v>
+      </c>
+      <c r="F561" t="n">
+        <v>3976.02</v>
+      </c>
+      <c r="G561" t="n">
+        <v>-2.28</v>
+      </c>
+      <c r="H561" t="n">
+        <v>4228.2001953125</v>
+      </c>
+      <c r="I561" t="n">
+        <v>3.920000076293945</v>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K561" t="n">
+        <v>0.8179999999999999</v>
+      </c>
+      <c r="L561" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M561" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N561" t="n">
+        <v>62.95</v>
+      </c>
+      <c r="O561" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
         </is>
       </c>
     </row>
@@ -34838,7 +36098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O271"/>
+  <dimension ref="A1:O281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52065,6 +53325,636 @@
       <c r="O271" t="inlineStr">
         <is>
           <t>03 Feb 2026, 07:14:01 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E272" t="n">
+        <v>1437.85</v>
+      </c>
+      <c r="F272" t="n">
+        <v>1488.55</v>
+      </c>
+      <c r="G272" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="H272" t="n">
+        <v>1670.329956054688</v>
+      </c>
+      <c r="I272" t="n">
+        <v>16.17000007629395</v>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K272" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N272" t="n">
+        <v>68.29000000000001</v>
+      </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E273" t="n">
+        <v>3223.7</v>
+      </c>
+      <c r="F273" t="n">
+        <v>3002.54</v>
+      </c>
+      <c r="G273" t="n">
+        <v>-6.86</v>
+      </c>
+      <c r="H273" t="n">
+        <v>3405.909912109375</v>
+      </c>
+      <c r="I273" t="n">
+        <v>5.650000095367432</v>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K273" t="n">
+        <v>-0.542</v>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N273" t="n">
+        <v>28.87</v>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E274" t="n">
+        <v>1654.95</v>
+      </c>
+      <c r="F274" t="n">
+        <v>1553.11</v>
+      </c>
+      <c r="G274" t="n">
+        <v>-6.15</v>
+      </c>
+      <c r="H274" t="n">
+        <v>1657.849975585938</v>
+      </c>
+      <c r="I274" t="n">
+        <v>0.1800000071525574</v>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K274" t="n">
+        <v>-0.511</v>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N274" t="n">
+        <v>30.55</v>
+      </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E275" t="n">
+        <v>948.4</v>
+      </c>
+      <c r="F275" t="n">
+        <v>922.26</v>
+      </c>
+      <c r="G275" t="n">
+        <v>-2.76</v>
+      </c>
+      <c r="H275" t="n">
+        <v>1055.150024414062</v>
+      </c>
+      <c r="I275" t="n">
+        <v>11.26000022888184</v>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K275" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N275" t="n">
+        <v>62.83</v>
+      </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E276" t="n">
+        <v>1389.6</v>
+      </c>
+      <c r="F276" t="n">
+        <v>1361.4</v>
+      </c>
+      <c r="G276" t="n">
+        <v>-2.03</v>
+      </c>
+      <c r="H276" t="n">
+        <v>1335.530029296875</v>
+      </c>
+      <c r="I276" t="n">
+        <v>-3.890000104904175</v>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K276" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N276" t="n">
+        <v>57.18</v>
+      </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E277" t="n">
+        <v>1064.25</v>
+      </c>
+      <c r="F277" t="n">
+        <v>1105.35</v>
+      </c>
+      <c r="G277" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="H277" t="n">
+        <v>1084.390014648438</v>
+      </c>
+      <c r="I277" t="n">
+        <v>1.889999985694885</v>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K277" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N277" t="n">
+        <v>68.79000000000001</v>
+      </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E278" t="n">
+        <v>310.2</v>
+      </c>
+      <c r="F278" t="n">
+        <v>304.62</v>
+      </c>
+      <c r="G278" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="H278" t="n">
+        <v>353.0199890136719</v>
+      </c>
+      <c r="I278" t="n">
+        <v>13.80000019073486</v>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K278" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N278" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E279" t="n">
+        <v>4037.65</v>
+      </c>
+      <c r="F279" t="n">
+        <v>3875.71</v>
+      </c>
+      <c r="G279" t="n">
+        <v>-4.01</v>
+      </c>
+      <c r="H279" t="n">
+        <v>3698.8798828125</v>
+      </c>
+      <c r="I279" t="n">
+        <v>-8.390000343322754</v>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K279" t="n">
+        <v>0</v>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N279" t="n">
+        <v>43.98</v>
+      </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E280" t="n">
+        <v>1355.55</v>
+      </c>
+      <c r="F280" t="n">
+        <v>1277.03</v>
+      </c>
+      <c r="G280" t="n">
+        <v>-5.79</v>
+      </c>
+      <c r="H280" t="n">
+        <v>1493.829956054688</v>
+      </c>
+      <c r="I280" t="n">
+        <v>10.19999980926514</v>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K280" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N280" t="n">
+        <v>52.45</v>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E281" t="n">
+        <v>14779.6</v>
+      </c>
+      <c r="F281" t="n">
+        <v>17170.84</v>
+      </c>
+      <c r="G281" t="n">
+        <v>16.18</v>
+      </c>
+      <c r="H281" t="n">
+        <v>15579.83984375</v>
+      </c>
+      <c r="I281" t="n">
+        <v>5.409999847412109</v>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K281" t="n">
+        <v>-0.637</v>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N281" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
         </is>
       </c>
     </row>
@@ -52079,7 +53969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O541"/>
+  <dimension ref="A1:O561"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -86459,6 +88349,1266 @@
         </is>
       </c>
     </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E542" t="n">
+        <v>269.48</v>
+      </c>
+      <c r="F542" t="n">
+        <v>258.53</v>
+      </c>
+      <c r="G542" t="n">
+        <v>-4.06</v>
+      </c>
+      <c r="H542" t="n">
+        <v>262.0199890136719</v>
+      </c>
+      <c r="I542" t="n">
+        <v>-2.769999980926514</v>
+      </c>
+      <c r="J542" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K542" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L542" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M542" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N542" t="n">
+        <v>53.78</v>
+      </c>
+      <c r="O542" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E543" t="n">
+        <v>411.21</v>
+      </c>
+      <c r="F543" t="n">
+        <v>427.86</v>
+      </c>
+      <c r="G543" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="H543" t="n">
+        <v>406.7699890136719</v>
+      </c>
+      <c r="I543" t="n">
+        <v>-1.080000042915344</v>
+      </c>
+      <c r="J543" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K543" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L543" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M543" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N543" t="n">
+        <v>69.06999999999999</v>
+      </c>
+      <c r="O543" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E544" t="n">
+        <v>339.71</v>
+      </c>
+      <c r="F544" t="n">
+        <v>347.45</v>
+      </c>
+      <c r="G544" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="H544" t="n">
+        <v>437.8200073242188</v>
+      </c>
+      <c r="I544" t="n">
+        <v>28.8799991607666</v>
+      </c>
+      <c r="J544" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K544" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="L544" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M544" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N544" t="n">
+        <v>67.23999999999999</v>
+      </c>
+      <c r="O544" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E545" t="n">
+        <v>238.62</v>
+      </c>
+      <c r="F545" t="n">
+        <v>238.33</v>
+      </c>
+      <c r="G545" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="H545" t="n">
+        <v>241.1399993896484</v>
+      </c>
+      <c r="I545" t="n">
+        <v>1.059999942779541</v>
+      </c>
+      <c r="J545" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K545" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L545" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M545" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N545" t="n">
+        <v>57.46</v>
+      </c>
+      <c r="O545" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E546" t="n">
+        <v>691.7</v>
+      </c>
+      <c r="F546" t="n">
+        <v>676.55</v>
+      </c>
+      <c r="G546" t="n">
+        <v>-2.19</v>
+      </c>
+      <c r="H546" t="n">
+        <v>663.6099853515625</v>
+      </c>
+      <c r="I546" t="n">
+        <v>-4.059999942779541</v>
+      </c>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K546" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L546" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M546" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N546" t="n">
+        <v>60.71</v>
+      </c>
+      <c r="O546" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E547" t="n">
+        <v>421.96</v>
+      </c>
+      <c r="F547" t="n">
+        <v>405.32</v>
+      </c>
+      <c r="G547" t="n">
+        <v>-3.94</v>
+      </c>
+      <c r="H547" t="n">
+        <v>371.3200073242188</v>
+      </c>
+      <c r="I547" t="n">
+        <v>-12</v>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K547" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L547" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M547" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N547" t="n">
+        <v>53.63</v>
+      </c>
+      <c r="O547" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E548" t="n">
+        <v>180.34</v>
+      </c>
+      <c r="F548" t="n">
+        <v>198.3</v>
+      </c>
+      <c r="G548" t="n">
+        <v>9.960000000000001</v>
+      </c>
+      <c r="H548" t="n">
+        <v>219.0099945068359</v>
+      </c>
+      <c r="I548" t="n">
+        <v>21.44000053405762</v>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K548" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L548" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M548" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N548" t="n">
+        <v>77.94</v>
+      </c>
+      <c r="O548" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E549" t="n">
+        <v>314.85</v>
+      </c>
+      <c r="F549" t="n">
+        <v>317.58</v>
+      </c>
+      <c r="G549" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="H549" t="n">
+        <v>319.8500061035156</v>
+      </c>
+      <c r="I549" t="n">
+        <v>1.590000033378601</v>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K549" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L549" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M549" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N549" t="n">
+        <v>62.74</v>
+      </c>
+      <c r="O549" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E550" t="n">
+        <v>328.93</v>
+      </c>
+      <c r="F550" t="n">
+        <v>334.59</v>
+      </c>
+      <c r="G550" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="H550" t="n">
+        <v>316.8999938964844</v>
+      </c>
+      <c r="I550" t="n">
+        <v>-3.660000085830688</v>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K550" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L550" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M550" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N550" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="O550" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E551" t="n">
+        <v>233.1</v>
+      </c>
+      <c r="F551" t="n">
+        <v>238.24</v>
+      </c>
+      <c r="G551" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="H551" t="n">
+        <v>222.9400024414062</v>
+      </c>
+      <c r="I551" t="n">
+        <v>-4.360000133514404</v>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K551" t="n">
+        <v>0</v>
+      </c>
+      <c r="L551" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M551" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N551" t="n">
+        <v>53.31</v>
+      </c>
+      <c r="O551" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E552" t="n">
+        <v>127.71</v>
+      </c>
+      <c r="F552" t="n">
+        <v>118.32</v>
+      </c>
+      <c r="G552" t="n">
+        <v>-7.35</v>
+      </c>
+      <c r="H552" t="n">
+        <v>109.120002746582</v>
+      </c>
+      <c r="I552" t="n">
+        <v>-14.55000019073486</v>
+      </c>
+      <c r="J552" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K552" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="L552" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M552" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N552" t="n">
+        <v>40.01</v>
+      </c>
+      <c r="O552" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E553" t="n">
+        <v>155.32</v>
+      </c>
+      <c r="F553" t="n">
+        <v>148.63</v>
+      </c>
+      <c r="G553" t="n">
+        <v>-4.31</v>
+      </c>
+      <c r="H553" t="n">
+        <v>157.8200073242188</v>
+      </c>
+      <c r="I553" t="n">
+        <v>1.610000014305115</v>
+      </c>
+      <c r="J553" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K553" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L553" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M553" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N553" t="n">
+        <v>56.53</v>
+      </c>
+      <c r="O553" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E554" t="n">
+        <v>550.72</v>
+      </c>
+      <c r="F554" t="n">
+        <v>543.4</v>
+      </c>
+      <c r="G554" t="n">
+        <v>-1.33</v>
+      </c>
+      <c r="H554" t="n">
+        <v>575.4500122070312</v>
+      </c>
+      <c r="I554" t="n">
+        <v>4.489999771118164</v>
+      </c>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K554" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L554" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M554" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N554" t="n">
+        <v>59.45</v>
+      </c>
+      <c r="O554" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E555" t="n">
+        <v>284.18</v>
+      </c>
+      <c r="F555" t="n">
+        <v>279.02</v>
+      </c>
+      <c r="G555" t="n">
+        <v>-1.82</v>
+      </c>
+      <c r="H555" t="n">
+        <v>321.6099853515625</v>
+      </c>
+      <c r="I555" t="n">
+        <v>13.17000007629395</v>
+      </c>
+      <c r="J555" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K555" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L555" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M555" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N555" t="n">
+        <v>58.72</v>
+      </c>
+      <c r="O555" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E556" t="n">
+        <v>381.1</v>
+      </c>
+      <c r="F556" t="n">
+        <v>338.74</v>
+      </c>
+      <c r="G556" t="n">
+        <v>-11.11</v>
+      </c>
+      <c r="H556" t="n">
+        <v>395.3900146484375</v>
+      </c>
+      <c r="I556" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J556" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K556" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L556" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M556" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N556" t="n">
+        <v>46.33</v>
+      </c>
+      <c r="O556" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E557" t="n">
+        <v>54.45</v>
+      </c>
+      <c r="F557" t="n">
+        <v>53.49</v>
+      </c>
+      <c r="G557" t="n">
+        <v>-1.77</v>
+      </c>
+      <c r="H557" t="n">
+        <v>55.29000091552734</v>
+      </c>
+      <c r="I557" t="n">
+        <v>1.529999971389771</v>
+      </c>
+      <c r="J557" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K557" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L557" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M557" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N557" t="n">
+        <v>60.35</v>
+      </c>
+      <c r="O557" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E558" t="n">
+        <v>143.73</v>
+      </c>
+      <c r="F558" t="n">
+        <v>137.17</v>
+      </c>
+      <c r="G558" t="n">
+        <v>-4.57</v>
+      </c>
+      <c r="H558" t="n">
+        <v>296.3800048828125</v>
+      </c>
+      <c r="I558" t="n">
+        <v>106.2099990844727</v>
+      </c>
+      <c r="J558" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K558" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L558" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M558" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N558" t="n">
+        <v>56.35</v>
+      </c>
+      <c r="O558" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E559" t="n">
+        <v>320.33</v>
+      </c>
+      <c r="F559" t="n">
+        <v>365.57</v>
+      </c>
+      <c r="G559" t="n">
+        <v>14.12</v>
+      </c>
+      <c r="H559" t="n">
+        <v>312.489990234375</v>
+      </c>
+      <c r="I559" t="n">
+        <v>-2.450000047683716</v>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K559" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L559" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M559" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N559" t="n">
+        <v>78.81999999999999</v>
+      </c>
+      <c r="O559" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E560" t="n">
+        <v>977.92</v>
+      </c>
+      <c r="F560" t="n">
+        <v>924.35</v>
+      </c>
+      <c r="G560" t="n">
+        <v>-5.48</v>
+      </c>
+      <c r="H560" t="n">
+        <v>991.3300170898438</v>
+      </c>
+      <c r="I560" t="n">
+        <v>1.370000004768372</v>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K560" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L560" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M560" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N560" t="n">
+        <v>28.78</v>
+      </c>
+      <c r="O560" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E561" t="n">
+        <v>162.85</v>
+      </c>
+      <c r="F561" t="n">
+        <v>153.38</v>
+      </c>
+      <c r="G561" t="n">
+        <v>-5.82</v>
+      </c>
+      <c r="H561" t="n">
+        <v>197.6199951171875</v>
+      </c>
+      <c r="I561" t="n">
+        <v>21.35000038146973</v>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K561" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L561" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M561" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N561" t="n">
+        <v>28.27</v>
+      </c>
+      <c r="O561" t="inlineStr">
+        <is>
+          <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-02-05)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O561"/>
+  <dimension ref="A1:O581"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36084,6 +36084,1266 @@
       <c r="O561" t="inlineStr">
         <is>
           <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E562" t="n">
+        <v>1456.8</v>
+      </c>
+      <c r="F562" t="n">
+        <v>1484.31</v>
+      </c>
+      <c r="G562" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="H562" t="n">
+        <v>1312.599975585938</v>
+      </c>
+      <c r="I562" t="n">
+        <v>-9.899999618530273</v>
+      </c>
+      <c r="J562" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K562" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L562" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M562" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N562" t="n">
+        <v>65.83</v>
+      </c>
+      <c r="O562" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E563" t="n">
+        <v>2999.1</v>
+      </c>
+      <c r="F563" t="n">
+        <v>2951.02</v>
+      </c>
+      <c r="G563" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="H563" t="n">
+        <v>3356.340087890625</v>
+      </c>
+      <c r="I563" t="n">
+        <v>11.90999984741211</v>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K563" t="n">
+        <v>0.421</v>
+      </c>
+      <c r="L563" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M563" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N563" t="n">
+        <v>56.02</v>
+      </c>
+      <c r="O563" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E564" t="n">
+        <v>1535.8</v>
+      </c>
+      <c r="F564" t="n">
+        <v>1527.4</v>
+      </c>
+      <c r="G564" t="n">
+        <v>-0.55</v>
+      </c>
+      <c r="H564" t="n">
+        <v>1587.949951171875</v>
+      </c>
+      <c r="I564" t="n">
+        <v>3.400000095367432</v>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K564" t="n">
+        <v>0.8129999999999999</v>
+      </c>
+      <c r="L564" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M564" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N564" t="n">
+        <v>65.44</v>
+      </c>
+      <c r="O564" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E565" t="n">
+        <v>953.1</v>
+      </c>
+      <c r="F565" t="n">
+        <v>918.79</v>
+      </c>
+      <c r="G565" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="H565" t="n">
+        <v>963.0800170898438</v>
+      </c>
+      <c r="I565" t="n">
+        <v>1.049999952316284</v>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K565" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="L565" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M565" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N565" t="n">
+        <v>61.56</v>
+      </c>
+      <c r="O565" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E566" t="n">
+        <v>1408.4</v>
+      </c>
+      <c r="F566" t="n">
+        <v>1366.31</v>
+      </c>
+      <c r="G566" t="n">
+        <v>-2.99</v>
+      </c>
+      <c r="H566" t="n">
+        <v>1349.93994140625</v>
+      </c>
+      <c r="I566" t="n">
+        <v>-4.150000095367432</v>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K566" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="L566" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M566" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N566" t="n">
+        <v>62.48</v>
+      </c>
+      <c r="O566" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E567" t="n">
+        <v>1068.2</v>
+      </c>
+      <c r="F567" t="n">
+        <v>1097.77</v>
+      </c>
+      <c r="G567" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="H567" t="n">
+        <v>939.1400146484375</v>
+      </c>
+      <c r="I567" t="n">
+        <v>-12.07999992370605</v>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K567" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L567" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M567" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N567" t="n">
+        <v>67.55</v>
+      </c>
+      <c r="O567" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E568" t="n">
+        <v>2371</v>
+      </c>
+      <c r="F568" t="n">
+        <v>2270.98</v>
+      </c>
+      <c r="G568" t="n">
+        <v>-4.22</v>
+      </c>
+      <c r="H568" t="n">
+        <v>2299.56005859375</v>
+      </c>
+      <c r="I568" t="n">
+        <v>-3.009999990463257</v>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K568" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L568" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M568" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N568" t="n">
+        <v>56.67</v>
+      </c>
+      <c r="O568" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E569" t="n">
+        <v>313.85</v>
+      </c>
+      <c r="F569" t="n">
+        <v>293.65</v>
+      </c>
+      <c r="G569" t="n">
+        <v>-6.43</v>
+      </c>
+      <c r="H569" t="n">
+        <v>342.3299865722656</v>
+      </c>
+      <c r="I569" t="n">
+        <v>9.079999923706055</v>
+      </c>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K569" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L569" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M569" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N569" t="n">
+        <v>51.49</v>
+      </c>
+      <c r="O569" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E570" t="n">
+        <v>4087.1</v>
+      </c>
+      <c r="F570" t="n">
+        <v>3878.21</v>
+      </c>
+      <c r="G570" t="n">
+        <v>-5.11</v>
+      </c>
+      <c r="H570" t="n">
+        <v>4200.97998046875</v>
+      </c>
+      <c r="I570" t="n">
+        <v>2.789999961853027</v>
+      </c>
+      <c r="J570" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K570" t="n">
+        <v>0</v>
+      </c>
+      <c r="L570" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M570" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N570" t="n">
+        <v>42.33</v>
+      </c>
+      <c r="O570" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E571" t="n">
+        <v>963.3</v>
+      </c>
+      <c r="F571" t="n">
+        <v>957.39</v>
+      </c>
+      <c r="G571" t="n">
+        <v>-0.61</v>
+      </c>
+      <c r="H571" t="n">
+        <v>959.6500244140625</v>
+      </c>
+      <c r="I571" t="n">
+        <v>-0.3799999952316284</v>
+      </c>
+      <c r="J571" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K571" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L571" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M571" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N571" t="n">
+        <v>63.08</v>
+      </c>
+      <c r="O571" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E572" t="n">
+        <v>2025.8</v>
+      </c>
+      <c r="F572" t="n">
+        <v>2051.44</v>
+      </c>
+      <c r="G572" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="H572" t="n">
+        <v>2137.56005859375</v>
+      </c>
+      <c r="I572" t="n">
+        <v>5.519999980926514</v>
+      </c>
+      <c r="J572" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K572" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L572" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M572" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N572" t="n">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="O572" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E573" t="n">
+        <v>2452.7</v>
+      </c>
+      <c r="F573" t="n">
+        <v>2553.28</v>
+      </c>
+      <c r="G573" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H573" t="n">
+        <v>2437</v>
+      </c>
+      <c r="I573" t="n">
+        <v>-0.6399999856948853</v>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K573" t="n">
+        <v>-0.511</v>
+      </c>
+      <c r="L573" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M573" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N573" t="n">
+        <v>45.93</v>
+      </c>
+      <c r="O573" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E574" t="n">
+        <v>1338.7</v>
+      </c>
+      <c r="F574" t="n">
+        <v>1282.5</v>
+      </c>
+      <c r="G574" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="H574" t="n">
+        <v>1134.5400390625</v>
+      </c>
+      <c r="I574" t="n">
+        <v>-15.25</v>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K574" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L574" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M574" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N574" t="n">
+        <v>59.26</v>
+      </c>
+      <c r="O574" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E575" t="n">
+        <v>15071</v>
+      </c>
+      <c r="F575" t="n">
+        <v>16957.9</v>
+      </c>
+      <c r="G575" t="n">
+        <v>12.52</v>
+      </c>
+      <c r="H575" t="n">
+        <v>16630.640625</v>
+      </c>
+      <c r="I575" t="n">
+        <v>10.35000038146973</v>
+      </c>
+      <c r="J575" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K575" t="n">
+        <v>-0.637</v>
+      </c>
+      <c r="L575" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M575" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N575" t="n">
+        <v>56.04</v>
+      </c>
+      <c r="O575" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E576" t="n">
+        <v>1693.4</v>
+      </c>
+      <c r="F576" t="n">
+        <v>1651.44</v>
+      </c>
+      <c r="G576" t="n">
+        <v>-2.48</v>
+      </c>
+      <c r="H576" t="n">
+        <v>1643.359985351562</v>
+      </c>
+      <c r="I576" t="n">
+        <v>-2.960000038146973</v>
+      </c>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K576" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L576" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M576" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N576" t="n">
+        <v>58.78</v>
+      </c>
+      <c r="O576" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E577" t="n">
+        <v>233.34</v>
+      </c>
+      <c r="F577" t="n">
+        <v>235.76</v>
+      </c>
+      <c r="G577" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="H577" t="n">
+        <v>234.0599975585938</v>
+      </c>
+      <c r="I577" t="n">
+        <v>0.3100000023841858</v>
+      </c>
+      <c r="J577" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K577" t="n">
+        <v>-0.8070000000000001</v>
+      </c>
+      <c r="L577" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M577" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N577" t="n">
+        <v>35.41</v>
+      </c>
+      <c r="O577" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E578" t="n">
+        <v>12806</v>
+      </c>
+      <c r="F578" t="n">
+        <v>11673.79</v>
+      </c>
+      <c r="G578" t="n">
+        <v>-8.84</v>
+      </c>
+      <c r="H578" t="n">
+        <v>11261.1103515625</v>
+      </c>
+      <c r="I578" t="n">
+        <v>-12.0600004196167</v>
+      </c>
+      <c r="J578" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K578" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="L578" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M578" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N578" t="n">
+        <v>44.78</v>
+      </c>
+      <c r="O578" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E579" t="n">
+        <v>367.25</v>
+      </c>
+      <c r="F579" t="n">
+        <v>347.04</v>
+      </c>
+      <c r="G579" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="H579" t="n">
+        <v>348.6499938964844</v>
+      </c>
+      <c r="I579" t="n">
+        <v>-5.059999942779541</v>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K579" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L579" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M579" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N579" t="n">
+        <v>51.63</v>
+      </c>
+      <c r="O579" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E580" t="n">
+        <v>289.4</v>
+      </c>
+      <c r="F580" t="n">
+        <v>259.29</v>
+      </c>
+      <c r="G580" t="n">
+        <v>-10.41</v>
+      </c>
+      <c r="H580" t="n">
+        <v>298.4500122070312</v>
+      </c>
+      <c r="I580" t="n">
+        <v>3.130000114440918</v>
+      </c>
+      <c r="J580" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K580" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L580" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M580" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N580" t="n">
+        <v>44.27</v>
+      </c>
+      <c r="O580" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E581" t="n">
+        <v>4144</v>
+      </c>
+      <c r="F581" t="n">
+        <v>3982.55</v>
+      </c>
+      <c r="G581" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="H581" t="n">
+        <v>3672.699951171875</v>
+      </c>
+      <c r="I581" t="n">
+        <v>-11.36999988555908</v>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K581" t="n">
+        <v>0.8179999999999999</v>
+      </c>
+      <c r="L581" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M581" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N581" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="O581" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
         </is>
       </c>
     </row>
@@ -36098,7 +37358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O281"/>
+  <dimension ref="A1:O291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53955,6 +55215,636 @@
       <c r="O281" t="inlineStr">
         <is>
           <t>04 Feb 2026, 07:14:00 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E282" t="n">
+        <v>1456.6</v>
+      </c>
+      <c r="F282" t="n">
+        <v>1488.05</v>
+      </c>
+      <c r="G282" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="H282" t="n">
+        <v>1358.219970703125</v>
+      </c>
+      <c r="I282" t="n">
+        <v>-6.75</v>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K282" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N282" t="n">
+        <v>66.23999999999999</v>
+      </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E283" t="n">
+        <v>2999.8</v>
+      </c>
+      <c r="F283" t="n">
+        <v>2993.05</v>
+      </c>
+      <c r="G283" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="H283" t="n">
+        <v>3245.030029296875</v>
+      </c>
+      <c r="I283" t="n">
+        <v>8.170000076293945</v>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K283" t="n">
+        <v>-0.511</v>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N283" t="n">
+        <v>39.44</v>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E284" t="n">
+        <v>1535.9</v>
+      </c>
+      <c r="F284" t="n">
+        <v>1536.8</v>
+      </c>
+      <c r="G284" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H284" t="n">
+        <v>1653.680053710938</v>
+      </c>
+      <c r="I284" t="n">
+        <v>7.670000076293945</v>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K284" t="n">
+        <v>0.8129999999999999</v>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N284" t="n">
+        <v>66.34999999999999</v>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E285" t="n">
+        <v>953.45</v>
+      </c>
+      <c r="F285" t="n">
+        <v>920.9400000000001</v>
+      </c>
+      <c r="G285" t="n">
+        <v>-3.41</v>
+      </c>
+      <c r="H285" t="n">
+        <v>997.739990234375</v>
+      </c>
+      <c r="I285" t="n">
+        <v>4.639999866485596</v>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K285" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N285" t="n">
+        <v>61.85</v>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E286" t="n">
+        <v>1408.7</v>
+      </c>
+      <c r="F286" t="n">
+        <v>1364.46</v>
+      </c>
+      <c r="G286" t="n">
+        <v>-3.14</v>
+      </c>
+      <c r="H286" t="n">
+        <v>1279.800048828125</v>
+      </c>
+      <c r="I286" t="n">
+        <v>-9.149999618530273</v>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K286" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N286" t="n">
+        <v>54.47</v>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E287" t="n">
+        <v>1068.1</v>
+      </c>
+      <c r="F287" t="n">
+        <v>1107.08</v>
+      </c>
+      <c r="G287" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="H287" t="n">
+        <v>1135.079956054688</v>
+      </c>
+      <c r="I287" t="n">
+        <v>6.269999980926514</v>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K287" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N287" t="n">
+        <v>68.87</v>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E288" t="n">
+        <v>313.85</v>
+      </c>
+      <c r="F288" t="n">
+        <v>306.92</v>
+      </c>
+      <c r="G288" t="n">
+        <v>-2.21</v>
+      </c>
+      <c r="H288" t="n">
+        <v>337.8399963378906</v>
+      </c>
+      <c r="I288" t="n">
+        <v>7.639999866485596</v>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K288" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N288" t="n">
+        <v>57.83</v>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E289" t="n">
+        <v>4086.5</v>
+      </c>
+      <c r="F289" t="n">
+        <v>3888.94</v>
+      </c>
+      <c r="G289" t="n">
+        <v>-4.83</v>
+      </c>
+      <c r="H289" t="n">
+        <v>3825.199951171875</v>
+      </c>
+      <c r="I289" t="n">
+        <v>-6.389999866485596</v>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K289" t="n">
+        <v>0</v>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N289" t="n">
+        <v>42.75</v>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E290" t="n">
+        <v>1338.35</v>
+      </c>
+      <c r="F290" t="n">
+        <v>1280.72</v>
+      </c>
+      <c r="G290" t="n">
+        <v>-4.31</v>
+      </c>
+      <c r="H290" t="n">
+        <v>1118.609985351562</v>
+      </c>
+      <c r="I290" t="n">
+        <v>-16.42000007629395</v>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K290" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N290" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E291" t="n">
+        <v>15077.5</v>
+      </c>
+      <c r="F291" t="n">
+        <v>17069.19</v>
+      </c>
+      <c r="G291" t="n">
+        <v>13.21</v>
+      </c>
+      <c r="H291" t="n">
+        <v>15431.98046875</v>
+      </c>
+      <c r="I291" t="n">
+        <v>2.349999904632568</v>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K291" t="n">
+        <v>-0.637</v>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N291" t="n">
+        <v>57.07</v>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
         </is>
       </c>
     </row>
@@ -53969,7 +55859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O561"/>
+  <dimension ref="A1:O581"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -89609,6 +91499,1266 @@
         </is>
       </c>
     </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E562" t="n">
+        <v>276.49</v>
+      </c>
+      <c r="F562" t="n">
+        <v>258.58</v>
+      </c>
+      <c r="G562" t="n">
+        <v>-6.48</v>
+      </c>
+      <c r="H562" t="n">
+        <v>253.6300048828125</v>
+      </c>
+      <c r="I562" t="n">
+        <v>-8.270000457763672</v>
+      </c>
+      <c r="J562" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K562" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L562" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M562" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N562" t="n">
+        <v>46.21</v>
+      </c>
+      <c r="O562" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E563" t="n">
+        <v>414.19</v>
+      </c>
+      <c r="F563" t="n">
+        <v>423.28</v>
+      </c>
+      <c r="G563" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H563" t="n">
+        <v>418.8399963378906</v>
+      </c>
+      <c r="I563" t="n">
+        <v>1.120000004768372</v>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K563" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L563" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M563" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N563" t="n">
+        <v>40.29</v>
+      </c>
+      <c r="O563" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E564" t="n">
+        <v>333.04</v>
+      </c>
+      <c r="F564" t="n">
+        <v>347.75</v>
+      </c>
+      <c r="G564" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="H564" t="n">
+        <v>368.8099975585938</v>
+      </c>
+      <c r="I564" t="n">
+        <v>10.73999977111816</v>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K564" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="L564" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M564" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N564" t="n">
+        <v>68.34999999999999</v>
+      </c>
+      <c r="O564" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E565" t="n">
+        <v>232.99</v>
+      </c>
+      <c r="F565" t="n">
+        <v>238.32</v>
+      </c>
+      <c r="G565" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="H565" t="n">
+        <v>201.3600006103516</v>
+      </c>
+      <c r="I565" t="n">
+        <v>-13.57999992370605</v>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K565" t="n">
+        <v>-0.79</v>
+      </c>
+      <c r="L565" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M565" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N565" t="n">
+        <v>37.63</v>
+      </c>
+      <c r="O565" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E566" t="n">
+        <v>668.99</v>
+      </c>
+      <c r="F566" t="n">
+        <v>678</v>
+      </c>
+      <c r="G566" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="H566" t="n">
+        <v>729.2899780273438</v>
+      </c>
+      <c r="I566" t="n">
+        <v>9.010000228881836</v>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K566" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="L566" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M566" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N566" t="n">
+        <v>66.88</v>
+      </c>
+      <c r="O566" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E567" t="n">
+        <v>406.01</v>
+      </c>
+      <c r="F567" t="n">
+        <v>400.32</v>
+      </c>
+      <c r="G567" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="H567" t="n">
+        <v>577.2899780273438</v>
+      </c>
+      <c r="I567" t="n">
+        <v>42.18999862670898</v>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K567" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L567" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M567" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N567" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="O567" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E568" t="n">
+        <v>174.19</v>
+      </c>
+      <c r="F568" t="n">
+        <v>196.97</v>
+      </c>
+      <c r="G568" t="n">
+        <v>13.08</v>
+      </c>
+      <c r="H568" t="n">
+        <v>207.1100006103516</v>
+      </c>
+      <c r="I568" t="n">
+        <v>18.89999961853027</v>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K568" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L568" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M568" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N568" t="n">
+        <v>75.54000000000001</v>
+      </c>
+      <c r="O568" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E569" t="n">
+        <v>317.27</v>
+      </c>
+      <c r="F569" t="n">
+        <v>317.14</v>
+      </c>
+      <c r="G569" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="H569" t="n">
+        <v>355.239990234375</v>
+      </c>
+      <c r="I569" t="n">
+        <v>11.97000026702881</v>
+      </c>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K569" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L569" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M569" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N569" t="n">
+        <v>55.86</v>
+      </c>
+      <c r="O569" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E570" t="n">
+        <v>329.95</v>
+      </c>
+      <c r="F570" t="n">
+        <v>333.64</v>
+      </c>
+      <c r="G570" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="H570" t="n">
+        <v>344.3699951171875</v>
+      </c>
+      <c r="I570" t="n">
+        <v>4.369999885559082</v>
+      </c>
+      <c r="J570" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K570" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L570" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M570" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N570" t="n">
+        <v>64.68000000000001</v>
+      </c>
+      <c r="O570" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E571" t="n">
+        <v>234.47</v>
+      </c>
+      <c r="F571" t="n">
+        <v>240.42</v>
+      </c>
+      <c r="G571" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="H571" t="n">
+        <v>334.25</v>
+      </c>
+      <c r="I571" t="n">
+        <v>42.56000137329102</v>
+      </c>
+      <c r="J571" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K571" t="n">
+        <v>0</v>
+      </c>
+      <c r="L571" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M571" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N571" t="n">
+        <v>53.81</v>
+      </c>
+      <c r="O571" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E572" t="n">
+        <v>128</v>
+      </c>
+      <c r="F572" t="n">
+        <v>118.5</v>
+      </c>
+      <c r="G572" t="n">
+        <v>-7.42</v>
+      </c>
+      <c r="H572" t="n">
+        <v>104.7099990844727</v>
+      </c>
+      <c r="I572" t="n">
+        <v>-18.20000076293945</v>
+      </c>
+      <c r="J572" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K572" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="L572" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M572" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N572" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="O572" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E573" t="n">
+        <v>156.87</v>
+      </c>
+      <c r="F573" t="n">
+        <v>148.89</v>
+      </c>
+      <c r="G573" t="n">
+        <v>-5.08</v>
+      </c>
+      <c r="H573" t="n">
+        <v>152.6499938964844</v>
+      </c>
+      <c r="I573" t="n">
+        <v>-2.690000057220459</v>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K573" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L573" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M573" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N573" t="n">
+        <v>55.37</v>
+      </c>
+      <c r="O573" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E574" t="n">
+        <v>553.52</v>
+      </c>
+      <c r="F574" t="n">
+        <v>542.65</v>
+      </c>
+      <c r="G574" t="n">
+        <v>-1.96</v>
+      </c>
+      <c r="H574" t="n">
+        <v>624.8499755859375</v>
+      </c>
+      <c r="I574" t="n">
+        <v>12.89000034332275</v>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K574" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L574" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M574" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N574" t="n">
+        <v>56.94</v>
+      </c>
+      <c r="O574" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E575" t="n">
+        <v>275.92</v>
+      </c>
+      <c r="F575" t="n">
+        <v>280.14</v>
+      </c>
+      <c r="G575" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="H575" t="n">
+        <v>297.1600036621094</v>
+      </c>
+      <c r="I575" t="n">
+        <v>7.699999809265137</v>
+      </c>
+      <c r="J575" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K575" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L575" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M575" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N575" t="n">
+        <v>58.22</v>
+      </c>
+      <c r="O575" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E576" t="n">
+        <v>387.2</v>
+      </c>
+      <c r="F576" t="n">
+        <v>338.91</v>
+      </c>
+      <c r="G576" t="n">
+        <v>-12.47</v>
+      </c>
+      <c r="H576" t="n">
+        <v>383.7099914550781</v>
+      </c>
+      <c r="I576" t="n">
+        <v>-0.8999999761581421</v>
+      </c>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K576" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="L576" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M576" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N576" t="n">
+        <v>33.59</v>
+      </c>
+      <c r="O576" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E577" t="n">
+        <v>55.38</v>
+      </c>
+      <c r="F577" t="n">
+        <v>53.43</v>
+      </c>
+      <c r="G577" t="n">
+        <v>-3.52</v>
+      </c>
+      <c r="H577" t="n">
+        <v>52.20999908447266</v>
+      </c>
+      <c r="I577" t="n">
+        <v>-5.71999979019165</v>
+      </c>
+      <c r="J577" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K577" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L577" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M577" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N577" t="n">
+        <v>57.72</v>
+      </c>
+      <c r="O577" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E578" t="n">
+        <v>147.59</v>
+      </c>
+      <c r="F578" t="n">
+        <v>138.35</v>
+      </c>
+      <c r="G578" t="n">
+        <v>-6.26</v>
+      </c>
+      <c r="H578" t="n">
+        <v>341.4200134277344</v>
+      </c>
+      <c r="I578" t="n">
+        <v>131.3300018310547</v>
+      </c>
+      <c r="J578" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K578" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="L578" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M578" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N578" t="n">
+        <v>51.15</v>
+      </c>
+      <c r="O578" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E579" t="n">
+        <v>308.05</v>
+      </c>
+      <c r="F579" t="n">
+        <v>358.19</v>
+      </c>
+      <c r="G579" t="n">
+        <v>16.28</v>
+      </c>
+      <c r="H579" t="n">
+        <v>384.2200012207031</v>
+      </c>
+      <c r="I579" t="n">
+        <v>24.72999954223633</v>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K579" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="L579" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M579" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N579" t="n">
+        <v>83.95999999999999</v>
+      </c>
+      <c r="O579" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E580" t="n">
+        <v>978.35</v>
+      </c>
+      <c r="F580" t="n">
+        <v>921.9400000000001</v>
+      </c>
+      <c r="G580" t="n">
+        <v>-5.77</v>
+      </c>
+      <c r="H580" t="n">
+        <v>909.1699829101562</v>
+      </c>
+      <c r="I580" t="n">
+        <v>-7.070000171661377</v>
+      </c>
+      <c r="J580" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K580" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L580" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M580" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N580" t="n">
+        <v>54.35</v>
+      </c>
+      <c r="O580" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E581" t="n">
+        <v>166.18</v>
+      </c>
+      <c r="F581" t="n">
+        <v>154.56</v>
+      </c>
+      <c r="G581" t="n">
+        <v>-6.99</v>
+      </c>
+      <c r="H581" t="n">
+        <v>171.7899932861328</v>
+      </c>
+      <c r="I581" t="n">
+        <v>3.380000114440918</v>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K581" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L581" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M581" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N581" t="n">
+        <v>50.95</v>
+      </c>
+      <c r="O581" t="inlineStr">
+        <is>
+          <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-02-06)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O581"/>
+  <dimension ref="A1:O601"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37344,6 +37344,1266 @@
       <c r="O581" t="inlineStr">
         <is>
           <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E582" t="n">
+        <v>1443.4</v>
+      </c>
+      <c r="F582" t="n">
+        <v>1554.77</v>
+      </c>
+      <c r="G582" t="n">
+        <v>7.72</v>
+      </c>
+      <c r="H582" t="n">
+        <v>1521.5400390625</v>
+      </c>
+      <c r="I582" t="n">
+        <v>5.409999847412109</v>
+      </c>
+      <c r="J582" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K582" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L582" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M582" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N582" t="n">
+        <v>74.56999999999999</v>
+      </c>
+      <c r="O582" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E583" t="n">
+        <v>2991.5</v>
+      </c>
+      <c r="F583" t="n">
+        <v>2942.2</v>
+      </c>
+      <c r="G583" t="n">
+        <v>-1.65</v>
+      </c>
+      <c r="H583" t="n">
+        <v>3301.35009765625</v>
+      </c>
+      <c r="I583" t="n">
+        <v>10.35999965667725</v>
+      </c>
+      <c r="J583" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K583" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="L583" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M583" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N583" t="n">
+        <v>50.09</v>
+      </c>
+      <c r="O583" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E584" t="n">
+        <v>1520.2</v>
+      </c>
+      <c r="F584" t="n">
+        <v>1489.8</v>
+      </c>
+      <c r="G584" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H584" t="n">
+        <v>1649.160034179688</v>
+      </c>
+      <c r="I584" t="n">
+        <v>8.479999542236328</v>
+      </c>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K584" t="n">
+        <v>0.8129999999999999</v>
+      </c>
+      <c r="L584" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M584" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N584" t="n">
+        <v>63.26</v>
+      </c>
+      <c r="O584" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E585" t="n">
+        <v>949.7</v>
+      </c>
+      <c r="F585" t="n">
+        <v>915.92</v>
+      </c>
+      <c r="G585" t="n">
+        <v>-3.56</v>
+      </c>
+      <c r="H585" t="n">
+        <v>925</v>
+      </c>
+      <c r="I585" t="n">
+        <v>-2.599999904632568</v>
+      </c>
+      <c r="J585" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K585" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="L585" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M585" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N585" t="n">
+        <v>61.62</v>
+      </c>
+      <c r="O585" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E586" t="n">
+        <v>1396.5</v>
+      </c>
+      <c r="F586" t="n">
+        <v>1381.32</v>
+      </c>
+      <c r="G586" t="n">
+        <v>-1.09</v>
+      </c>
+      <c r="H586" t="n">
+        <v>1478.670043945312</v>
+      </c>
+      <c r="I586" t="n">
+        <v>5.880000114440918</v>
+      </c>
+      <c r="J586" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K586" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L586" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M586" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N586" t="n">
+        <v>55.17</v>
+      </c>
+      <c r="O586" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E587" t="n">
+        <v>1073.5</v>
+      </c>
+      <c r="F587" t="n">
+        <v>1108.53</v>
+      </c>
+      <c r="G587" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="H587" t="n">
+        <v>1190.4599609375</v>
+      </c>
+      <c r="I587" t="n">
+        <v>10.89999961853027</v>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K587" t="n">
+        <v>0.832</v>
+      </c>
+      <c r="L587" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M587" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N587" t="n">
+        <v>71.53</v>
+      </c>
+      <c r="O587" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E588" t="n">
+        <v>2354.4</v>
+      </c>
+      <c r="F588" t="n">
+        <v>2411.54</v>
+      </c>
+      <c r="G588" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="H588" t="n">
+        <v>2336.199951171875</v>
+      </c>
+      <c r="I588" t="n">
+        <v>-0.7699999809265137</v>
+      </c>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K588" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L588" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M588" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N588" t="n">
+        <v>66.64</v>
+      </c>
+      <c r="O588" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E589" t="n">
+        <v>310.2</v>
+      </c>
+      <c r="F589" t="n">
+        <v>322.49</v>
+      </c>
+      <c r="G589" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="H589" t="n">
+        <v>373.1400146484375</v>
+      </c>
+      <c r="I589" t="n">
+        <v>20.29000091552734</v>
+      </c>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K589" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L589" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M589" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N589" t="n">
+        <v>71.5</v>
+      </c>
+      <c r="O589" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E590" t="n">
+        <v>4063.3</v>
+      </c>
+      <c r="F590" t="n">
+        <v>3916.02</v>
+      </c>
+      <c r="G590" t="n">
+        <v>-3.62</v>
+      </c>
+      <c r="H590" t="n">
+        <v>3901.840087890625</v>
+      </c>
+      <c r="I590" t="n">
+        <v>-3.970000028610229</v>
+      </c>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K590" t="n">
+        <v>-0.178</v>
+      </c>
+      <c r="L590" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M590" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N590" t="n">
+        <v>41</v>
+      </c>
+      <c r="O590" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E591" t="n">
+        <v>964.75</v>
+      </c>
+      <c r="F591" t="n">
+        <v>986.13</v>
+      </c>
+      <c r="G591" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="H591" t="n">
+        <v>1053.829956054688</v>
+      </c>
+      <c r="I591" t="n">
+        <v>9.229999542236328</v>
+      </c>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K591" t="n">
+        <v>0.649</v>
+      </c>
+      <c r="L591" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M591" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N591" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="O591" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E592" t="n">
+        <v>1992.4</v>
+      </c>
+      <c r="F592" t="n">
+        <v>2037.01</v>
+      </c>
+      <c r="G592" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="H592" t="n">
+        <v>1865.800048828125</v>
+      </c>
+      <c r="I592" t="n">
+        <v>-6.349999904632568</v>
+      </c>
+      <c r="J592" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K592" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L592" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M592" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N592" t="n">
+        <v>66.36</v>
+      </c>
+      <c r="O592" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E593" t="n">
+        <v>2432.1</v>
+      </c>
+      <c r="F593" t="n">
+        <v>2715.67</v>
+      </c>
+      <c r="G593" t="n">
+        <v>11.66</v>
+      </c>
+      <c r="H593" t="n">
+        <v>2268.8701171875</v>
+      </c>
+      <c r="I593" t="n">
+        <v>-6.710000038146973</v>
+      </c>
+      <c r="J593" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K593" t="n">
+        <v>-0.625</v>
+      </c>
+      <c r="L593" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M593" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N593" t="n">
+        <v>54.99</v>
+      </c>
+      <c r="O593" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E594" t="n">
+        <v>1330.6</v>
+      </c>
+      <c r="F594" t="n">
+        <v>1289.17</v>
+      </c>
+      <c r="G594" t="n">
+        <v>-3.11</v>
+      </c>
+      <c r="H594" t="n">
+        <v>1107.719970703125</v>
+      </c>
+      <c r="I594" t="n">
+        <v>-16.75</v>
+      </c>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K594" t="n">
+        <v>-0.494</v>
+      </c>
+      <c r="L594" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M594" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N594" t="n">
+        <v>35.45</v>
+      </c>
+      <c r="O594" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E595" t="n">
+        <v>15059</v>
+      </c>
+      <c r="F595" t="n">
+        <v>17897.56</v>
+      </c>
+      <c r="G595" t="n">
+        <v>18.85</v>
+      </c>
+      <c r="H595" t="n">
+        <v>17455.140625</v>
+      </c>
+      <c r="I595" t="n">
+        <v>15.90999984741211</v>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K595" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="L595" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M595" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N595" t="n">
+        <v>87.45</v>
+      </c>
+      <c r="O595" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E596" t="n">
+        <v>1702.6</v>
+      </c>
+      <c r="F596" t="n">
+        <v>1621.88</v>
+      </c>
+      <c r="G596" t="n">
+        <v>-4.74</v>
+      </c>
+      <c r="H596" t="n">
+        <v>1737.609985351562</v>
+      </c>
+      <c r="I596" t="n">
+        <v>2.059999942779541</v>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K596" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L596" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M596" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N596" t="n">
+        <v>48.81</v>
+      </c>
+      <c r="O596" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E597" t="n">
+        <v>233.39</v>
+      </c>
+      <c r="F597" t="n">
+        <v>238.69</v>
+      </c>
+      <c r="G597" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="H597" t="n">
+        <v>226.0800018310547</v>
+      </c>
+      <c r="I597" t="n">
+        <v>-3.130000114440918</v>
+      </c>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K597" t="n">
+        <v>-0.8070000000000001</v>
+      </c>
+      <c r="L597" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M597" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N597" t="n">
+        <v>37.26</v>
+      </c>
+      <c r="O597" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E598" t="n">
+        <v>12773</v>
+      </c>
+      <c r="F598" t="n">
+        <v>11540.76</v>
+      </c>
+      <c r="G598" t="n">
+        <v>-9.65</v>
+      </c>
+      <c r="H598" t="n">
+        <v>13657.419921875</v>
+      </c>
+      <c r="I598" t="n">
+        <v>6.920000076293945</v>
+      </c>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K598" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L598" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M598" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N598" t="n">
+        <v>48.73</v>
+      </c>
+      <c r="O598" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E599" t="n">
+        <v>364.25</v>
+      </c>
+      <c r="F599" t="n">
+        <v>345.43</v>
+      </c>
+      <c r="G599" t="n">
+        <v>-5.17</v>
+      </c>
+      <c r="H599" t="n">
+        <v>337.8500061035156</v>
+      </c>
+      <c r="I599" t="n">
+        <v>-7.25</v>
+      </c>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K599" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L599" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M599" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N599" t="n">
+        <v>51.05</v>
+      </c>
+      <c r="O599" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E600" t="n">
+        <v>289.35</v>
+      </c>
+      <c r="F600" t="n">
+        <v>258.46</v>
+      </c>
+      <c r="G600" t="n">
+        <v>-10.68</v>
+      </c>
+      <c r="H600" t="n">
+        <v>322.2200012207031</v>
+      </c>
+      <c r="I600" t="n">
+        <v>11.35999965667725</v>
+      </c>
+      <c r="J600" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K600" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L600" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M600" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N600" t="n">
+        <v>40.34</v>
+      </c>
+      <c r="O600" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E601" t="n">
+        <v>4097.6</v>
+      </c>
+      <c r="F601" t="n">
+        <v>4224.31</v>
+      </c>
+      <c r="G601" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="H601" t="n">
+        <v>3660.4599609375</v>
+      </c>
+      <c r="I601" t="n">
+        <v>-10.67000007629395</v>
+      </c>
+      <c r="J601" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K601" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L601" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M601" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N601" t="n">
+        <v>68.04000000000001</v>
+      </c>
+      <c r="O601" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
         </is>
       </c>
     </row>
@@ -37358,7 +38618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O291"/>
+  <dimension ref="A1:O301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55845,6 +57105,636 @@
       <c r="O291" t="inlineStr">
         <is>
           <t>05 Feb 2026, 07:16:48 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E292" t="n">
+        <v>1443.4</v>
+      </c>
+      <c r="F292" t="n">
+        <v>1524.74</v>
+      </c>
+      <c r="G292" t="n">
+        <v>5.64</v>
+      </c>
+      <c r="H292" t="n">
+        <v>1380</v>
+      </c>
+      <c r="I292" t="n">
+        <v>-4.389999866485596</v>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K292" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N292" t="n">
+        <v>71.45</v>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>2992.05</v>
+      </c>
+      <c r="F293" t="n">
+        <v>2984.31</v>
+      </c>
+      <c r="G293" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="H293" t="n">
+        <v>3119.489990234375</v>
+      </c>
+      <c r="I293" t="n">
+        <v>4.260000228881836</v>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K293" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N293" t="n">
+        <v>53.65</v>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E294" t="n">
+        <v>1519.8</v>
+      </c>
+      <c r="F294" t="n">
+        <v>1487.11</v>
+      </c>
+      <c r="G294" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="H294" t="n">
+        <v>1804.75</v>
+      </c>
+      <c r="I294" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K294" t="n">
+        <v>0.8129999999999999</v>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N294" t="n">
+        <v>63.03</v>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>949.5</v>
+      </c>
+      <c r="F295" t="n">
+        <v>918.1</v>
+      </c>
+      <c r="G295" t="n">
+        <v>-3.31</v>
+      </c>
+      <c r="H295" t="n">
+        <v>936.0399780273438</v>
+      </c>
+      <c r="I295" t="n">
+        <v>-1.419999957084656</v>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K295" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N295" t="n">
+        <v>62</v>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E296" t="n">
+        <v>1396.2</v>
+      </c>
+      <c r="F296" t="n">
+        <v>1374.85</v>
+      </c>
+      <c r="G296" t="n">
+        <v>-1.53</v>
+      </c>
+      <c r="H296" t="n">
+        <v>1378.47998046875</v>
+      </c>
+      <c r="I296" t="n">
+        <v>-1.269999980926514</v>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K296" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N296" t="n">
+        <v>57.93</v>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E297" t="n">
+        <v>1073.4</v>
+      </c>
+      <c r="F297" t="n">
+        <v>1129.82</v>
+      </c>
+      <c r="G297" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="H297" t="n">
+        <v>1205.319946289062</v>
+      </c>
+      <c r="I297" t="n">
+        <v>12.28999996185303</v>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K297" t="n">
+        <v>0.832</v>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N297" t="n">
+        <v>74.52</v>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E298" t="n">
+        <v>310.25</v>
+      </c>
+      <c r="F298" t="n">
+        <v>328.56</v>
+      </c>
+      <c r="G298" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="H298" t="n">
+        <v>355.9400024414062</v>
+      </c>
+      <c r="I298" t="n">
+        <v>14.72999954223633</v>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K298" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N298" t="n">
+        <v>69.39</v>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E299" t="n">
+        <v>4060.2</v>
+      </c>
+      <c r="F299" t="n">
+        <v>3915.52</v>
+      </c>
+      <c r="G299" t="n">
+        <v>-3.56</v>
+      </c>
+      <c r="H299" t="n">
+        <v>4043.9599609375</v>
+      </c>
+      <c r="I299" t="n">
+        <v>-0.4000000059604645</v>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K299" t="n">
+        <v>-0.178</v>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N299" t="n">
+        <v>41.09</v>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E300" t="n">
+        <v>1330.65</v>
+      </c>
+      <c r="F300" t="n">
+        <v>1274.73</v>
+      </c>
+      <c r="G300" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="H300" t="n">
+        <v>1234.380004882812</v>
+      </c>
+      <c r="I300" t="n">
+        <v>-7.230000019073486</v>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K300" t="n">
+        <v>-0.494</v>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N300" t="n">
+        <v>33.82</v>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E301" t="n">
+        <v>15051.2</v>
+      </c>
+      <c r="F301" t="n">
+        <v>18122.78</v>
+      </c>
+      <c r="G301" t="n">
+        <v>20.41</v>
+      </c>
+      <c r="H301" t="n">
+        <v>14909.9599609375</v>
+      </c>
+      <c r="I301" t="n">
+        <v>-0.9399999976158142</v>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K301" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N301" t="n">
+        <v>89.88</v>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
         </is>
       </c>
     </row>
@@ -55859,7 +57749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O581"/>
+  <dimension ref="A1:O601"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -92759,6 +94649,1266 @@
         </is>
       </c>
     </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E582" t="n">
+        <v>275.91</v>
+      </c>
+      <c r="F582" t="n">
+        <v>263.05</v>
+      </c>
+      <c r="G582" t="n">
+        <v>-4.66</v>
+      </c>
+      <c r="H582" t="n">
+        <v>290.239990234375</v>
+      </c>
+      <c r="I582" t="n">
+        <v>5.190000057220459</v>
+      </c>
+      <c r="J582" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K582" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="L582" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M582" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N582" t="n">
+        <v>53.23</v>
+      </c>
+      <c r="O582" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E583" t="n">
+        <v>393.67</v>
+      </c>
+      <c r="F583" t="n">
+        <v>419.52</v>
+      </c>
+      <c r="G583" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="H583" t="n">
+        <v>367.0199890136719</v>
+      </c>
+      <c r="I583" t="n">
+        <v>-6.769999980926514</v>
+      </c>
+      <c r="J583" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K583" t="n">
+        <v>-0.128</v>
+      </c>
+      <c r="L583" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M583" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N583" t="n">
+        <v>57.29</v>
+      </c>
+      <c r="O583" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E584" t="n">
+        <v>331.25</v>
+      </c>
+      <c r="F584" t="n">
+        <v>347.92</v>
+      </c>
+      <c r="G584" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="H584" t="n">
+        <v>319.1000061035156</v>
+      </c>
+      <c r="I584" t="n">
+        <v>-3.670000076293945</v>
+      </c>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K584" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L584" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M584" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N584" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="O584" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E585" t="n">
+        <v>222.69</v>
+      </c>
+      <c r="F585" t="n">
+        <v>234.69</v>
+      </c>
+      <c r="G585" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="H585" t="n">
+        <v>230</v>
+      </c>
+      <c r="I585" t="n">
+        <v>3.279999971389771</v>
+      </c>
+      <c r="J585" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K585" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L585" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M585" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N585" t="n">
+        <v>71.08</v>
+      </c>
+      <c r="O585" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E586" t="n">
+        <v>670.21</v>
+      </c>
+      <c r="F586" t="n">
+        <v>676.11</v>
+      </c>
+      <c r="G586" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="H586" t="n">
+        <v>790.530029296875</v>
+      </c>
+      <c r="I586" t="n">
+        <v>17.95000076293945</v>
+      </c>
+      <c r="J586" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K586" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L586" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M586" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N586" t="n">
+        <v>64.52</v>
+      </c>
+      <c r="O586" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E587" t="n">
+        <v>397.21</v>
+      </c>
+      <c r="F587" t="n">
+        <v>396.6</v>
+      </c>
+      <c r="G587" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="H587" t="n">
+        <v>319.5299987792969</v>
+      </c>
+      <c r="I587" t="n">
+        <v>-19.55999946594238</v>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K587" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L587" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M587" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N587" t="n">
+        <v>55.69</v>
+      </c>
+      <c r="O587" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E588" t="n">
+        <v>171.88</v>
+      </c>
+      <c r="F588" t="n">
+        <v>194.26</v>
+      </c>
+      <c r="G588" t="n">
+        <v>13.02</v>
+      </c>
+      <c r="H588" t="n">
+        <v>169.4900054931641</v>
+      </c>
+      <c r="I588" t="n">
+        <v>-1.389999985694885</v>
+      </c>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K588" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L588" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M588" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N588" t="n">
+        <v>82.53</v>
+      </c>
+      <c r="O588" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E589" t="n">
+        <v>310.16</v>
+      </c>
+      <c r="F589" t="n">
+        <v>316.02</v>
+      </c>
+      <c r="G589" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="H589" t="n">
+        <v>310.5700073242188</v>
+      </c>
+      <c r="I589" t="n">
+        <v>0.1299999952316284</v>
+      </c>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K589" t="n">
+        <v>0</v>
+      </c>
+      <c r="L589" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M589" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N589" t="n">
+        <v>52.83</v>
+      </c>
+      <c r="O589" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E590" t="n">
+        <v>329.13</v>
+      </c>
+      <c r="F590" t="n">
+        <v>331.84</v>
+      </c>
+      <c r="G590" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="H590" t="n">
+        <v>336.8999938964844</v>
+      </c>
+      <c r="I590" t="n">
+        <v>2.359999895095825</v>
+      </c>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K590" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L590" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M590" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N590" t="n">
+        <v>62.68</v>
+      </c>
+      <c r="O590" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E591" t="n">
+        <v>237.79</v>
+      </c>
+      <c r="F591" t="n">
+        <v>242.97</v>
+      </c>
+      <c r="G591" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="H591" t="n">
+        <v>421.3800048828125</v>
+      </c>
+      <c r="I591" t="n">
+        <v>77.20999908447266</v>
+      </c>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K591" t="n">
+        <v>0</v>
+      </c>
+      <c r="L591" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M591" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N591" t="n">
+        <v>53.27</v>
+      </c>
+      <c r="O591" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E592" t="n">
+        <v>126.94</v>
+      </c>
+      <c r="F592" t="n">
+        <v>119.59</v>
+      </c>
+      <c r="G592" t="n">
+        <v>-5.79</v>
+      </c>
+      <c r="H592" t="n">
+        <v>145.1000061035156</v>
+      </c>
+      <c r="I592" t="n">
+        <v>14.30000019073486</v>
+      </c>
+      <c r="J592" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K592" t="n">
+        <v>0</v>
+      </c>
+      <c r="L592" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M592" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N592" t="n">
+        <v>41.31</v>
+      </c>
+      <c r="O592" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E593" t="n">
+        <v>158.61</v>
+      </c>
+      <c r="F593" t="n">
+        <v>149.48</v>
+      </c>
+      <c r="G593" t="n">
+        <v>-5.76</v>
+      </c>
+      <c r="H593" t="n">
+        <v>150.75</v>
+      </c>
+      <c r="I593" t="n">
+        <v>-4.949999809265137</v>
+      </c>
+      <c r="J593" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K593" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L593" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M593" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N593" t="n">
+        <v>54.37</v>
+      </c>
+      <c r="O593" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E594" t="n">
+        <v>551.89</v>
+      </c>
+      <c r="F594" t="n">
+        <v>543.4299999999999</v>
+      </c>
+      <c r="G594" t="n">
+        <v>-1.53</v>
+      </c>
+      <c r="H594" t="n">
+        <v>581.6599731445312</v>
+      </c>
+      <c r="I594" t="n">
+        <v>5.389999866485596</v>
+      </c>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K594" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L594" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M594" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N594" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="O594" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E595" t="n">
+        <v>268.55</v>
+      </c>
+      <c r="F595" t="n">
+        <v>282.8</v>
+      </c>
+      <c r="G595" t="n">
+        <v>5.31</v>
+      </c>
+      <c r="H595" t="n">
+        <v>253.1399993896484</v>
+      </c>
+      <c r="I595" t="n">
+        <v>-5.739999771118164</v>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K595" t="n">
+        <v>0</v>
+      </c>
+      <c r="L595" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M595" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N595" t="n">
+        <v>57.96</v>
+      </c>
+      <c r="O595" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E596" t="n">
+        <v>382.37</v>
+      </c>
+      <c r="F596" t="n">
+        <v>339.44</v>
+      </c>
+      <c r="G596" t="n">
+        <v>-11.23</v>
+      </c>
+      <c r="H596" t="n">
+        <v>398.7900085449219</v>
+      </c>
+      <c r="I596" t="n">
+        <v>4.289999961853027</v>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K596" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="L596" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M596" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N596" t="n">
+        <v>35.46</v>
+      </c>
+      <c r="O596" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E597" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="F597" t="n">
+        <v>53.18</v>
+      </c>
+      <c r="G597" t="n">
+        <v>-3.2</v>
+      </c>
+      <c r="H597" t="n">
+        <v>53.15000152587891</v>
+      </c>
+      <c r="I597" t="n">
+        <v>-3.259999990463257</v>
+      </c>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K597" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L597" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M597" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N597" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="O597" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E598" t="n">
+        <v>146.08</v>
+      </c>
+      <c r="F598" t="n">
+        <v>138.6</v>
+      </c>
+      <c r="G598" t="n">
+        <v>-5.12</v>
+      </c>
+      <c r="H598" t="n">
+        <v>182.7700042724609</v>
+      </c>
+      <c r="I598" t="n">
+        <v>25.1200008392334</v>
+      </c>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K598" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L598" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M598" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N598" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="O598" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E599" t="n">
+        <v>310.51</v>
+      </c>
+      <c r="F599" t="n">
+        <v>363.05</v>
+      </c>
+      <c r="G599" t="n">
+        <v>16.92</v>
+      </c>
+      <c r="H599" t="n">
+        <v>315.4100036621094</v>
+      </c>
+      <c r="I599" t="n">
+        <v>1.580000042915344</v>
+      </c>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K599" t="n">
+        <v>0</v>
+      </c>
+      <c r="L599" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M599" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N599" t="n">
+        <v>75.38</v>
+      </c>
+      <c r="O599" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E600" t="n">
+        <v>989.29</v>
+      </c>
+      <c r="F600" t="n">
+        <v>918.16</v>
+      </c>
+      <c r="G600" t="n">
+        <v>-7.19</v>
+      </c>
+      <c r="H600" t="n">
+        <v>957.0599975585938</v>
+      </c>
+      <c r="I600" t="n">
+        <v>-3.259999990463257</v>
+      </c>
+      <c r="J600" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K600" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="L600" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M600" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N600" t="n">
+        <v>53.41</v>
+      </c>
+      <c r="O600" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E601" t="n">
+        <v>167.53</v>
+      </c>
+      <c r="F601" t="n">
+        <v>155.38</v>
+      </c>
+      <c r="G601" t="n">
+        <v>-7.26</v>
+      </c>
+      <c r="H601" t="n">
+        <v>149.9600067138672</v>
+      </c>
+      <c r="I601" t="n">
+        <v>-10.48999977111816</v>
+      </c>
+      <c r="J601" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K601" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L601" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M601" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N601" t="n">
+        <v>47.92</v>
+      </c>
+      <c r="O601" t="inlineStr">
+        <is>
+          <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily StockIQ Insights update (2026-02-07)
</commit_message>
<xml_diff>
--- a/Daily_StockIQ_Insights.xlsx
+++ b/Daily_StockIQ_Insights.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O601"/>
+  <dimension ref="A1:O621"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38604,6 +38604,1266 @@
       <c r="O601" t="inlineStr">
         <is>
           <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>RELIANCE.NS</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E602" t="n">
+        <v>1450.8</v>
+      </c>
+      <c r="F602" t="n">
+        <v>1504.57</v>
+      </c>
+      <c r="G602" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="H602" t="n">
+        <v>1389.660034179688</v>
+      </c>
+      <c r="I602" t="n">
+        <v>-4.210000038146973</v>
+      </c>
+      <c r="J602" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K602" t="n">
+        <v>0.577</v>
+      </c>
+      <c r="L602" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M602" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N602" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="O602" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>TCS.NS</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E603" t="n">
+        <v>2941.6</v>
+      </c>
+      <c r="F603" t="n">
+        <v>2922.15</v>
+      </c>
+      <c r="G603" t="n">
+        <v>-0.66</v>
+      </c>
+      <c r="H603" t="n">
+        <v>2951.35009765625</v>
+      </c>
+      <c r="I603" t="n">
+        <v>0.3300000131130219</v>
+      </c>
+      <c r="J603" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K603" t="n">
+        <v>0.421</v>
+      </c>
+      <c r="L603" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M603" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N603" t="n">
+        <v>57.43</v>
+      </c>
+      <c r="O603" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>INFY.NS</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E604" t="n">
+        <v>1507.1</v>
+      </c>
+      <c r="F604" t="n">
+        <v>1522.02</v>
+      </c>
+      <c r="G604" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H604" t="n">
+        <v>1611.280029296875</v>
+      </c>
+      <c r="I604" t="n">
+        <v>6.909999847412109</v>
+      </c>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K604" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L604" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M604" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N604" t="n">
+        <v>64.48999999999999</v>
+      </c>
+      <c r="O604" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>HDFCBANK.NS</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E605" t="n">
+        <v>941.1</v>
+      </c>
+      <c r="F605" t="n">
+        <v>917.45</v>
+      </c>
+      <c r="G605" t="n">
+        <v>-2.51</v>
+      </c>
+      <c r="H605" t="n">
+        <v>1095.699951171875</v>
+      </c>
+      <c r="I605" t="n">
+        <v>16.43000030517578</v>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K605" t="n">
+        <v>0.421</v>
+      </c>
+      <c r="L605" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M605" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N605" t="n">
+        <v>54.65</v>
+      </c>
+      <c r="O605" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>ICICIBANK.NS</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E606" t="n">
+        <v>1406.1</v>
+      </c>
+      <c r="F606" t="n">
+        <v>1374.59</v>
+      </c>
+      <c r="G606" t="n">
+        <v>-2.24</v>
+      </c>
+      <c r="H606" t="n">
+        <v>1447.329956054688</v>
+      </c>
+      <c r="I606" t="n">
+        <v>2.930000066757202</v>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K606" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L606" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M606" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N606" t="n">
+        <v>53.44</v>
+      </c>
+      <c r="O606" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>SBIN.NS</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E607" t="n">
+        <v>1066.4</v>
+      </c>
+      <c r="F607" t="n">
+        <v>1104.79</v>
+      </c>
+      <c r="G607" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H607" t="n">
+        <v>1198.650024414062</v>
+      </c>
+      <c r="I607" t="n">
+        <v>12.39999961853027</v>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K607" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="L607" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M607" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N607" t="n">
+        <v>72.28</v>
+      </c>
+      <c r="O607" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>HINDUNILVR.NS</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Limited</t>
+        </is>
+      </c>
+      <c r="E608" t="n">
+        <v>2424.2</v>
+      </c>
+      <c r="F608" t="n">
+        <v>2289.41</v>
+      </c>
+      <c r="G608" t="n">
+        <v>-5.56</v>
+      </c>
+      <c r="H608" t="n">
+        <v>2323.030029296875</v>
+      </c>
+      <c r="I608" t="n">
+        <v>-4.170000076293945</v>
+      </c>
+      <c r="J608" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K608" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L608" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M608" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N608" t="n">
+        <v>28.66</v>
+      </c>
+      <c r="O608" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>ITC.NS</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E609" t="n">
+        <v>325.8</v>
+      </c>
+      <c r="F609" t="n">
+        <v>295.31</v>
+      </c>
+      <c r="G609" t="n">
+        <v>-9.359999999999999</v>
+      </c>
+      <c r="H609" t="n">
+        <v>355.4599914550781</v>
+      </c>
+      <c r="I609" t="n">
+        <v>9.100000381469727</v>
+      </c>
+      <c r="J609" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K609" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L609" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M609" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N609" t="n">
+        <v>51.52</v>
+      </c>
+      <c r="O609" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>LT.NS</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E610" t="n">
+        <v>4068.1</v>
+      </c>
+      <c r="F610" t="n">
+        <v>3907.26</v>
+      </c>
+      <c r="G610" t="n">
+        <v>-3.95</v>
+      </c>
+      <c r="H610" t="n">
+        <v>3787.39990234375</v>
+      </c>
+      <c r="I610" t="n">
+        <v>-6.900000095367432</v>
+      </c>
+      <c r="J610" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K610" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L610" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M610" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N610" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="O610" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>BAJFINANCE.NS</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Limited</t>
+        </is>
+      </c>
+      <c r="E611" t="n">
+        <v>981.7</v>
+      </c>
+      <c r="F611" t="n">
+        <v>964.87</v>
+      </c>
+      <c r="G611" t="n">
+        <v>-1.71</v>
+      </c>
+      <c r="H611" t="n">
+        <v>881.47998046875</v>
+      </c>
+      <c r="I611" t="n">
+        <v>-10.21000003814697</v>
+      </c>
+      <c r="J611" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K611" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L611" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M611" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N611" t="n">
+        <v>60.43</v>
+      </c>
+      <c r="O611" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>BHARTIARTL.NS</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Limited</t>
+        </is>
+      </c>
+      <c r="E612" t="n">
+        <v>2038.4</v>
+      </c>
+      <c r="F612" t="n">
+        <v>2050.73</v>
+      </c>
+      <c r="G612" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H612" t="n">
+        <v>2093.06005859375</v>
+      </c>
+      <c r="I612" t="n">
+        <v>2.680000066757202</v>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K612" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L612" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M612" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N612" t="n">
+        <v>63.91</v>
+      </c>
+      <c r="O612" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>ASIANPAINT.NS</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Asian Paints Limited</t>
+        </is>
+      </c>
+      <c r="E613" t="n">
+        <v>2401.1</v>
+      </c>
+      <c r="F613" t="n">
+        <v>2604.34</v>
+      </c>
+      <c r="G613" t="n">
+        <v>8.460000000000001</v>
+      </c>
+      <c r="H613" t="n">
+        <v>2267.75</v>
+      </c>
+      <c r="I613" t="n">
+        <v>-5.550000190734863</v>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K613" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L613" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M613" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N613" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="O613" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>AXISBANK.NS</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E614" t="n">
+        <v>1341.6</v>
+      </c>
+      <c r="F614" t="n">
+        <v>1293.63</v>
+      </c>
+      <c r="G614" t="n">
+        <v>-3.58</v>
+      </c>
+      <c r="H614" t="n">
+        <v>1168.199951171875</v>
+      </c>
+      <c r="I614" t="n">
+        <v>-12.92000007629395</v>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K614" t="n">
+        <v>-0.494</v>
+      </c>
+      <c r="L614" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M614" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N614" t="n">
+        <v>34.76</v>
+      </c>
+      <c r="O614" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>MARUTI.NS</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E615" t="n">
+        <v>14997</v>
+      </c>
+      <c r="F615" t="n">
+        <v>16847.04</v>
+      </c>
+      <c r="G615" t="n">
+        <v>12.34</v>
+      </c>
+      <c r="H615" t="n">
+        <v>16271.4501953125</v>
+      </c>
+      <c r="I615" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="J615" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K615" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L615" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M615" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N615" t="n">
+        <v>81.5</v>
+      </c>
+      <c r="O615" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>SUNPHARMA.NS</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceutical Industries Limited</t>
+        </is>
+      </c>
+      <c r="E616" t="n">
+        <v>1695.1</v>
+      </c>
+      <c r="F616" t="n">
+        <v>1646.87</v>
+      </c>
+      <c r="G616" t="n">
+        <v>-2.84</v>
+      </c>
+      <c r="H616" t="n">
+        <v>1946.72998046875</v>
+      </c>
+      <c r="I616" t="n">
+        <v>14.84000015258789</v>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K616" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L616" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M616" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N616" t="n">
+        <v>51.65</v>
+      </c>
+      <c r="O616" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>WIPRO.NS</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Wipro Limited</t>
+        </is>
+      </c>
+      <c r="E617" t="n">
+        <v>230.72</v>
+      </c>
+      <c r="F617" t="n">
+        <v>234.7</v>
+      </c>
+      <c r="G617" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="H617" t="n">
+        <v>217.6499938964844</v>
+      </c>
+      <c r="I617" t="n">
+        <v>-5.670000076293945</v>
+      </c>
+      <c r="J617" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K617" t="n">
+        <v>0.802</v>
+      </c>
+      <c r="L617" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M617" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N617" t="n">
+        <v>68.63</v>
+      </c>
+      <c r="O617" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO.NS</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Limited</t>
+        </is>
+      </c>
+      <c r="E618" t="n">
+        <v>12722</v>
+      </c>
+      <c r="F618" t="n">
+        <v>11691.66</v>
+      </c>
+      <c r="G618" t="n">
+        <v>-8.1</v>
+      </c>
+      <c r="H618" t="n">
+        <v>12033.2001953125</v>
+      </c>
+      <c r="I618" t="n">
+        <v>-5.409999847412109</v>
+      </c>
+      <c r="J618" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K618" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="L618" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M618" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N618" t="n">
+        <v>51.05</v>
+      </c>
+      <c r="O618" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>NTPC.NS</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>NTPC Limited</t>
+        </is>
+      </c>
+      <c r="E619" t="n">
+        <v>365.05</v>
+      </c>
+      <c r="F619" t="n">
+        <v>347.76</v>
+      </c>
+      <c r="G619" t="n">
+        <v>-4.74</v>
+      </c>
+      <c r="H619" t="n">
+        <v>440.8399963378906</v>
+      </c>
+      <c r="I619" t="n">
+        <v>20.76000022888184</v>
+      </c>
+      <c r="J619" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K619" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L619" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M619" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N619" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="O619" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>POWERGRID.NS</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Limited</t>
+        </is>
+      </c>
+      <c r="E620" t="n">
+        <v>292.75</v>
+      </c>
+      <c r="F620" t="n">
+        <v>261.68</v>
+      </c>
+      <c r="G620" t="n">
+        <v>-10.61</v>
+      </c>
+      <c r="H620" t="n">
+        <v>305.1300048828125</v>
+      </c>
+      <c r="I620" t="n">
+        <v>4.230000019073486</v>
+      </c>
+      <c r="J620" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K620" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="L620" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M620" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N620" t="n">
+        <v>40.44</v>
+      </c>
+      <c r="O620" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>TITAN.NS</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>Titan Company Limited</t>
+        </is>
+      </c>
+      <c r="E621" t="n">
+        <v>4141</v>
+      </c>
+      <c r="F621" t="n">
+        <v>4054.38</v>
+      </c>
+      <c r="G621" t="n">
+        <v>-2.09</v>
+      </c>
+      <c r="H621" t="n">
+        <v>3952.320068359375</v>
+      </c>
+      <c r="I621" t="n">
+        <v>-4.559999942779541</v>
+      </c>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K621" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L621" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M621" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N621" t="n">
+        <v>59.86</v>
+      </c>
+      <c r="O621" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
         </is>
       </c>
     </row>
@@ -38618,7 +39878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O301"/>
+  <dimension ref="A1:O311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57735,6 +58995,636 @@
       <c r="O301" t="inlineStr">
         <is>
           <t>06 Feb 2026, 07:12:21 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>RELIANCE.BO</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Reliance Industries Limited</t>
+        </is>
+      </c>
+      <c r="E302" t="n">
+        <v>1450.85</v>
+      </c>
+      <c r="F302" t="n">
+        <v>1491.54</v>
+      </c>
+      <c r="G302" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H302" t="n">
+        <v>1328.180053710938</v>
+      </c>
+      <c r="I302" t="n">
+        <v>-8.460000038146973</v>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K302" t="n">
+        <v>0.577</v>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N302" t="n">
+        <v>65.75</v>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>TCS.BO</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Limited</t>
+        </is>
+      </c>
+      <c r="E303" t="n">
+        <v>2941.45</v>
+      </c>
+      <c r="F303" t="n">
+        <v>2955.59</v>
+      </c>
+      <c r="G303" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="H303" t="n">
+        <v>3050.7900390625</v>
+      </c>
+      <c r="I303" t="n">
+        <v>3.720000028610229</v>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K303" t="n">
+        <v>0.421</v>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N303" t="n">
+        <v>59.14</v>
+      </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>INFY.BO</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Infosys Limited</t>
+        </is>
+      </c>
+      <c r="E304" t="n">
+        <v>1506.9</v>
+      </c>
+      <c r="F304" t="n">
+        <v>1518.96</v>
+      </c>
+      <c r="G304" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H304" t="n">
+        <v>1722.599975585938</v>
+      </c>
+      <c r="I304" t="n">
+        <v>14.3100004196167</v>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K304" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N304" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>HDFCBANK.BO</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>HDFC Bank Limited</t>
+        </is>
+      </c>
+      <c r="E305" t="n">
+        <v>941.15</v>
+      </c>
+      <c r="F305" t="n">
+        <v>919.74</v>
+      </c>
+      <c r="G305" t="n">
+        <v>-2.27</v>
+      </c>
+      <c r="H305" t="n">
+        <v>886.1400146484375</v>
+      </c>
+      <c r="I305" t="n">
+        <v>-5.849999904632568</v>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K305" t="n">
+        <v>0.421</v>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N305" t="n">
+        <v>55.01</v>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>ICICIBANK.BO</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>ICICI Bank Limited</t>
+        </is>
+      </c>
+      <c r="E306" t="n">
+        <v>1406.65</v>
+      </c>
+      <c r="F306" t="n">
+        <v>1373.07</v>
+      </c>
+      <c r="G306" t="n">
+        <v>-2.39</v>
+      </c>
+      <c r="H306" t="n">
+        <v>1453.02001953125</v>
+      </c>
+      <c r="I306" t="n">
+        <v>3.299999952316284</v>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K306" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N306" t="n">
+        <v>53.22</v>
+      </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>SBIN.BO</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="E307" t="n">
+        <v>1066.4</v>
+      </c>
+      <c r="F307" t="n">
+        <v>1118.16</v>
+      </c>
+      <c r="G307" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="H307" t="n">
+        <v>1313.849975585938</v>
+      </c>
+      <c r="I307" t="n">
+        <v>23.20000076293945</v>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K307" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N307" t="n">
+        <v>74.16</v>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>ITC.BO</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>ITC Limited</t>
+        </is>
+      </c>
+      <c r="E308" t="n">
+        <v>326.05</v>
+      </c>
+      <c r="F308" t="n">
+        <v>306.19</v>
+      </c>
+      <c r="G308" t="n">
+        <v>-6.09</v>
+      </c>
+      <c r="H308" t="n">
+        <v>344.5</v>
+      </c>
+      <c r="I308" t="n">
+        <v>5.659999847412109</v>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K308" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N308" t="n">
+        <v>56.42</v>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>LT.BO</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Limited</t>
+        </is>
+      </c>
+      <c r="E309" t="n">
+        <v>4067.7</v>
+      </c>
+      <c r="F309" t="n">
+        <v>3916.42</v>
+      </c>
+      <c r="G309" t="n">
+        <v>-3.72</v>
+      </c>
+      <c r="H309" t="n">
+        <v>4119.66015625</v>
+      </c>
+      <c r="I309" t="n">
+        <v>1.279999971389771</v>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K309" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N309" t="n">
+        <v>53.22</v>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>AXISBANK.BO</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Axis Bank Limited</t>
+        </is>
+      </c>
+      <c r="E310" t="n">
+        <v>1341.55</v>
+      </c>
+      <c r="F310" t="n">
+        <v>1293.13</v>
+      </c>
+      <c r="G310" t="n">
+        <v>-3.61</v>
+      </c>
+      <c r="H310" t="n">
+        <v>1338.0400390625</v>
+      </c>
+      <c r="I310" t="n">
+        <v>-0.2599999904632568</v>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K310" t="n">
+        <v>-0.494</v>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N310" t="n">
+        <v>34.71</v>
+      </c>
+      <c r="O310" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>MARUTI.BO</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Limited</t>
+        </is>
+      </c>
+      <c r="E311" t="n">
+        <v>15001.4</v>
+      </c>
+      <c r="F311" t="n">
+        <v>16942.88</v>
+      </c>
+      <c r="G311" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="H311" t="n">
+        <v>14686.990234375</v>
+      </c>
+      <c r="I311" t="n">
+        <v>-2.099999904632568</v>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K311" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N311" t="n">
+        <v>82.41</v>
+      </c>
+      <c r="O311" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
         </is>
       </c>
     </row>
@@ -57749,7 +59639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O601"/>
+  <dimension ref="A1:O621"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -95909,6 +97799,1266 @@
         </is>
       </c>
     </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>Apple Inc.</t>
+        </is>
+      </c>
+      <c r="E602" t="n">
+        <v>278.12</v>
+      </c>
+      <c r="F602" t="n">
+        <v>261.09</v>
+      </c>
+      <c r="G602" t="n">
+        <v>-6.12</v>
+      </c>
+      <c r="H602" t="n">
+        <v>284.9500122070312</v>
+      </c>
+      <c r="I602" t="n">
+        <v>2.460000038146973</v>
+      </c>
+      <c r="J602" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K602" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L602" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M602" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N602" t="n">
+        <v>53.81</v>
+      </c>
+      <c r="O602" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Microsoft Corporation</t>
+        </is>
+      </c>
+      <c r="E603" t="n">
+        <v>401.14</v>
+      </c>
+      <c r="F603" t="n">
+        <v>414.82</v>
+      </c>
+      <c r="G603" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="H603" t="n">
+        <v>418.0400085449219</v>
+      </c>
+      <c r="I603" t="n">
+        <v>4.210000038146973</v>
+      </c>
+      <c r="J603" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K603" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L603" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M603" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N603" t="n">
+        <v>66.55</v>
+      </c>
+      <c r="O603" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>Alphabet Inc.</t>
+        </is>
+      </c>
+      <c r="E604" t="n">
+        <v>322.86</v>
+      </c>
+      <c r="F604" t="n">
+        <v>347.15</v>
+      </c>
+      <c r="G604" t="n">
+        <v>7.52</v>
+      </c>
+      <c r="H604" t="n">
+        <v>400.0599975585938</v>
+      </c>
+      <c r="I604" t="n">
+        <v>23.90999984741211</v>
+      </c>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K604" t="n">
+        <v>-0.696</v>
+      </c>
+      <c r="L604" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M604" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N604" t="n">
+        <v>47.36</v>
+      </c>
+      <c r="O604" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="E605" t="n">
+        <v>210.32</v>
+      </c>
+      <c r="F605" t="n">
+        <v>231.99</v>
+      </c>
+      <c r="G605" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="H605" t="n">
+        <v>235.4799957275391</v>
+      </c>
+      <c r="I605" t="n">
+        <v>11.96000003814697</v>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K605" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L605" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M605" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N605" t="n">
+        <v>78.45</v>
+      </c>
+      <c r="O605" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>Meta Platforms, Inc.</t>
+        </is>
+      </c>
+      <c r="E606" t="n">
+        <v>661.46</v>
+      </c>
+      <c r="F606" t="n">
+        <v>661.8099999999999</v>
+      </c>
+      <c r="G606" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H606" t="n">
+        <v>572.6699829101562</v>
+      </c>
+      <c r="I606" t="n">
+        <v>-13.42000007629395</v>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K606" t="n">
+        <v>-0.782</v>
+      </c>
+      <c r="L606" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M606" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N606" t="n">
+        <v>34.44</v>
+      </c>
+      <c r="O606" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>Tesla, Inc.</t>
+        </is>
+      </c>
+      <c r="E607" t="n">
+        <v>411.11</v>
+      </c>
+      <c r="F607" t="n">
+        <v>391.17</v>
+      </c>
+      <c r="G607" t="n">
+        <v>-4.85</v>
+      </c>
+      <c r="H607" t="n">
+        <v>336.7200012207031</v>
+      </c>
+      <c r="I607" t="n">
+        <v>-18.09000015258789</v>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K607" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="L607" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M607" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N607" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="O607" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="E608" t="n">
+        <v>185.41</v>
+      </c>
+      <c r="F608" t="n">
+        <v>193.57</v>
+      </c>
+      <c r="G608" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H608" t="n">
+        <v>167.0599975585938</v>
+      </c>
+      <c r="I608" t="n">
+        <v>-9.899999618530273</v>
+      </c>
+      <c r="J608" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K608" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L608" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M608" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N608" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="O608" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="E609" t="n">
+        <v>322.4</v>
+      </c>
+      <c r="F609" t="n">
+        <v>314.66</v>
+      </c>
+      <c r="G609" t="n">
+        <v>-2.4</v>
+      </c>
+      <c r="H609" t="n">
+        <v>324.5199890136719</v>
+      </c>
+      <c r="I609" t="n">
+        <v>0.6600000262260437</v>
+      </c>
+      <c r="J609" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K609" t="n">
+        <v>0</v>
+      </c>
+      <c r="L609" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M609" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N609" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="O609" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="E610" t="n">
+        <v>331.58</v>
+      </c>
+      <c r="F610" t="n">
+        <v>330.8</v>
+      </c>
+      <c r="G610" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="H610" t="n">
+        <v>326.25</v>
+      </c>
+      <c r="I610" t="n">
+        <v>-1.610000014305115</v>
+      </c>
+      <c r="J610" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K610" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="L610" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M610" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N610" t="n">
+        <v>61.09</v>
+      </c>
+      <c r="O610" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="E611" t="n">
+        <v>239.99</v>
+      </c>
+      <c r="F611" t="n">
+        <v>243.54</v>
+      </c>
+      <c r="G611" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="H611" t="n">
+        <v>326.3699951171875</v>
+      </c>
+      <c r="I611" t="n">
+        <v>35.9900016784668</v>
+      </c>
+      <c r="J611" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K611" t="n">
+        <v>0</v>
+      </c>
+      <c r="L611" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M611" t="inlineStr">
+        <is>
+          <t>🟢 Buy</t>
+        </is>
+      </c>
+      <c r="N611" t="n">
+        <v>52.22</v>
+      </c>
+      <c r="O611" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="E612" t="n">
+        <v>131.18</v>
+      </c>
+      <c r="F612" t="n">
+        <v>119.91</v>
+      </c>
+      <c r="G612" t="n">
+        <v>-8.59</v>
+      </c>
+      <c r="H612" t="n">
+        <v>111.2799987792969</v>
+      </c>
+      <c r="I612" t="n">
+        <v>-15.17000007629395</v>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K612" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="L612" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M612" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N612" t="n">
+        <v>40.67</v>
+      </c>
+      <c r="O612" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>The Procter &amp; Gamble Company</t>
+        </is>
+      </c>
+      <c r="E613" t="n">
+        <v>159.17</v>
+      </c>
+      <c r="F613" t="n">
+        <v>149.92</v>
+      </c>
+      <c r="G613" t="n">
+        <v>-5.81</v>
+      </c>
+      <c r="H613" t="n">
+        <v>148.3999938964844</v>
+      </c>
+      <c r="I613" t="n">
+        <v>-6.760000228881836</v>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K613" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L613" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M613" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N613" t="n">
+        <v>54.28</v>
+      </c>
+      <c r="O613" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="E614" t="n">
+        <v>548.74</v>
+      </c>
+      <c r="F614" t="n">
+        <v>537.87</v>
+      </c>
+      <c r="G614" t="n">
+        <v>-1.98</v>
+      </c>
+      <c r="H614" t="n">
+        <v>525.4000244140625</v>
+      </c>
+      <c r="I614" t="n">
+        <v>-4.25</v>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K614" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="L614" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M614" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N614" t="n">
+        <v>60.03</v>
+      </c>
+      <c r="O614" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group Incorporated</t>
+        </is>
+      </c>
+      <c r="E615" t="n">
+        <v>276.65</v>
+      </c>
+      <c r="F615" t="n">
+        <v>281.4</v>
+      </c>
+      <c r="G615" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="H615" t="n">
+        <v>270.3099975585938</v>
+      </c>
+      <c r="I615" t="n">
+        <v>-2.289999961853027</v>
+      </c>
+      <c r="J615" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K615" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L615" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M615" t="inlineStr">
+        <is>
+          <t>🚀 Strong Buy</t>
+        </is>
+      </c>
+      <c r="N615" t="n">
+        <v>61.37</v>
+      </c>
+      <c r="O615" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>The Home Depot, Inc.</t>
+        </is>
+      </c>
+      <c r="E616" t="n">
+        <v>385.15</v>
+      </c>
+      <c r="F616" t="n">
+        <v>339.28</v>
+      </c>
+      <c r="G616" t="n">
+        <v>-11.91</v>
+      </c>
+      <c r="H616" t="n">
+        <v>397.6199951171875</v>
+      </c>
+      <c r="I616" t="n">
+        <v>3.240000009536743</v>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K616" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L616" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M616" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N616" t="n">
+        <v>40.93</v>
+      </c>
+      <c r="O616" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Bank of America Corporation</t>
+        </is>
+      </c>
+      <c r="E617" t="n">
+        <v>56.53</v>
+      </c>
+      <c r="F617" t="n">
+        <v>53.11</v>
+      </c>
+      <c r="G617" t="n">
+        <v>-6.05</v>
+      </c>
+      <c r="H617" t="n">
+        <v>54.34000015258789</v>
+      </c>
+      <c r="I617" t="n">
+        <v>-3.869999885559082</v>
+      </c>
+      <c r="J617" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K617" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L617" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M617" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N617" t="n">
+        <v>54.32</v>
+      </c>
+      <c r="O617" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>Exxon Mobil Corporation</t>
+        </is>
+      </c>
+      <c r="E618" t="n">
+        <v>149.05</v>
+      </c>
+      <c r="F618" t="n">
+        <v>139.1</v>
+      </c>
+      <c r="G618" t="n">
+        <v>-6.67</v>
+      </c>
+      <c r="H618" t="n">
+        <v>354.8900146484375</v>
+      </c>
+      <c r="I618" t="n">
+        <v>138.1000061035156</v>
+      </c>
+      <c r="J618" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K618" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="L618" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M618" t="inlineStr">
+        <is>
+          <t>🔻 Avoid</t>
+        </is>
+      </c>
+      <c r="N618" t="n">
+        <v>45.91</v>
+      </c>
+      <c r="O618" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="E619" t="n">
+        <v>332.92</v>
+      </c>
+      <c r="F619" t="n">
+        <v>352.6</v>
+      </c>
+      <c r="G619" t="n">
+        <v>5.91</v>
+      </c>
+      <c r="H619" t="n">
+        <v>366.3900146484375</v>
+      </c>
+      <c r="I619" t="n">
+        <v>10.05000019073486</v>
+      </c>
+      <c r="J619" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K619" t="n">
+        <v>-0.477</v>
+      </c>
+      <c r="L619" t="inlineStr">
+        <is>
+          <t>Up</t>
+        </is>
+      </c>
+      <c r="M619" t="inlineStr">
+        <is>
+          <t>⚠️ Cautious Buy</t>
+        </is>
+      </c>
+      <c r="N619" t="n">
+        <v>49.33</v>
+      </c>
+      <c r="O619" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>Costco Wholesale Corporation</t>
+        </is>
+      </c>
+      <c r="E620" t="n">
+        <v>1001.16</v>
+      </c>
+      <c r="F620" t="n">
+        <v>915.61</v>
+      </c>
+      <c r="G620" t="n">
+        <v>-8.539999999999999</v>
+      </c>
+      <c r="H620" t="n">
+        <v>962.3200073242188</v>
+      </c>
+      <c r="I620" t="n">
+        <v>-3.880000114440918</v>
+      </c>
+      <c r="J620" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K620" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="L620" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M620" t="inlineStr">
+        <is>
+          <t>❌ Strong Avoid</t>
+        </is>
+      </c>
+      <c r="N620" t="n">
+        <v>24.18</v>
+      </c>
+      <c r="O620" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>NYSE</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc.</t>
+        </is>
+      </c>
+      <c r="E621" t="n">
+        <v>170.49</v>
+      </c>
+      <c r="F621" t="n">
+        <v>156.71</v>
+      </c>
+      <c r="G621" t="n">
+        <v>-8.08</v>
+      </c>
+      <c r="H621" t="n">
+        <v>169.2899932861328</v>
+      </c>
+      <c r="I621" t="n">
+        <v>-0.699999988079071</v>
+      </c>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K621" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L621" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="M621" t="inlineStr">
+        <is>
+          <t>⚠️ Speculative Buy</t>
+        </is>
+      </c>
+      <c r="N621" t="n">
+        <v>46.67</v>
+      </c>
+      <c r="O621" t="inlineStr">
+        <is>
+          <t>07 Feb 2026, 06:56:54 PM IST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>